<commit_message>
Updating the Sungrow model
</commit_message>
<xml_diff>
--- a/data_fetching/Entsoe/Actual_Production_Hydro_River.xlsx
+++ b/data_fetching/Entsoe/Actual_Production_Hydro_River.xlsx
@@ -394,799 +394,799 @@
     </row>
     <row r="2" spans="1:2">
       <c r="A2" s="2">
-        <v>46078</v>
+        <v>46093</v>
       </c>
       <c r="B2">
-        <v>1440</v>
+        <v>1280</v>
       </c>
     </row>
     <row r="3" spans="1:2">
       <c r="A3" s="2">
-        <v>46078.01041666666</v>
+        <v>46093.01041666666</v>
       </c>
       <c r="B3">
-        <v>1423</v>
+        <v>1237</v>
       </c>
     </row>
     <row r="4" spans="1:2">
       <c r="A4" s="2">
-        <v>46078.02083333334</v>
+        <v>46093.02083333334</v>
       </c>
       <c r="B4">
-        <v>1424</v>
+        <v>1238</v>
       </c>
     </row>
     <row r="5" spans="1:2">
       <c r="A5" s="2">
-        <v>46078.03125</v>
+        <v>46093.03125</v>
       </c>
       <c r="B5">
-        <v>1476</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6" spans="1:2">
       <c r="A6" s="2">
-        <v>46078.04166666666</v>
+        <v>46093.04166666666</v>
       </c>
       <c r="B6">
-        <v>1520</v>
+        <v>1231</v>
       </c>
     </row>
     <row r="7" spans="1:2">
       <c r="A7" s="2">
-        <v>46078.05208333334</v>
+        <v>46093.05208333334</v>
       </c>
       <c r="B7">
-        <v>1414</v>
+        <v>1228</v>
       </c>
     </row>
     <row r="8" spans="1:2">
       <c r="A8" s="2">
-        <v>46078.0625</v>
+        <v>46093.0625</v>
       </c>
       <c r="B8">
-        <v>1399</v>
+        <v>0</v>
       </c>
     </row>
     <row r="9" spans="1:2">
       <c r="A9" s="2">
-        <v>46078.07291666666</v>
+        <v>46093.07291666666</v>
       </c>
       <c r="B9">
-        <v>1364</v>
+        <v>1229</v>
       </c>
     </row>
     <row r="10" spans="1:2">
       <c r="A10" s="2">
-        <v>46078.08333333334</v>
+        <v>46093.08333333334</v>
       </c>
       <c r="B10">
-        <v>1387</v>
+        <v>1238</v>
       </c>
     </row>
     <row r="11" spans="1:2">
       <c r="A11" s="2">
-        <v>46078.09375</v>
+        <v>46093.09375</v>
       </c>
       <c r="B11">
-        <v>1379</v>
+        <v>1231</v>
       </c>
     </row>
     <row r="12" spans="1:2">
       <c r="A12" s="2">
-        <v>46078.10416666666</v>
+        <v>46093.10416666666</v>
       </c>
       <c r="B12">
-        <v>1381</v>
+        <v>0</v>
       </c>
     </row>
     <row r="13" spans="1:2">
       <c r="A13" s="2">
-        <v>46078.11458333334</v>
+        <v>46093.11458333334</v>
       </c>
       <c r="B13">
-        <v>1386</v>
+        <v>1229</v>
       </c>
     </row>
     <row r="14" spans="1:2">
       <c r="A14" s="2">
-        <v>46078.125</v>
+        <v>46093.125</v>
       </c>
       <c r="B14">
-        <v>1452</v>
+        <v>1237</v>
       </c>
     </row>
     <row r="15" spans="1:2">
       <c r="A15" s="2">
-        <v>46078.13541666666</v>
+        <v>46093.13541666666</v>
       </c>
       <c r="B15">
-        <v>1455</v>
+        <v>1246</v>
       </c>
     </row>
     <row r="16" spans="1:2">
       <c r="A16" s="2">
-        <v>46078.14583333334</v>
+        <v>46093.14583333334</v>
       </c>
       <c r="B16">
-        <v>0</v>
+        <v>1244</v>
       </c>
     </row>
     <row r="17" spans="1:2">
       <c r="A17" s="2">
-        <v>46078.15625</v>
+        <v>46093.15625</v>
       </c>
       <c r="B17">
-        <v>1454</v>
+        <v>1242</v>
       </c>
     </row>
     <row r="18" spans="1:2">
       <c r="A18" s="2">
-        <v>46078.16666666666</v>
+        <v>46093.16666666666</v>
       </c>
       <c r="B18">
-        <v>1497</v>
+        <v>1249</v>
       </c>
     </row>
     <row r="19" spans="1:2">
       <c r="A19" s="2">
-        <v>46078.17708333334</v>
+        <v>46093.17708333334</v>
       </c>
       <c r="B19">
-        <v>1500</v>
+        <v>1244</v>
       </c>
     </row>
     <row r="20" spans="1:2">
       <c r="A20" s="2">
-        <v>46078.1875</v>
+        <v>46093.1875</v>
       </c>
       <c r="B20">
-        <v>1502</v>
+        <v>1249</v>
       </c>
     </row>
     <row r="21" spans="1:2">
       <c r="A21" s="2">
-        <v>46078.19791666666</v>
+        <v>46093.19791666666</v>
       </c>
       <c r="B21">
-        <v>1510</v>
+        <v>1247</v>
       </c>
     </row>
     <row r="22" spans="1:2">
       <c r="A22" s="2">
-        <v>46078.20833333334</v>
+        <v>46093.20833333334</v>
       </c>
       <c r="B22">
-        <v>1557</v>
+        <v>1259</v>
       </c>
     </row>
     <row r="23" spans="1:2">
       <c r="A23" s="2">
-        <v>46078.21875</v>
+        <v>46093.21875</v>
       </c>
       <c r="B23">
-        <v>1619</v>
+        <v>1263</v>
       </c>
     </row>
     <row r="24" spans="1:2">
       <c r="A24" s="2">
-        <v>46078.22916666666</v>
+        <v>46093.22916666666</v>
       </c>
       <c r="B24">
-        <v>1584</v>
+        <v>1264</v>
       </c>
     </row>
     <row r="25" spans="1:2">
       <c r="A25" s="2">
-        <v>46078.23958333334</v>
+        <v>46093.23958333334</v>
       </c>
       <c r="B25">
-        <v>1585</v>
+        <v>1259</v>
       </c>
     </row>
     <row r="26" spans="1:2">
       <c r="A26" s="2">
-        <v>46078.25</v>
+        <v>46093.25</v>
       </c>
       <c r="B26">
-        <v>1658</v>
+        <v>1361</v>
       </c>
     </row>
     <row r="27" spans="1:2">
       <c r="A27" s="2">
-        <v>46078.26041666666</v>
+        <v>46093.26041666666</v>
       </c>
       <c r="B27">
-        <v>1690</v>
+        <v>1354</v>
       </c>
     </row>
     <row r="28" spans="1:2">
       <c r="A28" s="2">
-        <v>46078.27083333334</v>
+        <v>46093.27083333334</v>
       </c>
       <c r="B28">
-        <v>1692</v>
+        <v>0</v>
       </c>
     </row>
     <row r="29" spans="1:2">
       <c r="A29" s="2">
-        <v>46078.28125</v>
+        <v>46093.28125</v>
       </c>
       <c r="B29">
-        <v>1698</v>
+        <v>1355</v>
       </c>
     </row>
     <row r="30" spans="1:2">
       <c r="A30" s="2">
-        <v>46078.29166666666</v>
+        <v>46093.29166666666</v>
       </c>
       <c r="B30">
-        <v>1683</v>
+        <v>1342</v>
       </c>
     </row>
     <row r="31" spans="1:2">
       <c r="A31" s="2">
-        <v>46078.30208333334</v>
+        <v>46093.30208333334</v>
       </c>
       <c r="B31">
-        <v>1680</v>
+        <v>1329</v>
       </c>
     </row>
     <row r="32" spans="1:2">
       <c r="A32" s="2">
-        <v>46078.3125</v>
+        <v>46093.3125</v>
       </c>
       <c r="B32">
-        <v>1679</v>
+        <v>1327</v>
       </c>
     </row>
     <row r="33" spans="1:2">
       <c r="A33" s="2">
-        <v>46078.32291666666</v>
+        <v>46093.32291666666</v>
       </c>
       <c r="B33">
-        <v>1650</v>
+        <v>1328</v>
       </c>
     </row>
     <row r="34" spans="1:2">
       <c r="A34" s="2">
-        <v>46078.33333333334</v>
+        <v>46093.33333333334</v>
       </c>
       <c r="B34">
-        <v>1391</v>
+        <v>1351</v>
       </c>
     </row>
     <row r="35" spans="1:2">
       <c r="A35" s="2">
-        <v>46078.34375</v>
+        <v>46093.34375</v>
       </c>
       <c r="B35">
-        <v>1315</v>
+        <v>1349</v>
       </c>
     </row>
     <row r="36" spans="1:2">
       <c r="A36" s="2">
-        <v>46078.35416666666</v>
+        <v>46093.35416666666</v>
       </c>
       <c r="B36">
-        <v>1392</v>
+        <v>1348</v>
       </c>
     </row>
     <row r="37" spans="1:2">
       <c r="A37" s="2">
-        <v>46078.36458333334</v>
+        <v>46093.36458333334</v>
       </c>
       <c r="B37">
-        <v>1398</v>
+        <v>1337</v>
       </c>
     </row>
     <row r="38" spans="1:2">
       <c r="A38" s="2">
-        <v>46078.375</v>
+        <v>46093.375</v>
       </c>
       <c r="B38">
-        <v>984</v>
+        <v>1143</v>
       </c>
     </row>
     <row r="39" spans="1:2">
       <c r="A39" s="2">
-        <v>46078.38541666666</v>
+        <v>46093.38541666666</v>
       </c>
       <c r="B39">
-        <v>928</v>
+        <v>1144</v>
       </c>
     </row>
     <row r="40" spans="1:2">
       <c r="A40" s="2">
-        <v>46078.39583333334</v>
+        <v>46093.39583333334</v>
       </c>
       <c r="B40">
-        <v>932</v>
+        <v>1140</v>
       </c>
     </row>
     <row r="41" spans="1:2">
       <c r="A41" s="2">
-        <v>46078.40625</v>
+        <v>46093.40625</v>
       </c>
       <c r="B41">
-        <v>935</v>
+        <v>1143</v>
       </c>
     </row>
     <row r="42" spans="1:2">
       <c r="A42" s="2">
-        <v>46078.41666666666</v>
+        <v>46093.41666666666</v>
       </c>
       <c r="B42">
-        <v>902</v>
+        <v>1106</v>
       </c>
     </row>
     <row r="43" spans="1:2">
       <c r="A43" s="2">
-        <v>46078.42708333334</v>
+        <v>46093.42708333334</v>
       </c>
       <c r="B43">
-        <v>897</v>
+        <v>1098</v>
       </c>
     </row>
     <row r="44" spans="1:2">
       <c r="A44" s="2">
-        <v>46078.4375</v>
+        <v>46093.4375</v>
       </c>
       <c r="B44">
-        <v>898</v>
+        <v>1100</v>
       </c>
     </row>
     <row r="45" spans="1:2">
       <c r="A45" s="2">
-        <v>46078.44791666666</v>
+        <v>46093.44791666666</v>
       </c>
       <c r="B45">
-        <v>897</v>
+        <v>0</v>
       </c>
     </row>
     <row r="46" spans="1:2">
       <c r="A46" s="2">
-        <v>46078.45833333334</v>
+        <v>46093.45833333334</v>
       </c>
       <c r="B46">
-        <v>873</v>
+        <v>0</v>
       </c>
     </row>
     <row r="47" spans="1:2">
       <c r="A47" s="2">
-        <v>46078.46875</v>
+        <v>46093.46875</v>
       </c>
       <c r="B47">
-        <v>0</v>
+        <v>1099</v>
       </c>
     </row>
     <row r="48" spans="1:2">
       <c r="A48" s="2">
-        <v>46078.47916666666</v>
+        <v>46093.47916666666</v>
       </c>
       <c r="B48">
-        <v>971</v>
+        <v>1061</v>
       </c>
     </row>
     <row r="49" spans="1:2">
       <c r="A49" s="2">
-        <v>46078.48958333334</v>
+        <v>46093.48958333334</v>
       </c>
       <c r="B49">
-        <v>980</v>
+        <v>1082</v>
       </c>
     </row>
     <row r="50" spans="1:2">
       <c r="A50" s="2">
-        <v>46078.5</v>
+        <v>46093.5</v>
       </c>
       <c r="B50">
-        <v>1008</v>
+        <v>1119</v>
       </c>
     </row>
     <row r="51" spans="1:2">
       <c r="A51" s="2">
-        <v>46078.51041666666</v>
+        <v>46093.51041666666</v>
       </c>
       <c r="B51">
-        <v>1118</v>
+        <v>1133</v>
       </c>
     </row>
     <row r="52" spans="1:2">
       <c r="A52" s="2">
-        <v>46078.52083333334</v>
+        <v>46093.52083333334</v>
       </c>
       <c r="B52">
-        <v>1124</v>
+        <v>1131</v>
       </c>
     </row>
     <row r="53" spans="1:2">
       <c r="A53" s="2">
-        <v>46078.53125</v>
+        <v>46093.53125</v>
       </c>
       <c r="B53">
-        <v>1126</v>
+        <v>1120</v>
       </c>
     </row>
     <row r="54" spans="1:2">
       <c r="A54" s="2">
-        <v>46078.54166666666</v>
+        <v>46093.54166666666</v>
       </c>
       <c r="B54">
-        <v>1114</v>
+        <v>990</v>
       </c>
     </row>
     <row r="55" spans="1:2">
       <c r="A55" s="2">
-        <v>46078.55208333334</v>
+        <v>46093.55208333334</v>
       </c>
       <c r="B55">
-        <v>1113</v>
+        <v>867</v>
       </c>
     </row>
     <row r="56" spans="1:2">
       <c r="A56" s="2">
-        <v>46078.5625</v>
+        <v>46093.5625</v>
       </c>
       <c r="B56">
-        <v>1034</v>
+        <v>836</v>
       </c>
     </row>
     <row r="57" spans="1:2">
       <c r="A57" s="2">
-        <v>46078.57291666666</v>
+        <v>46093.57291666666</v>
       </c>
       <c r="B57">
-        <v>0</v>
+        <v>834</v>
       </c>
     </row>
     <row r="58" spans="1:2">
       <c r="A58" s="2">
-        <v>46078.58333333334</v>
+        <v>46093.58333333334</v>
       </c>
       <c r="B58">
-        <v>1201</v>
+        <v>887</v>
       </c>
     </row>
     <row r="59" spans="1:2">
       <c r="A59" s="2">
-        <v>46078.59375</v>
+        <v>46093.59375</v>
       </c>
       <c r="B59">
-        <v>1099</v>
+        <v>890</v>
       </c>
     </row>
     <row r="60" spans="1:2">
       <c r="A60" s="2">
-        <v>46078.60416666666</v>
+        <v>46093.60416666666</v>
       </c>
       <c r="B60">
-        <v>1095</v>
+        <v>889</v>
       </c>
     </row>
     <row r="61" spans="1:2">
       <c r="A61" s="2">
-        <v>46078.61458333334</v>
+        <v>46093.61458333334</v>
       </c>
       <c r="B61">
-        <v>1137</v>
+        <v>900</v>
       </c>
     </row>
     <row r="62" spans="1:2">
       <c r="A62" s="2">
-        <v>46078.625</v>
+        <v>46093.625</v>
       </c>
       <c r="B62">
-        <v>1614</v>
+        <v>1092</v>
       </c>
     </row>
     <row r="63" spans="1:2">
       <c r="A63" s="2">
-        <v>46078.63541666666</v>
+        <v>46093.63541666666</v>
       </c>
       <c r="B63">
-        <v>1654</v>
+        <v>1096</v>
       </c>
     </row>
     <row r="64" spans="1:2">
       <c r="A64" s="2">
-        <v>46078.64583333334</v>
+        <v>46093.64583333334</v>
       </c>
       <c r="B64">
-        <v>1635</v>
+        <v>1112</v>
       </c>
     </row>
     <row r="65" spans="1:2">
       <c r="A65" s="2">
-        <v>46078.65625</v>
+        <v>46093.65625</v>
       </c>
       <c r="B65">
-        <v>1633</v>
+        <v>1221</v>
       </c>
     </row>
     <row r="66" spans="1:2">
       <c r="A66" s="2">
-        <v>46078.66666666666</v>
+        <v>46093.66666666666</v>
       </c>
       <c r="B66">
-        <v>1754</v>
+        <v>1414</v>
       </c>
     </row>
     <row r="67" spans="1:2">
       <c r="A67" s="2">
-        <v>46078.67708333334</v>
+        <v>46093.67708333334</v>
       </c>
       <c r="B67">
-        <v>1770</v>
+        <v>1437</v>
       </c>
     </row>
     <row r="68" spans="1:2">
       <c r="A68" s="2">
-        <v>46078.6875</v>
+        <v>46093.6875</v>
       </c>
       <c r="B68">
-        <v>1769</v>
+        <v>1439</v>
       </c>
     </row>
     <row r="69" spans="1:2">
       <c r="A69" s="2">
-        <v>46078.69791666666</v>
+        <v>46093.69791666666</v>
       </c>
       <c r="B69">
-        <v>1766</v>
+        <v>1440</v>
       </c>
     </row>
     <row r="70" spans="1:2">
       <c r="A70" s="2">
-        <v>46078.70833333334</v>
+        <v>46093.70833333334</v>
       </c>
       <c r="B70">
-        <v>1774</v>
+        <v>1418</v>
       </c>
     </row>
     <row r="71" spans="1:2">
       <c r="A71" s="2">
-        <v>46078.71875</v>
+        <v>46093.71875</v>
       </c>
       <c r="B71">
-        <v>1779</v>
+        <v>1422</v>
       </c>
     </row>
     <row r="72" spans="1:2">
       <c r="A72" s="2">
-        <v>46078.72916666666</v>
+        <v>46093.72916666666</v>
       </c>
       <c r="B72">
-        <v>1776</v>
+        <v>1416</v>
       </c>
     </row>
     <row r="73" spans="1:2">
       <c r="A73" s="2">
-        <v>46078.73958333334</v>
+        <v>46093.73958333334</v>
       </c>
       <c r="B73">
-        <v>1765</v>
+        <v>0</v>
       </c>
     </row>
     <row r="74" spans="1:2">
       <c r="A74" s="2">
-        <v>46078.75</v>
+        <v>46093.75</v>
       </c>
       <c r="B74">
-        <v>1763</v>
+        <v>1441</v>
       </c>
     </row>
     <row r="75" spans="1:2">
       <c r="A75" s="2">
-        <v>46078.76041666666</v>
+        <v>46093.76041666666</v>
       </c>
       <c r="B75">
-        <v>1769</v>
+        <v>1447</v>
       </c>
     </row>
     <row r="76" spans="1:2">
       <c r="A76" s="2">
-        <v>46078.77083333334</v>
+        <v>46093.77083333334</v>
       </c>
       <c r="B76">
-        <v>1774</v>
+        <v>1443</v>
       </c>
     </row>
     <row r="77" spans="1:2">
       <c r="A77" s="2">
-        <v>46078.78125</v>
+        <v>46093.78125</v>
       </c>
       <c r="B77">
-        <v>1777</v>
+        <v>1442</v>
       </c>
     </row>
     <row r="78" spans="1:2">
       <c r="A78" s="2">
-        <v>46078.79166666666</v>
+        <v>46093.79166666666</v>
       </c>
       <c r="B78">
-        <v>1794</v>
+        <v>1400</v>
       </c>
     </row>
     <row r="79" spans="1:2">
       <c r="A79" s="2">
-        <v>46078.80208333334</v>
+        <v>46093.80208333334</v>
       </c>
       <c r="B79">
-        <v>1795</v>
+        <v>1387</v>
       </c>
     </row>
     <row r="80" spans="1:2">
       <c r="A80" s="2">
-        <v>46078.8125</v>
+        <v>46093.8125</v>
       </c>
       <c r="B80">
-        <v>1798</v>
+        <v>1385</v>
       </c>
     </row>
     <row r="81" spans="1:2">
       <c r="A81" s="2">
-        <v>46078.82291666666</v>
+        <v>46093.82291666666</v>
       </c>
       <c r="B81">
-        <v>1808</v>
+        <v>1387</v>
       </c>
     </row>
     <row r="82" spans="1:2">
       <c r="A82" s="2">
-        <v>46078.83333333334</v>
+        <v>46093.83333333334</v>
       </c>
       <c r="B82">
-        <v>1816</v>
+        <v>1357</v>
       </c>
     </row>
     <row r="83" spans="1:2">
       <c r="A83" s="2">
-        <v>46078.84375</v>
+        <v>46093.84375</v>
       </c>
       <c r="B83">
-        <v>1814</v>
+        <v>0</v>
       </c>
     </row>
     <row r="84" spans="1:2">
       <c r="A84" s="2">
-        <v>46078.85416666666</v>
+        <v>46093.85416666666</v>
       </c>
       <c r="B84">
-        <v>1816</v>
+        <v>1358</v>
       </c>
     </row>
     <row r="85" spans="1:2">
       <c r="A85" s="2">
-        <v>46078.86458333334</v>
+        <v>46093.86458333334</v>
       </c>
       <c r="B85">
-        <v>1809</v>
+        <v>1360</v>
       </c>
     </row>
     <row r="86" spans="1:2">
       <c r="A86" s="2">
-        <v>46078.875</v>
+        <v>46093.875</v>
       </c>
       <c r="B86">
-        <v>1892</v>
+        <v>1348</v>
       </c>
     </row>
     <row r="87" spans="1:2">
       <c r="A87" s="2">
-        <v>46078.88541666666</v>
+        <v>46093.88541666666</v>
       </c>
       <c r="B87">
-        <v>1896</v>
+        <v>1335</v>
       </c>
     </row>
     <row r="88" spans="1:2">
       <c r="A88" s="2">
-        <v>46078.89583333334</v>
+        <v>46093.89583333334</v>
       </c>
       <c r="B88">
-        <v>0</v>
+        <v>1338</v>
       </c>
     </row>
     <row r="89" spans="1:2">
       <c r="A89" s="2">
-        <v>46078.90625</v>
+        <v>46093.90625</v>
       </c>
       <c r="B89">
-        <v>1898</v>
+        <v>1336</v>
       </c>
     </row>
     <row r="90" spans="1:2">
       <c r="A90" s="2">
-        <v>46078.91666666666</v>
+        <v>46093.91666666666</v>
       </c>
       <c r="B90">
-        <v>1916</v>
+        <v>1389</v>
       </c>
     </row>
     <row r="91" spans="1:2">
       <c r="A91" s="2">
-        <v>46078.92708333334</v>
+        <v>46093.92708333334</v>
       </c>
       <c r="B91">
-        <v>1913</v>
+        <v>1360</v>
       </c>
     </row>
     <row r="92" spans="1:2">
       <c r="A92" s="2">
-        <v>46078.9375</v>
+        <v>46093.9375</v>
       </c>
       <c r="B92">
-        <v>1914</v>
+        <v>1357</v>
       </c>
     </row>
     <row r="93" spans="1:2">
       <c r="A93" s="2">
-        <v>46078.94791666666</v>
+        <v>46093.94791666666</v>
       </c>
       <c r="B93">
-        <v>0</v>
+        <v>1361</v>
       </c>
     </row>
     <row r="94" spans="1:2">
       <c r="A94" s="2">
-        <v>46078.95833333334</v>
+        <v>46093.95833333334</v>
       </c>
       <c r="B94">
-        <v>1556</v>
+        <v>1369</v>
       </c>
     </row>
     <row r="95" spans="1:2">
       <c r="A95" s="2">
-        <v>46078.96875</v>
+        <v>46093.96875</v>
       </c>
       <c r="B95">
-        <v>1511</v>
+        <v>1367</v>
       </c>
     </row>
     <row r="96" spans="1:2">
       <c r="A96" s="2">
-        <v>46078.97916666666</v>
+        <v>46093.97916666666</v>
       </c>
       <c r="B96">
-        <v>1459</v>
+        <v>1362</v>
       </c>
     </row>
     <row r="97" spans="1:2">
       <c r="A97" s="2">
-        <v>46078.98958333334</v>
+        <v>46093.98958333334</v>
       </c>
       <c r="B97">
-        <v>1507</v>
+        <v>1363</v>
       </c>
     </row>
     <row r="98" spans="1:2">
       <c r="A98" s="2">
-        <v>46079</v>
+        <v>46094</v>
       </c>
       <c r="B98">
-        <v>1878</v>
+        <v>1270</v>
       </c>
     </row>
     <row r="99" spans="1:2">
       <c r="A99" s="2">
-        <v>46079.01041666666</v>
+        <v>46094.01041666666</v>
       </c>
       <c r="B99">
-        <v>1906</v>
+        <v>1262</v>
       </c>
     </row>
     <row r="100" spans="1:2">
       <c r="A100" s="2">
-        <v>46079.02083333334</v>
+        <v>46094.02083333334</v>
       </c>
       <c r="B100">
-        <v>1905</v>
+        <v>0</v>
       </c>
     </row>
     <row r="101" spans="1:2">
       <c r="A101" s="2">
-        <v>46079.03125</v>
+        <v>46094.03125</v>
       </c>
       <c r="B101">
         <v>0</v>
@@ -1194,287 +1194,287 @@
     </row>
     <row r="102" spans="1:2">
       <c r="A102" s="2">
-        <v>46079.04166666666</v>
+        <v>46094.04166666666</v>
       </c>
       <c r="B102">
-        <v>1865</v>
+        <v>1173</v>
       </c>
     </row>
     <row r="103" spans="1:2">
       <c r="A103" s="2">
-        <v>46079.05208333334</v>
+        <v>46094.05208333334</v>
       </c>
       <c r="B103">
-        <v>1861</v>
+        <v>1163</v>
       </c>
     </row>
     <row r="104" spans="1:2">
       <c r="A104" s="2">
-        <v>46079.0625</v>
+        <v>46094.0625</v>
       </c>
       <c r="B104">
-        <v>1862</v>
+        <v>1161</v>
       </c>
     </row>
     <row r="105" spans="1:2">
       <c r="A105" s="2">
-        <v>46079.07291666666</v>
+        <v>46094.07291666666</v>
       </c>
       <c r="B105">
-        <v>1886</v>
+        <v>1162</v>
       </c>
     </row>
     <row r="106" spans="1:2">
       <c r="A106" s="2">
-        <v>46079.08333333334</v>
+        <v>46094.08333333334</v>
       </c>
       <c r="B106">
-        <v>1891</v>
+        <v>1113</v>
       </c>
     </row>
     <row r="107" spans="1:2">
       <c r="A107" s="2">
-        <v>46079.09375</v>
+        <v>46094.09375</v>
       </c>
       <c r="B107">
-        <v>1895</v>
+        <v>1112</v>
       </c>
     </row>
     <row r="108" spans="1:2">
       <c r="A108" s="2">
-        <v>46079.10416666666</v>
+        <v>46094.10416666666</v>
       </c>
       <c r="B108">
-        <v>1897</v>
+        <v>1110</v>
       </c>
     </row>
     <row r="109" spans="1:2">
       <c r="A109" s="2">
-        <v>46079.11458333334</v>
+        <v>46094.11458333334</v>
       </c>
       <c r="B109">
-        <v>1896</v>
+        <v>1111</v>
       </c>
     </row>
     <row r="110" spans="1:2">
       <c r="A110" s="2">
-        <v>46079.125</v>
+        <v>46094.125</v>
       </c>
       <c r="B110">
-        <v>1901</v>
+        <v>1108</v>
       </c>
     </row>
     <row r="111" spans="1:2">
       <c r="A111" s="2">
-        <v>46079.13541666666</v>
+        <v>46094.13541666666</v>
       </c>
       <c r="B111">
-        <v>1899</v>
+        <v>1109</v>
       </c>
     </row>
     <row r="112" spans="1:2">
       <c r="A112" s="2">
-        <v>46079.14583333334</v>
+        <v>46094.14583333334</v>
       </c>
       <c r="B112">
-        <v>1901</v>
+        <v>1108</v>
       </c>
     </row>
     <row r="113" spans="1:2">
       <c r="A113" s="2">
-        <v>46079.15625</v>
+        <v>46094.15625</v>
       </c>
       <c r="B113">
-        <v>1904</v>
+        <v>1126</v>
       </c>
     </row>
     <row r="114" spans="1:2">
       <c r="A114" s="2">
-        <v>46079.16666666666</v>
+        <v>46094.16666666666</v>
       </c>
       <c r="B114">
-        <v>1917</v>
+        <v>1257</v>
       </c>
     </row>
     <row r="115" spans="1:2">
       <c r="A115" s="2">
-        <v>46079.17708333334</v>
+        <v>46094.17708333334</v>
       </c>
       <c r="B115">
-        <v>1912</v>
+        <v>1261</v>
       </c>
     </row>
     <row r="116" spans="1:2">
       <c r="A116" s="2">
-        <v>46079.1875</v>
+        <v>46094.1875</v>
       </c>
       <c r="B116">
-        <v>1861</v>
+        <v>1262</v>
       </c>
     </row>
     <row r="117" spans="1:2">
       <c r="A117" s="2">
-        <v>46079.19791666666</v>
+        <v>46094.19791666666</v>
       </c>
       <c r="B117">
-        <v>1860</v>
+        <v>0</v>
       </c>
     </row>
     <row r="118" spans="1:2">
       <c r="A118" s="2">
-        <v>46079.20833333334</v>
+        <v>46094.20833333334</v>
       </c>
       <c r="B118">
-        <v>1899</v>
+        <v>1236</v>
       </c>
     </row>
     <row r="119" spans="1:2">
       <c r="A119" s="2">
-        <v>46079.21875</v>
+        <v>46094.21875</v>
       </c>
       <c r="B119">
-        <v>1895</v>
+        <v>1234</v>
       </c>
     </row>
     <row r="120" spans="1:2">
       <c r="A120" s="2">
-        <v>46079.22916666666</v>
+        <v>46094.22916666666</v>
       </c>
       <c r="B120">
-        <v>1888</v>
+        <v>0</v>
       </c>
     </row>
     <row r="121" spans="1:2">
       <c r="A121" s="2">
-        <v>46079.23958333334</v>
+        <v>46094.23958333334</v>
       </c>
       <c r="B121">
-        <v>1880</v>
+        <v>0</v>
       </c>
     </row>
     <row r="122" spans="1:2">
       <c r="A122" s="2">
-        <v>46079.25</v>
+        <v>46094.25</v>
       </c>
       <c r="B122">
-        <v>1867</v>
+        <v>1272</v>
       </c>
     </row>
     <row r="123" spans="1:2">
       <c r="A123" s="2">
-        <v>46079.26041666666</v>
+        <v>46094.26041666666</v>
       </c>
       <c r="B123">
-        <v>1872</v>
+        <v>1259</v>
       </c>
     </row>
     <row r="124" spans="1:2">
       <c r="A124" s="2">
-        <v>46079.27083333334</v>
+        <v>46094.27083333334</v>
       </c>
       <c r="B124">
-        <v>1893</v>
+        <v>1245</v>
       </c>
     </row>
     <row r="125" spans="1:2">
       <c r="A125" s="2">
-        <v>46079.28125</v>
+        <v>46094.28125</v>
       </c>
       <c r="B125">
-        <v>1879</v>
+        <v>1243</v>
       </c>
     </row>
     <row r="126" spans="1:2">
       <c r="A126" s="2">
-        <v>46079.29166666666</v>
+        <v>46094.29166666666</v>
       </c>
       <c r="B126">
-        <v>1823</v>
+        <v>1200</v>
       </c>
     </row>
     <row r="127" spans="1:2">
       <c r="A127" s="2">
-        <v>46079.30208333334</v>
+        <v>46094.30208333334</v>
       </c>
       <c r="B127">
-        <v>1849</v>
+        <v>0</v>
       </c>
     </row>
     <row r="128" spans="1:2">
       <c r="A128" s="2">
-        <v>46079.3125</v>
+        <v>46094.3125</v>
       </c>
       <c r="B128">
-        <v>1859</v>
+        <v>0</v>
       </c>
     </row>
     <row r="129" spans="1:2">
       <c r="A129" s="2">
-        <v>46079.32291666666</v>
+        <v>46094.32291666666</v>
       </c>
       <c r="B129">
-        <v>1833</v>
+        <v>0</v>
       </c>
     </row>
     <row r="130" spans="1:2">
       <c r="A130" s="2">
-        <v>46079.33333333334</v>
+        <v>46094.33333333334</v>
       </c>
       <c r="B130">
-        <v>1841</v>
+        <v>0</v>
       </c>
     </row>
     <row r="131" spans="1:2">
       <c r="A131" s="2">
-        <v>46079.34375</v>
+        <v>46094.34375</v>
       </c>
       <c r="B131">
-        <v>1833</v>
+        <v>0</v>
       </c>
     </row>
     <row r="132" spans="1:2">
       <c r="A132" s="2">
-        <v>46079.35416666666</v>
+        <v>46094.35416666666</v>
       </c>
       <c r="B132">
-        <v>1793</v>
+        <v>0</v>
       </c>
     </row>
     <row r="133" spans="1:2">
       <c r="A133" s="2">
-        <v>46079.36458333334</v>
+        <v>46094.36458333334</v>
       </c>
       <c r="B133">
-        <v>1784</v>
+        <v>0</v>
       </c>
     </row>
     <row r="134" spans="1:2">
       <c r="A134" s="2">
-        <v>46079.375</v>
+        <v>46094.375</v>
       </c>
       <c r="B134">
-        <v>1335</v>
+        <v>0</v>
       </c>
     </row>
     <row r="135" spans="1:2">
       <c r="A135" s="2">
-        <v>46079.38541666666</v>
+        <v>46094.38541666666</v>
       </c>
       <c r="B135">
-        <v>1267</v>
+        <v>0</v>
       </c>
     </row>
     <row r="136" spans="1:2">
       <c r="A136" s="2">
-        <v>46079.39583333334</v>
+        <v>46094.39583333334</v>
       </c>
       <c r="B136">
-        <v>1263</v>
+        <v>0</v>
       </c>
     </row>
     <row r="137" spans="1:2">
       <c r="A137" s="2">
-        <v>46079.40625</v>
+        <v>46094.40625</v>
       </c>
       <c r="B137">
         <v>0</v>
@@ -1482,7 +1482,7 @@
     </row>
     <row r="138" spans="1:2">
       <c r="A138" s="2">
-        <v>46079.41666666666</v>
+        <v>46094.41666666666</v>
       </c>
       <c r="B138">
         <v>0</v>
@@ -1490,7 +1490,7 @@
     </row>
     <row r="139" spans="1:2">
       <c r="A139" s="2">
-        <v>46079.42708333334</v>
+        <v>46094.42708333334</v>
       </c>
       <c r="B139">
         <v>0</v>
@@ -1498,7 +1498,7 @@
     </row>
     <row r="140" spans="1:2">
       <c r="A140" s="2">
-        <v>46079.4375</v>
+        <v>46094.4375</v>
       </c>
       <c r="B140">
         <v>0</v>
@@ -1506,7 +1506,7 @@
     </row>
     <row r="141" spans="1:2">
       <c r="A141" s="2">
-        <v>46079.44791666666</v>
+        <v>46094.44791666666</v>
       </c>
       <c r="B141">
         <v>0</v>
@@ -1514,7 +1514,7 @@
     </row>
     <row r="142" spans="1:2">
       <c r="A142" s="2">
-        <v>46079.45833333334</v>
+        <v>46094.45833333334</v>
       </c>
       <c r="B142">
         <v>0</v>
@@ -1522,7 +1522,7 @@
     </row>
     <row r="143" spans="1:2">
       <c r="A143" s="2">
-        <v>46079.46875</v>
+        <v>46094.46875</v>
       </c>
       <c r="B143">
         <v>0</v>
@@ -1530,7 +1530,7 @@
     </row>
     <row r="144" spans="1:2">
       <c r="A144" s="2">
-        <v>46079.47916666666</v>
+        <v>46094.47916666666</v>
       </c>
       <c r="B144">
         <v>0</v>
@@ -1538,7 +1538,7 @@
     </row>
     <row r="145" spans="1:2">
       <c r="A145" s="2">
-        <v>46079.48958333334</v>
+        <v>46094.48958333334</v>
       </c>
       <c r="B145">
         <v>0</v>
@@ -1546,7 +1546,7 @@
     </row>
     <row r="146" spans="1:2">
       <c r="A146" s="2">
-        <v>46079.5</v>
+        <v>46094.5</v>
       </c>
       <c r="B146">
         <v>0</v>
@@ -1554,7 +1554,7 @@
     </row>
     <row r="147" spans="1:2">
       <c r="A147" s="2">
-        <v>46079.51041666666</v>
+        <v>46094.51041666666</v>
       </c>
       <c r="B147">
         <v>0</v>
@@ -1562,7 +1562,7 @@
     </row>
     <row r="148" spans="1:2">
       <c r="A148" s="2">
-        <v>46079.52083333334</v>
+        <v>46094.52083333334</v>
       </c>
       <c r="B148">
         <v>0</v>
@@ -1570,7 +1570,7 @@
     </row>
     <row r="149" spans="1:2">
       <c r="A149" s="2">
-        <v>46079.53125</v>
+        <v>46094.53125</v>
       </c>
       <c r="B149">
         <v>0</v>
@@ -1578,7 +1578,7 @@
     </row>
     <row r="150" spans="1:2">
       <c r="A150" s="2">
-        <v>46079.54166666666</v>
+        <v>46094.54166666666</v>
       </c>
       <c r="B150">
         <v>0</v>
@@ -1586,7 +1586,7 @@
     </row>
     <row r="151" spans="1:2">
       <c r="A151" s="2">
-        <v>46079.55208333334</v>
+        <v>46094.55208333334</v>
       </c>
       <c r="B151">
         <v>0</v>
@@ -1594,7 +1594,7 @@
     </row>
     <row r="152" spans="1:2">
       <c r="A152" s="2">
-        <v>46079.5625</v>
+        <v>46094.5625</v>
       </c>
       <c r="B152">
         <v>0</v>
@@ -1602,7 +1602,7 @@
     </row>
     <row r="153" spans="1:2">
       <c r="A153" s="2">
-        <v>46079.57291666666</v>
+        <v>46094.57291666666</v>
       </c>
       <c r="B153">
         <v>0</v>
@@ -1610,7 +1610,7 @@
     </row>
     <row r="154" spans="1:2">
       <c r="A154" s="2">
-        <v>46079.58333333334</v>
+        <v>46094.58333333334</v>
       </c>
       <c r="B154">
         <v>0</v>
@@ -1618,7 +1618,7 @@
     </row>
     <row r="155" spans="1:2">
       <c r="A155" s="2">
-        <v>46079.59375</v>
+        <v>46094.59375</v>
       </c>
       <c r="B155">
         <v>0</v>
@@ -1626,7 +1626,7 @@
     </row>
     <row r="156" spans="1:2">
       <c r="A156" s="2">
-        <v>46079.60416666666</v>
+        <v>46094.60416666666</v>
       </c>
       <c r="B156">
         <v>0</v>
@@ -1634,7 +1634,7 @@
     </row>
     <row r="157" spans="1:2">
       <c r="A157" s="2">
-        <v>46079.61458333334</v>
+        <v>46094.61458333334</v>
       </c>
       <c r="B157">
         <v>0</v>
@@ -1642,7 +1642,7 @@
     </row>
     <row r="158" spans="1:2">
       <c r="A158" s="2">
-        <v>46079.625</v>
+        <v>46094.625</v>
       </c>
       <c r="B158">
         <v>0</v>
@@ -1650,7 +1650,7 @@
     </row>
     <row r="159" spans="1:2">
       <c r="A159" s="2">
-        <v>46079.63541666666</v>
+        <v>46094.63541666666</v>
       </c>
       <c r="B159">
         <v>0</v>
@@ -1658,7 +1658,7 @@
     </row>
     <row r="160" spans="1:2">
       <c r="A160" s="2">
-        <v>46079.64583333334</v>
+        <v>46094.64583333334</v>
       </c>
       <c r="B160">
         <v>0</v>
@@ -1666,7 +1666,7 @@
     </row>
     <row r="161" spans="1:2">
       <c r="A161" s="2">
-        <v>46079.65625</v>
+        <v>46094.65625</v>
       </c>
       <c r="B161">
         <v>0</v>
@@ -1674,7 +1674,7 @@
     </row>
     <row r="162" spans="1:2">
       <c r="A162" s="2">
-        <v>46079.66666666666</v>
+        <v>46094.66666666666</v>
       </c>
       <c r="B162">
         <v>0</v>
@@ -1682,7 +1682,7 @@
     </row>
     <row r="163" spans="1:2">
       <c r="A163" s="2">
-        <v>46079.67708333334</v>
+        <v>46094.67708333334</v>
       </c>
       <c r="B163">
         <v>0</v>
@@ -1690,7 +1690,7 @@
     </row>
     <row r="164" spans="1:2">
       <c r="A164" s="2">
-        <v>46079.6875</v>
+        <v>46094.6875</v>
       </c>
       <c r="B164">
         <v>0</v>
@@ -1698,7 +1698,7 @@
     </row>
     <row r="165" spans="1:2">
       <c r="A165" s="2">
-        <v>46079.69791666666</v>
+        <v>46094.69791666666</v>
       </c>
       <c r="B165">
         <v>0</v>
@@ -1706,7 +1706,7 @@
     </row>
     <row r="166" spans="1:2">
       <c r="A166" s="2">
-        <v>46079.70833333334</v>
+        <v>46094.70833333334</v>
       </c>
       <c r="B166">
         <v>0</v>
@@ -1714,7 +1714,7 @@
     </row>
     <row r="167" spans="1:2">
       <c r="A167" s="2">
-        <v>46079.71875</v>
+        <v>46094.71875</v>
       </c>
       <c r="B167">
         <v>0</v>
@@ -1722,7 +1722,7 @@
     </row>
     <row r="168" spans="1:2">
       <c r="A168" s="2">
-        <v>46079.72916666666</v>
+        <v>46094.72916666666</v>
       </c>
       <c r="B168">
         <v>0</v>
@@ -1730,7 +1730,7 @@
     </row>
     <row r="169" spans="1:2">
       <c r="A169" s="2">
-        <v>46079.73958333334</v>
+        <v>46094.73958333334</v>
       </c>
       <c r="B169">
         <v>0</v>
@@ -1738,7 +1738,7 @@
     </row>
     <row r="170" spans="1:2">
       <c r="A170" s="2">
-        <v>46079.75</v>
+        <v>46094.75</v>
       </c>
       <c r="B170">
         <v>0</v>
@@ -1746,7 +1746,7 @@
     </row>
     <row r="171" spans="1:2">
       <c r="A171" s="2">
-        <v>46079.76041666666</v>
+        <v>46094.76041666666</v>
       </c>
       <c r="B171">
         <v>0</v>
@@ -1754,7 +1754,7 @@
     </row>
     <row r="172" spans="1:2">
       <c r="A172" s="2">
-        <v>46079.77083333334</v>
+        <v>46094.77083333334</v>
       </c>
       <c r="B172">
         <v>0</v>
@@ -1762,7 +1762,7 @@
     </row>
     <row r="173" spans="1:2">
       <c r="A173" s="2">
-        <v>46079.78125</v>
+        <v>46094.78125</v>
       </c>
       <c r="B173">
         <v>0</v>
@@ -1770,7 +1770,7 @@
     </row>
     <row r="174" spans="1:2">
       <c r="A174" s="2">
-        <v>46079.79166666666</v>
+        <v>46094.79166666666</v>
       </c>
       <c r="B174">
         <v>0</v>
@@ -1778,7 +1778,7 @@
     </row>
     <row r="175" spans="1:2">
       <c r="A175" s="2">
-        <v>46079.80208333334</v>
+        <v>46094.80208333334</v>
       </c>
       <c r="B175">
         <v>0</v>
@@ -1786,7 +1786,7 @@
     </row>
     <row r="176" spans="1:2">
       <c r="A176" s="2">
-        <v>46079.8125</v>
+        <v>46094.8125</v>
       </c>
       <c r="B176">
         <v>0</v>
@@ -1794,7 +1794,7 @@
     </row>
     <row r="177" spans="1:2">
       <c r="A177" s="2">
-        <v>46079.82291666666</v>
+        <v>46094.82291666666</v>
       </c>
       <c r="B177">
         <v>0</v>
@@ -1802,7 +1802,7 @@
     </row>
     <row r="178" spans="1:2">
       <c r="A178" s="2">
-        <v>46079.83333333334</v>
+        <v>46094.83333333334</v>
       </c>
       <c r="B178">
         <v>0</v>
@@ -1810,7 +1810,7 @@
     </row>
     <row r="179" spans="1:2">
       <c r="A179" s="2">
-        <v>46079.84375</v>
+        <v>46094.84375</v>
       </c>
       <c r="B179">
         <v>0</v>
@@ -1818,7 +1818,7 @@
     </row>
     <row r="180" spans="1:2">
       <c r="A180" s="2">
-        <v>46079.85416666666</v>
+        <v>46094.85416666666</v>
       </c>
       <c r="B180">
         <v>0</v>
@@ -1826,7 +1826,7 @@
     </row>
     <row r="181" spans="1:2">
       <c r="A181" s="2">
-        <v>46079.86458333334</v>
+        <v>46094.86458333334</v>
       </c>
       <c r="B181">
         <v>0</v>
@@ -1834,7 +1834,7 @@
     </row>
     <row r="182" spans="1:2">
       <c r="A182" s="2">
-        <v>46079.875</v>
+        <v>46094.875</v>
       </c>
       <c r="B182">
         <v>0</v>
@@ -1842,7 +1842,7 @@
     </row>
     <row r="183" spans="1:2">
       <c r="A183" s="2">
-        <v>46079.88541666666</v>
+        <v>46094.88541666666</v>
       </c>
       <c r="B183">
         <v>0</v>
@@ -1850,7 +1850,7 @@
     </row>
     <row r="184" spans="1:2">
       <c r="A184" s="2">
-        <v>46079.89583333334</v>
+        <v>46094.89583333334</v>
       </c>
       <c r="B184">
         <v>0</v>
@@ -1858,7 +1858,7 @@
     </row>
     <row r="185" spans="1:2">
       <c r="A185" s="2">
-        <v>46079.90625</v>
+        <v>46094.90625</v>
       </c>
       <c r="B185">
         <v>0</v>
@@ -1866,7 +1866,7 @@
     </row>
     <row r="186" spans="1:2">
       <c r="A186" s="2">
-        <v>46079.91666666666</v>
+        <v>46094.91666666666</v>
       </c>
       <c r="B186">
         <v>0</v>
@@ -1874,7 +1874,7 @@
     </row>
     <row r="187" spans="1:2">
       <c r="A187" s="2">
-        <v>46079.92708333334</v>
+        <v>46094.92708333334</v>
       </c>
       <c r="B187">
         <v>0</v>
@@ -1882,7 +1882,7 @@
     </row>
     <row r="188" spans="1:2">
       <c r="A188" s="2">
-        <v>46079.9375</v>
+        <v>46094.9375</v>
       </c>
       <c r="B188">
         <v>0</v>
@@ -1890,7 +1890,7 @@
     </row>
     <row r="189" spans="1:2">
       <c r="A189" s="2">
-        <v>46079.94791666666</v>
+        <v>46094.94791666666</v>
       </c>
       <c r="B189">
         <v>0</v>
@@ -1898,7 +1898,7 @@
     </row>
     <row r="190" spans="1:2">
       <c r="A190" s="2">
-        <v>46079.95833333334</v>
+        <v>46094.95833333334</v>
       </c>
       <c r="B190">
         <v>0</v>
@@ -1906,7 +1906,7 @@
     </row>
     <row r="191" spans="1:2">
       <c r="A191" s="2">
-        <v>46079.96875</v>
+        <v>46094.96875</v>
       </c>
       <c r="B191">
         <v>0</v>
@@ -1914,7 +1914,7 @@
     </row>
     <row r="192" spans="1:2">
       <c r="A192" s="2">
-        <v>46079.97916666666</v>
+        <v>46094.97916666666</v>
       </c>
       <c r="B192">
         <v>0</v>
@@ -1922,7 +1922,7 @@
     </row>
     <row r="193" spans="1:2">
       <c r="A193" s="2">
-        <v>46079.98958333334</v>
+        <v>46094.98958333334</v>
       </c>
       <c r="B193">
         <v>0</v>

</xml_diff>

<commit_message>
Retraining the models for Rosiori and MM&MV
</commit_message>
<xml_diff>
--- a/data_fetching/Entsoe/Actual_Production_Hydro_River.xlsx
+++ b/data_fetching/Entsoe/Actual_Production_Hydro_River.xlsx
@@ -394,55 +394,55 @@
     </row>
     <row r="2" spans="1:2">
       <c r="A2" s="2">
-        <v>46121</v>
+        <v>46128</v>
       </c>
       <c r="B2">
-        <v>1765</v>
+        <v>1352</v>
       </c>
     </row>
     <row r="3" spans="1:2">
       <c r="A3" s="2">
-        <v>46121.01041666666</v>
+        <v>46128.01041666666</v>
       </c>
       <c r="B3">
-        <v>1752</v>
+        <v>1356</v>
       </c>
     </row>
     <row r="4" spans="1:2">
       <c r="A4" s="2">
-        <v>46121.02083333334</v>
+        <v>46128.02083333334</v>
       </c>
       <c r="B4">
-        <v>1736</v>
+        <v>1351</v>
       </c>
     </row>
     <row r="5" spans="1:2">
       <c r="A5" s="2">
-        <v>46121.03125</v>
+        <v>46128.03125</v>
       </c>
       <c r="B5">
-        <v>1732</v>
+        <v>1353</v>
       </c>
     </row>
     <row r="6" spans="1:2">
       <c r="A6" s="2">
-        <v>46121.04166666666</v>
+        <v>46128.04166666666</v>
       </c>
       <c r="B6">
-        <v>1758</v>
+        <v>1330</v>
       </c>
     </row>
     <row r="7" spans="1:2">
       <c r="A7" s="2">
-        <v>46121.05208333334</v>
+        <v>46128.05208333334</v>
       </c>
       <c r="B7">
-        <v>1757</v>
+        <v>1331</v>
       </c>
     </row>
     <row r="8" spans="1:2">
       <c r="A8" s="2">
-        <v>46121.0625</v>
+        <v>46128.0625</v>
       </c>
       <c r="B8">
         <v>0</v>
@@ -450,1087 +450,1087 @@
     </row>
     <row r="9" spans="1:2">
       <c r="A9" s="2">
-        <v>46121.07291666666</v>
+        <v>46128.07291666666</v>
       </c>
       <c r="B9">
-        <v>1758</v>
+        <v>1332</v>
       </c>
     </row>
     <row r="10" spans="1:2">
       <c r="A10" s="2">
-        <v>46121.08333333334</v>
+        <v>46128.08333333334</v>
       </c>
       <c r="B10">
-        <v>1718</v>
+        <v>1331</v>
       </c>
     </row>
     <row r="11" spans="1:2">
       <c r="A11" s="2">
-        <v>46121.09375</v>
+        <v>46128.09375</v>
       </c>
       <c r="B11">
-        <v>1695</v>
+        <v>1329</v>
       </c>
     </row>
     <row r="12" spans="1:2">
       <c r="A12" s="2">
-        <v>46121.10416666666</v>
+        <v>46128.10416666666</v>
       </c>
       <c r="B12">
-        <v>1667</v>
+        <v>0</v>
       </c>
     </row>
     <row r="13" spans="1:2">
       <c r="A13" s="2">
-        <v>46121.11458333334</v>
+        <v>46128.11458333334</v>
       </c>
       <c r="B13">
-        <v>1738</v>
+        <v>1327</v>
       </c>
     </row>
     <row r="14" spans="1:2">
       <c r="A14" s="2">
-        <v>46121.125</v>
+        <v>46128.125</v>
       </c>
       <c r="B14">
-        <v>1760</v>
+        <v>1334</v>
       </c>
     </row>
     <row r="15" spans="1:2">
       <c r="A15" s="2">
-        <v>46121.13541666666</v>
+        <v>46128.13541666666</v>
       </c>
       <c r="B15">
-        <v>1759</v>
+        <v>0</v>
       </c>
     </row>
     <row r="16" spans="1:2">
       <c r="A16" s="2">
-        <v>46121.14583333334</v>
+        <v>46128.14583333334</v>
       </c>
       <c r="B16">
-        <v>1758</v>
+        <v>0</v>
       </c>
     </row>
     <row r="17" spans="1:2">
       <c r="A17" s="2">
-        <v>46121.15625</v>
+        <v>46128.15625</v>
       </c>
       <c r="B17">
-        <v>0</v>
+        <v>1333</v>
       </c>
     </row>
     <row r="18" spans="1:2">
       <c r="A18" s="2">
-        <v>46121.16666666666</v>
+        <v>46128.16666666666</v>
       </c>
       <c r="B18">
-        <v>1760</v>
+        <v>1336</v>
       </c>
     </row>
     <row r="19" spans="1:2">
       <c r="A19" s="2">
-        <v>46121.17708333334</v>
+        <v>46128.17708333334</v>
       </c>
       <c r="B19">
-        <v>1758</v>
+        <v>1337</v>
       </c>
     </row>
     <row r="20" spans="1:2">
       <c r="A20" s="2">
-        <v>46121.1875</v>
+        <v>46128.1875</v>
       </c>
       <c r="B20">
-        <v>1763</v>
+        <v>0</v>
       </c>
     </row>
     <row r="21" spans="1:2">
       <c r="A21" s="2">
-        <v>46121.19791666666</v>
+        <v>46128.19791666666</v>
       </c>
       <c r="B21">
-        <v>1762</v>
+        <v>1336</v>
       </c>
     </row>
     <row r="22" spans="1:2">
       <c r="A22" s="2">
-        <v>46121.20833333334</v>
+        <v>46128.20833333334</v>
       </c>
       <c r="B22">
-        <v>1758</v>
+        <v>1374</v>
       </c>
     </row>
     <row r="23" spans="1:2">
       <c r="A23" s="2">
-        <v>46121.21875</v>
+        <v>46128.21875</v>
       </c>
       <c r="B23">
-        <v>1756</v>
+        <v>1373</v>
       </c>
     </row>
     <row r="24" spans="1:2">
       <c r="A24" s="2">
-        <v>46121.22916666666</v>
+        <v>46128.22916666666</v>
       </c>
       <c r="B24">
-        <v>1743</v>
+        <v>1375</v>
       </c>
     </row>
     <row r="25" spans="1:2">
       <c r="A25" s="2">
-        <v>46121.23958333334</v>
+        <v>46128.23958333334</v>
       </c>
       <c r="B25">
-        <v>1768</v>
+        <v>1374</v>
       </c>
     </row>
     <row r="26" spans="1:2">
       <c r="A26" s="2">
-        <v>46121.25</v>
+        <v>46128.25</v>
       </c>
       <c r="B26">
-        <v>1773</v>
+        <v>1376</v>
       </c>
     </row>
     <row r="27" spans="1:2">
       <c r="A27" s="2">
-        <v>46121.26041666666</v>
+        <v>46128.26041666666</v>
       </c>
       <c r="B27">
-        <v>1767</v>
+        <v>1370</v>
       </c>
     </row>
     <row r="28" spans="1:2">
       <c r="A28" s="2">
-        <v>46121.27083333334</v>
+        <v>46128.27083333334</v>
       </c>
       <c r="B28">
-        <v>1766</v>
+        <v>1367</v>
       </c>
     </row>
     <row r="29" spans="1:2">
       <c r="A29" s="2">
-        <v>46121.28125</v>
+        <v>46128.28125</v>
       </c>
       <c r="B29">
-        <v>1767</v>
+        <v>1369</v>
       </c>
     </row>
     <row r="30" spans="1:2">
       <c r="A30" s="2">
-        <v>46121.29166666666</v>
+        <v>46128.29166666666</v>
       </c>
       <c r="B30">
-        <v>1772</v>
+        <v>1370</v>
       </c>
     </row>
     <row r="31" spans="1:2">
       <c r="A31" s="2">
-        <v>46121.30208333334</v>
+        <v>46128.30208333334</v>
       </c>
       <c r="B31">
-        <v>1761</v>
+        <v>1365</v>
       </c>
     </row>
     <row r="32" spans="1:2">
       <c r="A32" s="2">
-        <v>46121.3125</v>
+        <v>46128.3125</v>
       </c>
       <c r="B32">
-        <v>1759</v>
+        <v>1302</v>
       </c>
     </row>
     <row r="33" spans="1:2">
       <c r="A33" s="2">
-        <v>46121.32291666666</v>
+        <v>46128.32291666666</v>
       </c>
       <c r="B33">
-        <v>0</v>
+        <v>1305</v>
       </c>
     </row>
     <row r="34" spans="1:2">
       <c r="A34" s="2">
-        <v>46121.33333333334</v>
+        <v>46128.33333333334</v>
       </c>
       <c r="B34">
-        <v>1757</v>
+        <v>1238</v>
       </c>
     </row>
     <row r="35" spans="1:2">
       <c r="A35" s="2">
-        <v>46121.34375</v>
+        <v>46128.34375</v>
       </c>
       <c r="B35">
-        <v>1715</v>
+        <v>1235</v>
       </c>
     </row>
     <row r="36" spans="1:2">
       <c r="A36" s="2">
-        <v>46121.35416666666</v>
+        <v>46128.35416666666</v>
       </c>
       <c r="B36">
-        <v>1709</v>
+        <v>1238</v>
       </c>
     </row>
     <row r="37" spans="1:2">
       <c r="A37" s="2">
-        <v>46121.36458333334</v>
+        <v>46128.36458333334</v>
       </c>
       <c r="B37">
-        <v>1704</v>
+        <v>1237</v>
       </c>
     </row>
     <row r="38" spans="1:2">
       <c r="A38" s="2">
-        <v>46121.375</v>
+        <v>46128.375</v>
       </c>
       <c r="B38">
-        <v>1478</v>
+        <v>1150</v>
       </c>
     </row>
     <row r="39" spans="1:2">
       <c r="A39" s="2">
-        <v>46121.38541666666</v>
+        <v>46128.38541666666</v>
       </c>
       <c r="B39">
-        <v>1397</v>
+        <v>1130</v>
       </c>
     </row>
     <row r="40" spans="1:2">
       <c r="A40" s="2">
-        <v>46121.39583333334</v>
+        <v>46128.39583333334</v>
       </c>
       <c r="B40">
-        <v>0</v>
+        <v>1127</v>
       </c>
     </row>
     <row r="41" spans="1:2">
       <c r="A41" s="2">
-        <v>46121.40625</v>
+        <v>46128.40625</v>
       </c>
       <c r="B41">
-        <v>1411</v>
+        <v>1126</v>
       </c>
     </row>
     <row r="42" spans="1:2">
       <c r="A42" s="2">
-        <v>46121.41666666666</v>
+        <v>46128.41666666666</v>
       </c>
       <c r="B42">
-        <v>1271</v>
+        <v>1044</v>
       </c>
     </row>
     <row r="43" spans="1:2">
       <c r="A43" s="2">
-        <v>46121.42708333334</v>
+        <v>46128.42708333334</v>
       </c>
       <c r="B43">
-        <v>1261</v>
+        <v>1001</v>
       </c>
     </row>
     <row r="44" spans="1:2">
       <c r="A44" s="2">
-        <v>46121.4375</v>
+        <v>46128.4375</v>
       </c>
       <c r="B44">
-        <v>1396</v>
+        <v>995</v>
       </c>
     </row>
     <row r="45" spans="1:2">
       <c r="A45" s="2">
-        <v>46121.44791666666</v>
+        <v>46128.44791666666</v>
       </c>
       <c r="B45">
-        <v>1413</v>
+        <v>994</v>
       </c>
     </row>
     <row r="46" spans="1:2">
       <c r="A46" s="2">
-        <v>46121.45833333334</v>
+        <v>46128.45833333334</v>
       </c>
       <c r="B46">
-        <v>1272</v>
+        <v>960</v>
       </c>
     </row>
     <row r="47" spans="1:2">
       <c r="A47" s="2">
-        <v>46121.46875</v>
+        <v>46128.46875</v>
       </c>
       <c r="B47">
-        <v>1260</v>
+        <v>941</v>
       </c>
     </row>
     <row r="48" spans="1:2">
       <c r="A48" s="2">
-        <v>46121.47916666666</v>
+        <v>46128.47916666666</v>
       </c>
       <c r="B48">
-        <v>0</v>
+        <v>856</v>
       </c>
     </row>
     <row r="49" spans="1:2">
       <c r="A49" s="2">
-        <v>46121.48958333334</v>
+        <v>46128.48958333334</v>
       </c>
       <c r="B49">
-        <v>1251</v>
+        <v>848</v>
       </c>
     </row>
     <row r="50" spans="1:2">
       <c r="A50" s="2">
-        <v>46121.5</v>
+        <v>46128.5</v>
       </c>
       <c r="B50">
-        <v>1295</v>
+        <v>866</v>
       </c>
     </row>
     <row r="51" spans="1:2">
       <c r="A51" s="2">
-        <v>46121.51041666666</v>
+        <v>46128.51041666666</v>
       </c>
       <c r="B51">
-        <v>1293</v>
+        <v>876</v>
       </c>
     </row>
     <row r="52" spans="1:2">
       <c r="A52" s="2">
-        <v>46121.52083333334</v>
+        <v>46128.52083333334</v>
       </c>
       <c r="B52">
-        <v>1266</v>
+        <v>1015</v>
       </c>
     </row>
     <row r="53" spans="1:2">
       <c r="A53" s="2">
-        <v>46121.53125</v>
+        <v>46128.53125</v>
       </c>
       <c r="B53">
-        <v>1293</v>
+        <v>977</v>
       </c>
     </row>
     <row r="54" spans="1:2">
       <c r="A54" s="2">
-        <v>46121.54166666666</v>
+        <v>46128.54166666666</v>
       </c>
       <c r="B54">
-        <v>1292</v>
+        <v>979</v>
       </c>
     </row>
     <row r="55" spans="1:2">
       <c r="A55" s="2">
-        <v>46121.55208333334</v>
+        <v>46128.55208333334</v>
       </c>
       <c r="B55">
-        <v>1285</v>
+        <v>1003</v>
       </c>
     </row>
     <row r="56" spans="1:2">
       <c r="A56" s="2">
-        <v>46121.5625</v>
+        <v>46128.5625</v>
       </c>
       <c r="B56">
-        <v>1302</v>
+        <v>1002</v>
       </c>
     </row>
     <row r="57" spans="1:2">
       <c r="A57" s="2">
-        <v>46121.57291666666</v>
+        <v>46128.57291666666</v>
       </c>
       <c r="B57">
-        <v>1139</v>
+        <v>1004</v>
       </c>
     </row>
     <row r="58" spans="1:2">
       <c r="A58" s="2">
-        <v>46121.58333333334</v>
+        <v>46128.58333333334</v>
       </c>
       <c r="B58">
-        <v>971</v>
+        <v>989</v>
       </c>
     </row>
     <row r="59" spans="1:2">
       <c r="A59" s="2">
-        <v>46121.59375</v>
+        <v>46128.59375</v>
       </c>
       <c r="B59">
-        <v>994</v>
+        <v>985</v>
       </c>
     </row>
     <row r="60" spans="1:2">
       <c r="A60" s="2">
-        <v>46121.60416666666</v>
+        <v>46128.60416666666</v>
       </c>
       <c r="B60">
-        <v>1209</v>
+        <v>982</v>
       </c>
     </row>
     <row r="61" spans="1:2">
       <c r="A61" s="2">
-        <v>46121.61458333334</v>
+        <v>46128.61458333334</v>
       </c>
       <c r="B61">
-        <v>1222</v>
+        <v>1040</v>
       </c>
     </row>
     <row r="62" spans="1:2">
       <c r="A62" s="2">
-        <v>46121.625</v>
+        <v>46128.625</v>
       </c>
       <c r="B62">
-        <v>1313</v>
+        <v>1083</v>
       </c>
     </row>
     <row r="63" spans="1:2">
       <c r="A63" s="2">
-        <v>46121.63541666666</v>
+        <v>46128.63541666666</v>
       </c>
       <c r="B63">
-        <v>1322</v>
+        <v>1090</v>
       </c>
     </row>
     <row r="64" spans="1:2">
       <c r="A64" s="2">
-        <v>46121.64583333334</v>
+        <v>46128.64583333334</v>
       </c>
       <c r="B64">
-        <v>1366</v>
+        <v>0</v>
       </c>
     </row>
     <row r="65" spans="1:2">
       <c r="A65" s="2">
-        <v>46121.65625</v>
+        <v>46128.65625</v>
       </c>
       <c r="B65">
-        <v>1368</v>
+        <v>1091</v>
       </c>
     </row>
     <row r="66" spans="1:2">
       <c r="A66" s="2">
-        <v>46121.66666666666</v>
+        <v>46128.66666666666</v>
       </c>
       <c r="B66">
-        <v>1358</v>
+        <v>1108</v>
       </c>
     </row>
     <row r="67" spans="1:2">
       <c r="A67" s="2">
-        <v>46121.67708333334</v>
+        <v>46128.67708333334</v>
       </c>
       <c r="B67">
-        <v>1417</v>
+        <v>1112</v>
       </c>
     </row>
     <row r="68" spans="1:2">
       <c r="A68" s="2">
-        <v>46121.6875</v>
+        <v>46128.6875</v>
       </c>
       <c r="B68">
-        <v>1440</v>
+        <v>0</v>
       </c>
     </row>
     <row r="69" spans="1:2">
       <c r="A69" s="2">
-        <v>46121.69791666666</v>
+        <v>46128.69791666666</v>
       </c>
       <c r="B69">
-        <v>1451</v>
+        <v>1122</v>
       </c>
     </row>
     <row r="70" spans="1:2">
       <c r="A70" s="2">
-        <v>46121.70833333334</v>
+        <v>46128.70833333334</v>
       </c>
       <c r="B70">
-        <v>1754</v>
+        <v>1396</v>
       </c>
     </row>
     <row r="71" spans="1:2">
       <c r="A71" s="2">
-        <v>46121.71875</v>
+        <v>46128.71875</v>
       </c>
       <c r="B71">
-        <v>1786</v>
+        <v>1420</v>
       </c>
     </row>
     <row r="72" spans="1:2">
       <c r="A72" s="2">
-        <v>46121.72916666666</v>
+        <v>46128.72916666666</v>
       </c>
       <c r="B72">
-        <v>1818</v>
+        <v>1425</v>
       </c>
     </row>
     <row r="73" spans="1:2">
       <c r="A73" s="2">
-        <v>46121.73958333334</v>
+        <v>46128.73958333334</v>
       </c>
       <c r="B73">
-        <v>1811</v>
+        <v>1423</v>
       </c>
     </row>
     <row r="74" spans="1:2">
       <c r="A74" s="2">
-        <v>46121.75</v>
+        <v>46128.75</v>
       </c>
       <c r="B74">
-        <v>1784</v>
+        <v>1444</v>
       </c>
     </row>
     <row r="75" spans="1:2">
       <c r="A75" s="2">
-        <v>46121.76041666666</v>
+        <v>46128.76041666666</v>
       </c>
       <c r="B75">
-        <v>1803</v>
+        <v>1450</v>
       </c>
     </row>
     <row r="76" spans="1:2">
       <c r="A76" s="2">
-        <v>46121.77083333334</v>
+        <v>46128.77083333334</v>
       </c>
       <c r="B76">
-        <v>1797</v>
+        <v>1440</v>
       </c>
     </row>
     <row r="77" spans="1:2">
       <c r="A77" s="2">
-        <v>46121.78125</v>
+        <v>46128.78125</v>
       </c>
       <c r="B77">
-        <v>1790</v>
+        <v>1435</v>
       </c>
     </row>
     <row r="78" spans="1:2">
       <c r="A78" s="2">
-        <v>46121.79166666666</v>
+        <v>46128.79166666666</v>
       </c>
       <c r="B78">
-        <v>1829</v>
+        <v>1450</v>
       </c>
     </row>
     <row r="79" spans="1:2">
       <c r="A79" s="2">
-        <v>46121.80208333334</v>
+        <v>46128.80208333334</v>
       </c>
       <c r="B79">
-        <v>1836</v>
+        <v>1455</v>
       </c>
     </row>
     <row r="80" spans="1:2">
       <c r="A80" s="2">
-        <v>46121.8125</v>
+        <v>46128.8125</v>
       </c>
       <c r="B80">
-        <v>1828</v>
+        <v>1453</v>
       </c>
     </row>
     <row r="81" spans="1:2">
       <c r="A81" s="2">
-        <v>46121.82291666666</v>
+        <v>46128.82291666666</v>
       </c>
       <c r="B81">
-        <v>1834</v>
+        <v>0</v>
       </c>
     </row>
     <row r="82" spans="1:2">
       <c r="A82" s="2">
-        <v>46121.83333333334</v>
+        <v>46128.83333333334</v>
       </c>
       <c r="B82">
-        <v>1831</v>
+        <v>1454</v>
       </c>
     </row>
     <row r="83" spans="1:2">
       <c r="A83" s="2">
-        <v>46121.84375</v>
+        <v>46128.84375</v>
       </c>
       <c r="B83">
-        <v>1830</v>
+        <v>1455</v>
       </c>
     </row>
     <row r="84" spans="1:2">
       <c r="A84" s="2">
-        <v>46121.85416666666</v>
+        <v>46128.85416666666</v>
       </c>
       <c r="B84">
-        <v>1831</v>
+        <v>1454</v>
       </c>
     </row>
     <row r="85" spans="1:2">
       <c r="A85" s="2">
-        <v>46121.86458333334</v>
+        <v>46128.86458333334</v>
       </c>
       <c r="B85">
-        <v>1827</v>
+        <v>1456</v>
       </c>
     </row>
     <row r="86" spans="1:2">
       <c r="A86" s="2">
-        <v>46121.875</v>
+        <v>46128.875</v>
       </c>
       <c r="B86">
-        <v>1865</v>
+        <v>1416</v>
       </c>
     </row>
     <row r="87" spans="1:2">
       <c r="A87" s="2">
-        <v>46121.88541666666</v>
+        <v>46128.88541666666</v>
       </c>
       <c r="B87">
-        <v>1861</v>
+        <v>1414</v>
       </c>
     </row>
     <row r="88" spans="1:2">
       <c r="A88" s="2">
-        <v>46121.89583333334</v>
+        <v>46128.89583333334</v>
       </c>
       <c r="B88">
-        <v>1857</v>
+        <v>1412</v>
       </c>
     </row>
     <row r="89" spans="1:2">
       <c r="A89" s="2">
-        <v>46121.90625</v>
+        <v>46128.90625</v>
       </c>
       <c r="B89">
-        <v>1856</v>
+        <v>1405</v>
       </c>
     </row>
     <row r="90" spans="1:2">
       <c r="A90" s="2">
-        <v>46121.91666666666</v>
+        <v>46128.91666666666</v>
       </c>
       <c r="B90">
-        <v>1877</v>
+        <v>1414</v>
       </c>
     </row>
     <row r="91" spans="1:2">
       <c r="A91" s="2">
-        <v>46121.92708333334</v>
+        <v>46128.92708333334</v>
       </c>
       <c r="B91">
-        <v>1865</v>
+        <v>1415</v>
       </c>
     </row>
     <row r="92" spans="1:2">
       <c r="A92" s="2">
-        <v>46121.9375</v>
+        <v>46128.9375</v>
       </c>
       <c r="B92">
-        <v>1869</v>
+        <v>1414</v>
       </c>
     </row>
     <row r="93" spans="1:2">
       <c r="A93" s="2">
-        <v>46121.94791666666</v>
+        <v>46128.94791666666</v>
       </c>
       <c r="B93">
-        <v>1867</v>
+        <v>1413</v>
       </c>
     </row>
     <row r="94" spans="1:2">
       <c r="A94" s="2">
-        <v>46121.95833333334</v>
+        <v>46128.95833333334</v>
       </c>
       <c r="B94">
-        <v>1828</v>
+        <v>1410</v>
       </c>
     </row>
     <row r="95" spans="1:2">
       <c r="A95" s="2">
-        <v>46121.96875</v>
+        <v>46128.96875</v>
       </c>
       <c r="B95">
-        <v>1818</v>
+        <v>0</v>
       </c>
     </row>
     <row r="96" spans="1:2">
       <c r="A96" s="2">
-        <v>46121.97916666666</v>
+        <v>46128.97916666666</v>
       </c>
       <c r="B96">
-        <v>0</v>
+        <v>1411</v>
       </c>
     </row>
     <row r="97" spans="1:2">
       <c r="A97" s="2">
-        <v>46121.98958333334</v>
+        <v>46128.98958333334</v>
       </c>
       <c r="B97">
-        <v>1814</v>
+        <v>1409</v>
       </c>
     </row>
     <row r="98" spans="1:2">
       <c r="A98" s="2">
-        <v>46122</v>
+        <v>46129</v>
       </c>
       <c r="B98">
-        <v>1647</v>
+        <v>1296</v>
       </c>
     </row>
     <row r="99" spans="1:2">
       <c r="A99" s="2">
-        <v>46122.01041666666</v>
+        <v>46129.01041666666</v>
       </c>
       <c r="B99">
-        <v>1595</v>
+        <v>1292</v>
       </c>
     </row>
     <row r="100" spans="1:2">
       <c r="A100" s="2">
-        <v>46122.02083333334</v>
+        <v>46129.02083333334</v>
       </c>
       <c r="B100">
-        <v>0</v>
+        <v>1289</v>
       </c>
     </row>
     <row r="101" spans="1:2">
       <c r="A101" s="2">
-        <v>46122.03125</v>
+        <v>46129.03125</v>
       </c>
       <c r="B101">
-        <v>1594</v>
+        <v>1291</v>
       </c>
     </row>
     <row r="102" spans="1:2">
       <c r="A102" s="2">
-        <v>46122.04166666666</v>
+        <v>46129.04166666666</v>
       </c>
       <c r="B102">
-        <v>1598</v>
+        <v>1227</v>
       </c>
     </row>
     <row r="103" spans="1:2">
       <c r="A103" s="2">
-        <v>46122.05208333334</v>
+        <v>46129.05208333334</v>
       </c>
       <c r="B103">
-        <v>0</v>
+        <v>1222</v>
       </c>
     </row>
     <row r="104" spans="1:2">
       <c r="A104" s="2">
-        <v>46122.0625</v>
+        <v>46129.0625</v>
       </c>
       <c r="B104">
-        <v>1594</v>
+        <v>0</v>
       </c>
     </row>
     <row r="105" spans="1:2">
       <c r="A105" s="2">
-        <v>46122.07291666666</v>
+        <v>46129.07291666666</v>
       </c>
       <c r="B105">
-        <v>1598</v>
+        <v>1221</v>
       </c>
     </row>
     <row r="106" spans="1:2">
       <c r="A106" s="2">
-        <v>46122.08333333334</v>
+        <v>46129.08333333334</v>
       </c>
       <c r="B106">
-        <v>1552</v>
+        <v>1220</v>
       </c>
     </row>
     <row r="107" spans="1:2">
       <c r="A107" s="2">
-        <v>46122.09375</v>
+        <v>46129.09375</v>
       </c>
       <c r="B107">
-        <v>1543</v>
+        <v>1216</v>
       </c>
     </row>
     <row r="108" spans="1:2">
       <c r="A108" s="2">
-        <v>46122.10416666666</v>
+        <v>46129.10416666666</v>
       </c>
       <c r="B108">
-        <v>1494</v>
+        <v>1217</v>
       </c>
     </row>
     <row r="109" spans="1:2">
       <c r="A109" s="2">
-        <v>46122.11458333334</v>
+        <v>46129.11458333334</v>
       </c>
       <c r="B109">
-        <v>1586</v>
+        <v>0</v>
       </c>
     </row>
     <row r="110" spans="1:2">
       <c r="A110" s="2">
-        <v>46122.125</v>
+        <v>46129.125</v>
       </c>
       <c r="B110">
-        <v>1560</v>
+        <v>1220</v>
       </c>
     </row>
     <row r="111" spans="1:2">
       <c r="A111" s="2">
-        <v>46122.13541666666</v>
+        <v>46129.13541666666</v>
       </c>
       <c r="B111">
-        <v>1540</v>
+        <v>1218</v>
       </c>
     </row>
     <row r="112" spans="1:2">
       <c r="A112" s="2">
-        <v>46122.14583333334</v>
+        <v>46129.14583333334</v>
       </c>
       <c r="B112">
-        <v>1521</v>
+        <v>0</v>
       </c>
     </row>
     <row r="113" spans="1:2">
       <c r="A113" s="2">
-        <v>46122.15625</v>
+        <v>46129.15625</v>
       </c>
       <c r="B113">
-        <v>1493</v>
+        <v>1219</v>
       </c>
     </row>
     <row r="114" spans="1:2">
       <c r="A114" s="2">
-        <v>46122.16666666666</v>
+        <v>46129.16666666666</v>
       </c>
       <c r="B114">
-        <v>1550</v>
+        <v>1221</v>
       </c>
     </row>
     <row r="115" spans="1:2">
       <c r="A115" s="2">
-        <v>46122.17708333334</v>
+        <v>46129.17708333334</v>
       </c>
       <c r="B115">
-        <v>1583</v>
+        <v>0</v>
       </c>
     </row>
     <row r="116" spans="1:2">
       <c r="A116" s="2">
-        <v>46122.1875</v>
+        <v>46129.1875</v>
       </c>
       <c r="B116">
-        <v>1585</v>
+        <v>1222</v>
       </c>
     </row>
     <row r="117" spans="1:2">
       <c r="A117" s="2">
-        <v>46122.19791666666</v>
+        <v>46129.19791666666</v>
       </c>
       <c r="B117">
-        <v>1584</v>
+        <v>1223</v>
       </c>
     </row>
     <row r="118" spans="1:2">
       <c r="A118" s="2">
-        <v>46122.20833333334</v>
+        <v>46129.20833333334</v>
       </c>
       <c r="B118">
-        <v>1582</v>
+        <v>1236</v>
       </c>
     </row>
     <row r="119" spans="1:2">
       <c r="A119" s="2">
-        <v>46122.21875</v>
+        <v>46129.21875</v>
       </c>
       <c r="B119">
-        <v>1584</v>
+        <v>1237</v>
       </c>
     </row>
     <row r="120" spans="1:2">
       <c r="A120" s="2">
-        <v>46122.22916666666</v>
+        <v>46129.22916666666</v>
       </c>
       <c r="B120">
-        <v>1570</v>
+        <v>1239</v>
       </c>
     </row>
     <row r="121" spans="1:2">
       <c r="A121" s="2">
-        <v>46122.23958333334</v>
+        <v>46129.23958333334</v>
       </c>
       <c r="B121">
-        <v>1578</v>
+        <v>1241</v>
       </c>
     </row>
     <row r="122" spans="1:2">
       <c r="A122" s="2">
-        <v>46122.25</v>
+        <v>46129.25</v>
       </c>
       <c r="B122">
-        <v>1763</v>
+        <v>1320</v>
       </c>
     </row>
     <row r="123" spans="1:2">
       <c r="A123" s="2">
-        <v>46122.26041666666</v>
+        <v>46129.26041666666</v>
       </c>
       <c r="B123">
-        <v>1821</v>
+        <v>1321</v>
       </c>
     </row>
     <row r="124" spans="1:2">
       <c r="A124" s="2">
-        <v>46122.27083333334</v>
+        <v>46129.27083333334</v>
       </c>
       <c r="B124">
-        <v>1827</v>
+        <v>1319</v>
       </c>
     </row>
     <row r="125" spans="1:2">
       <c r="A125" s="2">
-        <v>46122.28125</v>
+        <v>46129.28125</v>
       </c>
       <c r="B125">
-        <v>1836</v>
+        <v>1324</v>
       </c>
     </row>
     <row r="126" spans="1:2">
       <c r="A126" s="2">
-        <v>46122.29166666666</v>
+        <v>46129.29166666666</v>
       </c>
       <c r="B126">
-        <v>1831</v>
+        <v>1328</v>
       </c>
     </row>
     <row r="127" spans="1:2">
       <c r="A127" s="2">
-        <v>46122.30208333334</v>
+        <v>46129.30208333334</v>
       </c>
       <c r="B127">
-        <v>1824</v>
+        <v>1316</v>
       </c>
     </row>
     <row r="128" spans="1:2">
       <c r="A128" s="2">
-        <v>46122.3125</v>
+        <v>46129.3125</v>
       </c>
       <c r="B128">
-        <v>1832</v>
+        <v>1312</v>
       </c>
     </row>
     <row r="129" spans="1:2">
       <c r="A129" s="2">
-        <v>46122.32291666666</v>
+        <v>46129.32291666666</v>
       </c>
       <c r="B129">
-        <v>1831</v>
+        <v>1313</v>
       </c>
     </row>
     <row r="130" spans="1:2">
       <c r="A130" s="2">
-        <v>46122.33333333334</v>
+        <v>46129.33333333334</v>
       </c>
       <c r="B130">
-        <v>1827</v>
+        <v>1291</v>
       </c>
     </row>
     <row r="131" spans="1:2">
       <c r="A131" s="2">
-        <v>46122.34375</v>
+        <v>46129.34375</v>
       </c>
       <c r="B131">
-        <v>1820</v>
+        <v>1293</v>
       </c>
     </row>
     <row r="132" spans="1:2">
       <c r="A132" s="2">
-        <v>46122.35416666666</v>
+        <v>46129.35416666666</v>
       </c>
       <c r="B132">
-        <v>1815</v>
+        <v>1287</v>
       </c>
     </row>
     <row r="133" spans="1:2">
       <c r="A133" s="2">
-        <v>46122.36458333334</v>
+        <v>46129.36458333334</v>
       </c>
       <c r="B133">
-        <v>1812</v>
+        <v>0</v>
       </c>
     </row>
     <row r="134" spans="1:2">
       <c r="A134" s="2">
-        <v>46122.375</v>
+        <v>46129.375</v>
       </c>
       <c r="B134">
-        <v>1448</v>
+        <v>1026</v>
       </c>
     </row>
     <row r="135" spans="1:2">
       <c r="A135" s="2">
-        <v>46122.38541666666</v>
+        <v>46129.38541666666</v>
       </c>
       <c r="B135">
-        <v>1423</v>
+        <v>993</v>
       </c>
     </row>
     <row r="136" spans="1:2">
       <c r="A136" s="2">
-        <v>46122.39583333334</v>
+        <v>46129.39583333334</v>
       </c>
       <c r="B136">
-        <v>1424</v>
+        <v>999</v>
       </c>
     </row>
     <row r="137" spans="1:2">
       <c r="A137" s="2">
-        <v>46122.40625</v>
+        <v>46129.40625</v>
       </c>
       <c r="B137">
-        <v>1421</v>
+        <v>0</v>
       </c>
     </row>
     <row r="138" spans="1:2">
       <c r="A138" s="2">
-        <v>46122.41666666666</v>
+        <v>46129.41666666666</v>
       </c>
       <c r="B138">
-        <v>1166</v>
+        <v>911</v>
       </c>
     </row>
     <row r="139" spans="1:2">
       <c r="A139" s="2">
-        <v>46122.42708333334</v>
+        <v>46129.42708333334</v>
       </c>
       <c r="B139">
-        <v>0</v>
+        <v>900</v>
       </c>
     </row>
     <row r="140" spans="1:2">
       <c r="A140" s="2">
-        <v>46122.4375</v>
+        <v>46129.4375</v>
       </c>
       <c r="B140">
-        <v>0</v>
+        <v>903</v>
       </c>
     </row>
     <row r="141" spans="1:2">
       <c r="A141" s="2">
-        <v>46122.44791666666</v>
+        <v>46129.44791666666</v>
       </c>
       <c r="B141">
-        <v>0</v>
+        <v>899</v>
       </c>
     </row>
     <row r="142" spans="1:2">
       <c r="A142" s="2">
-        <v>46122.45833333334</v>
+        <v>46129.45833333334</v>
       </c>
       <c r="B142">
-        <v>0</v>
+        <v>876</v>
       </c>
     </row>
     <row r="143" spans="1:2">
       <c r="A143" s="2">
-        <v>46122.46875</v>
+        <v>46129.46875</v>
       </c>
       <c r="B143">
-        <v>0</v>
+        <v>866</v>
       </c>
     </row>
     <row r="144" spans="1:2">
       <c r="A144" s="2">
-        <v>46122.47916666666</v>
+        <v>46129.47916666666</v>
       </c>
       <c r="B144">
         <v>0</v>
@@ -1538,15 +1538,15 @@
     </row>
     <row r="145" spans="1:2">
       <c r="A145" s="2">
-        <v>46122.48958333334</v>
+        <v>46129.48958333334</v>
       </c>
       <c r="B145">
-        <v>0</v>
+        <v>864</v>
       </c>
     </row>
     <row r="146" spans="1:2">
       <c r="A146" s="2">
-        <v>46122.5</v>
+        <v>46129.5</v>
       </c>
       <c r="B146">
         <v>0</v>
@@ -1554,7 +1554,7 @@
     </row>
     <row r="147" spans="1:2">
       <c r="A147" s="2">
-        <v>46122.51041666666</v>
+        <v>46129.51041666666</v>
       </c>
       <c r="B147">
         <v>0</v>
@@ -1562,7 +1562,7 @@
     </row>
     <row r="148" spans="1:2">
       <c r="A148" s="2">
-        <v>46122.52083333334</v>
+        <v>46129.52083333334</v>
       </c>
       <c r="B148">
         <v>0</v>
@@ -1570,7 +1570,7 @@
     </row>
     <row r="149" spans="1:2">
       <c r="A149" s="2">
-        <v>46122.53125</v>
+        <v>46129.53125</v>
       </c>
       <c r="B149">
         <v>0</v>
@@ -1578,7 +1578,7 @@
     </row>
     <row r="150" spans="1:2">
       <c r="A150" s="2">
-        <v>46122.54166666666</v>
+        <v>46129.54166666666</v>
       </c>
       <c r="B150">
         <v>0</v>
@@ -1586,7 +1586,7 @@
     </row>
     <row r="151" spans="1:2">
       <c r="A151" s="2">
-        <v>46122.55208333334</v>
+        <v>46129.55208333334</v>
       </c>
       <c r="B151">
         <v>0</v>
@@ -1594,7 +1594,7 @@
     </row>
     <row r="152" spans="1:2">
       <c r="A152" s="2">
-        <v>46122.5625</v>
+        <v>46129.5625</v>
       </c>
       <c r="B152">
         <v>0</v>
@@ -1602,7 +1602,7 @@
     </row>
     <row r="153" spans="1:2">
       <c r="A153" s="2">
-        <v>46122.57291666666</v>
+        <v>46129.57291666666</v>
       </c>
       <c r="B153">
         <v>0</v>
@@ -1610,7 +1610,7 @@
     </row>
     <row r="154" spans="1:2">
       <c r="A154" s="2">
-        <v>46122.58333333334</v>
+        <v>46129.58333333334</v>
       </c>
       <c r="B154">
         <v>0</v>
@@ -1618,7 +1618,7 @@
     </row>
     <row r="155" spans="1:2">
       <c r="A155" s="2">
-        <v>46122.59375</v>
+        <v>46129.59375</v>
       </c>
       <c r="B155">
         <v>0</v>
@@ -1626,7 +1626,7 @@
     </row>
     <row r="156" spans="1:2">
       <c r="A156" s="2">
-        <v>46122.60416666666</v>
+        <v>46129.60416666666</v>
       </c>
       <c r="B156">
         <v>0</v>
@@ -1634,7 +1634,7 @@
     </row>
     <row r="157" spans="1:2">
       <c r="A157" s="2">
-        <v>46122.61458333334</v>
+        <v>46129.61458333334</v>
       </c>
       <c r="B157">
         <v>0</v>
@@ -1642,7 +1642,7 @@
     </row>
     <row r="158" spans="1:2">
       <c r="A158" s="2">
-        <v>46122.625</v>
+        <v>46129.625</v>
       </c>
       <c r="B158">
         <v>0</v>
@@ -1650,7 +1650,7 @@
     </row>
     <row r="159" spans="1:2">
       <c r="A159" s="2">
-        <v>46122.63541666666</v>
+        <v>46129.63541666666</v>
       </c>
       <c r="B159">
         <v>0</v>
@@ -1658,7 +1658,7 @@
     </row>
     <row r="160" spans="1:2">
       <c r="A160" s="2">
-        <v>46122.64583333334</v>
+        <v>46129.64583333334</v>
       </c>
       <c r="B160">
         <v>0</v>
@@ -1666,7 +1666,7 @@
     </row>
     <row r="161" spans="1:2">
       <c r="A161" s="2">
-        <v>46122.65625</v>
+        <v>46129.65625</v>
       </c>
       <c r="B161">
         <v>0</v>
@@ -1674,7 +1674,7 @@
     </row>
     <row r="162" spans="1:2">
       <c r="A162" s="2">
-        <v>46122.66666666666</v>
+        <v>46129.66666666666</v>
       </c>
       <c r="B162">
         <v>0</v>
@@ -1682,7 +1682,7 @@
     </row>
     <row r="163" spans="1:2">
       <c r="A163" s="2">
-        <v>46122.67708333334</v>
+        <v>46129.67708333334</v>
       </c>
       <c r="B163">
         <v>0</v>
@@ -1690,7 +1690,7 @@
     </row>
     <row r="164" spans="1:2">
       <c r="A164" s="2">
-        <v>46122.6875</v>
+        <v>46129.6875</v>
       </c>
       <c r="B164">
         <v>0</v>
@@ -1698,7 +1698,7 @@
     </row>
     <row r="165" spans="1:2">
       <c r="A165" s="2">
-        <v>46122.69791666666</v>
+        <v>46129.69791666666</v>
       </c>
       <c r="B165">
         <v>0</v>
@@ -1706,7 +1706,7 @@
     </row>
     <row r="166" spans="1:2">
       <c r="A166" s="2">
-        <v>46122.70833333334</v>
+        <v>46129.70833333334</v>
       </c>
       <c r="B166">
         <v>0</v>
@@ -1714,7 +1714,7 @@
     </row>
     <row r="167" spans="1:2">
       <c r="A167" s="2">
-        <v>46122.71875</v>
+        <v>46129.71875</v>
       </c>
       <c r="B167">
         <v>0</v>
@@ -1722,7 +1722,7 @@
     </row>
     <row r="168" spans="1:2">
       <c r="A168" s="2">
-        <v>46122.72916666666</v>
+        <v>46129.72916666666</v>
       </c>
       <c r="B168">
         <v>0</v>
@@ -1730,7 +1730,7 @@
     </row>
     <row r="169" spans="1:2">
       <c r="A169" s="2">
-        <v>46122.73958333334</v>
+        <v>46129.73958333334</v>
       </c>
       <c r="B169">
         <v>0</v>
@@ -1738,7 +1738,7 @@
     </row>
     <row r="170" spans="1:2">
       <c r="A170" s="2">
-        <v>46122.75</v>
+        <v>46129.75</v>
       </c>
       <c r="B170">
         <v>0</v>
@@ -1746,7 +1746,7 @@
     </row>
     <row r="171" spans="1:2">
       <c r="A171" s="2">
-        <v>46122.76041666666</v>
+        <v>46129.76041666666</v>
       </c>
       <c r="B171">
         <v>0</v>
@@ -1754,7 +1754,7 @@
     </row>
     <row r="172" spans="1:2">
       <c r="A172" s="2">
-        <v>46122.77083333334</v>
+        <v>46129.77083333334</v>
       </c>
       <c r="B172">
         <v>0</v>
@@ -1762,7 +1762,7 @@
     </row>
     <row r="173" spans="1:2">
       <c r="A173" s="2">
-        <v>46122.78125</v>
+        <v>46129.78125</v>
       </c>
       <c r="B173">
         <v>0</v>
@@ -1770,7 +1770,7 @@
     </row>
     <row r="174" spans="1:2">
       <c r="A174" s="2">
-        <v>46122.79166666666</v>
+        <v>46129.79166666666</v>
       </c>
       <c r="B174">
         <v>0</v>
@@ -1778,7 +1778,7 @@
     </row>
     <row r="175" spans="1:2">
       <c r="A175" s="2">
-        <v>46122.80208333334</v>
+        <v>46129.80208333334</v>
       </c>
       <c r="B175">
         <v>0</v>
@@ -1786,7 +1786,7 @@
     </row>
     <row r="176" spans="1:2">
       <c r="A176" s="2">
-        <v>46122.8125</v>
+        <v>46129.8125</v>
       </c>
       <c r="B176">
         <v>0</v>
@@ -1794,7 +1794,7 @@
     </row>
     <row r="177" spans="1:2">
       <c r="A177" s="2">
-        <v>46122.82291666666</v>
+        <v>46129.82291666666</v>
       </c>
       <c r="B177">
         <v>0</v>
@@ -1802,7 +1802,7 @@
     </row>
     <row r="178" spans="1:2">
       <c r="A178" s="2">
-        <v>46122.83333333334</v>
+        <v>46129.83333333334</v>
       </c>
       <c r="B178">
         <v>0</v>
@@ -1810,7 +1810,7 @@
     </row>
     <row r="179" spans="1:2">
       <c r="A179" s="2">
-        <v>46122.84375</v>
+        <v>46129.84375</v>
       </c>
       <c r="B179">
         <v>0</v>
@@ -1818,7 +1818,7 @@
     </row>
     <row r="180" spans="1:2">
       <c r="A180" s="2">
-        <v>46122.85416666666</v>
+        <v>46129.85416666666</v>
       </c>
       <c r="B180">
         <v>0</v>
@@ -1826,7 +1826,7 @@
     </row>
     <row r="181" spans="1:2">
       <c r="A181" s="2">
-        <v>46122.86458333334</v>
+        <v>46129.86458333334</v>
       </c>
       <c r="B181">
         <v>0</v>
@@ -1834,7 +1834,7 @@
     </row>
     <row r="182" spans="1:2">
       <c r="A182" s="2">
-        <v>46122.875</v>
+        <v>46129.875</v>
       </c>
       <c r="B182">
         <v>0</v>
@@ -1842,7 +1842,7 @@
     </row>
     <row r="183" spans="1:2">
       <c r="A183" s="2">
-        <v>46122.88541666666</v>
+        <v>46129.88541666666</v>
       </c>
       <c r="B183">
         <v>0</v>
@@ -1850,7 +1850,7 @@
     </row>
     <row r="184" spans="1:2">
       <c r="A184" s="2">
-        <v>46122.89583333334</v>
+        <v>46129.89583333334</v>
       </c>
       <c r="B184">
         <v>0</v>
@@ -1858,7 +1858,7 @@
     </row>
     <row r="185" spans="1:2">
       <c r="A185" s="2">
-        <v>46122.90625</v>
+        <v>46129.90625</v>
       </c>
       <c r="B185">
         <v>0</v>
@@ -1866,7 +1866,7 @@
     </row>
     <row r="186" spans="1:2">
       <c r="A186" s="2">
-        <v>46122.91666666666</v>
+        <v>46129.91666666666</v>
       </c>
       <c r="B186">
         <v>0</v>
@@ -1874,7 +1874,7 @@
     </row>
     <row r="187" spans="1:2">
       <c r="A187" s="2">
-        <v>46122.92708333334</v>
+        <v>46129.92708333334</v>
       </c>
       <c r="B187">
         <v>0</v>
@@ -1882,7 +1882,7 @@
     </row>
     <row r="188" spans="1:2">
       <c r="A188" s="2">
-        <v>46122.9375</v>
+        <v>46129.9375</v>
       </c>
       <c r="B188">
         <v>0</v>
@@ -1890,7 +1890,7 @@
     </row>
     <row r="189" spans="1:2">
       <c r="A189" s="2">
-        <v>46122.94791666666</v>
+        <v>46129.94791666666</v>
       </c>
       <c r="B189">
         <v>0</v>
@@ -1898,7 +1898,7 @@
     </row>
     <row r="190" spans="1:2">
       <c r="A190" s="2">
-        <v>46122.95833333334</v>
+        <v>46129.95833333334</v>
       </c>
       <c r="B190">
         <v>0</v>
@@ -1906,7 +1906,7 @@
     </row>
     <row r="191" spans="1:2">
       <c r="A191" s="2">
-        <v>46122.96875</v>
+        <v>46129.96875</v>
       </c>
       <c r="B191">
         <v>0</v>
@@ -1914,7 +1914,7 @@
     </row>
     <row r="192" spans="1:2">
       <c r="A192" s="2">
-        <v>46122.97916666666</v>
+        <v>46129.97916666666</v>
       </c>
       <c r="B192">
         <v>0</v>
@@ -1922,7 +1922,7 @@
     </row>
     <row r="193" spans="1:2">
       <c r="A193" s="2">
-        <v>46122.98958333334</v>
+        <v>46129.98958333334</v>
       </c>
       <c r="B193">
         <v>0</v>

</xml_diff>

<commit_message>
Retraining the model for MM&MV
</commit_message>
<xml_diff>
--- a/data_fetching/Entsoe/Actual_Production_Hydro_River.xlsx
+++ b/data_fetching/Entsoe/Actual_Production_Hydro_River.xlsx
@@ -381,7 +381,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B193"/>
+  <dimension ref="A1:B385"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:2">
@@ -394,55 +394,55 @@
     </row>
     <row r="2" spans="1:2">
       <c r="A2" s="2">
-        <v>46128</v>
+        <v>46129</v>
       </c>
       <c r="B2">
-        <v>1352</v>
+        <v>1296</v>
       </c>
     </row>
     <row r="3" spans="1:2">
       <c r="A3" s="2">
-        <v>46128.01041666666</v>
+        <v>46129.01041666666</v>
       </c>
       <c r="B3">
-        <v>1356</v>
+        <v>1292</v>
       </c>
     </row>
     <row r="4" spans="1:2">
       <c r="A4" s="2">
-        <v>46128.02083333334</v>
+        <v>46129.02083333334</v>
       </c>
       <c r="B4">
-        <v>1351</v>
+        <v>1289</v>
       </c>
     </row>
     <row r="5" spans="1:2">
       <c r="A5" s="2">
-        <v>46128.03125</v>
+        <v>46129.03125</v>
       </c>
       <c r="B5">
-        <v>1353</v>
+        <v>1291</v>
       </c>
     </row>
     <row r="6" spans="1:2">
       <c r="A6" s="2">
-        <v>46128.04166666666</v>
+        <v>46129.04166666666</v>
       </c>
       <c r="B6">
-        <v>1330</v>
+        <v>1227</v>
       </c>
     </row>
     <row r="7" spans="1:2">
       <c r="A7" s="2">
-        <v>46128.05208333334</v>
+        <v>46129.05208333334</v>
       </c>
       <c r="B7">
-        <v>1331</v>
+        <v>1222</v>
       </c>
     </row>
     <row r="8" spans="1:2">
       <c r="A8" s="2">
-        <v>46128.0625</v>
+        <v>46129.0625</v>
       </c>
       <c r="B8">
         <v>0</v>
@@ -450,63 +450,63 @@
     </row>
     <row r="9" spans="1:2">
       <c r="A9" s="2">
-        <v>46128.07291666666</v>
+        <v>46129.07291666666</v>
       </c>
       <c r="B9">
-        <v>1332</v>
+        <v>1221</v>
       </c>
     </row>
     <row r="10" spans="1:2">
       <c r="A10" s="2">
-        <v>46128.08333333334</v>
+        <v>46129.08333333334</v>
       </c>
       <c r="B10">
-        <v>1331</v>
+        <v>1220</v>
       </c>
     </row>
     <row r="11" spans="1:2">
       <c r="A11" s="2">
-        <v>46128.09375</v>
+        <v>46129.09375</v>
       </c>
       <c r="B11">
-        <v>1329</v>
+        <v>1216</v>
       </c>
     </row>
     <row r="12" spans="1:2">
       <c r="A12" s="2">
-        <v>46128.10416666666</v>
+        <v>46129.10416666666</v>
       </c>
       <c r="B12">
-        <v>0</v>
+        <v>1217</v>
       </c>
     </row>
     <row r="13" spans="1:2">
       <c r="A13" s="2">
-        <v>46128.11458333334</v>
+        <v>46129.11458333334</v>
       </c>
       <c r="B13">
-        <v>1327</v>
+        <v>0</v>
       </c>
     </row>
     <row r="14" spans="1:2">
       <c r="A14" s="2">
-        <v>46128.125</v>
+        <v>46129.125</v>
       </c>
       <c r="B14">
-        <v>1334</v>
+        <v>1220</v>
       </c>
     </row>
     <row r="15" spans="1:2">
       <c r="A15" s="2">
-        <v>46128.13541666666</v>
+        <v>46129.13541666666</v>
       </c>
       <c r="B15">
-        <v>0</v>
+        <v>1218</v>
       </c>
     </row>
     <row r="16" spans="1:2">
       <c r="A16" s="2">
-        <v>46128.14583333334</v>
+        <v>46129.14583333334</v>
       </c>
       <c r="B16">
         <v>0</v>
@@ -514,703 +514,703 @@
     </row>
     <row r="17" spans="1:2">
       <c r="A17" s="2">
-        <v>46128.15625</v>
+        <v>46129.15625</v>
       </c>
       <c r="B17">
-        <v>1333</v>
+        <v>1219</v>
       </c>
     </row>
     <row r="18" spans="1:2">
       <c r="A18" s="2">
-        <v>46128.16666666666</v>
+        <v>46129.16666666666</v>
       </c>
       <c r="B18">
-        <v>1336</v>
+        <v>1221</v>
       </c>
     </row>
     <row r="19" spans="1:2">
       <c r="A19" s="2">
-        <v>46128.17708333334</v>
+        <v>46129.17708333334</v>
       </c>
       <c r="B19">
-        <v>1337</v>
+        <v>0</v>
       </c>
     </row>
     <row r="20" spans="1:2">
       <c r="A20" s="2">
-        <v>46128.1875</v>
+        <v>46129.1875</v>
       </c>
       <c r="B20">
-        <v>0</v>
+        <v>1222</v>
       </c>
     </row>
     <row r="21" spans="1:2">
       <c r="A21" s="2">
-        <v>46128.19791666666</v>
+        <v>46129.19791666666</v>
       </c>
       <c r="B21">
-        <v>1336</v>
+        <v>1223</v>
       </c>
     </row>
     <row r="22" spans="1:2">
       <c r="A22" s="2">
-        <v>46128.20833333334</v>
+        <v>46129.20833333334</v>
       </c>
       <c r="B22">
-        <v>1374</v>
+        <v>1236</v>
       </c>
     </row>
     <row r="23" spans="1:2">
       <c r="A23" s="2">
-        <v>46128.21875</v>
+        <v>46129.21875</v>
       </c>
       <c r="B23">
-        <v>1373</v>
+        <v>1237</v>
       </c>
     </row>
     <row r="24" spans="1:2">
       <c r="A24" s="2">
-        <v>46128.22916666666</v>
+        <v>46129.22916666666</v>
       </c>
       <c r="B24">
-        <v>1375</v>
+        <v>1239</v>
       </c>
     </row>
     <row r="25" spans="1:2">
       <c r="A25" s="2">
-        <v>46128.23958333334</v>
+        <v>46129.23958333334</v>
       </c>
       <c r="B25">
-        <v>1374</v>
+        <v>1241</v>
       </c>
     </row>
     <row r="26" spans="1:2">
       <c r="A26" s="2">
-        <v>46128.25</v>
+        <v>46129.25</v>
       </c>
       <c r="B26">
-        <v>1376</v>
+        <v>1320</v>
       </c>
     </row>
     <row r="27" spans="1:2">
       <c r="A27" s="2">
-        <v>46128.26041666666</v>
+        <v>46129.26041666666</v>
       </c>
       <c r="B27">
-        <v>1370</v>
+        <v>1321</v>
       </c>
     </row>
     <row r="28" spans="1:2">
       <c r="A28" s="2">
-        <v>46128.27083333334</v>
+        <v>46129.27083333334</v>
       </c>
       <c r="B28">
-        <v>1367</v>
+        <v>1319</v>
       </c>
     </row>
     <row r="29" spans="1:2">
       <c r="A29" s="2">
-        <v>46128.28125</v>
+        <v>46129.28125</v>
       </c>
       <c r="B29">
-        <v>1369</v>
+        <v>1324</v>
       </c>
     </row>
     <row r="30" spans="1:2">
       <c r="A30" s="2">
-        <v>46128.29166666666</v>
+        <v>46129.29166666666</v>
       </c>
       <c r="B30">
-        <v>1370</v>
+        <v>1328</v>
       </c>
     </row>
     <row r="31" spans="1:2">
       <c r="A31" s="2">
-        <v>46128.30208333334</v>
+        <v>46129.30208333334</v>
       </c>
       <c r="B31">
-        <v>1365</v>
+        <v>1316</v>
       </c>
     </row>
     <row r="32" spans="1:2">
       <c r="A32" s="2">
-        <v>46128.3125</v>
+        <v>46129.3125</v>
       </c>
       <c r="B32">
-        <v>1302</v>
+        <v>1312</v>
       </c>
     </row>
     <row r="33" spans="1:2">
       <c r="A33" s="2">
-        <v>46128.32291666666</v>
+        <v>46129.32291666666</v>
       </c>
       <c r="B33">
-        <v>1305</v>
+        <v>1313</v>
       </c>
     </row>
     <row r="34" spans="1:2">
       <c r="A34" s="2">
-        <v>46128.33333333334</v>
+        <v>46129.33333333334</v>
       </c>
       <c r="B34">
-        <v>1238</v>
+        <v>1291</v>
       </c>
     </row>
     <row r="35" spans="1:2">
       <c r="A35" s="2">
-        <v>46128.34375</v>
+        <v>46129.34375</v>
       </c>
       <c r="B35">
-        <v>1235</v>
+        <v>1293</v>
       </c>
     </row>
     <row r="36" spans="1:2">
       <c r="A36" s="2">
-        <v>46128.35416666666</v>
+        <v>46129.35416666666</v>
       </c>
       <c r="B36">
-        <v>1238</v>
+        <v>1287</v>
       </c>
     </row>
     <row r="37" spans="1:2">
       <c r="A37" s="2">
-        <v>46128.36458333334</v>
+        <v>46129.36458333334</v>
       </c>
       <c r="B37">
-        <v>1237</v>
+        <v>0</v>
       </c>
     </row>
     <row r="38" spans="1:2">
       <c r="A38" s="2">
-        <v>46128.375</v>
+        <v>46129.375</v>
       </c>
       <c r="B38">
-        <v>1150</v>
+        <v>1026</v>
       </c>
     </row>
     <row r="39" spans="1:2">
       <c r="A39" s="2">
-        <v>46128.38541666666</v>
+        <v>46129.38541666666</v>
       </c>
       <c r="B39">
-        <v>1130</v>
+        <v>993</v>
       </c>
     </row>
     <row r="40" spans="1:2">
       <c r="A40" s="2">
-        <v>46128.39583333334</v>
+        <v>46129.39583333334</v>
       </c>
       <c r="B40">
-        <v>1127</v>
+        <v>999</v>
       </c>
     </row>
     <row r="41" spans="1:2">
       <c r="A41" s="2">
-        <v>46128.40625</v>
+        <v>46129.40625</v>
       </c>
       <c r="B41">
-        <v>1126</v>
+        <v>0</v>
       </c>
     </row>
     <row r="42" spans="1:2">
       <c r="A42" s="2">
-        <v>46128.41666666666</v>
+        <v>46129.41666666666</v>
       </c>
       <c r="B42">
-        <v>1044</v>
+        <v>911</v>
       </c>
     </row>
     <row r="43" spans="1:2">
       <c r="A43" s="2">
-        <v>46128.42708333334</v>
+        <v>46129.42708333334</v>
       </c>
       <c r="B43">
-        <v>1001</v>
+        <v>900</v>
       </c>
     </row>
     <row r="44" spans="1:2">
       <c r="A44" s="2">
-        <v>46128.4375</v>
+        <v>46129.4375</v>
       </c>
       <c r="B44">
-        <v>995</v>
+        <v>903</v>
       </c>
     </row>
     <row r="45" spans="1:2">
       <c r="A45" s="2">
-        <v>46128.44791666666</v>
+        <v>46129.44791666666</v>
       </c>
       <c r="B45">
-        <v>994</v>
+        <v>899</v>
       </c>
     </row>
     <row r="46" spans="1:2">
       <c r="A46" s="2">
-        <v>46128.45833333334</v>
+        <v>46129.45833333334</v>
       </c>
       <c r="B46">
-        <v>960</v>
+        <v>876</v>
       </c>
     </row>
     <row r="47" spans="1:2">
       <c r="A47" s="2">
-        <v>46128.46875</v>
+        <v>46129.46875</v>
       </c>
       <c r="B47">
-        <v>941</v>
+        <v>866</v>
       </c>
     </row>
     <row r="48" spans="1:2">
       <c r="A48" s="2">
-        <v>46128.47916666666</v>
+        <v>46129.47916666666</v>
       </c>
       <c r="B48">
-        <v>856</v>
+        <v>0</v>
       </c>
     </row>
     <row r="49" spans="1:2">
       <c r="A49" s="2">
-        <v>46128.48958333334</v>
+        <v>46129.48958333334</v>
       </c>
       <c r="B49">
-        <v>848</v>
+        <v>864</v>
       </c>
     </row>
     <row r="50" spans="1:2">
       <c r="A50" s="2">
-        <v>46128.5</v>
+        <v>46129.5</v>
       </c>
       <c r="B50">
-        <v>866</v>
+        <v>825</v>
       </c>
     </row>
     <row r="51" spans="1:2">
       <c r="A51" s="2">
-        <v>46128.51041666666</v>
+        <v>46129.51041666666</v>
       </c>
       <c r="B51">
-        <v>876</v>
+        <v>831</v>
       </c>
     </row>
     <row r="52" spans="1:2">
       <c r="A52" s="2">
-        <v>46128.52083333334</v>
+        <v>46129.52083333334</v>
       </c>
       <c r="B52">
-        <v>1015</v>
+        <v>803</v>
       </c>
     </row>
     <row r="53" spans="1:2">
       <c r="A53" s="2">
-        <v>46128.53125</v>
+        <v>46129.53125</v>
       </c>
       <c r="B53">
-        <v>977</v>
+        <v>800</v>
       </c>
     </row>
     <row r="54" spans="1:2">
       <c r="A54" s="2">
-        <v>46128.54166666666</v>
+        <v>46129.54166666666</v>
       </c>
       <c r="B54">
-        <v>979</v>
+        <v>818</v>
       </c>
     </row>
     <row r="55" spans="1:2">
       <c r="A55" s="2">
-        <v>46128.55208333334</v>
+        <v>46129.55208333334</v>
       </c>
       <c r="B55">
-        <v>1003</v>
+        <v>812</v>
       </c>
     </row>
     <row r="56" spans="1:2">
       <c r="A56" s="2">
-        <v>46128.5625</v>
+        <v>46129.5625</v>
       </c>
       <c r="B56">
-        <v>1002</v>
+        <v>0</v>
       </c>
     </row>
     <row r="57" spans="1:2">
       <c r="A57" s="2">
-        <v>46128.57291666666</v>
+        <v>46129.57291666666</v>
       </c>
       <c r="B57">
-        <v>1004</v>
+        <v>745</v>
       </c>
     </row>
     <row r="58" spans="1:2">
       <c r="A58" s="2">
-        <v>46128.58333333334</v>
+        <v>46129.58333333334</v>
       </c>
       <c r="B58">
-        <v>989</v>
+        <v>746</v>
       </c>
     </row>
     <row r="59" spans="1:2">
       <c r="A59" s="2">
-        <v>46128.59375</v>
+        <v>46129.59375</v>
       </c>
       <c r="B59">
-        <v>985</v>
+        <v>717</v>
       </c>
     </row>
     <row r="60" spans="1:2">
       <c r="A60" s="2">
-        <v>46128.60416666666</v>
+        <v>46129.60416666666</v>
       </c>
       <c r="B60">
-        <v>982</v>
+        <v>771</v>
       </c>
     </row>
     <row r="61" spans="1:2">
       <c r="A61" s="2">
-        <v>46128.61458333334</v>
+        <v>46129.61458333334</v>
       </c>
       <c r="B61">
-        <v>1040</v>
+        <v>778</v>
       </c>
     </row>
     <row r="62" spans="1:2">
       <c r="A62" s="2">
-        <v>46128.625</v>
+        <v>46129.625</v>
       </c>
       <c r="B62">
-        <v>1083</v>
+        <v>977</v>
       </c>
     </row>
     <row r="63" spans="1:2">
       <c r="A63" s="2">
-        <v>46128.63541666666</v>
+        <v>46129.63541666666</v>
       </c>
       <c r="B63">
-        <v>1090</v>
+        <v>996</v>
       </c>
     </row>
     <row r="64" spans="1:2">
       <c r="A64" s="2">
-        <v>46128.64583333334</v>
+        <v>46129.64583333334</v>
       </c>
       <c r="B64">
-        <v>0</v>
+        <v>1052</v>
       </c>
     </row>
     <row r="65" spans="1:2">
       <c r="A65" s="2">
-        <v>46128.65625</v>
+        <v>46129.65625</v>
       </c>
       <c r="B65">
-        <v>1091</v>
+        <v>1011</v>
       </c>
     </row>
     <row r="66" spans="1:2">
       <c r="A66" s="2">
-        <v>46128.66666666666</v>
+        <v>46129.66666666666</v>
       </c>
       <c r="B66">
-        <v>1108</v>
+        <v>1124</v>
       </c>
     </row>
     <row r="67" spans="1:2">
       <c r="A67" s="2">
-        <v>46128.67708333334</v>
+        <v>46129.67708333334</v>
       </c>
       <c r="B67">
-        <v>1112</v>
+        <v>1144</v>
       </c>
     </row>
     <row r="68" spans="1:2">
       <c r="A68" s="2">
-        <v>46128.6875</v>
+        <v>46129.6875</v>
       </c>
       <c r="B68">
-        <v>0</v>
+        <v>1229</v>
       </c>
     </row>
     <row r="69" spans="1:2">
       <c r="A69" s="2">
-        <v>46128.69791666666</v>
+        <v>46129.69791666666</v>
       </c>
       <c r="B69">
-        <v>1122</v>
+        <v>1278</v>
       </c>
     </row>
     <row r="70" spans="1:2">
       <c r="A70" s="2">
-        <v>46128.70833333334</v>
+        <v>46129.70833333334</v>
       </c>
       <c r="B70">
-        <v>1396</v>
+        <v>1399</v>
       </c>
     </row>
     <row r="71" spans="1:2">
       <c r="A71" s="2">
-        <v>46128.71875</v>
+        <v>46129.71875</v>
       </c>
       <c r="B71">
-        <v>1420</v>
+        <v>1424</v>
       </c>
     </row>
     <row r="72" spans="1:2">
       <c r="A72" s="2">
-        <v>46128.72916666666</v>
+        <v>46129.72916666666</v>
       </c>
       <c r="B72">
-        <v>1425</v>
+        <v>1421</v>
       </c>
     </row>
     <row r="73" spans="1:2">
       <c r="A73" s="2">
-        <v>46128.73958333334</v>
+        <v>46129.73958333334</v>
       </c>
       <c r="B73">
-        <v>1423</v>
+        <v>1418</v>
       </c>
     </row>
     <row r="74" spans="1:2">
       <c r="A74" s="2">
-        <v>46128.75</v>
+        <v>46129.75</v>
       </c>
       <c r="B74">
-        <v>1444</v>
+        <v>1404</v>
       </c>
     </row>
     <row r="75" spans="1:2">
       <c r="A75" s="2">
-        <v>46128.76041666666</v>
+        <v>46129.76041666666</v>
       </c>
       <c r="B75">
-        <v>1450</v>
+        <v>1412</v>
       </c>
     </row>
     <row r="76" spans="1:2">
       <c r="A76" s="2">
-        <v>46128.77083333334</v>
+        <v>46129.77083333334</v>
       </c>
       <c r="B76">
-        <v>1440</v>
+        <v>1415</v>
       </c>
     </row>
     <row r="77" spans="1:2">
       <c r="A77" s="2">
-        <v>46128.78125</v>
+        <v>46129.78125</v>
       </c>
       <c r="B77">
-        <v>1435</v>
+        <v>1413</v>
       </c>
     </row>
     <row r="78" spans="1:2">
       <c r="A78" s="2">
-        <v>46128.79166666666</v>
+        <v>46129.79166666666</v>
       </c>
       <c r="B78">
-        <v>1450</v>
+        <v>1416</v>
       </c>
     </row>
     <row r="79" spans="1:2">
       <c r="A79" s="2">
-        <v>46128.80208333334</v>
+        <v>46129.80208333334</v>
       </c>
       <c r="B79">
-        <v>1455</v>
+        <v>1429</v>
       </c>
     </row>
     <row r="80" spans="1:2">
       <c r="A80" s="2">
-        <v>46128.8125</v>
+        <v>46129.8125</v>
       </c>
       <c r="B80">
-        <v>1453</v>
+        <v>1417</v>
       </c>
     </row>
     <row r="81" spans="1:2">
       <c r="A81" s="2">
-        <v>46128.82291666666</v>
+        <v>46129.82291666666</v>
       </c>
       <c r="B81">
-        <v>0</v>
+        <v>1418</v>
       </c>
     </row>
     <row r="82" spans="1:2">
       <c r="A82" s="2">
-        <v>46128.83333333334</v>
+        <v>46129.83333333334</v>
       </c>
       <c r="B82">
-        <v>1454</v>
+        <v>1436</v>
       </c>
     </row>
     <row r="83" spans="1:2">
       <c r="A83" s="2">
-        <v>46128.84375</v>
+        <v>46129.84375</v>
       </c>
       <c r="B83">
-        <v>1455</v>
+        <v>1440</v>
       </c>
     </row>
     <row r="84" spans="1:2">
       <c r="A84" s="2">
-        <v>46128.85416666666</v>
+        <v>46129.85416666666</v>
       </c>
       <c r="B84">
-        <v>1454</v>
+        <v>1442</v>
       </c>
     </row>
     <row r="85" spans="1:2">
       <c r="A85" s="2">
-        <v>46128.86458333334</v>
+        <v>46129.86458333334</v>
       </c>
       <c r="B85">
-        <v>1456</v>
+        <v>1439</v>
       </c>
     </row>
     <row r="86" spans="1:2">
       <c r="A86" s="2">
-        <v>46128.875</v>
+        <v>46129.875</v>
       </c>
       <c r="B86">
-        <v>1416</v>
+        <v>1457</v>
       </c>
     </row>
     <row r="87" spans="1:2">
       <c r="A87" s="2">
-        <v>46128.88541666666</v>
+        <v>46129.88541666666</v>
       </c>
       <c r="B87">
-        <v>1414</v>
+        <v>1454</v>
       </c>
     </row>
     <row r="88" spans="1:2">
       <c r="A88" s="2">
-        <v>46128.89583333334</v>
+        <v>46129.89583333334</v>
       </c>
       <c r="B88">
-        <v>1412</v>
+        <v>1452</v>
       </c>
     </row>
     <row r="89" spans="1:2">
       <c r="A89" s="2">
-        <v>46128.90625</v>
+        <v>46129.90625</v>
       </c>
       <c r="B89">
-        <v>1405</v>
+        <v>1453</v>
       </c>
     </row>
     <row r="90" spans="1:2">
       <c r="A90" s="2">
-        <v>46128.91666666666</v>
+        <v>46129.91666666666</v>
       </c>
       <c r="B90">
-        <v>1414</v>
+        <v>1400</v>
       </c>
     </row>
     <row r="91" spans="1:2">
       <c r="A91" s="2">
-        <v>46128.92708333334</v>
+        <v>46129.92708333334</v>
       </c>
       <c r="B91">
-        <v>1415</v>
+        <v>1390</v>
       </c>
     </row>
     <row r="92" spans="1:2">
       <c r="A92" s="2">
-        <v>46128.9375</v>
+        <v>46129.9375</v>
       </c>
       <c r="B92">
-        <v>1414</v>
+        <v>0</v>
       </c>
     </row>
     <row r="93" spans="1:2">
       <c r="A93" s="2">
-        <v>46128.94791666666</v>
+        <v>46129.94791666666</v>
       </c>
       <c r="B93">
-        <v>1413</v>
+        <v>1385</v>
       </c>
     </row>
     <row r="94" spans="1:2">
       <c r="A94" s="2">
-        <v>46128.95833333334</v>
+        <v>46129.95833333334</v>
       </c>
       <c r="B94">
-        <v>1410</v>
+        <v>1444</v>
       </c>
     </row>
     <row r="95" spans="1:2">
       <c r="A95" s="2">
-        <v>46128.96875</v>
+        <v>46129.96875</v>
       </c>
       <c r="B95">
-        <v>0</v>
+        <v>1442</v>
       </c>
     </row>
     <row r="96" spans="1:2">
       <c r="A96" s="2">
-        <v>46128.97916666666</v>
+        <v>46129.97916666666</v>
       </c>
       <c r="B96">
-        <v>1411</v>
+        <v>1441</v>
       </c>
     </row>
     <row r="97" spans="1:2">
       <c r="A97" s="2">
-        <v>46128.98958333334</v>
+        <v>46129.98958333334</v>
       </c>
       <c r="B97">
-        <v>1409</v>
+        <v>1439</v>
       </c>
     </row>
     <row r="98" spans="1:2">
       <c r="A98" s="2">
-        <v>46129</v>
+        <v>46130</v>
       </c>
       <c r="B98">
-        <v>1296</v>
+        <v>1338</v>
       </c>
     </row>
     <row r="99" spans="1:2">
       <c r="A99" s="2">
-        <v>46129.01041666666</v>
+        <v>46130.01041666666</v>
       </c>
       <c r="B99">
-        <v>1292</v>
+        <v>1331</v>
       </c>
     </row>
     <row r="100" spans="1:2">
       <c r="A100" s="2">
-        <v>46129.02083333334</v>
+        <v>46130.02083333334</v>
       </c>
       <c r="B100">
-        <v>1289</v>
+        <v>1332</v>
       </c>
     </row>
     <row r="101" spans="1:2">
       <c r="A101" s="2">
-        <v>46129.03125</v>
+        <v>46130.03125</v>
       </c>
       <c r="B101">
-        <v>1291</v>
+        <v>1331</v>
       </c>
     </row>
     <row r="102" spans="1:2">
       <c r="A102" s="2">
-        <v>46129.04166666666</v>
+        <v>46130.04166666666</v>
       </c>
       <c r="B102">
-        <v>1227</v>
+        <v>1335</v>
       </c>
     </row>
     <row r="103" spans="1:2">
       <c r="A103" s="2">
-        <v>46129.05208333334</v>
+        <v>46130.05208333334</v>
       </c>
       <c r="B103">
-        <v>1222</v>
+        <v>1332</v>
       </c>
     </row>
     <row r="104" spans="1:2">
       <c r="A104" s="2">
-        <v>46129.0625</v>
+        <v>46130.0625</v>
       </c>
       <c r="B104">
         <v>0</v>
@@ -1218,335 +1218,335 @@
     </row>
     <row r="105" spans="1:2">
       <c r="A105" s="2">
-        <v>46129.07291666666</v>
+        <v>46130.07291666666</v>
       </c>
       <c r="B105">
-        <v>1221</v>
+        <v>1333</v>
       </c>
     </row>
     <row r="106" spans="1:2">
       <c r="A106" s="2">
-        <v>46129.08333333334</v>
+        <v>46130.08333333334</v>
       </c>
       <c r="B106">
-        <v>1220</v>
+        <v>1309</v>
       </c>
     </row>
     <row r="107" spans="1:2">
       <c r="A107" s="2">
-        <v>46129.09375</v>
+        <v>46130.09375</v>
       </c>
       <c r="B107">
-        <v>1216</v>
+        <v>1303</v>
       </c>
     </row>
     <row r="108" spans="1:2">
       <c r="A108" s="2">
-        <v>46129.10416666666</v>
+        <v>46130.10416666666</v>
       </c>
       <c r="B108">
-        <v>1217</v>
+        <v>1321</v>
       </c>
     </row>
     <row r="109" spans="1:2">
       <c r="A109" s="2">
-        <v>46129.11458333334</v>
+        <v>46130.11458333334</v>
       </c>
       <c r="B109">
-        <v>0</v>
+        <v>1323</v>
       </c>
     </row>
     <row r="110" spans="1:2">
       <c r="A110" s="2">
-        <v>46129.125</v>
+        <v>46130.125</v>
       </c>
       <c r="B110">
-        <v>1220</v>
+        <v>1326</v>
       </c>
     </row>
     <row r="111" spans="1:2">
       <c r="A111" s="2">
-        <v>46129.13541666666</v>
+        <v>46130.13541666666</v>
       </c>
       <c r="B111">
-        <v>1218</v>
+        <v>1321</v>
       </c>
     </row>
     <row r="112" spans="1:2">
       <c r="A112" s="2">
-        <v>46129.14583333334</v>
+        <v>46130.14583333334</v>
       </c>
       <c r="B112">
-        <v>0</v>
+        <v>1315</v>
       </c>
     </row>
     <row r="113" spans="1:2">
       <c r="A113" s="2">
-        <v>46129.15625</v>
+        <v>46130.15625</v>
       </c>
       <c r="B113">
-        <v>1219</v>
+        <v>1316</v>
       </c>
     </row>
     <row r="114" spans="1:2">
       <c r="A114" s="2">
-        <v>46129.16666666666</v>
+        <v>46130.16666666666</v>
       </c>
       <c r="B114">
-        <v>1221</v>
+        <v>1320</v>
       </c>
     </row>
     <row r="115" spans="1:2">
       <c r="A115" s="2">
-        <v>46129.17708333334</v>
+        <v>46130.17708333334</v>
       </c>
       <c r="B115">
-        <v>0</v>
+        <v>1327</v>
       </c>
     </row>
     <row r="116" spans="1:2">
       <c r="A116" s="2">
-        <v>46129.1875</v>
+        <v>46130.1875</v>
       </c>
       <c r="B116">
-        <v>1222</v>
+        <v>1330</v>
       </c>
     </row>
     <row r="117" spans="1:2">
       <c r="A117" s="2">
-        <v>46129.19791666666</v>
+        <v>46130.19791666666</v>
       </c>
       <c r="B117">
-        <v>1223</v>
+        <v>1329</v>
       </c>
     </row>
     <row r="118" spans="1:2">
       <c r="A118" s="2">
-        <v>46129.20833333334</v>
+        <v>46130.20833333334</v>
       </c>
       <c r="B118">
-        <v>1236</v>
+        <v>1369</v>
       </c>
     </row>
     <row r="119" spans="1:2">
       <c r="A119" s="2">
-        <v>46129.21875</v>
+        <v>46130.21875</v>
       </c>
       <c r="B119">
-        <v>1237</v>
+        <v>1371</v>
       </c>
     </row>
     <row r="120" spans="1:2">
       <c r="A120" s="2">
-        <v>46129.22916666666</v>
+        <v>46130.22916666666</v>
       </c>
       <c r="B120">
-        <v>1239</v>
+        <v>1362</v>
       </c>
     </row>
     <row r="121" spans="1:2">
       <c r="A121" s="2">
-        <v>46129.23958333334</v>
+        <v>46130.23958333334</v>
       </c>
       <c r="B121">
-        <v>1241</v>
+        <v>1360</v>
       </c>
     </row>
     <row r="122" spans="1:2">
       <c r="A122" s="2">
-        <v>46129.25</v>
+        <v>46130.25</v>
       </c>
       <c r="B122">
-        <v>1320</v>
+        <v>1406</v>
       </c>
     </row>
     <row r="123" spans="1:2">
       <c r="A123" s="2">
-        <v>46129.26041666666</v>
+        <v>46130.26041666666</v>
       </c>
       <c r="B123">
-        <v>1321</v>
+        <v>1415</v>
       </c>
     </row>
     <row r="124" spans="1:2">
       <c r="A124" s="2">
-        <v>46129.27083333334</v>
+        <v>46130.27083333334</v>
       </c>
       <c r="B124">
-        <v>1319</v>
+        <v>0</v>
       </c>
     </row>
     <row r="125" spans="1:2">
       <c r="A125" s="2">
-        <v>46129.28125</v>
+        <v>46130.28125</v>
       </c>
       <c r="B125">
-        <v>1324</v>
+        <v>1388</v>
       </c>
     </row>
     <row r="126" spans="1:2">
       <c r="A126" s="2">
-        <v>46129.29166666666</v>
+        <v>46130.29166666666</v>
       </c>
       <c r="B126">
-        <v>1328</v>
+        <v>1373</v>
       </c>
     </row>
     <row r="127" spans="1:2">
       <c r="A127" s="2">
-        <v>46129.30208333334</v>
+        <v>46130.30208333334</v>
       </c>
       <c r="B127">
-        <v>1316</v>
+        <v>1411</v>
       </c>
     </row>
     <row r="128" spans="1:2">
       <c r="A128" s="2">
-        <v>46129.3125</v>
+        <v>46130.3125</v>
       </c>
       <c r="B128">
-        <v>1312</v>
+        <v>1416</v>
       </c>
     </row>
     <row r="129" spans="1:2">
       <c r="A129" s="2">
-        <v>46129.32291666666</v>
+        <v>46130.32291666666</v>
       </c>
       <c r="B129">
-        <v>1313</v>
+        <v>1418</v>
       </c>
     </row>
     <row r="130" spans="1:2">
       <c r="A130" s="2">
-        <v>46129.33333333334</v>
+        <v>46130.33333333334</v>
       </c>
       <c r="B130">
-        <v>1291</v>
+        <v>1297</v>
       </c>
     </row>
     <row r="131" spans="1:2">
       <c r="A131" s="2">
-        <v>46129.34375</v>
+        <v>46130.34375</v>
       </c>
       <c r="B131">
-        <v>1293</v>
+        <v>1282</v>
       </c>
     </row>
     <row r="132" spans="1:2">
       <c r="A132" s="2">
-        <v>46129.35416666666</v>
+        <v>46130.35416666666</v>
       </c>
       <c r="B132">
-        <v>1287</v>
+        <v>1283</v>
       </c>
     </row>
     <row r="133" spans="1:2">
       <c r="A133" s="2">
-        <v>46129.36458333334</v>
+        <v>46130.36458333334</v>
       </c>
       <c r="B133">
-        <v>0</v>
+        <v>1258</v>
       </c>
     </row>
     <row r="134" spans="1:2">
       <c r="A134" s="2">
-        <v>46129.375</v>
+        <v>46130.375</v>
       </c>
       <c r="B134">
-        <v>1026</v>
+        <v>1110</v>
       </c>
     </row>
     <row r="135" spans="1:2">
       <c r="A135" s="2">
-        <v>46129.38541666666</v>
+        <v>46130.38541666666</v>
       </c>
       <c r="B135">
-        <v>993</v>
+        <v>1092</v>
       </c>
     </row>
     <row r="136" spans="1:2">
       <c r="A136" s="2">
-        <v>46129.39583333334</v>
+        <v>46130.39583333334</v>
       </c>
       <c r="B136">
-        <v>999</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="137" spans="1:2">
       <c r="A137" s="2">
-        <v>46129.40625</v>
+        <v>46130.40625</v>
       </c>
       <c r="B137">
-        <v>0</v>
+        <v>1040</v>
       </c>
     </row>
     <row r="138" spans="1:2">
       <c r="A138" s="2">
-        <v>46129.41666666666</v>
+        <v>46130.41666666666</v>
       </c>
       <c r="B138">
-        <v>911</v>
+        <v>853</v>
       </c>
     </row>
     <row r="139" spans="1:2">
       <c r="A139" s="2">
-        <v>46129.42708333334</v>
+        <v>46130.42708333334</v>
       </c>
       <c r="B139">
-        <v>900</v>
+        <v>840</v>
       </c>
     </row>
     <row r="140" spans="1:2">
       <c r="A140" s="2">
-        <v>46129.4375</v>
+        <v>46130.4375</v>
       </c>
       <c r="B140">
-        <v>903</v>
+        <v>839</v>
       </c>
     </row>
     <row r="141" spans="1:2">
       <c r="A141" s="2">
-        <v>46129.44791666666</v>
+        <v>46130.44791666666</v>
       </c>
       <c r="B141">
-        <v>899</v>
+        <v>790</v>
       </c>
     </row>
     <row r="142" spans="1:2">
       <c r="A142" s="2">
-        <v>46129.45833333334</v>
+        <v>46130.45833333334</v>
       </c>
       <c r="B142">
-        <v>876</v>
+        <v>693</v>
       </c>
     </row>
     <row r="143" spans="1:2">
       <c r="A143" s="2">
-        <v>46129.46875</v>
+        <v>46130.46875</v>
       </c>
       <c r="B143">
-        <v>866</v>
+        <v>681</v>
       </c>
     </row>
     <row r="144" spans="1:2">
       <c r="A144" s="2">
-        <v>46129.47916666666</v>
+        <v>46130.47916666666</v>
       </c>
       <c r="B144">
-        <v>0</v>
+        <v>680</v>
       </c>
     </row>
     <row r="145" spans="1:2">
       <c r="A145" s="2">
-        <v>46129.48958333334</v>
+        <v>46130.48958333334</v>
       </c>
       <c r="B145">
-        <v>864</v>
+        <v>0</v>
       </c>
     </row>
     <row r="146" spans="1:2">
       <c r="A146" s="2">
-        <v>46129.5</v>
+        <v>46130.5</v>
       </c>
       <c r="B146">
         <v>0</v>
@@ -1554,55 +1554,55 @@
     </row>
     <row r="147" spans="1:2">
       <c r="A147" s="2">
-        <v>46129.51041666666</v>
+        <v>46130.51041666666</v>
       </c>
       <c r="B147">
-        <v>0</v>
+        <v>683</v>
       </c>
     </row>
     <row r="148" spans="1:2">
       <c r="A148" s="2">
-        <v>46129.52083333334</v>
+        <v>46130.52083333334</v>
       </c>
       <c r="B148">
-        <v>0</v>
+        <v>680</v>
       </c>
     </row>
     <row r="149" spans="1:2">
       <c r="A149" s="2">
-        <v>46129.53125</v>
+        <v>46130.53125</v>
       </c>
       <c r="B149">
-        <v>0</v>
+        <v>664</v>
       </c>
     </row>
     <row r="150" spans="1:2">
       <c r="A150" s="2">
-        <v>46129.54166666666</v>
+        <v>46130.54166666666</v>
       </c>
       <c r="B150">
-        <v>0</v>
+        <v>677</v>
       </c>
     </row>
     <row r="151" spans="1:2">
       <c r="A151" s="2">
-        <v>46129.55208333334</v>
+        <v>46130.55208333334</v>
       </c>
       <c r="B151">
-        <v>0</v>
+        <v>673</v>
       </c>
     </row>
     <row r="152" spans="1:2">
       <c r="A152" s="2">
-        <v>46129.5625</v>
+        <v>46130.5625</v>
       </c>
       <c r="B152">
-        <v>0</v>
+        <v>669</v>
       </c>
     </row>
     <row r="153" spans="1:2">
       <c r="A153" s="2">
-        <v>46129.57291666666</v>
+        <v>46130.57291666666</v>
       </c>
       <c r="B153">
         <v>0</v>
@@ -1610,95 +1610,95 @@
     </row>
     <row r="154" spans="1:2">
       <c r="A154" s="2">
-        <v>46129.58333333334</v>
+        <v>46130.58333333334</v>
       </c>
       <c r="B154">
-        <v>0</v>
+        <v>673</v>
       </c>
     </row>
     <row r="155" spans="1:2">
       <c r="A155" s="2">
-        <v>46129.59375</v>
+        <v>46130.59375</v>
       </c>
       <c r="B155">
-        <v>0</v>
+        <v>692</v>
       </c>
     </row>
     <row r="156" spans="1:2">
       <c r="A156" s="2">
-        <v>46129.60416666666</v>
+        <v>46130.60416666666</v>
       </c>
       <c r="B156">
-        <v>0</v>
+        <v>740</v>
       </c>
     </row>
     <row r="157" spans="1:2">
       <c r="A157" s="2">
-        <v>46129.61458333334</v>
+        <v>46130.61458333334</v>
       </c>
       <c r="B157">
-        <v>0</v>
+        <v>746</v>
       </c>
     </row>
     <row r="158" spans="1:2">
       <c r="A158" s="2">
-        <v>46129.625</v>
+        <v>46130.625</v>
       </c>
       <c r="B158">
-        <v>0</v>
+        <v>841</v>
       </c>
     </row>
     <row r="159" spans="1:2">
       <c r="A159" s="2">
-        <v>46129.63541666666</v>
+        <v>46130.63541666666</v>
       </c>
       <c r="B159">
-        <v>0</v>
+        <v>845</v>
       </c>
     </row>
     <row r="160" spans="1:2">
       <c r="A160" s="2">
-        <v>46129.64583333334</v>
+        <v>46130.64583333334</v>
       </c>
       <c r="B160">
-        <v>0</v>
+        <v>900</v>
       </c>
     </row>
     <row r="161" spans="1:2">
       <c r="A161" s="2">
-        <v>46129.65625</v>
+        <v>46130.65625</v>
       </c>
       <c r="B161">
-        <v>0</v>
+        <v>921</v>
       </c>
     </row>
     <row r="162" spans="1:2">
       <c r="A162" s="2">
-        <v>46129.66666666666</v>
+        <v>46130.66666666666</v>
       </c>
       <c r="B162">
-        <v>0</v>
+        <v>1138</v>
       </c>
     </row>
     <row r="163" spans="1:2">
       <c r="A163" s="2">
-        <v>46129.67708333334</v>
+        <v>46130.67708333334</v>
       </c>
       <c r="B163">
-        <v>0</v>
+        <v>1170</v>
       </c>
     </row>
     <row r="164" spans="1:2">
       <c r="A164" s="2">
-        <v>46129.6875</v>
+        <v>46130.6875</v>
       </c>
       <c r="B164">
-        <v>0</v>
+        <v>1143</v>
       </c>
     </row>
     <row r="165" spans="1:2">
       <c r="A165" s="2">
-        <v>46129.69791666666</v>
+        <v>46130.69791666666</v>
       </c>
       <c r="B165">
         <v>0</v>
@@ -1706,225 +1706,1761 @@
     </row>
     <row r="166" spans="1:2">
       <c r="A166" s="2">
-        <v>46129.70833333334</v>
+        <v>46130.70833333334</v>
       </c>
       <c r="B166">
-        <v>0</v>
+        <v>1365</v>
       </c>
     </row>
     <row r="167" spans="1:2">
       <c r="A167" s="2">
-        <v>46129.71875</v>
+        <v>46130.71875</v>
       </c>
       <c r="B167">
-        <v>0</v>
+        <v>1391</v>
       </c>
     </row>
     <row r="168" spans="1:2">
       <c r="A168" s="2">
-        <v>46129.72916666666</v>
+        <v>46130.72916666666</v>
       </c>
       <c r="B168">
-        <v>0</v>
+        <v>1392</v>
       </c>
     </row>
     <row r="169" spans="1:2">
       <c r="A169" s="2">
-        <v>46129.73958333334</v>
+        <v>46130.73958333334</v>
       </c>
       <c r="B169">
-        <v>0</v>
+        <v>1395</v>
       </c>
     </row>
     <row r="170" spans="1:2">
       <c r="A170" s="2">
-        <v>46129.75</v>
+        <v>46130.75</v>
       </c>
       <c r="B170">
-        <v>0</v>
+        <v>1465</v>
       </c>
     </row>
     <row r="171" spans="1:2">
       <c r="A171" s="2">
-        <v>46129.76041666666</v>
+        <v>46130.76041666666</v>
       </c>
       <c r="B171">
-        <v>0</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="172" spans="1:2">
       <c r="A172" s="2">
-        <v>46129.77083333334</v>
+        <v>46130.77083333334</v>
       </c>
       <c r="B172">
-        <v>0</v>
+        <v>1488</v>
       </c>
     </row>
     <row r="173" spans="1:2">
       <c r="A173" s="2">
-        <v>46129.78125</v>
+        <v>46130.78125</v>
       </c>
       <c r="B173">
-        <v>0</v>
+        <v>1485</v>
       </c>
     </row>
     <row r="174" spans="1:2">
       <c r="A174" s="2">
-        <v>46129.79166666666</v>
+        <v>46130.79166666666</v>
       </c>
       <c r="B174">
-        <v>0</v>
+        <v>1471</v>
       </c>
     </row>
     <row r="175" spans="1:2">
       <c r="A175" s="2">
-        <v>46129.80208333334</v>
+        <v>46130.80208333334</v>
       </c>
       <c r="B175">
-        <v>0</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="176" spans="1:2">
       <c r="A176" s="2">
-        <v>46129.8125</v>
+        <v>46130.8125</v>
       </c>
       <c r="B176">
-        <v>0</v>
+        <v>1476</v>
       </c>
     </row>
     <row r="177" spans="1:2">
       <c r="A177" s="2">
-        <v>46129.82291666666</v>
+        <v>46130.82291666666</v>
       </c>
       <c r="B177">
-        <v>0</v>
+        <v>1480</v>
       </c>
     </row>
     <row r="178" spans="1:2">
       <c r="A178" s="2">
-        <v>46129.83333333334</v>
+        <v>46130.83333333334</v>
       </c>
       <c r="B178">
-        <v>0</v>
+        <v>1503</v>
       </c>
     </row>
     <row r="179" spans="1:2">
       <c r="A179" s="2">
-        <v>46129.84375</v>
+        <v>46130.84375</v>
       </c>
       <c r="B179">
-        <v>0</v>
+        <v>1511</v>
       </c>
     </row>
     <row r="180" spans="1:2">
       <c r="A180" s="2">
-        <v>46129.85416666666</v>
+        <v>46130.85416666666</v>
       </c>
       <c r="B180">
-        <v>0</v>
+        <v>1505</v>
       </c>
     </row>
     <row r="181" spans="1:2">
       <c r="A181" s="2">
-        <v>46129.86458333334</v>
+        <v>46130.86458333334</v>
       </c>
       <c r="B181">
-        <v>0</v>
+        <v>1504</v>
       </c>
     </row>
     <row r="182" spans="1:2">
       <c r="A182" s="2">
-        <v>46129.875</v>
+        <v>46130.875</v>
       </c>
       <c r="B182">
-        <v>0</v>
+        <v>1524</v>
       </c>
     </row>
     <row r="183" spans="1:2">
       <c r="A183" s="2">
-        <v>46129.88541666666</v>
+        <v>46130.88541666666</v>
       </c>
       <c r="B183">
-        <v>0</v>
+        <v>1551</v>
       </c>
     </row>
     <row r="184" spans="1:2">
       <c r="A184" s="2">
-        <v>46129.89583333334</v>
+        <v>46130.89583333334</v>
       </c>
       <c r="B184">
-        <v>0</v>
+        <v>1550</v>
       </c>
     </row>
     <row r="185" spans="1:2">
       <c r="A185" s="2">
-        <v>46129.90625</v>
+        <v>46130.90625</v>
       </c>
       <c r="B185">
-        <v>0</v>
+        <v>1528</v>
       </c>
     </row>
     <row r="186" spans="1:2">
       <c r="A186" s="2">
-        <v>46129.91666666666</v>
+        <v>46130.91666666666</v>
       </c>
       <c r="B186">
-        <v>0</v>
+        <v>1543</v>
       </c>
     </row>
     <row r="187" spans="1:2">
       <c r="A187" s="2">
-        <v>46129.92708333334</v>
+        <v>46130.92708333334</v>
       </c>
       <c r="B187">
-        <v>0</v>
+        <v>1539</v>
       </c>
     </row>
     <row r="188" spans="1:2">
       <c r="A188" s="2">
-        <v>46129.9375</v>
+        <v>46130.9375</v>
       </c>
       <c r="B188">
-        <v>0</v>
+        <v>1541</v>
       </c>
     </row>
     <row r="189" spans="1:2">
       <c r="A189" s="2">
-        <v>46129.94791666666</v>
+        <v>46130.94791666666</v>
       </c>
       <c r="B189">
-        <v>0</v>
+        <v>1527</v>
       </c>
     </row>
     <row r="190" spans="1:2">
       <c r="A190" s="2">
-        <v>46129.95833333334</v>
+        <v>46130.95833333334</v>
       </c>
       <c r="B190">
-        <v>0</v>
+        <v>1502</v>
       </c>
     </row>
     <row r="191" spans="1:2">
       <c r="A191" s="2">
-        <v>46129.96875</v>
+        <v>46130.96875</v>
       </c>
       <c r="B191">
-        <v>0</v>
+        <v>1493</v>
       </c>
     </row>
     <row r="192" spans="1:2">
       <c r="A192" s="2">
-        <v>46129.97916666666</v>
+        <v>46130.97916666666</v>
       </c>
       <c r="B192">
-        <v>0</v>
+        <v>1495</v>
       </c>
     </row>
     <row r="193" spans="1:2">
       <c r="A193" s="2">
-        <v>46129.98958333334</v>
+        <v>46130.98958333334</v>
       </c>
       <c r="B193">
+        <v>1492</v>
+      </c>
+    </row>
+    <row r="194" spans="1:2">
+      <c r="A194" s="2">
+        <v>46131</v>
+      </c>
+      <c r="B194">
+        <v>1368</v>
+      </c>
+    </row>
+    <row r="195" spans="1:2">
+      <c r="A195" s="2">
+        <v>46131.01041666666</v>
+      </c>
+      <c r="B195">
+        <v>1344</v>
+      </c>
+    </row>
+    <row r="196" spans="1:2">
+      <c r="A196" s="2">
+        <v>46131.02083333334</v>
+      </c>
+      <c r="B196">
+        <v>1342</v>
+      </c>
+    </row>
+    <row r="197" spans="1:2">
+      <c r="A197" s="2">
+        <v>46131.03125</v>
+      </c>
+      <c r="B197">
+        <v>1341</v>
+      </c>
+    </row>
+    <row r="198" spans="1:2">
+      <c r="A198" s="2">
+        <v>46131.04166666666</v>
+      </c>
+      <c r="B198">
+        <v>1362</v>
+      </c>
+    </row>
+    <row r="199" spans="1:2">
+      <c r="A199" s="2">
+        <v>46131.05208333334</v>
+      </c>
+      <c r="B199">
+        <v>1331</v>
+      </c>
+    </row>
+    <row r="200" spans="1:2">
+      <c r="A200" s="2">
+        <v>46131.0625</v>
+      </c>
+      <c r="B200">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="201" spans="1:2">
+      <c r="A201" s="2">
+        <v>46131.07291666666</v>
+      </c>
+      <c r="B201">
+        <v>1329</v>
+      </c>
+    </row>
+    <row r="202" spans="1:2">
+      <c r="A202" s="2">
+        <v>46131.08333333334</v>
+      </c>
+      <c r="B202">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="203" spans="1:2">
+      <c r="A203" s="2">
+        <v>46131.09375</v>
+      </c>
+      <c r="B203">
+        <v>1326</v>
+      </c>
+    </row>
+    <row r="204" spans="1:2">
+      <c r="A204" s="2">
+        <v>46131.10416666666</v>
+      </c>
+      <c r="B204">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="205" spans="1:2">
+      <c r="A205" s="2">
+        <v>46131.11458333334</v>
+      </c>
+      <c r="B205">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="206" spans="1:2">
+      <c r="A206" s="2">
+        <v>46131.125</v>
+      </c>
+      <c r="B206">
+        <v>1325</v>
+      </c>
+    </row>
+    <row r="207" spans="1:2">
+      <c r="A207" s="2">
+        <v>46131.13541666666</v>
+      </c>
+      <c r="B207">
+        <v>1338</v>
+      </c>
+    </row>
+    <row r="208" spans="1:2">
+      <c r="A208" s="2">
+        <v>46131.14583333334</v>
+      </c>
+      <c r="B208">
+        <v>1340</v>
+      </c>
+    </row>
+    <row r="209" spans="1:2">
+      <c r="A209" s="2">
+        <v>46131.15625</v>
+      </c>
+      <c r="B209">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="210" spans="1:2">
+      <c r="A210" s="2">
+        <v>46131.16666666666</v>
+      </c>
+      <c r="B210">
+        <v>1334</v>
+      </c>
+    </row>
+    <row r="211" spans="1:2">
+      <c r="A211" s="2">
+        <v>46131.17708333334</v>
+      </c>
+      <c r="B211">
+        <v>1333</v>
+      </c>
+    </row>
+    <row r="212" spans="1:2">
+      <c r="A212" s="2">
+        <v>46131.1875</v>
+      </c>
+      <c r="B212">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="213" spans="1:2">
+      <c r="A213" s="2">
+        <v>46131.19791666666</v>
+      </c>
+      <c r="B213">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="214" spans="1:2">
+      <c r="A214" s="2">
+        <v>46131.20833333334</v>
+      </c>
+      <c r="B214">
+        <v>1350</v>
+      </c>
+    </row>
+    <row r="215" spans="1:2">
+      <c r="A215" s="2">
+        <v>46131.21875</v>
+      </c>
+      <c r="B215">
+        <v>1347</v>
+      </c>
+    </row>
+    <row r="216" spans="1:2">
+      <c r="A216" s="2">
+        <v>46131.22916666666</v>
+      </c>
+      <c r="B216">
+        <v>1358</v>
+      </c>
+    </row>
+    <row r="217" spans="1:2">
+      <c r="A217" s="2">
+        <v>46131.23958333334</v>
+      </c>
+      <c r="B217">
+        <v>1359</v>
+      </c>
+    </row>
+    <row r="218" spans="1:2">
+      <c r="A218" s="2">
+        <v>46131.25</v>
+      </c>
+      <c r="B218">
+        <v>1384</v>
+      </c>
+    </row>
+    <row r="219" spans="1:2">
+      <c r="A219" s="2">
+        <v>46131.26041666666</v>
+      </c>
+      <c r="B219">
+        <v>1386</v>
+      </c>
+    </row>
+    <row r="220" spans="1:2">
+      <c r="A220" s="2">
+        <v>46131.27083333334</v>
+      </c>
+      <c r="B220">
+        <v>1385</v>
+      </c>
+    </row>
+    <row r="221" spans="1:2">
+      <c r="A221" s="2">
+        <v>46131.28125</v>
+      </c>
+      <c r="B221">
+        <v>1386</v>
+      </c>
+    </row>
+    <row r="222" spans="1:2">
+      <c r="A222" s="2">
+        <v>46131.29166666666</v>
+      </c>
+      <c r="B222">
+        <v>1227</v>
+      </c>
+    </row>
+    <row r="223" spans="1:2">
+      <c r="A223" s="2">
+        <v>46131.30208333334</v>
+      </c>
+      <c r="B223">
+        <v>1218</v>
+      </c>
+    </row>
+    <row r="224" spans="1:2">
+      <c r="A224" s="2">
+        <v>46131.3125</v>
+      </c>
+      <c r="B224">
+        <v>1221</v>
+      </c>
+    </row>
+    <row r="225" spans="1:2">
+      <c r="A225" s="2">
+        <v>46131.32291666666</v>
+      </c>
+      <c r="B225">
+        <v>1217</v>
+      </c>
+    </row>
+    <row r="226" spans="1:2">
+      <c r="A226" s="2">
+        <v>46131.33333333334</v>
+      </c>
+      <c r="B226">
+        <v>1027</v>
+      </c>
+    </row>
+    <row r="227" spans="1:2">
+      <c r="A227" s="2">
+        <v>46131.34375</v>
+      </c>
+      <c r="B227">
+        <v>1018</v>
+      </c>
+    </row>
+    <row r="228" spans="1:2">
+      <c r="A228" s="2">
+        <v>46131.35416666666</v>
+      </c>
+      <c r="B228">
+        <v>1013</v>
+      </c>
+    </row>
+    <row r="229" spans="1:2">
+      <c r="A229" s="2">
+        <v>46131.36458333334</v>
+      </c>
+      <c r="B229">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="230" spans="1:2">
+      <c r="A230" s="2">
+        <v>46131.375</v>
+      </c>
+      <c r="B230">
+        <v>954</v>
+      </c>
+    </row>
+    <row r="231" spans="1:2">
+      <c r="A231" s="2">
+        <v>46131.38541666666</v>
+      </c>
+      <c r="B231">
+        <v>950</v>
+      </c>
+    </row>
+    <row r="232" spans="1:2">
+      <c r="A232" s="2">
+        <v>46131.39583333334</v>
+      </c>
+      <c r="B232">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="233" spans="1:2">
+      <c r="A233" s="2">
+        <v>46131.40625</v>
+      </c>
+      <c r="B233">
+        <v>952</v>
+      </c>
+    </row>
+    <row r="234" spans="1:2">
+      <c r="A234" s="2">
+        <v>46131.41666666666</v>
+      </c>
+      <c r="B234">
+        <v>848</v>
+      </c>
+    </row>
+    <row r="235" spans="1:2">
+      <c r="A235" s="2">
+        <v>46131.42708333334</v>
+      </c>
+      <c r="B235">
+        <v>839</v>
+      </c>
+    </row>
+    <row r="236" spans="1:2">
+      <c r="A236" s="2">
+        <v>46131.4375</v>
+      </c>
+      <c r="B236">
+        <v>832</v>
+      </c>
+    </row>
+    <row r="237" spans="1:2">
+      <c r="A237" s="2">
+        <v>46131.44791666666</v>
+      </c>
+      <c r="B237">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="238" spans="1:2">
+      <c r="A238" s="2">
+        <v>46131.45833333334</v>
+      </c>
+      <c r="B238">
+        <v>837</v>
+      </c>
+    </row>
+    <row r="239" spans="1:2">
+      <c r="A239" s="2">
+        <v>46131.46875</v>
+      </c>
+      <c r="B239">
+        <v>816</v>
+      </c>
+    </row>
+    <row r="240" spans="1:2">
+      <c r="A240" s="2">
+        <v>46131.47916666666</v>
+      </c>
+      <c r="B240">
+        <v>806</v>
+      </c>
+    </row>
+    <row r="241" spans="1:2">
+      <c r="A241" s="2">
+        <v>46131.48958333334</v>
+      </c>
+      <c r="B241">
+        <v>800</v>
+      </c>
+    </row>
+    <row r="242" spans="1:2">
+      <c r="A242" s="2">
+        <v>46131.5</v>
+      </c>
+      <c r="B242">
+        <v>807</v>
+      </c>
+    </row>
+    <row r="243" spans="1:2">
+      <c r="A243" s="2">
+        <v>46131.51041666666</v>
+      </c>
+      <c r="B243">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="244" spans="1:2">
+      <c r="A244" s="2">
+        <v>46131.52083333334</v>
+      </c>
+      <c r="B244">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="245" spans="1:2">
+      <c r="A245" s="2">
+        <v>46131.53125</v>
+      </c>
+      <c r="B245">
+        <v>806</v>
+      </c>
+    </row>
+    <row r="246" spans="1:2">
+      <c r="A246" s="2">
+        <v>46131.54166666666</v>
+      </c>
+      <c r="B246">
+        <v>811</v>
+      </c>
+    </row>
+    <row r="247" spans="1:2">
+      <c r="A247" s="2">
+        <v>46131.55208333334</v>
+      </c>
+      <c r="B247">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="248" spans="1:2">
+      <c r="A248" s="2">
+        <v>46131.5625</v>
+      </c>
+      <c r="B248">
+        <v>818</v>
+      </c>
+    </row>
+    <row r="249" spans="1:2">
+      <c r="A249" s="2">
+        <v>46131.57291666666</v>
+      </c>
+      <c r="B249">
+        <v>816</v>
+      </c>
+    </row>
+    <row r="250" spans="1:2">
+      <c r="A250" s="2">
+        <v>46131.58333333334</v>
+      </c>
+      <c r="B250">
+        <v>801</v>
+      </c>
+    </row>
+    <row r="251" spans="1:2">
+      <c r="A251" s="2">
+        <v>46131.59375</v>
+      </c>
+      <c r="B251">
+        <v>799</v>
+      </c>
+    </row>
+    <row r="252" spans="1:2">
+      <c r="A252" s="2">
+        <v>46131.60416666666</v>
+      </c>
+      <c r="B252">
+        <v>809</v>
+      </c>
+    </row>
+    <row r="253" spans="1:2">
+      <c r="A253" s="2">
+        <v>46131.61458333334</v>
+      </c>
+      <c r="B253">
+        <v>813</v>
+      </c>
+    </row>
+    <row r="254" spans="1:2">
+      <c r="A254" s="2">
+        <v>46131.625</v>
+      </c>
+      <c r="B254">
+        <v>923</v>
+      </c>
+    </row>
+    <row r="255" spans="1:2">
+      <c r="A255" s="2">
+        <v>46131.63541666666</v>
+      </c>
+      <c r="B255">
+        <v>926</v>
+      </c>
+    </row>
+    <row r="256" spans="1:2">
+      <c r="A256" s="2">
+        <v>46131.64583333334</v>
+      </c>
+      <c r="B256">
+        <v>925</v>
+      </c>
+    </row>
+    <row r="257" spans="1:2">
+      <c r="A257" s="2">
+        <v>46131.65625</v>
+      </c>
+      <c r="B257">
+        <v>933</v>
+      </c>
+    </row>
+    <row r="258" spans="1:2">
+      <c r="A258" s="2">
+        <v>46131.66666666666</v>
+      </c>
+      <c r="B258">
+        <v>1193</v>
+      </c>
+    </row>
+    <row r="259" spans="1:2">
+      <c r="A259" s="2">
+        <v>46131.67708333334</v>
+      </c>
+      <c r="B259">
+        <v>1212</v>
+      </c>
+    </row>
+    <row r="260" spans="1:2">
+      <c r="A260" s="2">
+        <v>46131.6875</v>
+      </c>
+      <c r="B260">
+        <v>1213</v>
+      </c>
+    </row>
+    <row r="261" spans="1:2">
+      <c r="A261" s="2">
+        <v>46131.69791666666</v>
+      </c>
+      <c r="B261">
+        <v>1221</v>
+      </c>
+    </row>
+    <row r="262" spans="1:2">
+      <c r="A262" s="2">
+        <v>46131.70833333334</v>
+      </c>
+      <c r="B262">
+        <v>1359</v>
+      </c>
+    </row>
+    <row r="263" spans="1:2">
+      <c r="A263" s="2">
+        <v>46131.71875</v>
+      </c>
+      <c r="B263">
+        <v>1390</v>
+      </c>
+    </row>
+    <row r="264" spans="1:2">
+      <c r="A264" s="2">
+        <v>46131.72916666666</v>
+      </c>
+      <c r="B264">
+        <v>1392</v>
+      </c>
+    </row>
+    <row r="265" spans="1:2">
+      <c r="A265" s="2">
+        <v>46131.73958333334</v>
+      </c>
+      <c r="B265">
+        <v>1393</v>
+      </c>
+    </row>
+    <row r="266" spans="1:2">
+      <c r="A266" s="2">
+        <v>46131.75</v>
+      </c>
+      <c r="B266">
+        <v>1593</v>
+      </c>
+    </row>
+    <row r="267" spans="1:2">
+      <c r="A267" s="2">
+        <v>46131.76041666666</v>
+      </c>
+      <c r="B267">
+        <v>1605</v>
+      </c>
+    </row>
+    <row r="268" spans="1:2">
+      <c r="A268" s="2">
+        <v>46131.77083333334</v>
+      </c>
+      <c r="B268">
+        <v>1606</v>
+      </c>
+    </row>
+    <row r="269" spans="1:2">
+      <c r="A269" s="2">
+        <v>46131.78125</v>
+      </c>
+      <c r="B269">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="270" spans="1:2">
+      <c r="A270" s="2">
+        <v>46131.79166666666</v>
+      </c>
+      <c r="B270">
+        <v>1607</v>
+      </c>
+    </row>
+    <row r="271" spans="1:2">
+      <c r="A271" s="2">
+        <v>46131.80208333334</v>
+      </c>
+      <c r="B271">
+        <v>1614</v>
+      </c>
+    </row>
+    <row r="272" spans="1:2">
+      <c r="A272" s="2">
+        <v>46131.8125</v>
+      </c>
+      <c r="B272">
+        <v>1618</v>
+      </c>
+    </row>
+    <row r="273" spans="1:2">
+      <c r="A273" s="2">
+        <v>46131.82291666666</v>
+      </c>
+      <c r="B273">
+        <v>1616</v>
+      </c>
+    </row>
+    <row r="274" spans="1:2">
+      <c r="A274" s="2">
+        <v>46131.83333333334</v>
+      </c>
+      <c r="B274">
+        <v>1609</v>
+      </c>
+    </row>
+    <row r="275" spans="1:2">
+      <c r="A275" s="2">
+        <v>46131.84375</v>
+      </c>
+      <c r="B275">
+        <v>1606</v>
+      </c>
+    </row>
+    <row r="276" spans="1:2">
+      <c r="A276" s="2">
+        <v>46131.85416666666</v>
+      </c>
+      <c r="B276">
+        <v>1575</v>
+      </c>
+    </row>
+    <row r="277" spans="1:2">
+      <c r="A277" s="2">
+        <v>46131.86458333334</v>
+      </c>
+      <c r="B277">
+        <v>1572</v>
+      </c>
+    </row>
+    <row r="278" spans="1:2">
+      <c r="A278" s="2">
+        <v>46131.875</v>
+      </c>
+      <c r="B278">
+        <v>1601</v>
+      </c>
+    </row>
+    <row r="279" spans="1:2">
+      <c r="A279" s="2">
+        <v>46131.88541666666</v>
+      </c>
+      <c r="B279">
+        <v>1614</v>
+      </c>
+    </row>
+    <row r="280" spans="1:2">
+      <c r="A280" s="2">
+        <v>46131.89583333334</v>
+      </c>
+      <c r="B280">
+        <v>1615</v>
+      </c>
+    </row>
+    <row r="281" spans="1:2">
+      <c r="A281" s="2">
+        <v>46131.90625</v>
+      </c>
+      <c r="B281">
+        <v>1609</v>
+      </c>
+    </row>
+    <row r="282" spans="1:2">
+      <c r="A282" s="2">
+        <v>46131.91666666666</v>
+      </c>
+      <c r="B282">
+        <v>1557</v>
+      </c>
+    </row>
+    <row r="283" spans="1:2">
+      <c r="A283" s="2">
+        <v>46131.92708333334</v>
+      </c>
+      <c r="B283">
+        <v>1545</v>
+      </c>
+    </row>
+    <row r="284" spans="1:2">
+      <c r="A284" s="2">
+        <v>46131.9375</v>
+      </c>
+      <c r="B284">
+        <v>1544</v>
+      </c>
+    </row>
+    <row r="285" spans="1:2">
+      <c r="A285" s="2">
+        <v>46131.94791666666</v>
+      </c>
+      <c r="B285">
+        <v>1540</v>
+      </c>
+    </row>
+    <row r="286" spans="1:2">
+      <c r="A286" s="2">
+        <v>46131.95833333334</v>
+      </c>
+      <c r="B286">
+        <v>1372</v>
+      </c>
+    </row>
+    <row r="287" spans="1:2">
+      <c r="A287" s="2">
+        <v>46131.96875</v>
+      </c>
+      <c r="B287">
+        <v>1321</v>
+      </c>
+    </row>
+    <row r="288" spans="1:2">
+      <c r="A288" s="2">
+        <v>46131.97916666666</v>
+      </c>
+      <c r="B288">
+        <v>1322</v>
+      </c>
+    </row>
+    <row r="289" spans="1:2">
+      <c r="A289" s="2">
+        <v>46131.98958333334</v>
+      </c>
+      <c r="B289">
+        <v>1311</v>
+      </c>
+    </row>
+    <row r="290" spans="1:2">
+      <c r="A290" s="2">
+        <v>46132</v>
+      </c>
+      <c r="B290">
+        <v>1298</v>
+      </c>
+    </row>
+    <row r="291" spans="1:2">
+      <c r="A291" s="2">
+        <v>46132.01041666666</v>
+      </c>
+      <c r="B291">
+        <v>1290</v>
+      </c>
+    </row>
+    <row r="292" spans="1:2">
+      <c r="A292" s="2">
+        <v>46132.02083333334</v>
+      </c>
+      <c r="B292">
+        <v>1322</v>
+      </c>
+    </row>
+    <row r="293" spans="1:2">
+      <c r="A293" s="2">
+        <v>46132.03125</v>
+      </c>
+      <c r="B293">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="294" spans="1:2">
+      <c r="A294" s="2">
+        <v>46132.04166666666</v>
+      </c>
+      <c r="B294">
+        <v>1230</v>
+      </c>
+    </row>
+    <row r="295" spans="1:2">
+      <c r="A295" s="2">
+        <v>46132.05208333334</v>
+      </c>
+      <c r="B295">
+        <v>1226</v>
+      </c>
+    </row>
+    <row r="296" spans="1:2">
+      <c r="A296" s="2">
+        <v>46132.0625</v>
+      </c>
+      <c r="B296">
+        <v>1218</v>
+      </c>
+    </row>
+    <row r="297" spans="1:2">
+      <c r="A297" s="2">
+        <v>46132.07291666666</v>
+      </c>
+      <c r="B297">
+        <v>1156</v>
+      </c>
+    </row>
+    <row r="298" spans="1:2">
+      <c r="A298" s="2">
+        <v>46132.08333333334</v>
+      </c>
+      <c r="B298">
+        <v>1045</v>
+      </c>
+    </row>
+    <row r="299" spans="1:2">
+      <c r="A299" s="2">
+        <v>46132.09375</v>
+      </c>
+      <c r="B299">
+        <v>1038</v>
+      </c>
+    </row>
+    <row r="300" spans="1:2">
+      <c r="A300" s="2">
+        <v>46132.10416666666</v>
+      </c>
+      <c r="B300">
+        <v>1037</v>
+      </c>
+    </row>
+    <row r="301" spans="1:2">
+      <c r="A301" s="2">
+        <v>46132.11458333334</v>
+      </c>
+      <c r="B301">
+        <v>1054</v>
+      </c>
+    </row>
+    <row r="302" spans="1:2">
+      <c r="A302" s="2">
+        <v>46132.125</v>
+      </c>
+      <c r="B302">
+        <v>1091</v>
+      </c>
+    </row>
+    <row r="303" spans="1:2">
+      <c r="A303" s="2">
+        <v>46132.13541666666</v>
+      </c>
+      <c r="B303">
+        <v>1094</v>
+      </c>
+    </row>
+    <row r="304" spans="1:2">
+      <c r="A304" s="2">
+        <v>46132.14583333334</v>
+      </c>
+      <c r="B304">
+        <v>1079</v>
+      </c>
+    </row>
+    <row r="305" spans="1:2">
+      <c r="A305" s="2">
+        <v>46132.15625</v>
+      </c>
+      <c r="B305">
+        <v>1075</v>
+      </c>
+    </row>
+    <row r="306" spans="1:2">
+      <c r="A306" s="2">
+        <v>46132.16666666666</v>
+      </c>
+      <c r="B306">
+        <v>1214</v>
+      </c>
+    </row>
+    <row r="307" spans="1:2">
+      <c r="A307" s="2">
+        <v>46132.17708333334</v>
+      </c>
+      <c r="B307">
+        <v>1225</v>
+      </c>
+    </row>
+    <row r="308" spans="1:2">
+      <c r="A308" s="2">
+        <v>46132.1875</v>
+      </c>
+      <c r="B308">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="309" spans="1:2">
+      <c r="A309" s="2">
+        <v>46132.19791666666</v>
+      </c>
+      <c r="B309">
+        <v>1227</v>
+      </c>
+    </row>
+    <row r="310" spans="1:2">
+      <c r="A310" s="2">
+        <v>46132.20833333334</v>
+      </c>
+      <c r="B310">
+        <v>1176</v>
+      </c>
+    </row>
+    <row r="311" spans="1:2">
+      <c r="A311" s="2">
+        <v>46132.21875</v>
+      </c>
+      <c r="B311">
+        <v>1177</v>
+      </c>
+    </row>
+    <row r="312" spans="1:2">
+      <c r="A312" s="2">
+        <v>46132.22916666666</v>
+      </c>
+      <c r="B312">
+        <v>1197</v>
+      </c>
+    </row>
+    <row r="313" spans="1:2">
+      <c r="A313" s="2">
+        <v>46132.23958333334</v>
+      </c>
+      <c r="B313">
+        <v>1198</v>
+      </c>
+    </row>
+    <row r="314" spans="1:2">
+      <c r="A314" s="2">
+        <v>46132.25</v>
+      </c>
+      <c r="B314">
+        <v>1218</v>
+      </c>
+    </row>
+    <row r="315" spans="1:2">
+      <c r="A315" s="2">
+        <v>46132.26041666666</v>
+      </c>
+      <c r="B315">
+        <v>1217</v>
+      </c>
+    </row>
+    <row r="316" spans="1:2">
+      <c r="A316" s="2">
+        <v>46132.27083333334</v>
+      </c>
+      <c r="B316">
+        <v>1221</v>
+      </c>
+    </row>
+    <row r="317" spans="1:2">
+      <c r="A317" s="2">
+        <v>46132.28125</v>
+      </c>
+      <c r="B317">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="318" spans="1:2">
+      <c r="A318" s="2">
+        <v>46132.29166666666</v>
+      </c>
+      <c r="B318">
+        <v>1166</v>
+      </c>
+    </row>
+    <row r="319" spans="1:2">
+      <c r="A319" s="2">
+        <v>46132.30208333334</v>
+      </c>
+      <c r="B319">
+        <v>1193</v>
+      </c>
+    </row>
+    <row r="320" spans="1:2">
+      <c r="A320" s="2">
+        <v>46132.3125</v>
+      </c>
+      <c r="B320">
+        <v>1203</v>
+      </c>
+    </row>
+    <row r="321" spans="1:2">
+      <c r="A321" s="2">
+        <v>46132.32291666666</v>
+      </c>
+      <c r="B321">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="322" spans="1:2">
+      <c r="A322" s="2">
+        <v>46132.33333333334</v>
+      </c>
+      <c r="B322">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="323" spans="1:2">
+      <c r="A323" s="2">
+        <v>46132.34375</v>
+      </c>
+      <c r="B323">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="324" spans="1:2">
+      <c r="A324" s="2">
+        <v>46132.35416666666</v>
+      </c>
+      <c r="B324">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="325" spans="1:2">
+      <c r="A325" s="2">
+        <v>46132.36458333334</v>
+      </c>
+      <c r="B325">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="326" spans="1:2">
+      <c r="A326" s="2">
+        <v>46132.375</v>
+      </c>
+      <c r="B326">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="327" spans="1:2">
+      <c r="A327" s="2">
+        <v>46132.38541666666</v>
+      </c>
+      <c r="B327">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="328" spans="1:2">
+      <c r="A328" s="2">
+        <v>46132.39583333334</v>
+      </c>
+      <c r="B328">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="329" spans="1:2">
+      <c r="A329" s="2">
+        <v>46132.40625</v>
+      </c>
+      <c r="B329">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="330" spans="1:2">
+      <c r="A330" s="2">
+        <v>46132.41666666666</v>
+      </c>
+      <c r="B330">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="331" spans="1:2">
+      <c r="A331" s="2">
+        <v>46132.42708333334</v>
+      </c>
+      <c r="B331">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="332" spans="1:2">
+      <c r="A332" s="2">
+        <v>46132.4375</v>
+      </c>
+      <c r="B332">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="333" spans="1:2">
+      <c r="A333" s="2">
+        <v>46132.44791666666</v>
+      </c>
+      <c r="B333">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="334" spans="1:2">
+      <c r="A334" s="2">
+        <v>46132.45833333334</v>
+      </c>
+      <c r="B334">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="335" spans="1:2">
+      <c r="A335" s="2">
+        <v>46132.46875</v>
+      </c>
+      <c r="B335">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="336" spans="1:2">
+      <c r="A336" s="2">
+        <v>46132.47916666666</v>
+      </c>
+      <c r="B336">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="337" spans="1:2">
+      <c r="A337" s="2">
+        <v>46132.48958333334</v>
+      </c>
+      <c r="B337">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="338" spans="1:2">
+      <c r="A338" s="2">
+        <v>46132.5</v>
+      </c>
+      <c r="B338">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="339" spans="1:2">
+      <c r="A339" s="2">
+        <v>46132.51041666666</v>
+      </c>
+      <c r="B339">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="340" spans="1:2">
+      <c r="A340" s="2">
+        <v>46132.52083333334</v>
+      </c>
+      <c r="B340">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="341" spans="1:2">
+      <c r="A341" s="2">
+        <v>46132.53125</v>
+      </c>
+      <c r="B341">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="342" spans="1:2">
+      <c r="A342" s="2">
+        <v>46132.54166666666</v>
+      </c>
+      <c r="B342">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="343" spans="1:2">
+      <c r="A343" s="2">
+        <v>46132.55208333334</v>
+      </c>
+      <c r="B343">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="344" spans="1:2">
+      <c r="A344" s="2">
+        <v>46132.5625</v>
+      </c>
+      <c r="B344">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="345" spans="1:2">
+      <c r="A345" s="2">
+        <v>46132.57291666666</v>
+      </c>
+      <c r="B345">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="346" spans="1:2">
+      <c r="A346" s="2">
+        <v>46132.58333333334</v>
+      </c>
+      <c r="B346">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="347" spans="1:2">
+      <c r="A347" s="2">
+        <v>46132.59375</v>
+      </c>
+      <c r="B347">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="348" spans="1:2">
+      <c r="A348" s="2">
+        <v>46132.60416666666</v>
+      </c>
+      <c r="B348">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="349" spans="1:2">
+      <c r="A349" s="2">
+        <v>46132.61458333334</v>
+      </c>
+      <c r="B349">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="350" spans="1:2">
+      <c r="A350" s="2">
+        <v>46132.625</v>
+      </c>
+      <c r="B350">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="351" spans="1:2">
+      <c r="A351" s="2">
+        <v>46132.63541666666</v>
+      </c>
+      <c r="B351">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="352" spans="1:2">
+      <c r="A352" s="2">
+        <v>46132.64583333334</v>
+      </c>
+      <c r="B352">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="353" spans="1:2">
+      <c r="A353" s="2">
+        <v>46132.65625</v>
+      </c>
+      <c r="B353">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="354" spans="1:2">
+      <c r="A354" s="2">
+        <v>46132.66666666666</v>
+      </c>
+      <c r="B354">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="355" spans="1:2">
+      <c r="A355" s="2">
+        <v>46132.67708333334</v>
+      </c>
+      <c r="B355">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="356" spans="1:2">
+      <c r="A356" s="2">
+        <v>46132.6875</v>
+      </c>
+      <c r="B356">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="357" spans="1:2">
+      <c r="A357" s="2">
+        <v>46132.69791666666</v>
+      </c>
+      <c r="B357">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="358" spans="1:2">
+      <c r="A358" s="2">
+        <v>46132.70833333334</v>
+      </c>
+      <c r="B358">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="359" spans="1:2">
+      <c r="A359" s="2">
+        <v>46132.71875</v>
+      </c>
+      <c r="B359">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="360" spans="1:2">
+      <c r="A360" s="2">
+        <v>46132.72916666666</v>
+      </c>
+      <c r="B360">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="361" spans="1:2">
+      <c r="A361" s="2">
+        <v>46132.73958333334</v>
+      </c>
+      <c r="B361">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="362" spans="1:2">
+      <c r="A362" s="2">
+        <v>46132.75</v>
+      </c>
+      <c r="B362">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="363" spans="1:2">
+      <c r="A363" s="2">
+        <v>46132.76041666666</v>
+      </c>
+      <c r="B363">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="364" spans="1:2">
+      <c r="A364" s="2">
+        <v>46132.77083333334</v>
+      </c>
+      <c r="B364">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="365" spans="1:2">
+      <c r="A365" s="2">
+        <v>46132.78125</v>
+      </c>
+      <c r="B365">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="366" spans="1:2">
+      <c r="A366" s="2">
+        <v>46132.79166666666</v>
+      </c>
+      <c r="B366">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="367" spans="1:2">
+      <c r="A367" s="2">
+        <v>46132.80208333334</v>
+      </c>
+      <c r="B367">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="368" spans="1:2">
+      <c r="A368" s="2">
+        <v>46132.8125</v>
+      </c>
+      <c r="B368">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="369" spans="1:2">
+      <c r="A369" s="2">
+        <v>46132.82291666666</v>
+      </c>
+      <c r="B369">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="370" spans="1:2">
+      <c r="A370" s="2">
+        <v>46132.83333333334</v>
+      </c>
+      <c r="B370">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="371" spans="1:2">
+      <c r="A371" s="2">
+        <v>46132.84375</v>
+      </c>
+      <c r="B371">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="372" spans="1:2">
+      <c r="A372" s="2">
+        <v>46132.85416666666</v>
+      </c>
+      <c r="B372">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="373" spans="1:2">
+      <c r="A373" s="2">
+        <v>46132.86458333334</v>
+      </c>
+      <c r="B373">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="374" spans="1:2">
+      <c r="A374" s="2">
+        <v>46132.875</v>
+      </c>
+      <c r="B374">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="375" spans="1:2">
+      <c r="A375" s="2">
+        <v>46132.88541666666</v>
+      </c>
+      <c r="B375">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="376" spans="1:2">
+      <c r="A376" s="2">
+        <v>46132.89583333334</v>
+      </c>
+      <c r="B376">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="377" spans="1:2">
+      <c r="A377" s="2">
+        <v>46132.90625</v>
+      </c>
+      <c r="B377">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="378" spans="1:2">
+      <c r="A378" s="2">
+        <v>46132.91666666666</v>
+      </c>
+      <c r="B378">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="379" spans="1:2">
+      <c r="A379" s="2">
+        <v>46132.92708333334</v>
+      </c>
+      <c r="B379">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="380" spans="1:2">
+      <c r="A380" s="2">
+        <v>46132.9375</v>
+      </c>
+      <c r="B380">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="381" spans="1:2">
+      <c r="A381" s="2">
+        <v>46132.94791666666</v>
+      </c>
+      <c r="B381">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="382" spans="1:2">
+      <c r="A382" s="2">
+        <v>46132.95833333334</v>
+      </c>
+      <c r="B382">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="383" spans="1:2">
+      <c r="A383" s="2">
+        <v>46132.96875</v>
+      </c>
+      <c r="B383">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="384" spans="1:2">
+      <c r="A384" s="2">
+        <v>46132.97916666666</v>
+      </c>
+      <c r="B384">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="385" spans="1:2">
+      <c r="A385" s="2">
+        <v>46132.98958333334</v>
+      </c>
+      <c r="B385">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Updating the model for GESS with the latest historical data
</commit_message>
<xml_diff>
--- a/data_fetching/Entsoe/Actual_Production_Hydro_River.xlsx
+++ b/data_fetching/Entsoe/Actual_Production_Hydro_River.xlsx
@@ -381,7 +381,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B385"/>
+  <dimension ref="A1:B289"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:2">
@@ -394,127 +394,127 @@
     </row>
     <row r="2" spans="1:2">
       <c r="A2" s="2">
-        <v>46136</v>
+        <v>46140</v>
       </c>
       <c r="B2">
-        <v>1545</v>
+        <v>1123</v>
       </c>
     </row>
     <row r="3" spans="1:2">
       <c r="A3" s="2">
-        <v>46136.01041666666</v>
+        <v>46140.01041666666</v>
       </c>
       <c r="B3">
-        <v>1533</v>
+        <v>1112</v>
       </c>
     </row>
     <row r="4" spans="1:2">
       <c r="A4" s="2">
-        <v>46136.02083333334</v>
+        <v>46140.02083333334</v>
       </c>
       <c r="B4">
-        <v>1539</v>
+        <v>1119</v>
       </c>
     </row>
     <row r="5" spans="1:2">
       <c r="A5" s="2">
-        <v>46136.03125</v>
+        <v>46140.03125</v>
       </c>
       <c r="B5">
-        <v>1542</v>
+        <v>1154</v>
       </c>
     </row>
     <row r="6" spans="1:2">
       <c r="A6" s="2">
-        <v>46136.04166666666</v>
+        <v>46140.04166666666</v>
       </c>
       <c r="B6">
-        <v>1372</v>
+        <v>1058</v>
       </c>
     </row>
     <row r="7" spans="1:2">
       <c r="A7" s="2">
-        <v>46136.05208333334</v>
+        <v>46140.05208333334</v>
       </c>
       <c r="B7">
-        <v>1338</v>
+        <v>1044</v>
       </c>
     </row>
     <row r="8" spans="1:2">
       <c r="A8" s="2">
-        <v>46136.0625</v>
+        <v>46140.0625</v>
       </c>
       <c r="B8">
-        <v>1340</v>
+        <v>1050</v>
       </c>
     </row>
     <row r="9" spans="1:2">
       <c r="A9" s="2">
-        <v>46136.07291666666</v>
+        <v>46140.07291666666</v>
       </c>
       <c r="B9">
-        <v>1338</v>
+        <v>1052</v>
       </c>
     </row>
     <row r="10" spans="1:2">
       <c r="A10" s="2">
-        <v>46136.08333333334</v>
+        <v>46140.08333333334</v>
       </c>
       <c r="B10">
-        <v>1322</v>
+        <v>1057</v>
       </c>
     </row>
     <row r="11" spans="1:2">
       <c r="A11" s="2">
-        <v>46136.09375</v>
+        <v>46140.09375</v>
       </c>
       <c r="B11">
-        <v>1319</v>
+        <v>1058</v>
       </c>
     </row>
     <row r="12" spans="1:2">
       <c r="A12" s="2">
-        <v>46136.10416666666</v>
+        <v>46140.10416666666</v>
       </c>
       <c r="B12">
-        <v>1321</v>
+        <v>1056</v>
       </c>
     </row>
     <row r="13" spans="1:2">
       <c r="A13" s="2">
-        <v>46136.11458333334</v>
+        <v>46140.11458333334</v>
       </c>
       <c r="B13">
-        <v>1319</v>
+        <v>1055</v>
       </c>
     </row>
     <row r="14" spans="1:2">
       <c r="A14" s="2">
-        <v>46136.125</v>
+        <v>46140.125</v>
       </c>
       <c r="B14">
-        <v>1285</v>
+        <v>926</v>
       </c>
     </row>
     <row r="15" spans="1:2">
       <c r="A15" s="2">
-        <v>46136.13541666666</v>
+        <v>46140.13541666666</v>
       </c>
       <c r="B15">
-        <v>1281</v>
+        <v>921</v>
       </c>
     </row>
     <row r="16" spans="1:2">
       <c r="A16" s="2">
-        <v>46136.14583333334</v>
+        <v>46140.14583333334</v>
       </c>
       <c r="B16">
-        <v>1283</v>
+        <v>0</v>
       </c>
     </row>
     <row r="17" spans="1:2">
       <c r="A17" s="2">
-        <v>46136.15625</v>
+        <v>46140.15625</v>
       </c>
       <c r="B17">
         <v>0</v>
@@ -522,191 +522,191 @@
     </row>
     <row r="18" spans="1:2">
       <c r="A18" s="2">
-        <v>46136.16666666666</v>
+        <v>46140.16666666666</v>
       </c>
       <c r="B18">
-        <v>1279</v>
+        <v>927</v>
       </c>
     </row>
     <row r="19" spans="1:2">
       <c r="A19" s="2">
-        <v>46136.17708333334</v>
+        <v>46140.17708333334</v>
       </c>
       <c r="B19">
-        <v>1276</v>
+        <v>926</v>
       </c>
     </row>
     <row r="20" spans="1:2">
       <c r="A20" s="2">
-        <v>46136.1875</v>
+        <v>46140.1875</v>
       </c>
       <c r="B20">
-        <v>1277</v>
+        <v>927</v>
       </c>
     </row>
     <row r="21" spans="1:2">
       <c r="A21" s="2">
-        <v>46136.19791666666</v>
+        <v>46140.19791666666</v>
       </c>
       <c r="B21">
-        <v>1274</v>
+        <v>923</v>
       </c>
     </row>
     <row r="22" spans="1:2">
       <c r="A22" s="2">
-        <v>46136.20833333334</v>
+        <v>46140.20833333334</v>
       </c>
       <c r="B22">
-        <v>1267</v>
+        <v>1116</v>
       </c>
     </row>
     <row r="23" spans="1:2">
       <c r="A23" s="2">
-        <v>46136.21875</v>
+        <v>46140.21875</v>
       </c>
       <c r="B23">
-        <v>1261</v>
+        <v>1135</v>
       </c>
     </row>
     <row r="24" spans="1:2">
       <c r="A24" s="2">
-        <v>46136.22916666666</v>
+        <v>46140.22916666666</v>
       </c>
       <c r="B24">
-        <v>1264</v>
+        <v>1134</v>
       </c>
     </row>
     <row r="25" spans="1:2">
       <c r="A25" s="2">
-        <v>46136.23958333334</v>
+        <v>46140.23958333334</v>
       </c>
       <c r="B25">
-        <v>1263</v>
+        <v>1132</v>
       </c>
     </row>
     <row r="26" spans="1:2">
       <c r="A26" s="2">
-        <v>46136.25</v>
+        <v>46140.25</v>
       </c>
       <c r="B26">
-        <v>1188</v>
+        <v>1209</v>
       </c>
     </row>
     <row r="27" spans="1:2">
       <c r="A27" s="2">
-        <v>46136.26041666666</v>
+        <v>46140.26041666666</v>
       </c>
       <c r="B27">
-        <v>1185</v>
+        <v>1202</v>
       </c>
     </row>
     <row r="28" spans="1:2">
       <c r="A28" s="2">
-        <v>46136.27083333334</v>
+        <v>46140.27083333334</v>
       </c>
       <c r="B28">
-        <v>1186</v>
+        <v>1203</v>
       </c>
     </row>
     <row r="29" spans="1:2">
       <c r="A29" s="2">
-        <v>46136.28125</v>
+        <v>46140.28125</v>
       </c>
       <c r="B29">
-        <v>1183</v>
+        <v>1204</v>
       </c>
     </row>
     <row r="30" spans="1:2">
       <c r="A30" s="2">
-        <v>46136.29166666666</v>
+        <v>46140.29166666666</v>
       </c>
       <c r="B30">
-        <v>1172</v>
+        <v>1191</v>
       </c>
     </row>
     <row r="31" spans="1:2">
       <c r="A31" s="2">
-        <v>46136.30208333334</v>
+        <v>46140.30208333334</v>
       </c>
       <c r="B31">
-        <v>1166</v>
+        <v>0</v>
       </c>
     </row>
     <row r="32" spans="1:2">
       <c r="A32" s="2">
-        <v>46136.3125</v>
+        <v>46140.3125</v>
       </c>
       <c r="B32">
-        <v>0</v>
+        <v>1187</v>
       </c>
     </row>
     <row r="33" spans="1:2">
       <c r="A33" s="2">
-        <v>46136.32291666666</v>
+        <v>46140.32291666666</v>
       </c>
       <c r="B33">
-        <v>1167</v>
+        <v>0</v>
       </c>
     </row>
     <row r="34" spans="1:2">
       <c r="A34" s="2">
-        <v>46136.33333333334</v>
+        <v>46140.33333333334</v>
       </c>
       <c r="B34">
-        <v>1197</v>
+        <v>995</v>
       </c>
     </row>
     <row r="35" spans="1:2">
       <c r="A35" s="2">
-        <v>46136.34375</v>
+        <v>46140.34375</v>
       </c>
       <c r="B35">
-        <v>1199</v>
+        <v>989</v>
       </c>
     </row>
     <row r="36" spans="1:2">
       <c r="A36" s="2">
-        <v>46136.35416666666</v>
+        <v>46140.35416666666</v>
       </c>
       <c r="B36">
-        <v>1204</v>
+        <v>980</v>
       </c>
     </row>
     <row r="37" spans="1:2">
       <c r="A37" s="2">
-        <v>46136.36458333334</v>
+        <v>46140.36458333334</v>
       </c>
       <c r="B37">
-        <v>1116</v>
+        <v>938</v>
       </c>
     </row>
     <row r="38" spans="1:2">
       <c r="A38" s="2">
-        <v>46136.375</v>
+        <v>46140.375</v>
       </c>
       <c r="B38">
-        <v>976</v>
+        <v>954</v>
       </c>
     </row>
     <row r="39" spans="1:2">
       <c r="A39" s="2">
-        <v>46136.38541666666</v>
+        <v>46140.38541666666</v>
       </c>
       <c r="B39">
-        <v>958</v>
+        <v>952</v>
       </c>
     </row>
     <row r="40" spans="1:2">
       <c r="A40" s="2">
-        <v>46136.39583333334</v>
+        <v>46140.39583333334</v>
       </c>
       <c r="B40">
-        <v>954</v>
+        <v>953</v>
       </c>
     </row>
     <row r="41" spans="1:2">
       <c r="A41" s="2">
-        <v>46136.40625</v>
+        <v>46140.40625</v>
       </c>
       <c r="B41">
         <v>950</v>
@@ -714,63 +714,63 @@
     </row>
     <row r="42" spans="1:2">
       <c r="A42" s="2">
-        <v>46136.41666666666</v>
+        <v>46140.41666666666</v>
       </c>
       <c r="B42">
-        <v>786</v>
+        <v>607</v>
       </c>
     </row>
     <row r="43" spans="1:2">
       <c r="A43" s="2">
-        <v>46136.42708333334</v>
+        <v>46140.42708333334</v>
       </c>
       <c r="B43">
-        <v>759</v>
+        <v>587</v>
       </c>
     </row>
     <row r="44" spans="1:2">
       <c r="A44" s="2">
-        <v>46136.4375</v>
+        <v>46140.4375</v>
       </c>
       <c r="B44">
-        <v>763</v>
+        <v>0</v>
       </c>
     </row>
     <row r="45" spans="1:2">
       <c r="A45" s="2">
-        <v>46136.44791666666</v>
+        <v>46140.44791666666</v>
       </c>
       <c r="B45">
-        <v>762</v>
+        <v>588</v>
       </c>
     </row>
     <row r="46" spans="1:2">
       <c r="A46" s="2">
-        <v>46136.45833333334</v>
+        <v>46140.45833333334</v>
       </c>
       <c r="B46">
-        <v>764</v>
+        <v>519</v>
       </c>
     </row>
     <row r="47" spans="1:2">
       <c r="A47" s="2">
-        <v>46136.46875</v>
+        <v>46140.46875</v>
       </c>
       <c r="B47">
-        <v>760</v>
+        <v>517</v>
       </c>
     </row>
     <row r="48" spans="1:2">
       <c r="A48" s="2">
-        <v>46136.47916666666</v>
+        <v>46140.47916666666</v>
       </c>
       <c r="B48">
-        <v>762</v>
+        <v>515</v>
       </c>
     </row>
     <row r="49" spans="1:2">
       <c r="A49" s="2">
-        <v>46136.48958333334</v>
+        <v>46140.48958333334</v>
       </c>
       <c r="B49">
         <v>0</v>
@@ -778,1175 +778,1175 @@
     </row>
     <row r="50" spans="1:2">
       <c r="A50" s="2">
-        <v>46136.5</v>
+        <v>46140.5</v>
       </c>
       <c r="B50">
-        <v>701</v>
+        <v>513</v>
       </c>
     </row>
     <row r="51" spans="1:2">
       <c r="A51" s="2">
-        <v>46136.51041666666</v>
+        <v>46140.51041666666</v>
       </c>
       <c r="B51">
-        <v>702</v>
+        <v>511</v>
       </c>
     </row>
     <row r="52" spans="1:2">
       <c r="A52" s="2">
-        <v>46136.52083333334</v>
+        <v>46140.52083333334</v>
       </c>
       <c r="B52">
-        <v>700</v>
+        <v>512</v>
       </c>
     </row>
     <row r="53" spans="1:2">
       <c r="A53" s="2">
-        <v>46136.53125</v>
+        <v>46140.53125</v>
       </c>
       <c r="B53">
-        <v>699</v>
+        <v>0</v>
       </c>
     </row>
     <row r="54" spans="1:2">
       <c r="A54" s="2">
-        <v>46136.54166666666</v>
+        <v>46140.54166666666</v>
       </c>
       <c r="B54">
-        <v>704</v>
+        <v>474</v>
       </c>
     </row>
     <row r="55" spans="1:2">
       <c r="A55" s="2">
-        <v>46136.55208333334</v>
+        <v>46140.55208333334</v>
       </c>
       <c r="B55">
-        <v>675</v>
+        <v>468</v>
       </c>
     </row>
     <row r="56" spans="1:2">
       <c r="A56" s="2">
-        <v>46136.5625</v>
+        <v>46140.5625</v>
       </c>
       <c r="B56">
-        <v>674</v>
+        <v>466</v>
       </c>
     </row>
     <row r="57" spans="1:2">
       <c r="A57" s="2">
-        <v>46136.57291666666</v>
+        <v>46140.57291666666</v>
       </c>
       <c r="B57">
-        <v>675</v>
+        <v>0</v>
       </c>
     </row>
     <row r="58" spans="1:2">
       <c r="A58" s="2">
-        <v>46136.58333333334</v>
+        <v>46140.58333333334</v>
       </c>
       <c r="B58">
-        <v>706</v>
+        <v>474</v>
       </c>
     </row>
     <row r="59" spans="1:2">
       <c r="A59" s="2">
-        <v>46136.59375</v>
+        <v>46140.59375</v>
       </c>
       <c r="B59">
-        <v>0</v>
+        <v>476</v>
       </c>
     </row>
     <row r="60" spans="1:2">
       <c r="A60" s="2">
-        <v>46136.60416666666</v>
+        <v>46140.60416666666</v>
       </c>
       <c r="B60">
-        <v>0</v>
+        <v>475</v>
       </c>
     </row>
     <row r="61" spans="1:2">
       <c r="A61" s="2">
-        <v>46136.61458333334</v>
+        <v>46140.61458333334</v>
       </c>
       <c r="B61">
-        <v>708</v>
+        <v>486</v>
       </c>
     </row>
     <row r="62" spans="1:2">
       <c r="A62" s="2">
-        <v>46136.625</v>
+        <v>46140.625</v>
       </c>
       <c r="B62">
-        <v>760</v>
+        <v>603</v>
       </c>
     </row>
     <row r="63" spans="1:2">
       <c r="A63" s="2">
-        <v>46136.63541666666</v>
+        <v>46140.63541666666</v>
       </c>
       <c r="B63">
-        <v>762</v>
+        <v>607</v>
       </c>
     </row>
     <row r="64" spans="1:2">
       <c r="A64" s="2">
-        <v>46136.64583333334</v>
+        <v>46140.64583333334</v>
       </c>
       <c r="B64">
-        <v>770</v>
+        <v>616</v>
       </c>
     </row>
     <row r="65" spans="1:2">
       <c r="A65" s="2">
-        <v>46136.65625</v>
+        <v>46140.65625</v>
       </c>
       <c r="B65">
-        <v>781</v>
+        <v>628</v>
       </c>
     </row>
     <row r="66" spans="1:2">
       <c r="A66" s="2">
-        <v>46136.66666666666</v>
+        <v>46140.66666666666</v>
       </c>
       <c r="B66">
-        <v>900</v>
+        <v>950</v>
       </c>
     </row>
     <row r="67" spans="1:2">
       <c r="A67" s="2">
-        <v>46136.67708333334</v>
+        <v>46140.67708333334</v>
       </c>
       <c r="B67">
-        <v>923</v>
+        <v>969</v>
       </c>
     </row>
     <row r="68" spans="1:2">
       <c r="A68" s="2">
-        <v>46136.6875</v>
+        <v>46140.6875</v>
       </c>
       <c r="B68">
-        <v>926</v>
+        <v>973</v>
       </c>
     </row>
     <row r="69" spans="1:2">
       <c r="A69" s="2">
-        <v>46136.69791666666</v>
+        <v>46140.69791666666</v>
       </c>
       <c r="B69">
-        <v>795</v>
+        <v>976</v>
       </c>
     </row>
     <row r="70" spans="1:2">
       <c r="A70" s="2">
-        <v>46136.70833333334</v>
+        <v>46140.70833333334</v>
       </c>
       <c r="B70">
-        <v>987</v>
+        <v>1241</v>
       </c>
     </row>
     <row r="71" spans="1:2">
       <c r="A71" s="2">
-        <v>46136.71875</v>
+        <v>46140.71875</v>
       </c>
       <c r="B71">
-        <v>1003</v>
+        <v>1285</v>
       </c>
     </row>
     <row r="72" spans="1:2">
       <c r="A72" s="2">
-        <v>46136.72916666666</v>
+        <v>46140.72916666666</v>
       </c>
       <c r="B72">
-        <v>1094</v>
+        <v>1287</v>
       </c>
     </row>
     <row r="73" spans="1:2">
       <c r="A73" s="2">
-        <v>46136.73958333334</v>
+        <v>46140.73958333334</v>
       </c>
       <c r="B73">
-        <v>1117</v>
+        <v>1285</v>
       </c>
     </row>
     <row r="74" spans="1:2">
       <c r="A74" s="2">
-        <v>46136.75</v>
+        <v>46140.75</v>
       </c>
       <c r="B74">
-        <v>1327</v>
+        <v>1318</v>
       </c>
     </row>
     <row r="75" spans="1:2">
       <c r="A75" s="2">
-        <v>46136.76041666666</v>
+        <v>46140.76041666666</v>
       </c>
       <c r="B75">
-        <v>1339</v>
+        <v>1320</v>
       </c>
     </row>
     <row r="76" spans="1:2">
       <c r="A76" s="2">
-        <v>46136.77083333334</v>
+        <v>46140.77083333334</v>
       </c>
       <c r="B76">
-        <v>1375</v>
+        <v>1353</v>
       </c>
     </row>
     <row r="77" spans="1:2">
       <c r="A77" s="2">
-        <v>46136.78125</v>
+        <v>46140.78125</v>
       </c>
       <c r="B77">
-        <v>1395</v>
+        <v>1358</v>
       </c>
     </row>
     <row r="78" spans="1:2">
       <c r="A78" s="2">
-        <v>46136.79166666666</v>
+        <v>46140.79166666666</v>
       </c>
       <c r="B78">
-        <v>1483</v>
+        <v>0</v>
       </c>
     </row>
     <row r="79" spans="1:2">
       <c r="A79" s="2">
-        <v>46136.80208333334</v>
+        <v>46140.80208333334</v>
       </c>
       <c r="B79">
-        <v>1496</v>
+        <v>1361</v>
       </c>
     </row>
     <row r="80" spans="1:2">
       <c r="A80" s="2">
-        <v>46136.8125</v>
+        <v>46140.8125</v>
       </c>
       <c r="B80">
-        <v>1487</v>
+        <v>1362</v>
       </c>
     </row>
     <row r="81" spans="1:2">
       <c r="A81" s="2">
-        <v>46136.82291666666</v>
+        <v>46140.82291666666</v>
       </c>
       <c r="B81">
-        <v>1490</v>
+        <v>1360</v>
       </c>
     </row>
     <row r="82" spans="1:2">
       <c r="A82" s="2">
-        <v>46136.83333333334</v>
+        <v>46140.83333333334</v>
       </c>
       <c r="B82">
-        <v>1483</v>
+        <v>1382</v>
       </c>
     </row>
     <row r="83" spans="1:2">
       <c r="A83" s="2">
-        <v>46136.84375</v>
+        <v>46140.84375</v>
       </c>
       <c r="B83">
-        <v>1482</v>
+        <v>1379</v>
       </c>
     </row>
     <row r="84" spans="1:2">
       <c r="A84" s="2">
-        <v>46136.85416666666</v>
+        <v>46140.85416666666</v>
       </c>
       <c r="B84">
-        <v>1481</v>
+        <v>1369</v>
       </c>
     </row>
     <row r="85" spans="1:2">
       <c r="A85" s="2">
-        <v>46136.86458333334</v>
+        <v>46140.86458333334</v>
       </c>
       <c r="B85">
-        <v>1483</v>
+        <v>1370</v>
       </c>
     </row>
     <row r="86" spans="1:2">
       <c r="A86" s="2">
-        <v>46136.875</v>
+        <v>46140.875</v>
       </c>
       <c r="B86">
-        <v>1422</v>
+        <v>1365</v>
       </c>
     </row>
     <row r="87" spans="1:2">
       <c r="A87" s="2">
-        <v>46136.88541666666</v>
+        <v>46140.88541666666</v>
       </c>
       <c r="B87">
-        <v>1414</v>
+        <v>1387</v>
       </c>
     </row>
     <row r="88" spans="1:2">
       <c r="A88" s="2">
-        <v>46136.89583333334</v>
+        <v>46140.89583333334</v>
       </c>
       <c r="B88">
-        <v>1416</v>
+        <v>1393</v>
       </c>
     </row>
     <row r="89" spans="1:2">
       <c r="A89" s="2">
-        <v>46136.90625</v>
+        <v>46140.90625</v>
       </c>
       <c r="B89">
-        <v>1411</v>
+        <v>1390</v>
       </c>
     </row>
     <row r="90" spans="1:2">
       <c r="A90" s="2">
-        <v>46136.91666666666</v>
+        <v>46140.91666666666</v>
       </c>
       <c r="B90">
-        <v>1383</v>
+        <v>1311</v>
       </c>
     </row>
     <row r="91" spans="1:2">
       <c r="A91" s="2">
-        <v>46136.92708333334</v>
+        <v>46140.92708333334</v>
       </c>
       <c r="B91">
-        <v>1382</v>
+        <v>1297</v>
       </c>
     </row>
     <row r="92" spans="1:2">
       <c r="A92" s="2">
-        <v>46136.9375</v>
+        <v>46140.9375</v>
       </c>
       <c r="B92">
-        <v>1354</v>
+        <v>0</v>
       </c>
     </row>
     <row r="93" spans="1:2">
       <c r="A93" s="2">
-        <v>46136.94791666666</v>
+        <v>46140.94791666666</v>
       </c>
       <c r="B93">
-        <v>1350</v>
+        <v>1298</v>
       </c>
     </row>
     <row r="94" spans="1:2">
       <c r="A94" s="2">
-        <v>46136.95833333334</v>
+        <v>46140.95833333334</v>
       </c>
       <c r="B94">
-        <v>1416</v>
+        <v>1230</v>
       </c>
     </row>
     <row r="95" spans="1:2">
       <c r="A95" s="2">
-        <v>46136.96875</v>
+        <v>46140.96875</v>
       </c>
       <c r="B95">
-        <v>1392</v>
+        <v>1225</v>
       </c>
     </row>
     <row r="96" spans="1:2">
       <c r="A96" s="2">
-        <v>46136.97916666666</v>
+        <v>46140.97916666666</v>
       </c>
       <c r="B96">
-        <v>0</v>
+        <v>1222</v>
       </c>
     </row>
     <row r="97" spans="1:2">
       <c r="A97" s="2">
-        <v>46136.98958333334</v>
+        <v>46140.98958333334</v>
       </c>
       <c r="B97">
-        <v>1389</v>
+        <v>1221</v>
       </c>
     </row>
     <row r="98" spans="1:2">
       <c r="A98" s="2">
-        <v>46137</v>
+        <v>46141</v>
       </c>
       <c r="B98">
-        <v>1423</v>
+        <v>1055</v>
       </c>
     </row>
     <row r="99" spans="1:2">
       <c r="A99" s="2">
-        <v>46137.01041666666</v>
+        <v>46141.01041666666</v>
       </c>
       <c r="B99">
-        <v>1406</v>
+        <v>1032</v>
       </c>
     </row>
     <row r="100" spans="1:2">
       <c r="A100" s="2">
-        <v>46137.02083333334</v>
+        <v>46141.02083333334</v>
       </c>
       <c r="B100">
-        <v>1411</v>
+        <v>1031</v>
       </c>
     </row>
     <row r="101" spans="1:2">
       <c r="A101" s="2">
-        <v>46137.03125</v>
+        <v>46141.03125</v>
       </c>
       <c r="B101">
-        <v>1409</v>
+        <v>1023</v>
       </c>
     </row>
     <row r="102" spans="1:2">
       <c r="A102" s="2">
-        <v>46137.04166666666</v>
+        <v>46141.04166666666</v>
       </c>
       <c r="B102">
-        <v>1335</v>
+        <v>1015</v>
       </c>
     </row>
     <row r="103" spans="1:2">
       <c r="A103" s="2">
-        <v>46137.05208333334</v>
+        <v>46141.05208333334</v>
       </c>
       <c r="B103">
-        <v>1330</v>
+        <v>1012</v>
       </c>
     </row>
     <row r="104" spans="1:2">
       <c r="A104" s="2">
-        <v>46137.0625</v>
+        <v>46141.0625</v>
       </c>
       <c r="B104">
-        <v>1342</v>
+        <v>1013</v>
       </c>
     </row>
     <row r="105" spans="1:2">
       <c r="A105" s="2">
-        <v>46137.07291666666</v>
+        <v>46141.07291666666</v>
       </c>
       <c r="B105">
-        <v>1343</v>
+        <v>1012</v>
       </c>
     </row>
     <row r="106" spans="1:2">
       <c r="A106" s="2">
-        <v>46137.08333333334</v>
+        <v>46141.08333333334</v>
       </c>
       <c r="B106">
-        <v>1208</v>
+        <v>1013</v>
       </c>
     </row>
     <row r="107" spans="1:2">
       <c r="A107" s="2">
-        <v>46137.09375</v>
+        <v>46141.09375</v>
       </c>
       <c r="B107">
-        <v>1195</v>
+        <v>1012</v>
       </c>
     </row>
     <row r="108" spans="1:2">
       <c r="A108" s="2">
-        <v>46137.10416666666</v>
+        <v>46141.10416666666</v>
       </c>
       <c r="B108">
-        <v>1197</v>
+        <v>1014</v>
       </c>
     </row>
     <row r="109" spans="1:2">
       <c r="A109" s="2">
-        <v>46137.11458333334</v>
+        <v>46141.11458333334</v>
       </c>
       <c r="B109">
-        <v>1196</v>
+        <v>1011</v>
       </c>
     </row>
     <row r="110" spans="1:2">
       <c r="A110" s="2">
-        <v>46137.125</v>
+        <v>46141.125</v>
       </c>
       <c r="B110">
-        <v>1168</v>
+        <v>0</v>
       </c>
     </row>
     <row r="111" spans="1:2">
       <c r="A111" s="2">
-        <v>46137.13541666666</v>
+        <v>46141.13541666666</v>
       </c>
       <c r="B111">
-        <v>1166</v>
+        <v>1012</v>
       </c>
     </row>
     <row r="112" spans="1:2">
       <c r="A112" s="2">
-        <v>46137.14583333334</v>
+        <v>46141.14583333334</v>
       </c>
       <c r="B112">
-        <v>1167</v>
+        <v>0</v>
       </c>
     </row>
     <row r="113" spans="1:2">
       <c r="A113" s="2">
-        <v>46137.15625</v>
+        <v>46141.15625</v>
       </c>
       <c r="B113">
-        <v>1166</v>
+        <v>1009</v>
       </c>
     </row>
     <row r="114" spans="1:2">
       <c r="A114" s="2">
-        <v>46137.16666666666</v>
+        <v>46141.16666666666</v>
       </c>
       <c r="B114">
-        <v>1227</v>
+        <v>1015</v>
       </c>
     </row>
     <row r="115" spans="1:2">
       <c r="A115" s="2">
-        <v>46137.17708333334</v>
+        <v>46141.17708333334</v>
       </c>
       <c r="B115">
-        <v>1230</v>
+        <v>0</v>
       </c>
     </row>
     <row r="116" spans="1:2">
       <c r="A116" s="2">
-        <v>46137.1875</v>
+        <v>46141.1875</v>
       </c>
       <c r="B116">
-        <v>1231</v>
+        <v>1018</v>
       </c>
     </row>
     <row r="117" spans="1:2">
       <c r="A117" s="2">
-        <v>46137.19791666666</v>
+        <v>46141.19791666666</v>
       </c>
       <c r="B117">
-        <v>1234</v>
+        <v>1025</v>
       </c>
     </row>
     <row r="118" spans="1:2">
       <c r="A118" s="2">
-        <v>46137.20833333334</v>
+        <v>46141.20833333334</v>
       </c>
       <c r="B118">
-        <v>1348</v>
+        <v>1235</v>
       </c>
     </row>
     <row r="119" spans="1:2">
       <c r="A119" s="2">
-        <v>46137.21875</v>
+        <v>46141.21875</v>
       </c>
       <c r="B119">
-        <v>1350</v>
+        <v>1243</v>
       </c>
     </row>
     <row r="120" spans="1:2">
       <c r="A120" s="2">
-        <v>46137.22916666666</v>
+        <v>46141.22916666666</v>
       </c>
       <c r="B120">
-        <v>1351</v>
+        <v>1244</v>
       </c>
     </row>
     <row r="121" spans="1:2">
       <c r="A121" s="2">
-        <v>46137.23958333334</v>
+        <v>46141.23958333334</v>
       </c>
       <c r="B121">
-        <v>1359</v>
+        <v>0</v>
       </c>
     </row>
     <row r="122" spans="1:2">
       <c r="A122" s="2">
-        <v>46137.25</v>
+        <v>46141.25</v>
       </c>
       <c r="B122">
-        <v>1245</v>
+        <v>1211</v>
       </c>
     </row>
     <row r="123" spans="1:2">
       <c r="A123" s="2">
-        <v>46137.26041666666</v>
+        <v>46141.26041666666</v>
       </c>
       <c r="B123">
-        <v>1243</v>
+        <v>1200</v>
       </c>
     </row>
     <row r="124" spans="1:2">
       <c r="A124" s="2">
-        <v>46137.27083333334</v>
+        <v>46141.27083333334</v>
       </c>
       <c r="B124">
-        <v>1240</v>
+        <v>1205</v>
       </c>
     </row>
     <row r="125" spans="1:2">
       <c r="A125" s="2">
-        <v>46137.28125</v>
+        <v>46141.28125</v>
       </c>
       <c r="B125">
-        <v>1243</v>
+        <v>1204</v>
       </c>
     </row>
     <row r="126" spans="1:2">
       <c r="A126" s="2">
-        <v>46137.29166666666</v>
+        <v>46141.29166666666</v>
       </c>
       <c r="B126">
-        <v>1158</v>
+        <v>1185</v>
       </c>
     </row>
     <row r="127" spans="1:2">
       <c r="A127" s="2">
-        <v>46137.30208333334</v>
+        <v>46141.30208333334</v>
       </c>
       <c r="B127">
-        <v>1161</v>
+        <v>1183</v>
       </c>
     </row>
     <row r="128" spans="1:2">
       <c r="A128" s="2">
-        <v>46137.3125</v>
+        <v>46141.3125</v>
       </c>
       <c r="B128">
-        <v>1162</v>
+        <v>1184</v>
       </c>
     </row>
     <row r="129" spans="1:2">
       <c r="A129" s="2">
-        <v>46137.32291666666</v>
+        <v>46141.32291666666</v>
       </c>
       <c r="B129">
-        <v>1163</v>
+        <v>1183</v>
       </c>
     </row>
     <row r="130" spans="1:2">
       <c r="A130" s="2">
-        <v>46137.33333333334</v>
+        <v>46141.33333333334</v>
       </c>
       <c r="B130">
-        <v>1054</v>
+        <v>930</v>
       </c>
     </row>
     <row r="131" spans="1:2">
       <c r="A131" s="2">
-        <v>46137.34375</v>
+        <v>46141.34375</v>
       </c>
       <c r="B131">
-        <v>1048</v>
+        <v>831</v>
       </c>
     </row>
     <row r="132" spans="1:2">
       <c r="A132" s="2">
-        <v>46137.35416666666</v>
+        <v>46141.35416666666</v>
       </c>
       <c r="B132">
-        <v>1046</v>
+        <v>830</v>
       </c>
     </row>
     <row r="133" spans="1:2">
       <c r="A133" s="2">
-        <v>46137.36458333334</v>
+        <v>46141.36458333334</v>
       </c>
       <c r="B133">
-        <v>1049</v>
+        <v>821</v>
       </c>
     </row>
     <row r="134" spans="1:2">
       <c r="A134" s="2">
-        <v>46137.375</v>
+        <v>46141.375</v>
       </c>
       <c r="B134">
-        <v>904</v>
+        <v>794</v>
       </c>
     </row>
     <row r="135" spans="1:2">
       <c r="A135" s="2">
-        <v>46137.38541666666</v>
+        <v>46141.38541666666</v>
       </c>
       <c r="B135">
-        <v>891</v>
+        <v>871</v>
       </c>
     </row>
     <row r="136" spans="1:2">
       <c r="A136" s="2">
-        <v>46137.39583333334</v>
+        <v>46141.39583333334</v>
       </c>
       <c r="B136">
-        <v>884</v>
+        <v>885</v>
       </c>
     </row>
     <row r="137" spans="1:2">
       <c r="A137" s="2">
-        <v>46137.40625</v>
+        <v>46141.40625</v>
       </c>
       <c r="B137">
-        <v>713</v>
+        <v>888</v>
       </c>
     </row>
     <row r="138" spans="1:2">
       <c r="A138" s="2">
-        <v>46137.41666666666</v>
+        <v>46141.41666666666</v>
       </c>
       <c r="B138">
-        <v>622</v>
+        <v>577</v>
       </c>
     </row>
     <row r="139" spans="1:2">
       <c r="A139" s="2">
-        <v>46137.42708333334</v>
+        <v>46141.42708333334</v>
       </c>
       <c r="B139">
-        <v>616</v>
+        <v>508</v>
       </c>
     </row>
     <row r="140" spans="1:2">
       <c r="A140" s="2">
-        <v>46137.4375</v>
+        <v>46141.4375</v>
       </c>
       <c r="B140">
-        <v>698</v>
+        <v>444</v>
       </c>
     </row>
     <row r="141" spans="1:2">
       <c r="A141" s="2">
-        <v>46137.44791666666</v>
+        <v>46141.44791666666</v>
       </c>
       <c r="B141">
-        <v>705</v>
+        <v>0</v>
       </c>
     </row>
     <row r="142" spans="1:2">
       <c r="A142" s="2">
-        <v>46137.45833333334</v>
+        <v>46141.45833333334</v>
       </c>
       <c r="B142">
-        <v>672</v>
+        <v>460</v>
       </c>
     </row>
     <row r="143" spans="1:2">
       <c r="A143" s="2">
-        <v>46137.46875</v>
+        <v>46141.46875</v>
       </c>
       <c r="B143">
-        <v>656</v>
+        <v>462</v>
       </c>
     </row>
     <row r="144" spans="1:2">
       <c r="A144" s="2">
-        <v>46137.47916666666</v>
+        <v>46141.47916666666</v>
       </c>
       <c r="B144">
-        <v>747</v>
+        <v>459</v>
       </c>
     </row>
     <row r="145" spans="1:2">
       <c r="A145" s="2">
-        <v>46137.48958333334</v>
+        <v>46141.48958333334</v>
       </c>
       <c r="B145">
-        <v>754</v>
+        <v>458</v>
       </c>
     </row>
     <row r="146" spans="1:2">
       <c r="A146" s="2">
-        <v>46137.5</v>
+        <v>46141.5</v>
       </c>
       <c r="B146">
-        <v>737</v>
+        <v>456</v>
       </c>
     </row>
     <row r="147" spans="1:2">
       <c r="A147" s="2">
-        <v>46137.51041666666</v>
+        <v>46141.51041666666</v>
       </c>
       <c r="B147">
-        <v>740</v>
+        <v>449</v>
       </c>
     </row>
     <row r="148" spans="1:2">
       <c r="A148" s="2">
-        <v>46137.52083333334</v>
+        <v>46141.52083333334</v>
       </c>
       <c r="B148">
-        <v>738</v>
+        <v>418</v>
       </c>
     </row>
     <row r="149" spans="1:2">
       <c r="A149" s="2">
-        <v>46137.53125</v>
+        <v>46141.53125</v>
       </c>
       <c r="B149">
-        <v>737</v>
+        <v>417</v>
       </c>
     </row>
     <row r="150" spans="1:2">
       <c r="A150" s="2">
-        <v>46137.54166666666</v>
+        <v>46141.54166666666</v>
       </c>
       <c r="B150">
-        <v>748</v>
+        <v>413</v>
       </c>
     </row>
     <row r="151" spans="1:2">
       <c r="A151" s="2">
-        <v>46137.55208333334</v>
+        <v>46141.55208333334</v>
       </c>
       <c r="B151">
-        <v>0</v>
+        <v>412</v>
       </c>
     </row>
     <row r="152" spans="1:2">
       <c r="A152" s="2">
-        <v>46137.5625</v>
+        <v>46141.5625</v>
       </c>
       <c r="B152">
-        <v>0</v>
+        <v>411</v>
       </c>
     </row>
     <row r="153" spans="1:2">
       <c r="A153" s="2">
-        <v>46137.57291666666</v>
+        <v>46141.57291666666</v>
       </c>
       <c r="B153">
-        <v>0</v>
+        <v>414</v>
       </c>
     </row>
     <row r="154" spans="1:2">
       <c r="A154" s="2">
-        <v>46137.58333333334</v>
+        <v>46141.58333333334</v>
       </c>
       <c r="B154">
-        <v>735</v>
+        <v>427</v>
       </c>
     </row>
     <row r="155" spans="1:2">
       <c r="A155" s="2">
-        <v>46137.59375</v>
+        <v>46141.59375</v>
       </c>
       <c r="B155">
-        <v>738</v>
+        <v>426</v>
       </c>
     </row>
     <row r="156" spans="1:2">
       <c r="A156" s="2">
-        <v>46137.60416666666</v>
+        <v>46141.60416666666</v>
       </c>
       <c r="B156">
-        <v>603</v>
+        <v>485</v>
       </c>
     </row>
     <row r="157" spans="1:2">
       <c r="A157" s="2">
-        <v>46137.61458333334</v>
+        <v>46141.61458333334</v>
       </c>
       <c r="B157">
-        <v>587</v>
+        <v>484</v>
       </c>
     </row>
     <row r="158" spans="1:2">
       <c r="A158" s="2">
-        <v>46137.625</v>
+        <v>46141.625</v>
       </c>
       <c r="B158">
-        <v>591</v>
+        <v>559</v>
       </c>
     </row>
     <row r="159" spans="1:2">
       <c r="A159" s="2">
-        <v>46137.63541666666</v>
+        <v>46141.63541666666</v>
       </c>
       <c r="B159">
-        <v>593</v>
+        <v>564</v>
       </c>
     </row>
     <row r="160" spans="1:2">
       <c r="A160" s="2">
-        <v>46137.64583333334</v>
+        <v>46141.64583333334</v>
       </c>
       <c r="B160">
-        <v>0</v>
+        <v>554</v>
       </c>
     </row>
     <row r="161" spans="1:2">
       <c r="A161" s="2">
-        <v>46137.65625</v>
+        <v>46141.65625</v>
       </c>
       <c r="B161">
-        <v>598</v>
+        <v>589</v>
       </c>
     </row>
     <row r="162" spans="1:2">
       <c r="A162" s="2">
-        <v>46137.66666666666</v>
+        <v>46141.66666666666</v>
       </c>
       <c r="B162">
-        <v>766</v>
+        <v>929</v>
       </c>
     </row>
     <row r="163" spans="1:2">
       <c r="A163" s="2">
-        <v>46137.67708333334</v>
+        <v>46141.67708333334</v>
       </c>
       <c r="B163">
-        <v>776</v>
+        <v>919</v>
       </c>
     </row>
     <row r="164" spans="1:2">
       <c r="A164" s="2">
-        <v>46137.6875</v>
+        <v>46141.6875</v>
       </c>
       <c r="B164">
-        <v>0</v>
+        <v>923</v>
       </c>
     </row>
     <row r="165" spans="1:2">
       <c r="A165" s="2">
-        <v>46137.69791666666</v>
+        <v>46141.69791666666</v>
       </c>
       <c r="B165">
-        <v>783</v>
+        <v>924</v>
       </c>
     </row>
     <row r="166" spans="1:2">
       <c r="A166" s="2">
-        <v>46137.70833333334</v>
+        <v>46141.70833333334</v>
       </c>
       <c r="B166">
-        <v>1083</v>
+        <v>1050</v>
       </c>
     </row>
     <row r="167" spans="1:2">
       <c r="A167" s="2">
-        <v>46137.71875</v>
+        <v>46141.71875</v>
       </c>
       <c r="B167">
-        <v>1116</v>
+        <v>1068</v>
       </c>
     </row>
     <row r="168" spans="1:2">
       <c r="A168" s="2">
-        <v>46137.72916666666</v>
+        <v>46141.72916666666</v>
       </c>
       <c r="B168">
-        <v>0</v>
+        <v>1083</v>
       </c>
     </row>
     <row r="169" spans="1:2">
       <c r="A169" s="2">
-        <v>46137.73958333334</v>
+        <v>46141.73958333334</v>
       </c>
       <c r="B169">
-        <v>1216</v>
+        <v>0</v>
       </c>
     </row>
     <row r="170" spans="1:2">
       <c r="A170" s="2">
-        <v>46137.75</v>
+        <v>46141.75</v>
       </c>
       <c r="B170">
-        <v>1381</v>
+        <v>1145</v>
       </c>
     </row>
     <row r="171" spans="1:2">
       <c r="A171" s="2">
-        <v>46137.76041666666</v>
+        <v>46141.76041666666</v>
       </c>
       <c r="B171">
-        <v>1406</v>
+        <v>1152</v>
       </c>
     </row>
     <row r="172" spans="1:2">
       <c r="A172" s="2">
-        <v>46137.77083333334</v>
+        <v>46141.77083333334</v>
       </c>
       <c r="B172">
-        <v>1401</v>
+        <v>1141</v>
       </c>
     </row>
     <row r="173" spans="1:2">
       <c r="A173" s="2">
-        <v>46137.78125</v>
+        <v>46141.78125</v>
       </c>
       <c r="B173">
-        <v>1400</v>
+        <v>1147</v>
       </c>
     </row>
     <row r="174" spans="1:2">
       <c r="A174" s="2">
-        <v>46137.79166666666</v>
+        <v>46141.79166666666</v>
       </c>
       <c r="B174">
-        <v>1403</v>
+        <v>1140</v>
       </c>
     </row>
     <row r="175" spans="1:2">
       <c r="A175" s="2">
-        <v>46137.80208333334</v>
+        <v>46141.80208333334</v>
       </c>
       <c r="B175">
-        <v>1415</v>
+        <v>1179</v>
       </c>
     </row>
     <row r="176" spans="1:2">
       <c r="A176" s="2">
-        <v>46137.8125</v>
+        <v>46141.8125</v>
       </c>
       <c r="B176">
-        <v>1435</v>
+        <v>1196</v>
       </c>
     </row>
     <row r="177" spans="1:2">
       <c r="A177" s="2">
-        <v>46137.82291666666</v>
+        <v>46141.82291666666</v>
       </c>
       <c r="B177">
-        <v>1434</v>
+        <v>1197</v>
       </c>
     </row>
     <row r="178" spans="1:2">
       <c r="A178" s="2">
-        <v>46137.83333333334</v>
+        <v>46141.83333333334</v>
       </c>
       <c r="B178">
-        <v>1403</v>
+        <v>1150</v>
       </c>
     </row>
     <row r="179" spans="1:2">
       <c r="A179" s="2">
-        <v>46137.84375</v>
+        <v>46141.84375</v>
       </c>
       <c r="B179">
-        <v>1398</v>
+        <v>1140</v>
       </c>
     </row>
     <row r="180" spans="1:2">
       <c r="A180" s="2">
-        <v>46137.85416666666</v>
+        <v>46141.85416666666</v>
       </c>
       <c r="B180">
-        <v>1394</v>
+        <v>1141</v>
       </c>
     </row>
     <row r="181" spans="1:2">
       <c r="A181" s="2">
-        <v>46137.86458333334</v>
+        <v>46141.86458333334</v>
       </c>
       <c r="B181">
-        <v>1396</v>
+        <v>1142</v>
       </c>
     </row>
     <row r="182" spans="1:2">
       <c r="A182" s="2">
-        <v>46137.875</v>
+        <v>46141.875</v>
       </c>
       <c r="B182">
-        <v>1414</v>
+        <v>1179</v>
       </c>
     </row>
     <row r="183" spans="1:2">
       <c r="A183" s="2">
-        <v>46137.88541666666</v>
+        <v>46141.88541666666</v>
       </c>
       <c r="B183">
-        <v>1430</v>
+        <v>1187</v>
       </c>
     </row>
     <row r="184" spans="1:2">
       <c r="A184" s="2">
-        <v>46137.89583333334</v>
+        <v>46141.89583333334</v>
       </c>
       <c r="B184">
-        <v>1428</v>
+        <v>1184</v>
       </c>
     </row>
     <row r="185" spans="1:2">
       <c r="A185" s="2">
-        <v>46137.90625</v>
+        <v>46141.90625</v>
       </c>
       <c r="B185">
-        <v>1432</v>
+        <v>1195</v>
       </c>
     </row>
     <row r="186" spans="1:2">
       <c r="A186" s="2">
-        <v>46137.91666666666</v>
+        <v>46141.91666666666</v>
       </c>
       <c r="B186">
-        <v>1436</v>
+        <v>1315</v>
       </c>
     </row>
     <row r="187" spans="1:2">
       <c r="A187" s="2">
-        <v>46137.92708333334</v>
+        <v>46141.92708333334</v>
       </c>
       <c r="B187">
-        <v>1433</v>
+        <v>1294</v>
       </c>
     </row>
     <row r="188" spans="1:2">
       <c r="A188" s="2">
-        <v>46137.9375</v>
+        <v>46141.9375</v>
       </c>
       <c r="B188">
-        <v>1445</v>
+        <v>1283</v>
       </c>
     </row>
     <row r="189" spans="1:2">
       <c r="A189" s="2">
-        <v>46137.94791666666</v>
+        <v>46141.94791666666</v>
       </c>
       <c r="B189">
-        <v>1442</v>
+        <v>1284</v>
       </c>
     </row>
     <row r="190" spans="1:2">
       <c r="A190" s="2">
-        <v>46137.95833333334</v>
+        <v>46141.95833333334</v>
       </c>
       <c r="B190">
-        <v>1494</v>
+        <v>1013</v>
       </c>
     </row>
     <row r="191" spans="1:2">
       <c r="A191" s="2">
-        <v>46137.96875</v>
+        <v>46141.96875</v>
       </c>
       <c r="B191">
-        <v>1497</v>
+        <v>971</v>
       </c>
     </row>
     <row r="192" spans="1:2">
       <c r="A192" s="2">
-        <v>46137.97916666666</v>
+        <v>46141.97916666666</v>
       </c>
       <c r="B192">
-        <v>1501</v>
+        <v>973</v>
       </c>
     </row>
     <row r="193" spans="1:2">
       <c r="A193" s="2">
-        <v>46137.98958333334</v>
+        <v>46141.98958333334</v>
       </c>
       <c r="B193">
-        <v>1496</v>
+        <v>0</v>
       </c>
     </row>
     <row r="194" spans="1:2">
       <c r="A194" s="2">
-        <v>46138</v>
+        <v>46142</v>
       </c>
       <c r="B194">
-        <v>1471</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="195" spans="1:2">
       <c r="A195" s="2">
-        <v>46138.01041666666</v>
+        <v>46142.01041666666</v>
       </c>
       <c r="B195">
-        <v>1465</v>
+        <v>995</v>
       </c>
     </row>
     <row r="196" spans="1:2">
       <c r="A196" s="2">
-        <v>46138.02083333334</v>
+        <v>46142.02083333334</v>
       </c>
       <c r="B196">
         <v>0</v>
@@ -1954,119 +1954,119 @@
     </row>
     <row r="197" spans="1:2">
       <c r="A197" s="2">
-        <v>46138.03125</v>
+        <v>46142.03125</v>
       </c>
       <c r="B197">
-        <v>1466</v>
+        <v>993</v>
       </c>
     </row>
     <row r="198" spans="1:2">
       <c r="A198" s="2">
-        <v>46138.04166666666</v>
+        <v>46142.04166666666</v>
       </c>
       <c r="B198">
-        <v>1390</v>
+        <v>954</v>
       </c>
     </row>
     <row r="199" spans="1:2">
       <c r="A199" s="2">
-        <v>46138.05208333334</v>
+        <v>46142.05208333334</v>
       </c>
       <c r="B199">
-        <v>1377</v>
+        <v>955</v>
       </c>
     </row>
     <row r="200" spans="1:2">
       <c r="A200" s="2">
-        <v>46138.0625</v>
+        <v>46142.0625</v>
       </c>
       <c r="B200">
-        <v>1378</v>
+        <v>0</v>
       </c>
     </row>
     <row r="201" spans="1:2">
       <c r="A201" s="2">
-        <v>46138.07291666666</v>
+        <v>46142.07291666666</v>
       </c>
       <c r="B201">
-        <v>1377</v>
+        <v>954</v>
       </c>
     </row>
     <row r="202" spans="1:2">
       <c r="A202" s="2">
-        <v>46138.08333333334</v>
+        <v>46142.08333333334</v>
       </c>
       <c r="B202">
-        <v>1230</v>
+        <v>955</v>
       </c>
     </row>
     <row r="203" spans="1:2">
       <c r="A203" s="2">
-        <v>46138.09375</v>
+        <v>46142.09375</v>
       </c>
       <c r="B203">
-        <v>1184</v>
+        <v>956</v>
       </c>
     </row>
     <row r="204" spans="1:2">
       <c r="A204" s="2">
-        <v>46138.10416666666</v>
+        <v>46142.10416666666</v>
       </c>
       <c r="B204">
-        <v>1188</v>
+        <v>969</v>
       </c>
     </row>
     <row r="205" spans="1:2">
       <c r="A205" s="2">
-        <v>46138.11458333334</v>
+        <v>46142.11458333334</v>
       </c>
       <c r="B205">
-        <v>1185</v>
+        <v>966</v>
       </c>
     </row>
     <row r="206" spans="1:2">
       <c r="A206" s="2">
-        <v>46138.125</v>
+        <v>46142.125</v>
       </c>
       <c r="B206">
-        <v>1202</v>
+        <v>970</v>
       </c>
     </row>
     <row r="207" spans="1:2">
       <c r="A207" s="2">
-        <v>46138.13541666666</v>
+        <v>46142.13541666666</v>
       </c>
       <c r="B207">
-        <v>1201</v>
+        <v>969</v>
       </c>
     </row>
     <row r="208" spans="1:2">
       <c r="A208" s="2">
-        <v>46138.14583333334</v>
+        <v>46142.14583333334</v>
       </c>
       <c r="B208">
-        <v>1195</v>
+        <v>970</v>
       </c>
     </row>
     <row r="209" spans="1:2">
       <c r="A209" s="2">
-        <v>46138.15625</v>
+        <v>46142.15625</v>
       </c>
       <c r="B209">
-        <v>1186</v>
+        <v>969</v>
       </c>
     </row>
     <row r="210" spans="1:2">
       <c r="A210" s="2">
-        <v>46138.16666666666</v>
+        <v>46142.16666666666</v>
       </c>
       <c r="B210">
-        <v>1181</v>
+        <v>972</v>
       </c>
     </row>
     <row r="211" spans="1:2">
       <c r="A211" s="2">
-        <v>46138.17708333334</v>
+        <v>46142.17708333334</v>
       </c>
       <c r="B211">
         <v>0</v>
@@ -2074,319 +2074,319 @@
     </row>
     <row r="212" spans="1:2">
       <c r="A212" s="2">
-        <v>46138.1875</v>
+        <v>46142.1875</v>
       </c>
       <c r="B212">
-        <v>1182</v>
+        <v>971</v>
       </c>
     </row>
     <row r="213" spans="1:2">
       <c r="A213" s="2">
-        <v>46138.19791666666</v>
+        <v>46142.19791666666</v>
       </c>
       <c r="B213">
-        <v>0</v>
+        <v>975</v>
       </c>
     </row>
     <row r="214" spans="1:2">
       <c r="A214" s="2">
-        <v>46138.20833333334</v>
+        <v>46142.20833333334</v>
       </c>
       <c r="B214">
-        <v>1141</v>
+        <v>1057</v>
       </c>
     </row>
     <row r="215" spans="1:2">
       <c r="A215" s="2">
-        <v>46138.21875</v>
+        <v>46142.21875</v>
       </c>
       <c r="B215">
-        <v>1138</v>
+        <v>1067</v>
       </c>
     </row>
     <row r="216" spans="1:2">
       <c r="A216" s="2">
-        <v>46138.22916666666</v>
+        <v>46142.22916666666</v>
       </c>
       <c r="B216">
-        <v>1140</v>
+        <v>1064</v>
       </c>
     </row>
     <row r="217" spans="1:2">
       <c r="A217" s="2">
-        <v>46138.23958333334</v>
+        <v>46142.23958333334</v>
       </c>
       <c r="B217">
-        <v>1139</v>
+        <v>1069</v>
       </c>
     </row>
     <row r="218" spans="1:2">
       <c r="A218" s="2">
-        <v>46138.25</v>
+        <v>46142.25</v>
       </c>
       <c r="B218">
-        <v>1203</v>
+        <v>1132</v>
       </c>
     </row>
     <row r="219" spans="1:2">
       <c r="A219" s="2">
-        <v>46138.26041666666</v>
+        <v>46142.26041666666</v>
       </c>
       <c r="B219">
-        <v>1194</v>
+        <v>1138</v>
       </c>
     </row>
     <row r="220" spans="1:2">
       <c r="A220" s="2">
-        <v>46138.27083333334</v>
+        <v>46142.27083333334</v>
       </c>
       <c r="B220">
-        <v>1188</v>
+        <v>1137</v>
       </c>
     </row>
     <row r="221" spans="1:2">
       <c r="A221" s="2">
-        <v>46138.28125</v>
+        <v>46142.28125</v>
       </c>
       <c r="B221">
-        <v>1189</v>
+        <v>0</v>
       </c>
     </row>
     <row r="222" spans="1:2">
       <c r="A222" s="2">
-        <v>46138.29166666666</v>
+        <v>46142.29166666666</v>
       </c>
       <c r="B222">
-        <v>1163</v>
+        <v>1138</v>
       </c>
     </row>
     <row r="223" spans="1:2">
       <c r="A223" s="2">
-        <v>46138.30208333334</v>
+        <v>46142.30208333334</v>
       </c>
       <c r="B223">
-        <v>1162</v>
+        <v>1148</v>
       </c>
     </row>
     <row r="224" spans="1:2">
       <c r="A224" s="2">
-        <v>46138.3125</v>
+        <v>46142.3125</v>
       </c>
       <c r="B224">
-        <v>1165</v>
+        <v>1152</v>
       </c>
     </row>
     <row r="225" spans="1:2">
       <c r="A225" s="2">
-        <v>46138.32291666666</v>
+        <v>46142.32291666666</v>
       </c>
       <c r="B225">
-        <v>1180</v>
+        <v>0</v>
       </c>
     </row>
     <row r="226" spans="1:2">
       <c r="A226" s="2">
-        <v>46138.33333333334</v>
+        <v>46142.33333333334</v>
       </c>
       <c r="B226">
-        <v>904</v>
+        <v>936</v>
       </c>
     </row>
     <row r="227" spans="1:2">
       <c r="A227" s="2">
-        <v>46138.34375</v>
+        <v>46142.34375</v>
       </c>
       <c r="B227">
-        <v>844</v>
+        <v>916</v>
       </c>
     </row>
     <row r="228" spans="1:2">
       <c r="A228" s="2">
-        <v>46138.35416666666</v>
+        <v>46142.35416666666</v>
       </c>
       <c r="B228">
-        <v>847</v>
+        <v>955</v>
       </c>
     </row>
     <row r="229" spans="1:2">
       <c r="A229" s="2">
-        <v>46138.36458333334</v>
+        <v>46142.36458333334</v>
       </c>
       <c r="B229">
-        <v>926</v>
+        <v>959</v>
       </c>
     </row>
     <row r="230" spans="1:2">
       <c r="A230" s="2">
-        <v>46138.375</v>
+        <v>46142.375</v>
       </c>
       <c r="B230">
-        <v>908</v>
+        <v>904</v>
       </c>
     </row>
     <row r="231" spans="1:2">
       <c r="A231" s="2">
-        <v>46138.38541666666</v>
+        <v>46142.38541666666</v>
       </c>
       <c r="B231">
-        <v>903</v>
+        <v>899</v>
       </c>
     </row>
     <row r="232" spans="1:2">
       <c r="A232" s="2">
-        <v>46138.39583333334</v>
+        <v>46142.39583333334</v>
       </c>
       <c r="B232">
-        <v>890</v>
+        <v>0</v>
       </c>
     </row>
     <row r="233" spans="1:2">
       <c r="A233" s="2">
-        <v>46138.40625</v>
+        <v>46142.40625</v>
       </c>
       <c r="B233">
-        <v>861</v>
+        <v>898</v>
       </c>
     </row>
     <row r="234" spans="1:2">
       <c r="A234" s="2">
-        <v>46138.41666666666</v>
+        <v>46142.41666666666</v>
       </c>
       <c r="B234">
-        <v>767</v>
+        <v>658</v>
       </c>
     </row>
     <row r="235" spans="1:2">
       <c r="A235" s="2">
-        <v>46138.42708333334</v>
+        <v>46142.42708333334</v>
       </c>
       <c r="B235">
-        <v>750</v>
+        <v>643</v>
       </c>
     </row>
     <row r="236" spans="1:2">
       <c r="A236" s="2">
-        <v>46138.4375</v>
+        <v>46142.4375</v>
       </c>
       <c r="B236">
-        <v>722</v>
+        <v>650</v>
       </c>
     </row>
     <row r="237" spans="1:2">
       <c r="A237" s="2">
-        <v>46138.44791666666</v>
+        <v>46142.44791666666</v>
       </c>
       <c r="B237">
-        <v>647</v>
+        <v>595</v>
       </c>
     </row>
     <row r="238" spans="1:2">
       <c r="A238" s="2">
-        <v>46138.45833333334</v>
+        <v>46142.45833333334</v>
       </c>
       <c r="B238">
-        <v>614</v>
+        <v>563</v>
       </c>
     </row>
     <row r="239" spans="1:2">
       <c r="A239" s="2">
-        <v>46138.46875</v>
+        <v>46142.46875</v>
       </c>
       <c r="B239">
-        <v>608</v>
+        <v>0</v>
       </c>
     </row>
     <row r="240" spans="1:2">
       <c r="A240" s="2">
-        <v>46138.47916666666</v>
+        <v>46142.47916666666</v>
       </c>
       <c r="B240">
-        <v>620</v>
+        <v>0</v>
       </c>
     </row>
     <row r="241" spans="1:2">
       <c r="A241" s="2">
-        <v>46138.48958333334</v>
+        <v>46142.48958333334</v>
       </c>
       <c r="B241">
-        <v>628</v>
+        <v>0</v>
       </c>
     </row>
     <row r="242" spans="1:2">
       <c r="A242" s="2">
-        <v>46138.5</v>
+        <v>46142.5</v>
       </c>
       <c r="B242">
-        <v>625</v>
+        <v>0</v>
       </c>
     </row>
     <row r="243" spans="1:2">
       <c r="A243" s="2">
-        <v>46138.51041666666</v>
+        <v>46142.51041666666</v>
       </c>
       <c r="B243">
-        <v>613</v>
+        <v>0</v>
       </c>
     </row>
     <row r="244" spans="1:2">
       <c r="A244" s="2">
-        <v>46138.52083333334</v>
+        <v>46142.52083333334</v>
       </c>
       <c r="B244">
-        <v>555</v>
+        <v>0</v>
       </c>
     </row>
     <row r="245" spans="1:2">
       <c r="A245" s="2">
-        <v>46138.53125</v>
+        <v>46142.53125</v>
       </c>
       <c r="B245">
-        <v>466</v>
+        <v>0</v>
       </c>
     </row>
     <row r="246" spans="1:2">
       <c r="A246" s="2">
-        <v>46138.54166666666</v>
+        <v>46142.54166666666</v>
       </c>
       <c r="B246">
-        <v>460</v>
+        <v>0</v>
       </c>
     </row>
     <row r="247" spans="1:2">
       <c r="A247" s="2">
-        <v>46138.55208333334</v>
+        <v>46142.55208333334</v>
       </c>
       <c r="B247">
-        <v>465</v>
+        <v>0</v>
       </c>
     </row>
     <row r="248" spans="1:2">
       <c r="A248" s="2">
-        <v>46138.5625</v>
+        <v>46142.5625</v>
       </c>
       <c r="B248">
-        <v>467</v>
+        <v>0</v>
       </c>
     </row>
     <row r="249" spans="1:2">
       <c r="A249" s="2">
-        <v>46138.57291666666</v>
+        <v>46142.57291666666</v>
       </c>
       <c r="B249">
-        <v>468</v>
+        <v>0</v>
       </c>
     </row>
     <row r="250" spans="1:2">
       <c r="A250" s="2">
-        <v>46138.58333333334</v>
+        <v>46142.58333333334</v>
       </c>
       <c r="B250">
-        <v>471</v>
+        <v>0</v>
       </c>
     </row>
     <row r="251" spans="1:2">
       <c r="A251" s="2">
-        <v>46138.59375</v>
+        <v>46142.59375</v>
       </c>
       <c r="B251">
         <v>0</v>
@@ -2394,7 +2394,7 @@
     </row>
     <row r="252" spans="1:2">
       <c r="A252" s="2">
-        <v>46138.60416666666</v>
+        <v>46142.60416666666</v>
       </c>
       <c r="B252">
         <v>0</v>
@@ -2402,63 +2402,63 @@
     </row>
     <row r="253" spans="1:2">
       <c r="A253" s="2">
-        <v>46138.61458333334</v>
+        <v>46142.61458333334</v>
       </c>
       <c r="B253">
-        <v>472</v>
+        <v>0</v>
       </c>
     </row>
     <row r="254" spans="1:2">
       <c r="A254" s="2">
-        <v>46138.625</v>
+        <v>46142.625</v>
       </c>
       <c r="B254">
-        <v>445</v>
+        <v>0</v>
       </c>
     </row>
     <row r="255" spans="1:2">
       <c r="A255" s="2">
-        <v>46138.63541666666</v>
+        <v>46142.63541666666</v>
       </c>
       <c r="B255">
-        <v>443</v>
+        <v>0</v>
       </c>
     </row>
     <row r="256" spans="1:2">
       <c r="A256" s="2">
-        <v>46138.64583333334</v>
+        <v>46142.64583333334</v>
       </c>
       <c r="B256">
-        <v>488</v>
+        <v>0</v>
       </c>
     </row>
     <row r="257" spans="1:2">
       <c r="A257" s="2">
-        <v>46138.65625</v>
+        <v>46142.65625</v>
       </c>
       <c r="B257">
-        <v>494</v>
+        <v>0</v>
       </c>
     </row>
     <row r="258" spans="1:2">
       <c r="A258" s="2">
-        <v>46138.66666666666</v>
+        <v>46142.66666666666</v>
       </c>
       <c r="B258">
-        <v>536</v>
+        <v>0</v>
       </c>
     </row>
     <row r="259" spans="1:2">
       <c r="A259" s="2">
-        <v>46138.67708333334</v>
+        <v>46142.67708333334</v>
       </c>
       <c r="B259">
-        <v>625</v>
+        <v>0</v>
       </c>
     </row>
     <row r="260" spans="1:2">
       <c r="A260" s="2">
-        <v>46138.6875</v>
+        <v>46142.6875</v>
       </c>
       <c r="B260">
         <v>0</v>
@@ -2466,95 +2466,95 @@
     </row>
     <row r="261" spans="1:2">
       <c r="A261" s="2">
-        <v>46138.69791666666</v>
+        <v>46142.69791666666</v>
       </c>
       <c r="B261">
-        <v>636</v>
+        <v>0</v>
       </c>
     </row>
     <row r="262" spans="1:2">
       <c r="A262" s="2">
-        <v>46138.70833333334</v>
+        <v>46142.70833333334</v>
       </c>
       <c r="B262">
-        <v>958</v>
+        <v>0</v>
       </c>
     </row>
     <row r="263" spans="1:2">
       <c r="A263" s="2">
-        <v>46138.71875</v>
+        <v>46142.71875</v>
       </c>
       <c r="B263">
-        <v>925</v>
+        <v>0</v>
       </c>
     </row>
     <row r="264" spans="1:2">
       <c r="A264" s="2">
-        <v>46138.72916666666</v>
+        <v>46142.72916666666</v>
       </c>
       <c r="B264">
-        <v>920</v>
+        <v>0</v>
       </c>
     </row>
     <row r="265" spans="1:2">
       <c r="A265" s="2">
-        <v>46138.73958333334</v>
+        <v>46142.73958333334</v>
       </c>
       <c r="B265">
-        <v>1031</v>
+        <v>0</v>
       </c>
     </row>
     <row r="266" spans="1:2">
       <c r="A266" s="2">
-        <v>46138.75</v>
+        <v>46142.75</v>
       </c>
       <c r="B266">
-        <v>1111</v>
+        <v>0</v>
       </c>
     </row>
     <row r="267" spans="1:2">
       <c r="A267" s="2">
-        <v>46138.76041666666</v>
+        <v>46142.76041666666</v>
       </c>
       <c r="B267">
-        <v>1132</v>
+        <v>0</v>
       </c>
     </row>
     <row r="268" spans="1:2">
       <c r="A268" s="2">
-        <v>46138.77083333334</v>
+        <v>46142.77083333334</v>
       </c>
       <c r="B268">
-        <v>1227</v>
+        <v>0</v>
       </c>
     </row>
     <row r="269" spans="1:2">
       <c r="A269" s="2">
-        <v>46138.78125</v>
+        <v>46142.78125</v>
       </c>
       <c r="B269">
-        <v>1235</v>
+        <v>0</v>
       </c>
     </row>
     <row r="270" spans="1:2">
       <c r="A270" s="2">
-        <v>46138.79166666666</v>
+        <v>46142.79166666666</v>
       </c>
       <c r="B270">
-        <v>1372</v>
+        <v>0</v>
       </c>
     </row>
     <row r="271" spans="1:2">
       <c r="A271" s="2">
-        <v>46138.80208333334</v>
+        <v>46142.80208333334</v>
       </c>
       <c r="B271">
-        <v>1385</v>
+        <v>0</v>
       </c>
     </row>
     <row r="272" spans="1:2">
       <c r="A272" s="2">
-        <v>46138.8125</v>
+        <v>46142.8125</v>
       </c>
       <c r="B272">
         <v>0</v>
@@ -2562,31 +2562,31 @@
     </row>
     <row r="273" spans="1:2">
       <c r="A273" s="2">
-        <v>46138.82291666666</v>
+        <v>46142.82291666666</v>
       </c>
       <c r="B273">
-        <v>1392</v>
+        <v>0</v>
       </c>
     </row>
     <row r="274" spans="1:2">
       <c r="A274" s="2">
-        <v>46138.83333333334</v>
+        <v>46142.83333333334</v>
       </c>
       <c r="B274">
-        <v>1468</v>
+        <v>0</v>
       </c>
     </row>
     <row r="275" spans="1:2">
       <c r="A275" s="2">
-        <v>46138.84375</v>
+        <v>46142.84375</v>
       </c>
       <c r="B275">
-        <v>1474</v>
+        <v>0</v>
       </c>
     </row>
     <row r="276" spans="1:2">
       <c r="A276" s="2">
-        <v>46138.85416666666</v>
+        <v>46142.85416666666</v>
       </c>
       <c r="B276">
         <v>0</v>
@@ -2594,7 +2594,7 @@
     </row>
     <row r="277" spans="1:2">
       <c r="A277" s="2">
-        <v>46138.86458333334</v>
+        <v>46142.86458333334</v>
       </c>
       <c r="B277">
         <v>0</v>
@@ -2602,23 +2602,23 @@
     </row>
     <row r="278" spans="1:2">
       <c r="A278" s="2">
-        <v>46138.875</v>
+        <v>46142.875</v>
       </c>
       <c r="B278">
-        <v>1481</v>
+        <v>0</v>
       </c>
     </row>
     <row r="279" spans="1:2">
       <c r="A279" s="2">
-        <v>46138.88541666666</v>
+        <v>46142.88541666666</v>
       </c>
       <c r="B279">
-        <v>1484</v>
+        <v>0</v>
       </c>
     </row>
     <row r="280" spans="1:2">
       <c r="A280" s="2">
-        <v>46138.89583333334</v>
+        <v>46142.89583333334</v>
       </c>
       <c r="B280">
         <v>0</v>
@@ -2626,7 +2626,7 @@
     </row>
     <row r="281" spans="1:2">
       <c r="A281" s="2">
-        <v>46138.90625</v>
+        <v>46142.90625</v>
       </c>
       <c r="B281">
         <v>0</v>
@@ -2634,833 +2634,65 @@
     </row>
     <row r="282" spans="1:2">
       <c r="A282" s="2">
-        <v>46138.91666666666</v>
+        <v>46142.91666666666</v>
       </c>
       <c r="B282">
-        <v>1507</v>
+        <v>0</v>
       </c>
     </row>
     <row r="283" spans="1:2">
       <c r="A283" s="2">
-        <v>46138.92708333334</v>
+        <v>46142.92708333334</v>
       </c>
       <c r="B283">
-        <v>1502</v>
+        <v>0</v>
       </c>
     </row>
     <row r="284" spans="1:2">
       <c r="A284" s="2">
-        <v>46138.9375</v>
+        <v>46142.9375</v>
       </c>
       <c r="B284">
-        <v>1495</v>
+        <v>0</v>
       </c>
     </row>
     <row r="285" spans="1:2">
       <c r="A285" s="2">
-        <v>46138.94791666666</v>
+        <v>46142.94791666666</v>
       </c>
       <c r="B285">
-        <v>1494</v>
+        <v>0</v>
       </c>
     </row>
     <row r="286" spans="1:2">
       <c r="A286" s="2">
-        <v>46138.95833333334</v>
+        <v>46142.95833333334</v>
       </c>
       <c r="B286">
-        <v>1397</v>
+        <v>0</v>
       </c>
     </row>
     <row r="287" spans="1:2">
       <c r="A287" s="2">
-        <v>46138.96875</v>
+        <v>46142.96875</v>
       </c>
       <c r="B287">
-        <v>1374</v>
+        <v>0</v>
       </c>
     </row>
     <row r="288" spans="1:2">
       <c r="A288" s="2">
-        <v>46138.97916666666</v>
+        <v>46142.97916666666</v>
       </c>
       <c r="B288">
-        <v>1407</v>
+        <v>0</v>
       </c>
     </row>
     <row r="289" spans="1:2">
       <c r="A289" s="2">
-        <v>46138.98958333334</v>
+        <v>46142.98958333334</v>
       </c>
       <c r="B289">
-        <v>1402</v>
-      </c>
-    </row>
-    <row r="290" spans="1:2">
-      <c r="A290" s="2">
-        <v>46139</v>
-      </c>
-      <c r="B290">
-        <v>1215</v>
-      </c>
-    </row>
-    <row r="291" spans="1:2">
-      <c r="A291" s="2">
-        <v>46139.01041666666</v>
-      </c>
-      <c r="B291">
-        <v>1174</v>
-      </c>
-    </row>
-    <row r="292" spans="1:2">
-      <c r="A292" s="2">
-        <v>46139.02083333334</v>
-      </c>
-      <c r="B292">
-        <v>1173</v>
-      </c>
-    </row>
-    <row r="293" spans="1:2">
-      <c r="A293" s="2">
-        <v>46139.03125</v>
-      </c>
-      <c r="B293">
-        <v>1171</v>
-      </c>
-    </row>
-    <row r="294" spans="1:2">
-      <c r="A294" s="2">
-        <v>46139.04166666666</v>
-      </c>
-      <c r="B294">
-        <v>1158</v>
-      </c>
-    </row>
-    <row r="295" spans="1:2">
-      <c r="A295" s="2">
-        <v>46139.05208333334</v>
-      </c>
-      <c r="B295">
-        <v>1146</v>
-      </c>
-    </row>
-    <row r="296" spans="1:2">
-      <c r="A296" s="2">
-        <v>46139.0625</v>
-      </c>
-      <c r="B296">
-        <v>1134</v>
-      </c>
-    </row>
-    <row r="297" spans="1:2">
-      <c r="A297" s="2">
-        <v>46139.07291666666</v>
-      </c>
-      <c r="B297">
-        <v>1196</v>
-      </c>
-    </row>
-    <row r="298" spans="1:2">
-      <c r="A298" s="2">
-        <v>46139.08333333334</v>
-      </c>
-      <c r="B298">
-        <v>1201</v>
-      </c>
-    </row>
-    <row r="299" spans="1:2">
-      <c r="A299" s="2">
-        <v>46139.09375</v>
-      </c>
-      <c r="B299">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="300" spans="1:2">
-      <c r="A300" s="2">
-        <v>46139.10416666666</v>
-      </c>
-      <c r="B300">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="301" spans="1:2">
-      <c r="A301" s="2">
-        <v>46139.11458333334</v>
-      </c>
-      <c r="B301">
-        <v>1203</v>
-      </c>
-    </row>
-    <row r="302" spans="1:2">
-      <c r="A302" s="2">
-        <v>46139.125</v>
-      </c>
-      <c r="B302">
-        <v>1208</v>
-      </c>
-    </row>
-    <row r="303" spans="1:2">
-      <c r="A303" s="2">
-        <v>46139.13541666666</v>
-      </c>
-      <c r="B303">
-        <v>1206</v>
-      </c>
-    </row>
-    <row r="304" spans="1:2">
-      <c r="A304" s="2">
-        <v>46139.14583333334</v>
-      </c>
-      <c r="B304">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="305" spans="1:2">
-      <c r="A305" s="2">
-        <v>46139.15625</v>
-      </c>
-      <c r="B305">
-        <v>1229</v>
-      </c>
-    </row>
-    <row r="306" spans="1:2">
-      <c r="A306" s="2">
-        <v>46139.16666666666</v>
-      </c>
-      <c r="B306">
-        <v>1332</v>
-      </c>
-    </row>
-    <row r="307" spans="1:2">
-      <c r="A307" s="2">
-        <v>46139.17708333334</v>
-      </c>
-      <c r="B307">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="308" spans="1:2">
-      <c r="A308" s="2">
-        <v>46139.1875</v>
-      </c>
-      <c r="B308">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="309" spans="1:2">
-      <c r="A309" s="2">
-        <v>46139.19791666666</v>
-      </c>
-      <c r="B309">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="310" spans="1:2">
-      <c r="A310" s="2">
-        <v>46139.20833333334</v>
-      </c>
-      <c r="B310">
-        <v>1323</v>
-      </c>
-    </row>
-    <row r="311" spans="1:2">
-      <c r="A311" s="2">
-        <v>46139.21875</v>
-      </c>
-      <c r="B311">
-        <v>1329</v>
-      </c>
-    </row>
-    <row r="312" spans="1:2">
-      <c r="A312" s="2">
-        <v>46139.22916666666</v>
-      </c>
-      <c r="B312">
-        <v>1332</v>
-      </c>
-    </row>
-    <row r="313" spans="1:2">
-      <c r="A313" s="2">
-        <v>46139.23958333334</v>
-      </c>
-      <c r="B313">
-        <v>1331</v>
-      </c>
-    </row>
-    <row r="314" spans="1:2">
-      <c r="A314" s="2">
-        <v>46139.25</v>
-      </c>
-      <c r="B314">
-        <v>1369</v>
-      </c>
-    </row>
-    <row r="315" spans="1:2">
-      <c r="A315" s="2">
-        <v>46139.26041666666</v>
-      </c>
-      <c r="B315">
-        <v>1366</v>
-      </c>
-    </row>
-    <row r="316" spans="1:2">
-      <c r="A316" s="2">
-        <v>46139.27083333334</v>
-      </c>
-      <c r="B316">
-        <v>1362</v>
-      </c>
-    </row>
-    <row r="317" spans="1:2">
-      <c r="A317" s="2">
-        <v>46139.28125</v>
-      </c>
-      <c r="B317">
-        <v>1360</v>
-      </c>
-    </row>
-    <row r="318" spans="1:2">
-      <c r="A318" s="2">
-        <v>46139.29166666666</v>
-      </c>
-      <c r="B318">
-        <v>1324</v>
-      </c>
-    </row>
-    <row r="319" spans="1:2">
-      <c r="A319" s="2">
-        <v>46139.30208333334</v>
-      </c>
-      <c r="B319">
-        <v>1316</v>
-      </c>
-    </row>
-    <row r="320" spans="1:2">
-      <c r="A320" s="2">
-        <v>46139.3125</v>
-      </c>
-      <c r="B320">
-        <v>1309</v>
-      </c>
-    </row>
-    <row r="321" spans="1:2">
-      <c r="A321" s="2">
-        <v>46139.32291666666</v>
-      </c>
-      <c r="B321">
-        <v>1313</v>
-      </c>
-    </row>
-    <row r="322" spans="1:2">
-      <c r="A322" s="2">
-        <v>46139.33333333334</v>
-      </c>
-      <c r="B322">
-        <v>1311</v>
-      </c>
-    </row>
-    <row r="323" spans="1:2">
-      <c r="A323" s="2">
-        <v>46139.34375</v>
-      </c>
-      <c r="B323">
-        <v>1310</v>
-      </c>
-    </row>
-    <row r="324" spans="1:2">
-      <c r="A324" s="2">
-        <v>46139.35416666666</v>
-      </c>
-      <c r="B324">
-        <v>1255</v>
-      </c>
-    </row>
-    <row r="325" spans="1:2">
-      <c r="A325" s="2">
-        <v>46139.36458333334</v>
-      </c>
-      <c r="B325">
-        <v>1252</v>
-      </c>
-    </row>
-    <row r="326" spans="1:2">
-      <c r="A326" s="2">
-        <v>46139.375</v>
-      </c>
-      <c r="B326">
-        <v>1013</v>
-      </c>
-    </row>
-    <row r="327" spans="1:2">
-      <c r="A327" s="2">
-        <v>46139.38541666666</v>
-      </c>
-      <c r="B327">
-        <v>981</v>
-      </c>
-    </row>
-    <row r="328" spans="1:2">
-      <c r="A328" s="2">
-        <v>46139.39583333334</v>
-      </c>
-      <c r="B328">
-        <v>976</v>
-      </c>
-    </row>
-    <row r="329" spans="1:2">
-      <c r="A329" s="2">
-        <v>46139.40625</v>
-      </c>
-      <c r="B329">
-        <v>1007</v>
-      </c>
-    </row>
-    <row r="330" spans="1:2">
-      <c r="A330" s="2">
-        <v>46139.41666666666</v>
-      </c>
-      <c r="B330">
-        <v>641</v>
-      </c>
-    </row>
-    <row r="331" spans="1:2">
-      <c r="A331" s="2">
-        <v>46139.42708333334</v>
-      </c>
-      <c r="B331">
-        <v>574</v>
-      </c>
-    </row>
-    <row r="332" spans="1:2">
-      <c r="A332" s="2">
-        <v>46139.4375</v>
-      </c>
-      <c r="B332">
-        <v>573</v>
-      </c>
-    </row>
-    <row r="333" spans="1:2">
-      <c r="A333" s="2">
-        <v>46139.44791666666</v>
-      </c>
-      <c r="B333">
-        <v>572</v>
-      </c>
-    </row>
-    <row r="334" spans="1:2">
-      <c r="A334" s="2">
-        <v>46139.45833333334</v>
-      </c>
-      <c r="B334">
-        <v>569</v>
-      </c>
-    </row>
-    <row r="335" spans="1:2">
-      <c r="A335" s="2">
-        <v>46139.46875</v>
-      </c>
-      <c r="B335">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="336" spans="1:2">
-      <c r="A336" s="2">
-        <v>46139.47916666666</v>
-      </c>
-      <c r="B336">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="337" spans="1:2">
-      <c r="A337" s="2">
-        <v>46139.48958333334</v>
-      </c>
-      <c r="B337">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="338" spans="1:2">
-      <c r="A338" s="2">
-        <v>46139.5</v>
-      </c>
-      <c r="B338">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="339" spans="1:2">
-      <c r="A339" s="2">
-        <v>46139.51041666666</v>
-      </c>
-      <c r="B339">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="340" spans="1:2">
-      <c r="A340" s="2">
-        <v>46139.52083333334</v>
-      </c>
-      <c r="B340">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="341" spans="1:2">
-      <c r="A341" s="2">
-        <v>46139.53125</v>
-      </c>
-      <c r="B341">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="342" spans="1:2">
-      <c r="A342" s="2">
-        <v>46139.54166666666</v>
-      </c>
-      <c r="B342">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="343" spans="1:2">
-      <c r="A343" s="2">
-        <v>46139.55208333334</v>
-      </c>
-      <c r="B343">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="344" spans="1:2">
-      <c r="A344" s="2">
-        <v>46139.5625</v>
-      </c>
-      <c r="B344">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="345" spans="1:2">
-      <c r="A345" s="2">
-        <v>46139.57291666666</v>
-      </c>
-      <c r="B345">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="346" spans="1:2">
-      <c r="A346" s="2">
-        <v>46139.58333333334</v>
-      </c>
-      <c r="B346">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="347" spans="1:2">
-      <c r="A347" s="2">
-        <v>46139.59375</v>
-      </c>
-      <c r="B347">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="348" spans="1:2">
-      <c r="A348" s="2">
-        <v>46139.60416666666</v>
-      </c>
-      <c r="B348">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="349" spans="1:2">
-      <c r="A349" s="2">
-        <v>46139.61458333334</v>
-      </c>
-      <c r="B349">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="350" spans="1:2">
-      <c r="A350" s="2">
-        <v>46139.625</v>
-      </c>
-      <c r="B350">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="351" spans="1:2">
-      <c r="A351" s="2">
-        <v>46139.63541666666</v>
-      </c>
-      <c r="B351">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="352" spans="1:2">
-      <c r="A352" s="2">
-        <v>46139.64583333334</v>
-      </c>
-      <c r="B352">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="353" spans="1:2">
-      <c r="A353" s="2">
-        <v>46139.65625</v>
-      </c>
-      <c r="B353">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="354" spans="1:2">
-      <c r="A354" s="2">
-        <v>46139.66666666666</v>
-      </c>
-      <c r="B354">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="355" spans="1:2">
-      <c r="A355" s="2">
-        <v>46139.67708333334</v>
-      </c>
-      <c r="B355">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="356" spans="1:2">
-      <c r="A356" s="2">
-        <v>46139.6875</v>
-      </c>
-      <c r="B356">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="357" spans="1:2">
-      <c r="A357" s="2">
-        <v>46139.69791666666</v>
-      </c>
-      <c r="B357">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="358" spans="1:2">
-      <c r="A358" s="2">
-        <v>46139.70833333334</v>
-      </c>
-      <c r="B358">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="359" spans="1:2">
-      <c r="A359" s="2">
-        <v>46139.71875</v>
-      </c>
-      <c r="B359">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="360" spans="1:2">
-      <c r="A360" s="2">
-        <v>46139.72916666666</v>
-      </c>
-      <c r="B360">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="361" spans="1:2">
-      <c r="A361" s="2">
-        <v>46139.73958333334</v>
-      </c>
-      <c r="B361">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="362" spans="1:2">
-      <c r="A362" s="2">
-        <v>46139.75</v>
-      </c>
-      <c r="B362">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="363" spans="1:2">
-      <c r="A363" s="2">
-        <v>46139.76041666666</v>
-      </c>
-      <c r="B363">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="364" spans="1:2">
-      <c r="A364" s="2">
-        <v>46139.77083333334</v>
-      </c>
-      <c r="B364">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="365" spans="1:2">
-      <c r="A365" s="2">
-        <v>46139.78125</v>
-      </c>
-      <c r="B365">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="366" spans="1:2">
-      <c r="A366" s="2">
-        <v>46139.79166666666</v>
-      </c>
-      <c r="B366">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="367" spans="1:2">
-      <c r="A367" s="2">
-        <v>46139.80208333334</v>
-      </c>
-      <c r="B367">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="368" spans="1:2">
-      <c r="A368" s="2">
-        <v>46139.8125</v>
-      </c>
-      <c r="B368">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="369" spans="1:2">
-      <c r="A369" s="2">
-        <v>46139.82291666666</v>
-      </c>
-      <c r="B369">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="370" spans="1:2">
-      <c r="A370" s="2">
-        <v>46139.83333333334</v>
-      </c>
-      <c r="B370">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="371" spans="1:2">
-      <c r="A371" s="2">
-        <v>46139.84375</v>
-      </c>
-      <c r="B371">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="372" spans="1:2">
-      <c r="A372" s="2">
-        <v>46139.85416666666</v>
-      </c>
-      <c r="B372">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="373" spans="1:2">
-      <c r="A373" s="2">
-        <v>46139.86458333334</v>
-      </c>
-      <c r="B373">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="374" spans="1:2">
-      <c r="A374" s="2">
-        <v>46139.875</v>
-      </c>
-      <c r="B374">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="375" spans="1:2">
-      <c r="A375" s="2">
-        <v>46139.88541666666</v>
-      </c>
-      <c r="B375">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="376" spans="1:2">
-      <c r="A376" s="2">
-        <v>46139.89583333334</v>
-      </c>
-      <c r="B376">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="377" spans="1:2">
-      <c r="A377" s="2">
-        <v>46139.90625</v>
-      </c>
-      <c r="B377">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="378" spans="1:2">
-      <c r="A378" s="2">
-        <v>46139.91666666666</v>
-      </c>
-      <c r="B378">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="379" spans="1:2">
-      <c r="A379" s="2">
-        <v>46139.92708333334</v>
-      </c>
-      <c r="B379">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="380" spans="1:2">
-      <c r="A380" s="2">
-        <v>46139.9375</v>
-      </c>
-      <c r="B380">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="381" spans="1:2">
-      <c r="A381" s="2">
-        <v>46139.94791666666</v>
-      </c>
-      <c r="B381">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="382" spans="1:2">
-      <c r="A382" s="2">
-        <v>46139.95833333334</v>
-      </c>
-      <c r="B382">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="383" spans="1:2">
-      <c r="A383" s="2">
-        <v>46139.96875</v>
-      </c>
-      <c r="B383">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="384" spans="1:2">
-      <c r="A384" s="2">
-        <v>46139.97916666666</v>
-      </c>
-      <c r="B384">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="385" spans="1:2">
-      <c r="A385" s="2">
-        <v>46139.98958333334</v>
-      </c>
-      <c r="B385">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Updating the model for Necaluxan
</commit_message>
<xml_diff>
--- a/data_fetching/Entsoe/Actual_Production_Hydro_River.xlsx
+++ b/data_fetching/Entsoe/Actual_Production_Hydro_River.xlsx
@@ -381,7 +381,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B289"/>
+  <dimension ref="A1:B481"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:2">
@@ -394,255 +394,255 @@
     </row>
     <row r="2" spans="1:2">
       <c r="A2" s="2">
-        <v>46140</v>
+        <v>46142</v>
       </c>
       <c r="B2">
-        <v>1123</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="3" spans="1:2">
       <c r="A3" s="2">
-        <v>46140.01041666666</v>
+        <v>46142.01041666666</v>
       </c>
       <c r="B3">
-        <v>1112</v>
+        <v>995</v>
       </c>
     </row>
     <row r="4" spans="1:2">
       <c r="A4" s="2">
-        <v>46140.02083333334</v>
+        <v>46142.02083333334</v>
       </c>
       <c r="B4">
-        <v>1119</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5" spans="1:2">
       <c r="A5" s="2">
-        <v>46140.03125</v>
+        <v>46142.03125</v>
       </c>
       <c r="B5">
-        <v>1154</v>
+        <v>993</v>
       </c>
     </row>
     <row r="6" spans="1:2">
       <c r="A6" s="2">
-        <v>46140.04166666666</v>
+        <v>46142.04166666666</v>
       </c>
       <c r="B6">
-        <v>1058</v>
+        <v>954</v>
       </c>
     </row>
     <row r="7" spans="1:2">
       <c r="A7" s="2">
-        <v>46140.05208333334</v>
+        <v>46142.05208333334</v>
       </c>
       <c r="B7">
-        <v>1044</v>
+        <v>955</v>
       </c>
     </row>
     <row r="8" spans="1:2">
       <c r="A8" s="2">
-        <v>46140.0625</v>
+        <v>46142.0625</v>
       </c>
       <c r="B8">
-        <v>1050</v>
+        <v>0</v>
       </c>
     </row>
     <row r="9" spans="1:2">
       <c r="A9" s="2">
-        <v>46140.07291666666</v>
+        <v>46142.07291666666</v>
       </c>
       <c r="B9">
-        <v>1052</v>
+        <v>954</v>
       </c>
     </row>
     <row r="10" spans="1:2">
       <c r="A10" s="2">
-        <v>46140.08333333334</v>
+        <v>46142.08333333334</v>
       </c>
       <c r="B10">
-        <v>1057</v>
+        <v>955</v>
       </c>
     </row>
     <row r="11" spans="1:2">
       <c r="A11" s="2">
-        <v>46140.09375</v>
+        <v>46142.09375</v>
       </c>
       <c r="B11">
-        <v>1058</v>
+        <v>956</v>
       </c>
     </row>
     <row r="12" spans="1:2">
       <c r="A12" s="2">
-        <v>46140.10416666666</v>
+        <v>46142.10416666666</v>
       </c>
       <c r="B12">
-        <v>1056</v>
+        <v>969</v>
       </c>
     </row>
     <row r="13" spans="1:2">
       <c r="A13" s="2">
-        <v>46140.11458333334</v>
+        <v>46142.11458333334</v>
       </c>
       <c r="B13">
-        <v>1055</v>
+        <v>966</v>
       </c>
     </row>
     <row r="14" spans="1:2">
       <c r="A14" s="2">
-        <v>46140.125</v>
+        <v>46142.125</v>
       </c>
       <c r="B14">
-        <v>926</v>
+        <v>970</v>
       </c>
     </row>
     <row r="15" spans="1:2">
       <c r="A15" s="2">
-        <v>46140.13541666666</v>
+        <v>46142.13541666666</v>
       </c>
       <c r="B15">
-        <v>921</v>
+        <v>969</v>
       </c>
     </row>
     <row r="16" spans="1:2">
       <c r="A16" s="2">
-        <v>46140.14583333334</v>
+        <v>46142.14583333334</v>
       </c>
       <c r="B16">
-        <v>0</v>
+        <v>970</v>
       </c>
     </row>
     <row r="17" spans="1:2">
       <c r="A17" s="2">
-        <v>46140.15625</v>
+        <v>46142.15625</v>
       </c>
       <c r="B17">
-        <v>0</v>
+        <v>969</v>
       </c>
     </row>
     <row r="18" spans="1:2">
       <c r="A18" s="2">
-        <v>46140.16666666666</v>
+        <v>46142.16666666666</v>
       </c>
       <c r="B18">
-        <v>927</v>
+        <v>972</v>
       </c>
     </row>
     <row r="19" spans="1:2">
       <c r="A19" s="2">
-        <v>46140.17708333334</v>
+        <v>46142.17708333334</v>
       </c>
       <c r="B19">
-        <v>926</v>
+        <v>0</v>
       </c>
     </row>
     <row r="20" spans="1:2">
       <c r="A20" s="2">
-        <v>46140.1875</v>
+        <v>46142.1875</v>
       </c>
       <c r="B20">
-        <v>927</v>
+        <v>971</v>
       </c>
     </row>
     <row r="21" spans="1:2">
       <c r="A21" s="2">
-        <v>46140.19791666666</v>
+        <v>46142.19791666666</v>
       </c>
       <c r="B21">
-        <v>923</v>
+        <v>975</v>
       </c>
     </row>
     <row r="22" spans="1:2">
       <c r="A22" s="2">
-        <v>46140.20833333334</v>
+        <v>46142.20833333334</v>
       </c>
       <c r="B22">
-        <v>1116</v>
+        <v>1057</v>
       </c>
     </row>
     <row r="23" spans="1:2">
       <c r="A23" s="2">
-        <v>46140.21875</v>
+        <v>46142.21875</v>
       </c>
       <c r="B23">
-        <v>1135</v>
+        <v>1067</v>
       </c>
     </row>
     <row r="24" spans="1:2">
       <c r="A24" s="2">
-        <v>46140.22916666666</v>
+        <v>46142.22916666666</v>
       </c>
       <c r="B24">
-        <v>1134</v>
+        <v>1064</v>
       </c>
     </row>
     <row r="25" spans="1:2">
       <c r="A25" s="2">
-        <v>46140.23958333334</v>
+        <v>46142.23958333334</v>
       </c>
       <c r="B25">
-        <v>1132</v>
+        <v>1069</v>
       </c>
     </row>
     <row r="26" spans="1:2">
       <c r="A26" s="2">
-        <v>46140.25</v>
+        <v>46142.25</v>
       </c>
       <c r="B26">
-        <v>1209</v>
+        <v>1132</v>
       </c>
     </row>
     <row r="27" spans="1:2">
       <c r="A27" s="2">
-        <v>46140.26041666666</v>
+        <v>46142.26041666666</v>
       </c>
       <c r="B27">
-        <v>1202</v>
+        <v>1138</v>
       </c>
     </row>
     <row r="28" spans="1:2">
       <c r="A28" s="2">
-        <v>46140.27083333334</v>
+        <v>46142.27083333334</v>
       </c>
       <c r="B28">
-        <v>1203</v>
+        <v>1137</v>
       </c>
     </row>
     <row r="29" spans="1:2">
       <c r="A29" s="2">
-        <v>46140.28125</v>
+        <v>46142.28125</v>
       </c>
       <c r="B29">
-        <v>1204</v>
+        <v>0</v>
       </c>
     </row>
     <row r="30" spans="1:2">
       <c r="A30" s="2">
-        <v>46140.29166666666</v>
+        <v>46142.29166666666</v>
       </c>
       <c r="B30">
-        <v>1191</v>
+        <v>1138</v>
       </c>
     </row>
     <row r="31" spans="1:2">
       <c r="A31" s="2">
-        <v>46140.30208333334</v>
+        <v>46142.30208333334</v>
       </c>
       <c r="B31">
-        <v>0</v>
+        <v>1148</v>
       </c>
     </row>
     <row r="32" spans="1:2">
       <c r="A32" s="2">
-        <v>46140.3125</v>
+        <v>46142.3125</v>
       </c>
       <c r="B32">
-        <v>1187</v>
+        <v>1152</v>
       </c>
     </row>
     <row r="33" spans="1:2">
       <c r="A33" s="2">
-        <v>46140.32291666666</v>
+        <v>46142.32291666666</v>
       </c>
       <c r="B33">
         <v>0</v>
@@ -650,159 +650,159 @@
     </row>
     <row r="34" spans="1:2">
       <c r="A34" s="2">
-        <v>46140.33333333334</v>
+        <v>46142.33333333334</v>
       </c>
       <c r="B34">
-        <v>995</v>
+        <v>936</v>
       </c>
     </row>
     <row r="35" spans="1:2">
       <c r="A35" s="2">
-        <v>46140.34375</v>
+        <v>46142.34375</v>
       </c>
       <c r="B35">
-        <v>989</v>
+        <v>916</v>
       </c>
     </row>
     <row r="36" spans="1:2">
       <c r="A36" s="2">
-        <v>46140.35416666666</v>
+        <v>46142.35416666666</v>
       </c>
       <c r="B36">
-        <v>980</v>
+        <v>955</v>
       </c>
     </row>
     <row r="37" spans="1:2">
       <c r="A37" s="2">
-        <v>46140.36458333334</v>
+        <v>46142.36458333334</v>
       </c>
       <c r="B37">
-        <v>938</v>
+        <v>959</v>
       </c>
     </row>
     <row r="38" spans="1:2">
       <c r="A38" s="2">
-        <v>46140.375</v>
+        <v>46142.375</v>
       </c>
       <c r="B38">
-        <v>954</v>
+        <v>904</v>
       </c>
     </row>
     <row r="39" spans="1:2">
       <c r="A39" s="2">
-        <v>46140.38541666666</v>
+        <v>46142.38541666666</v>
       </c>
       <c r="B39">
-        <v>952</v>
+        <v>899</v>
       </c>
     </row>
     <row r="40" spans="1:2">
       <c r="A40" s="2">
-        <v>46140.39583333334</v>
+        <v>46142.39583333334</v>
       </c>
       <c r="B40">
-        <v>953</v>
+        <v>0</v>
       </c>
     </row>
     <row r="41" spans="1:2">
       <c r="A41" s="2">
-        <v>46140.40625</v>
+        <v>46142.40625</v>
       </c>
       <c r="B41">
-        <v>950</v>
+        <v>898</v>
       </c>
     </row>
     <row r="42" spans="1:2">
       <c r="A42" s="2">
-        <v>46140.41666666666</v>
+        <v>46142.41666666666</v>
       </c>
       <c r="B42">
-        <v>607</v>
+        <v>658</v>
       </c>
     </row>
     <row r="43" spans="1:2">
       <c r="A43" s="2">
-        <v>46140.42708333334</v>
+        <v>46142.42708333334</v>
       </c>
       <c r="B43">
-        <v>587</v>
+        <v>643</v>
       </c>
     </row>
     <row r="44" spans="1:2">
       <c r="A44" s="2">
-        <v>46140.4375</v>
+        <v>46142.4375</v>
       </c>
       <c r="B44">
-        <v>0</v>
+        <v>650</v>
       </c>
     </row>
     <row r="45" spans="1:2">
       <c r="A45" s="2">
-        <v>46140.44791666666</v>
+        <v>46142.44791666666</v>
       </c>
       <c r="B45">
-        <v>588</v>
+        <v>595</v>
       </c>
     </row>
     <row r="46" spans="1:2">
       <c r="A46" s="2">
-        <v>46140.45833333334</v>
+        <v>46142.45833333334</v>
       </c>
       <c r="B46">
-        <v>519</v>
+        <v>563</v>
       </c>
     </row>
     <row r="47" spans="1:2">
       <c r="A47" s="2">
-        <v>46140.46875</v>
+        <v>46142.46875</v>
       </c>
       <c r="B47">
-        <v>517</v>
+        <v>561</v>
       </c>
     </row>
     <row r="48" spans="1:2">
       <c r="A48" s="2">
-        <v>46140.47916666666</v>
+        <v>46142.47916666666</v>
       </c>
       <c r="B48">
-        <v>515</v>
+        <v>643</v>
       </c>
     </row>
     <row r="49" spans="1:2">
       <c r="A49" s="2">
-        <v>46140.48958333334</v>
+        <v>46142.48958333334</v>
       </c>
       <c r="B49">
-        <v>0</v>
+        <v>669</v>
       </c>
     </row>
     <row r="50" spans="1:2">
       <c r="A50" s="2">
-        <v>46140.5</v>
+        <v>46142.5</v>
       </c>
       <c r="B50">
-        <v>513</v>
+        <v>662</v>
       </c>
     </row>
     <row r="51" spans="1:2">
       <c r="A51" s="2">
-        <v>46140.51041666666</v>
+        <v>46142.51041666666</v>
       </c>
       <c r="B51">
-        <v>511</v>
+        <v>659</v>
       </c>
     </row>
     <row r="52" spans="1:2">
       <c r="A52" s="2">
-        <v>46140.52083333334</v>
+        <v>46142.52083333334</v>
       </c>
       <c r="B52">
-        <v>512</v>
+        <v>0</v>
       </c>
     </row>
     <row r="53" spans="1:2">
       <c r="A53" s="2">
-        <v>46140.53125</v>
+        <v>46142.53125</v>
       </c>
       <c r="B53">
         <v>0</v>
@@ -810,1143 +810,1143 @@
     </row>
     <row r="54" spans="1:2">
       <c r="A54" s="2">
-        <v>46140.54166666666</v>
+        <v>46142.54166666666</v>
       </c>
       <c r="B54">
-        <v>474</v>
+        <v>670</v>
       </c>
     </row>
     <row r="55" spans="1:2">
       <c r="A55" s="2">
-        <v>46140.55208333334</v>
+        <v>46142.55208333334</v>
       </c>
       <c r="B55">
-        <v>468</v>
+        <v>672</v>
       </c>
     </row>
     <row r="56" spans="1:2">
       <c r="A56" s="2">
-        <v>46140.5625</v>
+        <v>46142.5625</v>
       </c>
       <c r="B56">
-        <v>466</v>
+        <v>0</v>
       </c>
     </row>
     <row r="57" spans="1:2">
       <c r="A57" s="2">
-        <v>46140.57291666666</v>
+        <v>46142.57291666666</v>
       </c>
       <c r="B57">
-        <v>0</v>
+        <v>673</v>
       </c>
     </row>
     <row r="58" spans="1:2">
       <c r="A58" s="2">
-        <v>46140.58333333334</v>
+        <v>46142.58333333334</v>
       </c>
       <c r="B58">
-        <v>474</v>
+        <v>668</v>
       </c>
     </row>
     <row r="59" spans="1:2">
       <c r="A59" s="2">
-        <v>46140.59375</v>
+        <v>46142.59375</v>
       </c>
       <c r="B59">
-        <v>476</v>
+        <v>667</v>
       </c>
     </row>
     <row r="60" spans="1:2">
       <c r="A60" s="2">
-        <v>46140.60416666666</v>
+        <v>46142.60416666666</v>
       </c>
       <c r="B60">
-        <v>475</v>
+        <v>0</v>
       </c>
     </row>
     <row r="61" spans="1:2">
       <c r="A61" s="2">
-        <v>46140.61458333334</v>
+        <v>46142.61458333334</v>
       </c>
       <c r="B61">
-        <v>486</v>
+        <v>668</v>
       </c>
     </row>
     <row r="62" spans="1:2">
       <c r="A62" s="2">
-        <v>46140.625</v>
+        <v>46142.625</v>
       </c>
       <c r="B62">
-        <v>603</v>
+        <v>664</v>
       </c>
     </row>
     <row r="63" spans="1:2">
       <c r="A63" s="2">
-        <v>46140.63541666666</v>
+        <v>46142.63541666666</v>
       </c>
       <c r="B63">
-        <v>607</v>
+        <v>682</v>
       </c>
     </row>
     <row r="64" spans="1:2">
       <c r="A64" s="2">
-        <v>46140.64583333334</v>
+        <v>46142.64583333334</v>
       </c>
       <c r="B64">
-        <v>616</v>
+        <v>658</v>
       </c>
     </row>
     <row r="65" spans="1:2">
       <c r="A65" s="2">
-        <v>46140.65625</v>
+        <v>46142.65625</v>
       </c>
       <c r="B65">
-        <v>628</v>
+        <v>666</v>
       </c>
     </row>
     <row r="66" spans="1:2">
       <c r="A66" s="2">
-        <v>46140.66666666666</v>
+        <v>46142.66666666666</v>
       </c>
       <c r="B66">
-        <v>950</v>
+        <v>928</v>
       </c>
     </row>
     <row r="67" spans="1:2">
       <c r="A67" s="2">
-        <v>46140.67708333334</v>
+        <v>46142.67708333334</v>
       </c>
       <c r="B67">
-        <v>969</v>
+        <v>950</v>
       </c>
     </row>
     <row r="68" spans="1:2">
       <c r="A68" s="2">
-        <v>46140.6875</v>
+        <v>46142.6875</v>
       </c>
       <c r="B68">
-        <v>973</v>
+        <v>951</v>
       </c>
     </row>
     <row r="69" spans="1:2">
       <c r="A69" s="2">
-        <v>46140.69791666666</v>
+        <v>46142.69791666666</v>
       </c>
       <c r="B69">
-        <v>976</v>
+        <v>959</v>
       </c>
     </row>
     <row r="70" spans="1:2">
       <c r="A70" s="2">
-        <v>46140.70833333334</v>
+        <v>46142.70833333334</v>
       </c>
       <c r="B70">
-        <v>1241</v>
+        <v>1090</v>
       </c>
     </row>
     <row r="71" spans="1:2">
       <c r="A71" s="2">
-        <v>46140.71875</v>
+        <v>46142.71875</v>
       </c>
       <c r="B71">
-        <v>1285</v>
+        <v>1101</v>
       </c>
     </row>
     <row r="72" spans="1:2">
       <c r="A72" s="2">
-        <v>46140.72916666666</v>
+        <v>46142.72916666666</v>
       </c>
       <c r="B72">
-        <v>1287</v>
+        <v>1096</v>
       </c>
     </row>
     <row r="73" spans="1:2">
       <c r="A73" s="2">
-        <v>46140.73958333334</v>
+        <v>46142.73958333334</v>
       </c>
       <c r="B73">
-        <v>1285</v>
+        <v>1104</v>
       </c>
     </row>
     <row r="74" spans="1:2">
       <c r="A74" s="2">
-        <v>46140.75</v>
+        <v>46142.75</v>
       </c>
       <c r="B74">
-        <v>1318</v>
+        <v>1256</v>
       </c>
     </row>
     <row r="75" spans="1:2">
       <c r="A75" s="2">
-        <v>46140.76041666666</v>
+        <v>46142.76041666666</v>
       </c>
       <c r="B75">
-        <v>1320</v>
+        <v>1268</v>
       </c>
     </row>
     <row r="76" spans="1:2">
       <c r="A76" s="2">
-        <v>46140.77083333334</v>
+        <v>46142.77083333334</v>
       </c>
       <c r="B76">
-        <v>1353</v>
+        <v>1260</v>
       </c>
     </row>
     <row r="77" spans="1:2">
       <c r="A77" s="2">
-        <v>46140.78125</v>
+        <v>46142.78125</v>
       </c>
       <c r="B77">
-        <v>1358</v>
+        <v>1230</v>
       </c>
     </row>
     <row r="78" spans="1:2">
       <c r="A78" s="2">
-        <v>46140.79166666666</v>
+        <v>46142.79166666666</v>
       </c>
       <c r="B78">
-        <v>0</v>
+        <v>1254</v>
       </c>
     </row>
     <row r="79" spans="1:2">
       <c r="A79" s="2">
-        <v>46140.80208333334</v>
+        <v>46142.80208333334</v>
       </c>
       <c r="B79">
-        <v>1361</v>
+        <v>1270</v>
       </c>
     </row>
     <row r="80" spans="1:2">
       <c r="A80" s="2">
-        <v>46140.8125</v>
+        <v>46142.8125</v>
       </c>
       <c r="B80">
-        <v>1362</v>
+        <v>1272</v>
       </c>
     </row>
     <row r="81" spans="1:2">
       <c r="A81" s="2">
-        <v>46140.82291666666</v>
+        <v>46142.82291666666</v>
       </c>
       <c r="B81">
-        <v>1360</v>
+        <v>1268</v>
       </c>
     </row>
     <row r="82" spans="1:2">
       <c r="A82" s="2">
-        <v>46140.83333333334</v>
+        <v>46142.83333333334</v>
       </c>
       <c r="B82">
-        <v>1382</v>
+        <v>1260</v>
       </c>
     </row>
     <row r="83" spans="1:2">
       <c r="A83" s="2">
-        <v>46140.84375</v>
+        <v>46142.84375</v>
       </c>
       <c r="B83">
-        <v>1379</v>
+        <v>1259</v>
       </c>
     </row>
     <row r="84" spans="1:2">
       <c r="A84" s="2">
-        <v>46140.85416666666</v>
+        <v>46142.85416666666</v>
       </c>
       <c r="B84">
-        <v>1369</v>
+        <v>1256</v>
       </c>
     </row>
     <row r="85" spans="1:2">
       <c r="A85" s="2">
-        <v>46140.86458333334</v>
+        <v>46142.86458333334</v>
       </c>
       <c r="B85">
-        <v>1370</v>
+        <v>1259</v>
       </c>
     </row>
     <row r="86" spans="1:2">
       <c r="A86" s="2">
-        <v>46140.875</v>
+        <v>46142.875</v>
       </c>
       <c r="B86">
-        <v>1365</v>
+        <v>1217</v>
       </c>
     </row>
     <row r="87" spans="1:2">
       <c r="A87" s="2">
-        <v>46140.88541666666</v>
+        <v>46142.88541666666</v>
       </c>
       <c r="B87">
-        <v>1387</v>
+        <v>1214</v>
       </c>
     </row>
     <row r="88" spans="1:2">
       <c r="A88" s="2">
-        <v>46140.89583333334</v>
+        <v>46142.89583333334</v>
       </c>
       <c r="B88">
-        <v>1393</v>
+        <v>1210</v>
       </c>
     </row>
     <row r="89" spans="1:2">
       <c r="A89" s="2">
-        <v>46140.90625</v>
+        <v>46142.90625</v>
       </c>
       <c r="B89">
-        <v>1390</v>
+        <v>1212</v>
       </c>
     </row>
     <row r="90" spans="1:2">
       <c r="A90" s="2">
-        <v>46140.91666666666</v>
+        <v>46142.91666666666</v>
       </c>
       <c r="B90">
-        <v>1311</v>
+        <v>1088</v>
       </c>
     </row>
     <row r="91" spans="1:2">
       <c r="A91" s="2">
-        <v>46140.92708333334</v>
+        <v>46142.92708333334</v>
       </c>
       <c r="B91">
-        <v>1297</v>
+        <v>1065</v>
       </c>
     </row>
     <row r="92" spans="1:2">
       <c r="A92" s="2">
-        <v>46140.9375</v>
+        <v>46142.9375</v>
       </c>
       <c r="B92">
-        <v>0</v>
+        <v>1061</v>
       </c>
     </row>
     <row r="93" spans="1:2">
       <c r="A93" s="2">
-        <v>46140.94791666666</v>
+        <v>46142.94791666666</v>
       </c>
       <c r="B93">
-        <v>1298</v>
+        <v>1064</v>
       </c>
     </row>
     <row r="94" spans="1:2">
       <c r="A94" s="2">
-        <v>46140.95833333334</v>
+        <v>46142.95833333334</v>
       </c>
       <c r="B94">
-        <v>1230</v>
+        <v>1062</v>
       </c>
     </row>
     <row r="95" spans="1:2">
       <c r="A95" s="2">
-        <v>46140.96875</v>
+        <v>46142.96875</v>
       </c>
       <c r="B95">
-        <v>1225</v>
+        <v>1050</v>
       </c>
     </row>
     <row r="96" spans="1:2">
       <c r="A96" s="2">
-        <v>46140.97916666666</v>
+        <v>46142.97916666666</v>
       </c>
       <c r="B96">
-        <v>1222</v>
+        <v>0</v>
       </c>
     </row>
     <row r="97" spans="1:2">
       <c r="A97" s="2">
-        <v>46140.98958333334</v>
+        <v>46142.98958333334</v>
       </c>
       <c r="B97">
-        <v>1221</v>
+        <v>1052</v>
       </c>
     </row>
     <row r="98" spans="1:2">
       <c r="A98" s="2">
-        <v>46141</v>
+        <v>46143</v>
       </c>
       <c r="B98">
-        <v>1055</v>
+        <v>1046</v>
       </c>
     </row>
     <row r="99" spans="1:2">
       <c r="A99" s="2">
-        <v>46141.01041666666</v>
+        <v>46143.01041666666</v>
       </c>
       <c r="B99">
-        <v>1032</v>
+        <v>1042</v>
       </c>
     </row>
     <row r="100" spans="1:2">
       <c r="A100" s="2">
-        <v>46141.02083333334</v>
+        <v>46143.02083333334</v>
       </c>
       <c r="B100">
-        <v>1031</v>
+        <v>1095</v>
       </c>
     </row>
     <row r="101" spans="1:2">
       <c r="A101" s="2">
-        <v>46141.03125</v>
+        <v>46143.03125</v>
       </c>
       <c r="B101">
-        <v>1023</v>
+        <v>1107</v>
       </c>
     </row>
     <row r="102" spans="1:2">
       <c r="A102" s="2">
-        <v>46141.04166666666</v>
+        <v>46143.04166666666</v>
       </c>
       <c r="B102">
-        <v>1015</v>
+        <v>1138</v>
       </c>
     </row>
     <row r="103" spans="1:2">
       <c r="A103" s="2">
-        <v>46141.05208333334</v>
+        <v>46143.05208333334</v>
       </c>
       <c r="B103">
-        <v>1012</v>
+        <v>1135</v>
       </c>
     </row>
     <row r="104" spans="1:2">
       <c r="A104" s="2">
-        <v>46141.0625</v>
+        <v>46143.0625</v>
       </c>
       <c r="B104">
-        <v>1013</v>
+        <v>1137</v>
       </c>
     </row>
     <row r="105" spans="1:2">
       <c r="A105" s="2">
-        <v>46141.07291666666</v>
+        <v>46143.07291666666</v>
       </c>
       <c r="B105">
-        <v>1012</v>
+        <v>1135</v>
       </c>
     </row>
     <row r="106" spans="1:2">
       <c r="A106" s="2">
-        <v>46141.08333333334</v>
+        <v>46143.08333333334</v>
       </c>
       <c r="B106">
-        <v>1013</v>
+        <v>1122</v>
       </c>
     </row>
     <row r="107" spans="1:2">
       <c r="A107" s="2">
-        <v>46141.09375</v>
+        <v>46143.09375</v>
       </c>
       <c r="B107">
-        <v>1012</v>
+        <v>1118</v>
       </c>
     </row>
     <row r="108" spans="1:2">
       <c r="A108" s="2">
-        <v>46141.10416666666</v>
+        <v>46143.10416666666</v>
       </c>
       <c r="B108">
-        <v>1014</v>
+        <v>1117</v>
       </c>
     </row>
     <row r="109" spans="1:2">
       <c r="A109" s="2">
-        <v>46141.11458333334</v>
+        <v>46143.11458333334</v>
       </c>
       <c r="B109">
-        <v>1011</v>
+        <v>0</v>
       </c>
     </row>
     <row r="110" spans="1:2">
       <c r="A110" s="2">
-        <v>46141.125</v>
+        <v>46143.125</v>
       </c>
       <c r="B110">
-        <v>0</v>
+        <v>1095</v>
       </c>
     </row>
     <row r="111" spans="1:2">
       <c r="A111" s="2">
-        <v>46141.13541666666</v>
+        <v>46143.13541666666</v>
       </c>
       <c r="B111">
-        <v>1012</v>
+        <v>1090</v>
       </c>
     </row>
     <row r="112" spans="1:2">
       <c r="A112" s="2">
-        <v>46141.14583333334</v>
+        <v>46143.14583333334</v>
       </c>
       <c r="B112">
-        <v>0</v>
+        <v>1094</v>
       </c>
     </row>
     <row r="113" spans="1:2">
       <c r="A113" s="2">
-        <v>46141.15625</v>
+        <v>46143.15625</v>
       </c>
       <c r="B113">
-        <v>1009</v>
+        <v>1095</v>
       </c>
     </row>
     <row r="114" spans="1:2">
       <c r="A114" s="2">
-        <v>46141.16666666666</v>
+        <v>46143.16666666666</v>
       </c>
       <c r="B114">
-        <v>1015</v>
+        <v>1094</v>
       </c>
     </row>
     <row r="115" spans="1:2">
       <c r="A115" s="2">
-        <v>46141.17708333334</v>
+        <v>46143.17708333334</v>
       </c>
       <c r="B115">
-        <v>0</v>
+        <v>1092</v>
       </c>
     </row>
     <row r="116" spans="1:2">
       <c r="A116" s="2">
-        <v>46141.1875</v>
+        <v>46143.1875</v>
       </c>
       <c r="B116">
-        <v>1018</v>
+        <v>1048</v>
       </c>
     </row>
     <row r="117" spans="1:2">
       <c r="A117" s="2">
-        <v>46141.19791666666</v>
+        <v>46143.19791666666</v>
       </c>
       <c r="B117">
-        <v>1025</v>
+        <v>1046</v>
       </c>
     </row>
     <row r="118" spans="1:2">
       <c r="A118" s="2">
-        <v>46141.20833333334</v>
+        <v>46143.20833333334</v>
       </c>
       <c r="B118">
-        <v>1235</v>
+        <v>1070</v>
       </c>
     </row>
     <row r="119" spans="1:2">
       <c r="A119" s="2">
-        <v>46141.21875</v>
+        <v>46143.21875</v>
       </c>
       <c r="B119">
-        <v>1243</v>
+        <v>1073</v>
       </c>
     </row>
     <row r="120" spans="1:2">
       <c r="A120" s="2">
-        <v>46141.22916666666</v>
+        <v>46143.22916666666</v>
       </c>
       <c r="B120">
-        <v>1244</v>
+        <v>1074</v>
       </c>
     </row>
     <row r="121" spans="1:2">
       <c r="A121" s="2">
-        <v>46141.23958333334</v>
+        <v>46143.23958333334</v>
       </c>
       <c r="B121">
-        <v>0</v>
+        <v>1065</v>
       </c>
     </row>
     <row r="122" spans="1:2">
       <c r="A122" s="2">
-        <v>46141.25</v>
+        <v>46143.25</v>
       </c>
       <c r="B122">
-        <v>1211</v>
+        <v>1048</v>
       </c>
     </row>
     <row r="123" spans="1:2">
       <c r="A123" s="2">
-        <v>46141.26041666666</v>
+        <v>46143.26041666666</v>
       </c>
       <c r="B123">
-        <v>1200</v>
+        <v>1052</v>
       </c>
     </row>
     <row r="124" spans="1:2">
       <c r="A124" s="2">
-        <v>46141.27083333334</v>
+        <v>46143.27083333334</v>
       </c>
       <c r="B124">
-        <v>1205</v>
+        <v>1051</v>
       </c>
     </row>
     <row r="125" spans="1:2">
       <c r="A125" s="2">
-        <v>46141.28125</v>
+        <v>46143.28125</v>
       </c>
       <c r="B125">
-        <v>1204</v>
+        <v>1052</v>
       </c>
     </row>
     <row r="126" spans="1:2">
       <c r="A126" s="2">
-        <v>46141.29166666666</v>
+        <v>46143.29166666666</v>
       </c>
       <c r="B126">
-        <v>1185</v>
+        <v>1108</v>
       </c>
     </row>
     <row r="127" spans="1:2">
       <c r="A127" s="2">
-        <v>46141.30208333334</v>
+        <v>46143.30208333334</v>
       </c>
       <c r="B127">
-        <v>1183</v>
+        <v>1103</v>
       </c>
     </row>
     <row r="128" spans="1:2">
       <c r="A128" s="2">
-        <v>46141.3125</v>
+        <v>46143.3125</v>
       </c>
       <c r="B128">
-        <v>1184</v>
+        <v>1094</v>
       </c>
     </row>
     <row r="129" spans="1:2">
       <c r="A129" s="2">
-        <v>46141.32291666666</v>
+        <v>46143.32291666666</v>
       </c>
       <c r="B129">
-        <v>1183</v>
+        <v>1082</v>
       </c>
     </row>
     <row r="130" spans="1:2">
       <c r="A130" s="2">
-        <v>46141.33333333334</v>
+        <v>46143.33333333334</v>
       </c>
       <c r="B130">
-        <v>930</v>
+        <v>703</v>
       </c>
     </row>
     <row r="131" spans="1:2">
       <c r="A131" s="2">
-        <v>46141.34375</v>
+        <v>46143.34375</v>
       </c>
       <c r="B131">
-        <v>831</v>
+        <v>692</v>
       </c>
     </row>
     <row r="132" spans="1:2">
       <c r="A132" s="2">
-        <v>46141.35416666666</v>
+        <v>46143.35416666666</v>
       </c>
       <c r="B132">
-        <v>830</v>
+        <v>688</v>
       </c>
     </row>
     <row r="133" spans="1:2">
       <c r="A133" s="2">
-        <v>46141.36458333334</v>
+        <v>46143.36458333334</v>
       </c>
       <c r="B133">
-        <v>821</v>
+        <v>0</v>
       </c>
     </row>
     <row r="134" spans="1:2">
       <c r="A134" s="2">
-        <v>46141.375</v>
+        <v>46143.375</v>
       </c>
       <c r="B134">
-        <v>794</v>
+        <v>583</v>
       </c>
     </row>
     <row r="135" spans="1:2">
       <c r="A135" s="2">
-        <v>46141.38541666666</v>
+        <v>46143.38541666666</v>
       </c>
       <c r="B135">
-        <v>871</v>
+        <v>577</v>
       </c>
     </row>
     <row r="136" spans="1:2">
       <c r="A136" s="2">
-        <v>46141.39583333334</v>
+        <v>46143.39583333334</v>
       </c>
       <c r="B136">
-        <v>885</v>
+        <v>451</v>
       </c>
     </row>
     <row r="137" spans="1:2">
       <c r="A137" s="2">
-        <v>46141.40625</v>
+        <v>46143.40625</v>
       </c>
       <c r="B137">
-        <v>888</v>
+        <v>440</v>
       </c>
     </row>
     <row r="138" spans="1:2">
       <c r="A138" s="2">
-        <v>46141.41666666666</v>
+        <v>46143.41666666666</v>
       </c>
       <c r="B138">
-        <v>577</v>
+        <v>431</v>
       </c>
     </row>
     <row r="139" spans="1:2">
       <c r="A139" s="2">
-        <v>46141.42708333334</v>
+        <v>46143.42708333334</v>
       </c>
       <c r="B139">
-        <v>508</v>
+        <v>428</v>
       </c>
     </row>
     <row r="140" spans="1:2">
       <c r="A140" s="2">
-        <v>46141.4375</v>
+        <v>46143.4375</v>
       </c>
       <c r="B140">
-        <v>444</v>
+        <v>560</v>
       </c>
     </row>
     <row r="141" spans="1:2">
       <c r="A141" s="2">
-        <v>46141.44791666666</v>
+        <v>46143.44791666666</v>
       </c>
       <c r="B141">
-        <v>0</v>
+        <v>579</v>
       </c>
     </row>
     <row r="142" spans="1:2">
       <c r="A142" s="2">
-        <v>46141.45833333334</v>
+        <v>46143.45833333334</v>
       </c>
       <c r="B142">
-        <v>460</v>
+        <v>594</v>
       </c>
     </row>
     <row r="143" spans="1:2">
       <c r="A143" s="2">
-        <v>46141.46875</v>
+        <v>46143.46875</v>
       </c>
       <c r="B143">
-        <v>462</v>
+        <v>602</v>
       </c>
     </row>
     <row r="144" spans="1:2">
       <c r="A144" s="2">
-        <v>46141.47916666666</v>
+        <v>46143.47916666666</v>
       </c>
       <c r="B144">
-        <v>459</v>
+        <v>611</v>
       </c>
     </row>
     <row r="145" spans="1:2">
       <c r="A145" s="2">
-        <v>46141.48958333334</v>
+        <v>46143.48958333334</v>
       </c>
       <c r="B145">
-        <v>458</v>
+        <v>617</v>
       </c>
     </row>
     <row r="146" spans="1:2">
       <c r="A146" s="2">
-        <v>46141.5</v>
+        <v>46143.5</v>
       </c>
       <c r="B146">
-        <v>456</v>
+        <v>594</v>
       </c>
     </row>
     <row r="147" spans="1:2">
       <c r="A147" s="2">
-        <v>46141.51041666666</v>
+        <v>46143.51041666666</v>
       </c>
       <c r="B147">
-        <v>449</v>
+        <v>0</v>
       </c>
     </row>
     <row r="148" spans="1:2">
       <c r="A148" s="2">
-        <v>46141.52083333334</v>
+        <v>46143.52083333334</v>
       </c>
       <c r="B148">
-        <v>418</v>
+        <v>591</v>
       </c>
     </row>
     <row r="149" spans="1:2">
       <c r="A149" s="2">
-        <v>46141.53125</v>
+        <v>46143.53125</v>
       </c>
       <c r="B149">
-        <v>417</v>
+        <v>0</v>
       </c>
     </row>
     <row r="150" spans="1:2">
       <c r="A150" s="2">
-        <v>46141.54166666666</v>
+        <v>46143.54166666666</v>
       </c>
       <c r="B150">
-        <v>413</v>
+        <v>584</v>
       </c>
     </row>
     <row r="151" spans="1:2">
       <c r="A151" s="2">
-        <v>46141.55208333334</v>
+        <v>46143.55208333334</v>
       </c>
       <c r="B151">
-        <v>412</v>
+        <v>594</v>
       </c>
     </row>
     <row r="152" spans="1:2">
       <c r="A152" s="2">
-        <v>46141.5625</v>
+        <v>46143.5625</v>
       </c>
       <c r="B152">
-        <v>411</v>
+        <v>566</v>
       </c>
     </row>
     <row r="153" spans="1:2">
       <c r="A153" s="2">
-        <v>46141.57291666666</v>
+        <v>46143.57291666666</v>
       </c>
       <c r="B153">
-        <v>414</v>
+        <v>564</v>
       </c>
     </row>
     <row r="154" spans="1:2">
       <c r="A154" s="2">
-        <v>46141.58333333334</v>
+        <v>46143.58333333334</v>
       </c>
       <c r="B154">
-        <v>427</v>
+        <v>573</v>
       </c>
     </row>
     <row r="155" spans="1:2">
       <c r="A155" s="2">
-        <v>46141.59375</v>
+        <v>46143.59375</v>
       </c>
       <c r="B155">
-        <v>426</v>
+        <v>589</v>
       </c>
     </row>
     <row r="156" spans="1:2">
       <c r="A156" s="2">
-        <v>46141.60416666666</v>
+        <v>46143.60416666666</v>
       </c>
       <c r="B156">
-        <v>485</v>
+        <v>581</v>
       </c>
     </row>
     <row r="157" spans="1:2">
       <c r="A157" s="2">
-        <v>46141.61458333334</v>
+        <v>46143.61458333334</v>
       </c>
       <c r="B157">
-        <v>484</v>
+        <v>519</v>
       </c>
     </row>
     <row r="158" spans="1:2">
       <c r="A158" s="2">
-        <v>46141.625</v>
+        <v>46143.625</v>
       </c>
       <c r="B158">
-        <v>559</v>
+        <v>512</v>
       </c>
     </row>
     <row r="159" spans="1:2">
       <c r="A159" s="2">
-        <v>46141.63541666666</v>
+        <v>46143.63541666666</v>
       </c>
       <c r="B159">
-        <v>564</v>
+        <v>530</v>
       </c>
     </row>
     <row r="160" spans="1:2">
       <c r="A160" s="2">
-        <v>46141.64583333334</v>
+        <v>46143.64583333334</v>
       </c>
       <c r="B160">
-        <v>554</v>
+        <v>546</v>
       </c>
     </row>
     <row r="161" spans="1:2">
       <c r="A161" s="2">
-        <v>46141.65625</v>
+        <v>46143.65625</v>
       </c>
       <c r="B161">
-        <v>589</v>
+        <v>555</v>
       </c>
     </row>
     <row r="162" spans="1:2">
       <c r="A162" s="2">
-        <v>46141.66666666666</v>
+        <v>46143.66666666666</v>
       </c>
       <c r="B162">
-        <v>929</v>
+        <v>664</v>
       </c>
     </row>
     <row r="163" spans="1:2">
       <c r="A163" s="2">
-        <v>46141.67708333334</v>
+        <v>46143.67708333334</v>
       </c>
       <c r="B163">
-        <v>919</v>
+        <v>662</v>
       </c>
     </row>
     <row r="164" spans="1:2">
       <c r="A164" s="2">
-        <v>46141.6875</v>
+        <v>46143.6875</v>
       </c>
       <c r="B164">
-        <v>923</v>
+        <v>661</v>
       </c>
     </row>
     <row r="165" spans="1:2">
       <c r="A165" s="2">
-        <v>46141.69791666666</v>
+        <v>46143.69791666666</v>
       </c>
       <c r="B165">
-        <v>924</v>
+        <v>736</v>
       </c>
     </row>
     <row r="166" spans="1:2">
       <c r="A166" s="2">
-        <v>46141.70833333334</v>
+        <v>46143.70833333334</v>
       </c>
       <c r="B166">
-        <v>1050</v>
+        <v>866</v>
       </c>
     </row>
     <row r="167" spans="1:2">
       <c r="A167" s="2">
-        <v>46141.71875</v>
+        <v>46143.71875</v>
       </c>
       <c r="B167">
-        <v>1068</v>
+        <v>858</v>
       </c>
     </row>
     <row r="168" spans="1:2">
       <c r="A168" s="2">
-        <v>46141.72916666666</v>
+        <v>46143.72916666666</v>
       </c>
       <c r="B168">
-        <v>1083</v>
+        <v>885</v>
       </c>
     </row>
     <row r="169" spans="1:2">
       <c r="A169" s="2">
-        <v>46141.73958333334</v>
+        <v>46143.73958333334</v>
       </c>
       <c r="B169">
-        <v>0</v>
+        <v>894</v>
       </c>
     </row>
     <row r="170" spans="1:2">
       <c r="A170" s="2">
-        <v>46141.75</v>
+        <v>46143.75</v>
       </c>
       <c r="B170">
-        <v>1145</v>
+        <v>1168</v>
       </c>
     </row>
     <row r="171" spans="1:2">
       <c r="A171" s="2">
-        <v>46141.76041666666</v>
+        <v>46143.76041666666</v>
       </c>
       <c r="B171">
-        <v>1152</v>
+        <v>1178</v>
       </c>
     </row>
     <row r="172" spans="1:2">
       <c r="A172" s="2">
-        <v>46141.77083333334</v>
+        <v>46143.77083333334</v>
       </c>
       <c r="B172">
-        <v>1141</v>
+        <v>1180</v>
       </c>
     </row>
     <row r="173" spans="1:2">
       <c r="A173" s="2">
-        <v>46141.78125</v>
+        <v>46143.78125</v>
       </c>
       <c r="B173">
-        <v>1147</v>
+        <v>1181</v>
       </c>
     </row>
     <row r="174" spans="1:2">
       <c r="A174" s="2">
-        <v>46141.79166666666</v>
+        <v>46143.79166666666</v>
       </c>
       <c r="B174">
-        <v>1140</v>
+        <v>1190</v>
       </c>
     </row>
     <row r="175" spans="1:2">
       <c r="A175" s="2">
-        <v>46141.80208333334</v>
+        <v>46143.80208333334</v>
       </c>
       <c r="B175">
-        <v>1179</v>
+        <v>1189</v>
       </c>
     </row>
     <row r="176" spans="1:2">
       <c r="A176" s="2">
-        <v>46141.8125</v>
+        <v>46143.8125</v>
       </c>
       <c r="B176">
-        <v>1196</v>
+        <v>1187</v>
       </c>
     </row>
     <row r="177" spans="1:2">
       <c r="A177" s="2">
-        <v>46141.82291666666</v>
+        <v>46143.82291666666</v>
       </c>
       <c r="B177">
-        <v>1197</v>
+        <v>1191</v>
       </c>
     </row>
     <row r="178" spans="1:2">
       <c r="A178" s="2">
-        <v>46141.83333333334</v>
+        <v>46143.83333333334</v>
       </c>
       <c r="B178">
-        <v>1150</v>
+        <v>1183</v>
       </c>
     </row>
     <row r="179" spans="1:2">
       <c r="A179" s="2">
-        <v>46141.84375</v>
+        <v>46143.84375</v>
       </c>
       <c r="B179">
-        <v>1140</v>
+        <v>1182</v>
       </c>
     </row>
     <row r="180" spans="1:2">
       <c r="A180" s="2">
-        <v>46141.85416666666</v>
+        <v>46143.85416666666</v>
       </c>
       <c r="B180">
-        <v>1141</v>
+        <v>1183</v>
       </c>
     </row>
     <row r="181" spans="1:2">
       <c r="A181" s="2">
-        <v>46141.86458333334</v>
+        <v>46143.86458333334</v>
       </c>
       <c r="B181">
-        <v>1142</v>
+        <v>0</v>
       </c>
     </row>
     <row r="182" spans="1:2">
       <c r="A182" s="2">
-        <v>46141.875</v>
+        <v>46143.875</v>
       </c>
       <c r="B182">
-        <v>1179</v>
+        <v>1186</v>
       </c>
     </row>
     <row r="183" spans="1:2">
       <c r="A183" s="2">
-        <v>46141.88541666666</v>
+        <v>46143.88541666666</v>
       </c>
       <c r="B183">
-        <v>1187</v>
+        <v>1188</v>
       </c>
     </row>
     <row r="184" spans="1:2">
       <c r="A184" s="2">
-        <v>46141.89583333334</v>
+        <v>46143.89583333334</v>
       </c>
       <c r="B184">
-        <v>1184</v>
+        <v>1201</v>
       </c>
     </row>
     <row r="185" spans="1:2">
       <c r="A185" s="2">
-        <v>46141.90625</v>
+        <v>46143.90625</v>
       </c>
       <c r="B185">
-        <v>1195</v>
+        <v>0</v>
       </c>
     </row>
     <row r="186" spans="1:2">
       <c r="A186" s="2">
-        <v>46141.91666666666</v>
+        <v>46143.91666666666</v>
       </c>
       <c r="B186">
-        <v>1315</v>
+        <v>1213</v>
       </c>
     </row>
     <row r="187" spans="1:2">
       <c r="A187" s="2">
-        <v>46141.92708333334</v>
+        <v>46143.92708333334</v>
       </c>
       <c r="B187">
-        <v>1294</v>
+        <v>1204</v>
       </c>
     </row>
     <row r="188" spans="1:2">
       <c r="A188" s="2">
-        <v>46141.9375</v>
+        <v>46143.9375</v>
       </c>
       <c r="B188">
-        <v>1283</v>
+        <v>0</v>
       </c>
     </row>
     <row r="189" spans="1:2">
       <c r="A189" s="2">
-        <v>46141.94791666666</v>
+        <v>46143.94791666666</v>
       </c>
       <c r="B189">
-        <v>1284</v>
+        <v>0</v>
       </c>
     </row>
     <row r="190" spans="1:2">
       <c r="A190" s="2">
-        <v>46141.95833333334</v>
+        <v>46143.95833333334</v>
       </c>
       <c r="B190">
-        <v>1013</v>
+        <v>1178</v>
       </c>
     </row>
     <row r="191" spans="1:2">
       <c r="A191" s="2">
-        <v>46141.96875</v>
+        <v>46143.96875</v>
       </c>
       <c r="B191">
-        <v>971</v>
+        <v>1173</v>
       </c>
     </row>
     <row r="192" spans="1:2">
       <c r="A192" s="2">
-        <v>46141.97916666666</v>
+        <v>46143.97916666666</v>
       </c>
       <c r="B192">
-        <v>973</v>
+        <v>1172</v>
       </c>
     </row>
     <row r="193" spans="1:2">
       <c r="A193" s="2">
-        <v>46141.98958333334</v>
+        <v>46143.98958333334</v>
       </c>
       <c r="B193">
-        <v>0</v>
+        <v>1169</v>
       </c>
     </row>
     <row r="194" spans="1:2">
       <c r="A194" s="2">
-        <v>46142</v>
+        <v>46144</v>
       </c>
       <c r="B194">
-        <v>1000</v>
+        <v>960</v>
       </c>
     </row>
     <row r="195" spans="1:2">
       <c r="A195" s="2">
-        <v>46142.01041666666</v>
+        <v>46144.01041666666</v>
       </c>
       <c r="B195">
-        <v>995</v>
+        <v>950</v>
       </c>
     </row>
     <row r="196" spans="1:2">
       <c r="A196" s="2">
-        <v>46142.02083333334</v>
+        <v>46144.02083333334</v>
       </c>
       <c r="B196">
         <v>0</v>
@@ -1954,31 +1954,31 @@
     </row>
     <row r="197" spans="1:2">
       <c r="A197" s="2">
-        <v>46142.03125</v>
+        <v>46144.03125</v>
       </c>
       <c r="B197">
-        <v>993</v>
+        <v>947</v>
       </c>
     </row>
     <row r="198" spans="1:2">
       <c r="A198" s="2">
-        <v>46142.04166666666</v>
+        <v>46144.04166666666</v>
       </c>
       <c r="B198">
-        <v>954</v>
+        <v>946</v>
       </c>
     </row>
     <row r="199" spans="1:2">
       <c r="A199" s="2">
-        <v>46142.05208333334</v>
+        <v>46144.05208333334</v>
       </c>
       <c r="B199">
-        <v>955</v>
+        <v>945</v>
       </c>
     </row>
     <row r="200" spans="1:2">
       <c r="A200" s="2">
-        <v>46142.0625</v>
+        <v>46144.0625</v>
       </c>
       <c r="B200">
         <v>0</v>
@@ -1986,87 +1986,87 @@
     </row>
     <row r="201" spans="1:2">
       <c r="A201" s="2">
-        <v>46142.07291666666</v>
+        <v>46144.07291666666</v>
       </c>
       <c r="B201">
-        <v>954</v>
+        <v>943</v>
       </c>
     </row>
     <row r="202" spans="1:2">
       <c r="A202" s="2">
-        <v>46142.08333333334</v>
+        <v>46144.08333333334</v>
       </c>
       <c r="B202">
-        <v>955</v>
+        <v>944</v>
       </c>
     </row>
     <row r="203" spans="1:2">
       <c r="A203" s="2">
-        <v>46142.09375</v>
+        <v>46144.09375</v>
       </c>
       <c r="B203">
-        <v>956</v>
+        <v>0</v>
       </c>
     </row>
     <row r="204" spans="1:2">
       <c r="A204" s="2">
-        <v>46142.10416666666</v>
+        <v>46144.10416666666</v>
       </c>
       <c r="B204">
-        <v>969</v>
+        <v>946</v>
       </c>
     </row>
     <row r="205" spans="1:2">
       <c r="A205" s="2">
-        <v>46142.11458333334</v>
+        <v>46144.11458333334</v>
       </c>
       <c r="B205">
-        <v>966</v>
+        <v>0</v>
       </c>
     </row>
     <row r="206" spans="1:2">
       <c r="A206" s="2">
-        <v>46142.125</v>
+        <v>46144.125</v>
       </c>
       <c r="B206">
-        <v>970</v>
+        <v>939</v>
       </c>
     </row>
     <row r="207" spans="1:2">
       <c r="A207" s="2">
-        <v>46142.13541666666</v>
+        <v>46144.13541666666</v>
       </c>
       <c r="B207">
-        <v>969</v>
+        <v>0</v>
       </c>
     </row>
     <row r="208" spans="1:2">
       <c r="A208" s="2">
-        <v>46142.14583333334</v>
+        <v>46144.14583333334</v>
       </c>
       <c r="B208">
-        <v>970</v>
+        <v>0</v>
       </c>
     </row>
     <row r="209" spans="1:2">
       <c r="A209" s="2">
-        <v>46142.15625</v>
+        <v>46144.15625</v>
       </c>
       <c r="B209">
-        <v>969</v>
+        <v>0</v>
       </c>
     </row>
     <row r="210" spans="1:2">
       <c r="A210" s="2">
-        <v>46142.16666666666</v>
+        <v>46144.16666666666</v>
       </c>
       <c r="B210">
-        <v>972</v>
+        <v>934</v>
       </c>
     </row>
     <row r="211" spans="1:2">
       <c r="A211" s="2">
-        <v>46142.17708333334</v>
+        <v>46144.17708333334</v>
       </c>
       <c r="B211">
         <v>0</v>
@@ -2074,255 +2074,255 @@
     </row>
     <row r="212" spans="1:2">
       <c r="A212" s="2">
-        <v>46142.1875</v>
+        <v>46144.1875</v>
       </c>
       <c r="B212">
-        <v>971</v>
+        <v>933</v>
       </c>
     </row>
     <row r="213" spans="1:2">
       <c r="A213" s="2">
-        <v>46142.19791666666</v>
+        <v>46144.19791666666</v>
       </c>
       <c r="B213">
-        <v>975</v>
+        <v>932</v>
       </c>
     </row>
     <row r="214" spans="1:2">
       <c r="A214" s="2">
-        <v>46142.20833333334</v>
+        <v>46144.20833333334</v>
       </c>
       <c r="B214">
-        <v>1057</v>
+        <v>962</v>
       </c>
     </row>
     <row r="215" spans="1:2">
       <c r="A215" s="2">
-        <v>46142.21875</v>
+        <v>46144.21875</v>
       </c>
       <c r="B215">
-        <v>1067</v>
+        <v>964</v>
       </c>
     </row>
     <row r="216" spans="1:2">
       <c r="A216" s="2">
-        <v>46142.22916666666</v>
+        <v>46144.22916666666</v>
       </c>
       <c r="B216">
-        <v>1064</v>
+        <v>965</v>
       </c>
     </row>
     <row r="217" spans="1:2">
       <c r="A217" s="2">
-        <v>46142.23958333334</v>
+        <v>46144.23958333334</v>
       </c>
       <c r="B217">
-        <v>1069</v>
+        <v>964</v>
       </c>
     </row>
     <row r="218" spans="1:2">
       <c r="A218" s="2">
-        <v>46142.25</v>
+        <v>46144.25</v>
       </c>
       <c r="B218">
-        <v>1132</v>
+        <v>845</v>
       </c>
     </row>
     <row r="219" spans="1:2">
       <c r="A219" s="2">
-        <v>46142.26041666666</v>
+        <v>46144.26041666666</v>
       </c>
       <c r="B219">
-        <v>1138</v>
+        <v>811</v>
       </c>
     </row>
     <row r="220" spans="1:2">
       <c r="A220" s="2">
-        <v>46142.27083333334</v>
+        <v>46144.27083333334</v>
       </c>
       <c r="B220">
-        <v>1137</v>
+        <v>812</v>
       </c>
     </row>
     <row r="221" spans="1:2">
       <c r="A221" s="2">
-        <v>46142.28125</v>
+        <v>46144.28125</v>
       </c>
       <c r="B221">
-        <v>0</v>
+        <v>810</v>
       </c>
     </row>
     <row r="222" spans="1:2">
       <c r="A222" s="2">
-        <v>46142.29166666666</v>
+        <v>46144.29166666666</v>
       </c>
       <c r="B222">
-        <v>1138</v>
+        <v>822</v>
       </c>
     </row>
     <row r="223" spans="1:2">
       <c r="A223" s="2">
-        <v>46142.30208333334</v>
+        <v>46144.30208333334</v>
       </c>
       <c r="B223">
-        <v>1148</v>
+        <v>827</v>
       </c>
     </row>
     <row r="224" spans="1:2">
       <c r="A224" s="2">
-        <v>46142.3125</v>
+        <v>46144.3125</v>
       </c>
       <c r="B224">
-        <v>1152</v>
+        <v>917</v>
       </c>
     </row>
     <row r="225" spans="1:2">
       <c r="A225" s="2">
-        <v>46142.32291666666</v>
+        <v>46144.32291666666</v>
       </c>
       <c r="B225">
-        <v>0</v>
+        <v>920</v>
       </c>
     </row>
     <row r="226" spans="1:2">
       <c r="A226" s="2">
-        <v>46142.33333333334</v>
+        <v>46144.33333333334</v>
       </c>
       <c r="B226">
-        <v>936</v>
+        <v>702</v>
       </c>
     </row>
     <row r="227" spans="1:2">
       <c r="A227" s="2">
-        <v>46142.34375</v>
+        <v>46144.34375</v>
       </c>
       <c r="B227">
-        <v>916</v>
+        <v>688</v>
       </c>
     </row>
     <row r="228" spans="1:2">
       <c r="A228" s="2">
-        <v>46142.35416666666</v>
+        <v>46144.35416666666</v>
       </c>
       <c r="B228">
-        <v>955</v>
+        <v>690</v>
       </c>
     </row>
     <row r="229" spans="1:2">
       <c r="A229" s="2">
-        <v>46142.36458333334</v>
+        <v>46144.36458333334</v>
       </c>
       <c r="B229">
-        <v>959</v>
+        <v>689</v>
       </c>
     </row>
     <row r="230" spans="1:2">
       <c r="A230" s="2">
-        <v>46142.375</v>
+        <v>46144.375</v>
       </c>
       <c r="B230">
-        <v>904</v>
+        <v>627</v>
       </c>
     </row>
     <row r="231" spans="1:2">
       <c r="A231" s="2">
-        <v>46142.38541666666</v>
+        <v>46144.38541666666</v>
       </c>
       <c r="B231">
-        <v>899</v>
+        <v>597</v>
       </c>
     </row>
     <row r="232" spans="1:2">
       <c r="A232" s="2">
-        <v>46142.39583333334</v>
+        <v>46144.39583333334</v>
       </c>
       <c r="B232">
-        <v>0</v>
+        <v>600</v>
       </c>
     </row>
     <row r="233" spans="1:2">
       <c r="A233" s="2">
-        <v>46142.40625</v>
+        <v>46144.40625</v>
       </c>
       <c r="B233">
-        <v>898</v>
+        <v>599</v>
       </c>
     </row>
     <row r="234" spans="1:2">
       <c r="A234" s="2">
-        <v>46142.41666666666</v>
+        <v>46144.41666666666</v>
       </c>
       <c r="B234">
-        <v>658</v>
+        <v>584</v>
       </c>
     </row>
     <row r="235" spans="1:2">
       <c r="A235" s="2">
-        <v>46142.42708333334</v>
+        <v>46144.42708333334</v>
       </c>
       <c r="B235">
-        <v>643</v>
+        <v>579</v>
       </c>
     </row>
     <row r="236" spans="1:2">
       <c r="A236" s="2">
-        <v>46142.4375</v>
+        <v>46144.4375</v>
       </c>
       <c r="B236">
-        <v>650</v>
+        <v>0</v>
       </c>
     </row>
     <row r="237" spans="1:2">
       <c r="A237" s="2">
-        <v>46142.44791666666</v>
+        <v>46144.44791666666</v>
       </c>
       <c r="B237">
-        <v>595</v>
+        <v>578</v>
       </c>
     </row>
     <row r="238" spans="1:2">
       <c r="A238" s="2">
-        <v>46142.45833333334</v>
+        <v>46144.45833333334</v>
       </c>
       <c r="B238">
-        <v>563</v>
+        <v>599</v>
       </c>
     </row>
     <row r="239" spans="1:2">
       <c r="A239" s="2">
-        <v>46142.46875</v>
+        <v>46144.46875</v>
       </c>
       <c r="B239">
-        <v>0</v>
+        <v>600</v>
       </c>
     </row>
     <row r="240" spans="1:2">
       <c r="A240" s="2">
-        <v>46142.47916666666</v>
+        <v>46144.47916666666</v>
       </c>
       <c r="B240">
-        <v>0</v>
+        <v>601</v>
       </c>
     </row>
     <row r="241" spans="1:2">
       <c r="A241" s="2">
-        <v>46142.48958333334</v>
+        <v>46144.48958333334</v>
       </c>
       <c r="B241">
-        <v>0</v>
+        <v>600</v>
       </c>
     </row>
     <row r="242" spans="1:2">
       <c r="A242" s="2">
-        <v>46142.5</v>
+        <v>46144.5</v>
       </c>
       <c r="B242">
-        <v>0</v>
+        <v>599</v>
       </c>
     </row>
     <row r="243" spans="1:2">
       <c r="A243" s="2">
-        <v>46142.51041666666</v>
+        <v>46144.51041666666</v>
       </c>
       <c r="B243">
         <v>0</v>
@@ -2330,63 +2330,63 @@
     </row>
     <row r="244" spans="1:2">
       <c r="A244" s="2">
-        <v>46142.52083333334</v>
+        <v>46144.52083333334</v>
       </c>
       <c r="B244">
-        <v>0</v>
+        <v>600</v>
       </c>
     </row>
     <row r="245" spans="1:2">
       <c r="A245" s="2">
-        <v>46142.53125</v>
+        <v>46144.53125</v>
       </c>
       <c r="B245">
-        <v>0</v>
+        <v>599</v>
       </c>
     </row>
     <row r="246" spans="1:2">
       <c r="A246" s="2">
-        <v>46142.54166666666</v>
+        <v>46144.54166666666</v>
       </c>
       <c r="B246">
-        <v>0</v>
+        <v>590</v>
       </c>
     </row>
     <row r="247" spans="1:2">
       <c r="A247" s="2">
-        <v>46142.55208333334</v>
+        <v>46144.55208333334</v>
       </c>
       <c r="B247">
-        <v>0</v>
+        <v>575</v>
       </c>
     </row>
     <row r="248" spans="1:2">
       <c r="A248" s="2">
-        <v>46142.5625</v>
+        <v>46144.5625</v>
       </c>
       <c r="B248">
-        <v>0</v>
+        <v>553</v>
       </c>
     </row>
     <row r="249" spans="1:2">
       <c r="A249" s="2">
-        <v>46142.57291666666</v>
+        <v>46144.57291666666</v>
       </c>
       <c r="B249">
-        <v>0</v>
+        <v>583</v>
       </c>
     </row>
     <row r="250" spans="1:2">
       <c r="A250" s="2">
-        <v>46142.58333333334</v>
+        <v>46144.58333333334</v>
       </c>
       <c r="B250">
-        <v>0</v>
+        <v>590</v>
       </c>
     </row>
     <row r="251" spans="1:2">
       <c r="A251" s="2">
-        <v>46142.59375</v>
+        <v>46144.59375</v>
       </c>
       <c r="B251">
         <v>0</v>
@@ -2394,175 +2394,175 @@
     </row>
     <row r="252" spans="1:2">
       <c r="A252" s="2">
-        <v>46142.60416666666</v>
+        <v>46144.60416666666</v>
       </c>
       <c r="B252">
-        <v>0</v>
+        <v>591</v>
       </c>
     </row>
     <row r="253" spans="1:2">
       <c r="A253" s="2">
-        <v>46142.61458333334</v>
+        <v>46144.61458333334</v>
       </c>
       <c r="B253">
-        <v>0</v>
+        <v>597</v>
       </c>
     </row>
     <row r="254" spans="1:2">
       <c r="A254" s="2">
-        <v>46142.625</v>
+        <v>46144.625</v>
       </c>
       <c r="B254">
-        <v>0</v>
+        <v>718</v>
       </c>
     </row>
     <row r="255" spans="1:2">
       <c r="A255" s="2">
-        <v>46142.63541666666</v>
+        <v>46144.63541666666</v>
       </c>
       <c r="B255">
-        <v>0</v>
+        <v>683</v>
       </c>
     </row>
     <row r="256" spans="1:2">
       <c r="A256" s="2">
-        <v>46142.64583333334</v>
+        <v>46144.64583333334</v>
       </c>
       <c r="B256">
-        <v>0</v>
+        <v>654</v>
       </c>
     </row>
     <row r="257" spans="1:2">
       <c r="A257" s="2">
-        <v>46142.65625</v>
+        <v>46144.65625</v>
       </c>
       <c r="B257">
-        <v>0</v>
+        <v>655</v>
       </c>
     </row>
     <row r="258" spans="1:2">
       <c r="A258" s="2">
-        <v>46142.66666666666</v>
+        <v>46144.66666666666</v>
       </c>
       <c r="B258">
-        <v>0</v>
+        <v>669</v>
       </c>
     </row>
     <row r="259" spans="1:2">
       <c r="A259" s="2">
-        <v>46142.67708333334</v>
+        <v>46144.67708333334</v>
       </c>
       <c r="B259">
-        <v>0</v>
+        <v>709</v>
       </c>
     </row>
     <row r="260" spans="1:2">
       <c r="A260" s="2">
-        <v>46142.6875</v>
+        <v>46144.6875</v>
       </c>
       <c r="B260">
-        <v>0</v>
+        <v>718</v>
       </c>
     </row>
     <row r="261" spans="1:2">
       <c r="A261" s="2">
-        <v>46142.69791666666</v>
+        <v>46144.69791666666</v>
       </c>
       <c r="B261">
-        <v>0</v>
+        <v>727</v>
       </c>
     </row>
     <row r="262" spans="1:2">
       <c r="A262" s="2">
-        <v>46142.70833333334</v>
+        <v>46144.70833333334</v>
       </c>
       <c r="B262">
-        <v>0</v>
+        <v>769</v>
       </c>
     </row>
     <row r="263" spans="1:2">
       <c r="A263" s="2">
-        <v>46142.71875</v>
+        <v>46144.71875</v>
       </c>
       <c r="B263">
-        <v>0</v>
+        <v>783</v>
       </c>
     </row>
     <row r="264" spans="1:2">
       <c r="A264" s="2">
-        <v>46142.72916666666</v>
+        <v>46144.72916666666</v>
       </c>
       <c r="B264">
-        <v>0</v>
+        <v>795</v>
       </c>
     </row>
     <row r="265" spans="1:2">
       <c r="A265" s="2">
-        <v>46142.73958333334</v>
+        <v>46144.73958333334</v>
       </c>
       <c r="B265">
-        <v>0</v>
+        <v>800</v>
       </c>
     </row>
     <row r="266" spans="1:2">
       <c r="A266" s="2">
-        <v>46142.75</v>
+        <v>46144.75</v>
       </c>
       <c r="B266">
-        <v>0</v>
+        <v>1070</v>
       </c>
     </row>
     <row r="267" spans="1:2">
       <c r="A267" s="2">
-        <v>46142.76041666666</v>
+        <v>46144.76041666666</v>
       </c>
       <c r="B267">
-        <v>0</v>
+        <v>1128</v>
       </c>
     </row>
     <row r="268" spans="1:2">
       <c r="A268" s="2">
-        <v>46142.77083333334</v>
+        <v>46144.77083333334</v>
       </c>
       <c r="B268">
-        <v>0</v>
+        <v>1124</v>
       </c>
     </row>
     <row r="269" spans="1:2">
       <c r="A269" s="2">
-        <v>46142.78125</v>
+        <v>46144.78125</v>
       </c>
       <c r="B269">
-        <v>0</v>
+        <v>1123</v>
       </c>
     </row>
     <row r="270" spans="1:2">
       <c r="A270" s="2">
-        <v>46142.79166666666</v>
+        <v>46144.79166666666</v>
       </c>
       <c r="B270">
-        <v>0</v>
+        <v>1206</v>
       </c>
     </row>
     <row r="271" spans="1:2">
       <c r="A271" s="2">
-        <v>46142.80208333334</v>
+        <v>46144.80208333334</v>
       </c>
       <c r="B271">
-        <v>0</v>
+        <v>1208</v>
       </c>
     </row>
     <row r="272" spans="1:2">
       <c r="A272" s="2">
-        <v>46142.8125</v>
+        <v>46144.8125</v>
       </c>
       <c r="B272">
-        <v>0</v>
+        <v>1214</v>
       </c>
     </row>
     <row r="273" spans="1:2">
       <c r="A273" s="2">
-        <v>46142.82291666666</v>
+        <v>46144.82291666666</v>
       </c>
       <c r="B273">
         <v>0</v>
@@ -2570,23 +2570,23 @@
     </row>
     <row r="274" spans="1:2">
       <c r="A274" s="2">
-        <v>46142.83333333334</v>
+        <v>46144.83333333334</v>
       </c>
       <c r="B274">
-        <v>0</v>
+        <v>1185</v>
       </c>
     </row>
     <row r="275" spans="1:2">
       <c r="A275" s="2">
-        <v>46142.84375</v>
+        <v>46144.84375</v>
       </c>
       <c r="B275">
-        <v>0</v>
+        <v>1188</v>
       </c>
     </row>
     <row r="276" spans="1:2">
       <c r="A276" s="2">
-        <v>46142.85416666666</v>
+        <v>46144.85416666666</v>
       </c>
       <c r="B276">
         <v>0</v>
@@ -2594,7 +2594,7 @@
     </row>
     <row r="277" spans="1:2">
       <c r="A277" s="2">
-        <v>46142.86458333334</v>
+        <v>46144.86458333334</v>
       </c>
       <c r="B277">
         <v>0</v>
@@ -2602,47 +2602,47 @@
     </row>
     <row r="278" spans="1:2">
       <c r="A278" s="2">
-        <v>46142.875</v>
+        <v>46144.875</v>
       </c>
       <c r="B278">
-        <v>0</v>
+        <v>1187</v>
       </c>
     </row>
     <row r="279" spans="1:2">
       <c r="A279" s="2">
-        <v>46142.88541666666</v>
+        <v>46144.88541666666</v>
       </c>
       <c r="B279">
-        <v>0</v>
+        <v>1183</v>
       </c>
     </row>
     <row r="280" spans="1:2">
       <c r="A280" s="2">
-        <v>46142.89583333334</v>
+        <v>46144.89583333334</v>
       </c>
       <c r="B280">
-        <v>0</v>
+        <v>1161</v>
       </c>
     </row>
     <row r="281" spans="1:2">
       <c r="A281" s="2">
-        <v>46142.90625</v>
+        <v>46144.90625</v>
       </c>
       <c r="B281">
-        <v>0</v>
+        <v>1165</v>
       </c>
     </row>
     <row r="282" spans="1:2">
       <c r="A282" s="2">
-        <v>46142.91666666666</v>
+        <v>46144.91666666666</v>
       </c>
       <c r="B282">
-        <v>0</v>
+        <v>1180</v>
       </c>
     </row>
     <row r="283" spans="1:2">
       <c r="A283" s="2">
-        <v>46142.92708333334</v>
+        <v>46144.92708333334</v>
       </c>
       <c r="B283">
         <v>0</v>
@@ -2650,49 +2650,1585 @@
     </row>
     <row r="284" spans="1:2">
       <c r="A284" s="2">
-        <v>46142.9375</v>
+        <v>46144.9375</v>
       </c>
       <c r="B284">
-        <v>0</v>
+        <v>1190</v>
       </c>
     </row>
     <row r="285" spans="1:2">
       <c r="A285" s="2">
-        <v>46142.94791666666</v>
+        <v>46144.94791666666</v>
       </c>
       <c r="B285">
-        <v>0</v>
+        <v>1192</v>
       </c>
     </row>
     <row r="286" spans="1:2">
       <c r="A286" s="2">
-        <v>46142.95833333334</v>
+        <v>46144.95833333334</v>
       </c>
       <c r="B286">
-        <v>0</v>
+        <v>976</v>
       </c>
     </row>
     <row r="287" spans="1:2">
       <c r="A287" s="2">
-        <v>46142.96875</v>
+        <v>46144.96875</v>
       </c>
       <c r="B287">
-        <v>0</v>
+        <v>944</v>
       </c>
     </row>
     <row r="288" spans="1:2">
       <c r="A288" s="2">
-        <v>46142.97916666666</v>
+        <v>46144.97916666666</v>
       </c>
       <c r="B288">
-        <v>0</v>
+        <v>945</v>
       </c>
     </row>
     <row r="289" spans="1:2">
       <c r="A289" s="2">
-        <v>46142.98958333334</v>
+        <v>46144.98958333334</v>
       </c>
       <c r="B289">
+        <v>940</v>
+      </c>
+    </row>
+    <row r="290" spans="1:2">
+      <c r="A290" s="2">
+        <v>46145</v>
+      </c>
+      <c r="B290">
+        <v>883</v>
+      </c>
+    </row>
+    <row r="291" spans="1:2">
+      <c r="A291" s="2">
+        <v>46145.01041666666</v>
+      </c>
+      <c r="B291">
+        <v>880</v>
+      </c>
+    </row>
+    <row r="292" spans="1:2">
+      <c r="A292" s="2">
+        <v>46145.02083333334</v>
+      </c>
+      <c r="B292">
+        <v>879</v>
+      </c>
+    </row>
+    <row r="293" spans="1:2">
+      <c r="A293" s="2">
+        <v>46145.03125</v>
+      </c>
+      <c r="B293">
+        <v>878</v>
+      </c>
+    </row>
+    <row r="294" spans="1:2">
+      <c r="A294" s="2">
+        <v>46145.04166666666</v>
+      </c>
+      <c r="B294">
+        <v>877</v>
+      </c>
+    </row>
+    <row r="295" spans="1:2">
+      <c r="A295" s="2">
+        <v>46145.05208333334</v>
+      </c>
+      <c r="B295">
+        <v>873</v>
+      </c>
+    </row>
+    <row r="296" spans="1:2">
+      <c r="A296" s="2">
+        <v>46145.0625</v>
+      </c>
+      <c r="B296">
+        <v>874</v>
+      </c>
+    </row>
+    <row r="297" spans="1:2">
+      <c r="A297" s="2">
+        <v>46145.07291666666</v>
+      </c>
+      <c r="B297">
+        <v>873</v>
+      </c>
+    </row>
+    <row r="298" spans="1:2">
+      <c r="A298" s="2">
+        <v>46145.08333333334</v>
+      </c>
+      <c r="B298">
+        <v>863</v>
+      </c>
+    </row>
+    <row r="299" spans="1:2">
+      <c r="A299" s="2">
+        <v>46145.09375</v>
+      </c>
+      <c r="B299">
+        <v>859</v>
+      </c>
+    </row>
+    <row r="300" spans="1:2">
+      <c r="A300" s="2">
+        <v>46145.10416666666</v>
+      </c>
+      <c r="B300">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="301" spans="1:2">
+      <c r="A301" s="2">
+        <v>46145.11458333334</v>
+      </c>
+      <c r="B301">
+        <v>858</v>
+      </c>
+    </row>
+    <row r="302" spans="1:2">
+      <c r="A302" s="2">
+        <v>46145.125</v>
+      </c>
+      <c r="B302">
+        <v>848</v>
+      </c>
+    </row>
+    <row r="303" spans="1:2">
+      <c r="A303" s="2">
+        <v>46145.13541666666</v>
+      </c>
+      <c r="B303">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="304" spans="1:2">
+      <c r="A304" s="2">
+        <v>46145.14583333334</v>
+      </c>
+      <c r="B304">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="305" spans="1:2">
+      <c r="A305" s="2">
+        <v>46145.15625</v>
+      </c>
+      <c r="B305">
+        <v>849</v>
+      </c>
+    </row>
+    <row r="306" spans="1:2">
+      <c r="A306" s="2">
+        <v>46145.16666666666</v>
+      </c>
+      <c r="B306">
+        <v>878</v>
+      </c>
+    </row>
+    <row r="307" spans="1:2">
+      <c r="A307" s="2">
+        <v>46145.17708333334</v>
+      </c>
+      <c r="B307">
+        <v>887</v>
+      </c>
+    </row>
+    <row r="308" spans="1:2">
+      <c r="A308" s="2">
+        <v>46145.1875</v>
+      </c>
+      <c r="B308">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="309" spans="1:2">
+      <c r="A309" s="2">
+        <v>46145.19791666666</v>
+      </c>
+      <c r="B309">
+        <v>891</v>
+      </c>
+    </row>
+    <row r="310" spans="1:2">
+      <c r="A310" s="2">
+        <v>46145.20833333334</v>
+      </c>
+      <c r="B310">
+        <v>812</v>
+      </c>
+    </row>
+    <row r="311" spans="1:2">
+      <c r="A311" s="2">
+        <v>46145.21875</v>
+      </c>
+      <c r="B311">
+        <v>803</v>
+      </c>
+    </row>
+    <row r="312" spans="1:2">
+      <c r="A312" s="2">
+        <v>46145.22916666666</v>
+      </c>
+      <c r="B312">
+        <v>804</v>
+      </c>
+    </row>
+    <row r="313" spans="1:2">
+      <c r="A313" s="2">
+        <v>46145.23958333334</v>
+      </c>
+      <c r="B313">
+        <v>801</v>
+      </c>
+    </row>
+    <row r="314" spans="1:2">
+      <c r="A314" s="2">
+        <v>46145.25</v>
+      </c>
+      <c r="B314">
+        <v>815</v>
+      </c>
+    </row>
+    <row r="315" spans="1:2">
+      <c r="A315" s="2">
+        <v>46145.26041666666</v>
+      </c>
+      <c r="B315">
+        <v>816</v>
+      </c>
+    </row>
+    <row r="316" spans="1:2">
+      <c r="A316" s="2">
+        <v>46145.27083333334</v>
+      </c>
+      <c r="B316">
+        <v>815</v>
+      </c>
+    </row>
+    <row r="317" spans="1:2">
+      <c r="A317" s="2">
+        <v>46145.28125</v>
+      </c>
+      <c r="B317">
+        <v>814</v>
+      </c>
+    </row>
+    <row r="318" spans="1:2">
+      <c r="A318" s="2">
+        <v>46145.29166666666</v>
+      </c>
+      <c r="B318">
+        <v>810</v>
+      </c>
+    </row>
+    <row r="319" spans="1:2">
+      <c r="A319" s="2">
+        <v>46145.30208333334</v>
+      </c>
+      <c r="B319">
+        <v>806</v>
+      </c>
+    </row>
+    <row r="320" spans="1:2">
+      <c r="A320" s="2">
+        <v>46145.3125</v>
+      </c>
+      <c r="B320">
+        <v>807</v>
+      </c>
+    </row>
+    <row r="321" spans="1:2">
+      <c r="A321" s="2">
+        <v>46145.32291666666</v>
+      </c>
+      <c r="B321">
+        <v>841</v>
+      </c>
+    </row>
+    <row r="322" spans="1:2">
+      <c r="A322" s="2">
+        <v>46145.33333333334</v>
+      </c>
+      <c r="B322">
+        <v>621</v>
+      </c>
+    </row>
+    <row r="323" spans="1:2">
+      <c r="A323" s="2">
+        <v>46145.34375</v>
+      </c>
+      <c r="B323">
+        <v>586</v>
+      </c>
+    </row>
+    <row r="324" spans="1:2">
+      <c r="A324" s="2">
+        <v>46145.35416666666</v>
+      </c>
+      <c r="B324">
+        <v>566</v>
+      </c>
+    </row>
+    <row r="325" spans="1:2">
+      <c r="A325" s="2">
+        <v>46145.36458333334</v>
+      </c>
+      <c r="B325">
+        <v>543</v>
+      </c>
+    </row>
+    <row r="326" spans="1:2">
+      <c r="A326" s="2">
+        <v>46145.375</v>
+      </c>
+      <c r="B326">
+        <v>535</v>
+      </c>
+    </row>
+    <row r="327" spans="1:2">
+      <c r="A327" s="2">
+        <v>46145.38541666666</v>
+      </c>
+      <c r="B327">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="328" spans="1:2">
+      <c r="A328" s="2">
+        <v>46145.39583333334</v>
+      </c>
+      <c r="B328">
+        <v>540</v>
+      </c>
+    </row>
+    <row r="329" spans="1:2">
+      <c r="A329" s="2">
+        <v>46145.40625</v>
+      </c>
+      <c r="B329">
+        <v>541</v>
+      </c>
+    </row>
+    <row r="330" spans="1:2">
+      <c r="A330" s="2">
+        <v>46145.41666666666</v>
+      </c>
+      <c r="B330">
+        <v>560</v>
+      </c>
+    </row>
+    <row r="331" spans="1:2">
+      <c r="A331" s="2">
+        <v>46145.42708333334</v>
+      </c>
+      <c r="B331">
+        <v>562</v>
+      </c>
+    </row>
+    <row r="332" spans="1:2">
+      <c r="A332" s="2">
+        <v>46145.4375</v>
+      </c>
+      <c r="B332">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="333" spans="1:2">
+      <c r="A333" s="2">
+        <v>46145.44791666666</v>
+      </c>
+      <c r="B333">
+        <v>563</v>
+      </c>
+    </row>
+    <row r="334" spans="1:2">
+      <c r="A334" s="2">
+        <v>46145.45833333334</v>
+      </c>
+      <c r="B334">
+        <v>567</v>
+      </c>
+    </row>
+    <row r="335" spans="1:2">
+      <c r="A335" s="2">
+        <v>46145.46875</v>
+      </c>
+      <c r="B335">
+        <v>566</v>
+      </c>
+    </row>
+    <row r="336" spans="1:2">
+      <c r="A336" s="2">
+        <v>46145.47916666666</v>
+      </c>
+      <c r="B336">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="337" spans="1:2">
+      <c r="A337" s="2">
+        <v>46145.48958333334</v>
+      </c>
+      <c r="B337">
+        <v>567</v>
+      </c>
+    </row>
+    <row r="338" spans="1:2">
+      <c r="A338" s="2">
+        <v>46145.5</v>
+      </c>
+      <c r="B338">
+        <v>592</v>
+      </c>
+    </row>
+    <row r="339" spans="1:2">
+      <c r="A339" s="2">
+        <v>46145.51041666666</v>
+      </c>
+      <c r="B339">
+        <v>593</v>
+      </c>
+    </row>
+    <row r="340" spans="1:2">
+      <c r="A340" s="2">
+        <v>46145.52083333334</v>
+      </c>
+      <c r="B340">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="341" spans="1:2">
+      <c r="A341" s="2">
+        <v>46145.53125</v>
+      </c>
+      <c r="B341">
+        <v>594</v>
+      </c>
+    </row>
+    <row r="342" spans="1:2">
+      <c r="A342" s="2">
+        <v>46145.54166666666</v>
+      </c>
+      <c r="B342">
+        <v>575</v>
+      </c>
+    </row>
+    <row r="343" spans="1:2">
+      <c r="A343" s="2">
+        <v>46145.55208333334</v>
+      </c>
+      <c r="B343">
+        <v>573</v>
+      </c>
+    </row>
+    <row r="344" spans="1:2">
+      <c r="A344" s="2">
+        <v>46145.5625</v>
+      </c>
+      <c r="B344">
+        <v>585</v>
+      </c>
+    </row>
+    <row r="345" spans="1:2">
+      <c r="A345" s="2">
+        <v>46145.57291666666</v>
+      </c>
+      <c r="B345">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="346" spans="1:2">
+      <c r="A346" s="2">
+        <v>46145.58333333334</v>
+      </c>
+      <c r="B346">
+        <v>574</v>
+      </c>
+    </row>
+    <row r="347" spans="1:2">
+      <c r="A347" s="2">
+        <v>46145.59375</v>
+      </c>
+      <c r="B347">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="348" spans="1:2">
+      <c r="A348" s="2">
+        <v>46145.60416666666</v>
+      </c>
+      <c r="B348">
+        <v>575</v>
+      </c>
+    </row>
+    <row r="349" spans="1:2">
+      <c r="A349" s="2">
+        <v>46145.61458333334</v>
+      </c>
+      <c r="B349">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="350" spans="1:2">
+      <c r="A350" s="2">
+        <v>46145.625</v>
+      </c>
+      <c r="B350">
+        <v>572</v>
+      </c>
+    </row>
+    <row r="351" spans="1:2">
+      <c r="A351" s="2">
+        <v>46145.63541666666</v>
+      </c>
+      <c r="B351">
+        <v>582</v>
+      </c>
+    </row>
+    <row r="352" spans="1:2">
+      <c r="A352" s="2">
+        <v>46145.64583333334</v>
+      </c>
+      <c r="B352">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="353" spans="1:2">
+      <c r="A353" s="2">
+        <v>46145.65625</v>
+      </c>
+      <c r="B353">
+        <v>584</v>
+      </c>
+    </row>
+    <row r="354" spans="1:2">
+      <c r="A354" s="2">
+        <v>46145.66666666666</v>
+      </c>
+      <c r="B354">
+        <v>569</v>
+      </c>
+    </row>
+    <row r="355" spans="1:2">
+      <c r="A355" s="2">
+        <v>46145.67708333334</v>
+      </c>
+      <c r="B355">
+        <v>568</v>
+      </c>
+    </row>
+    <row r="356" spans="1:2">
+      <c r="A356" s="2">
+        <v>46145.6875</v>
+      </c>
+      <c r="B356">
+        <v>496</v>
+      </c>
+    </row>
+    <row r="357" spans="1:2">
+      <c r="A357" s="2">
+        <v>46145.69791666666</v>
+      </c>
+      <c r="B357">
+        <v>503</v>
+      </c>
+    </row>
+    <row r="358" spans="1:2">
+      <c r="A358" s="2">
+        <v>46145.70833333334</v>
+      </c>
+      <c r="B358">
+        <v>832</v>
+      </c>
+    </row>
+    <row r="359" spans="1:2">
+      <c r="A359" s="2">
+        <v>46145.71875</v>
+      </c>
+      <c r="B359">
+        <v>857</v>
+      </c>
+    </row>
+    <row r="360" spans="1:2">
+      <c r="A360" s="2">
+        <v>46145.72916666666</v>
+      </c>
+      <c r="B360">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="361" spans="1:2">
+      <c r="A361" s="2">
+        <v>46145.73958333334</v>
+      </c>
+      <c r="B361">
+        <v>884</v>
+      </c>
+    </row>
+    <row r="362" spans="1:2">
+      <c r="A362" s="2">
+        <v>46145.75</v>
+      </c>
+      <c r="B362">
+        <v>1073</v>
+      </c>
+    </row>
+    <row r="363" spans="1:2">
+      <c r="A363" s="2">
+        <v>46145.76041666666</v>
+      </c>
+      <c r="B363">
+        <v>1083</v>
+      </c>
+    </row>
+    <row r="364" spans="1:2">
+      <c r="A364" s="2">
+        <v>46145.77083333334</v>
+      </c>
+      <c r="B364">
+        <v>1084</v>
+      </c>
+    </row>
+    <row r="365" spans="1:2">
+      <c r="A365" s="2">
+        <v>46145.78125</v>
+      </c>
+      <c r="B365">
+        <v>1079</v>
+      </c>
+    </row>
+    <row r="366" spans="1:2">
+      <c r="A366" s="2">
+        <v>46145.79166666666</v>
+      </c>
+      <c r="B366">
+        <v>1118</v>
+      </c>
+    </row>
+    <row r="367" spans="1:2">
+      <c r="A367" s="2">
+        <v>46145.80208333334</v>
+      </c>
+      <c r="B367">
+        <v>1119</v>
+      </c>
+    </row>
+    <row r="368" spans="1:2">
+      <c r="A368" s="2">
+        <v>46145.8125</v>
+      </c>
+      <c r="B368">
+        <v>1123</v>
+      </c>
+    </row>
+    <row r="369" spans="1:2">
+      <c r="A369" s="2">
+        <v>46145.82291666666</v>
+      </c>
+      <c r="B369">
+        <v>1125</v>
+      </c>
+    </row>
+    <row r="370" spans="1:2">
+      <c r="A370" s="2">
+        <v>46145.83333333334</v>
+      </c>
+      <c r="B370">
+        <v>1131</v>
+      </c>
+    </row>
+    <row r="371" spans="1:2">
+      <c r="A371" s="2">
+        <v>46145.84375</v>
+      </c>
+      <c r="B371">
+        <v>1221</v>
+      </c>
+    </row>
+    <row r="372" spans="1:2">
+      <c r="A372" s="2">
+        <v>46145.85416666666</v>
+      </c>
+      <c r="B372">
+        <v>1225</v>
+      </c>
+    </row>
+    <row r="373" spans="1:2">
+      <c r="A373" s="2">
+        <v>46145.86458333334</v>
+      </c>
+      <c r="B373">
+        <v>1224</v>
+      </c>
+    </row>
+    <row r="374" spans="1:2">
+      <c r="A374" s="2">
+        <v>46145.875</v>
+      </c>
+      <c r="B374">
+        <v>1119</v>
+      </c>
+    </row>
+    <row r="375" spans="1:2">
+      <c r="A375" s="2">
+        <v>46145.88541666666</v>
+      </c>
+      <c r="B375">
+        <v>1108</v>
+      </c>
+    </row>
+    <row r="376" spans="1:2">
+      <c r="A376" s="2">
+        <v>46145.89583333334</v>
+      </c>
+      <c r="B376">
+        <v>1107</v>
+      </c>
+    </row>
+    <row r="377" spans="1:2">
+      <c r="A377" s="2">
+        <v>46145.90625</v>
+      </c>
+      <c r="B377">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="378" spans="1:2">
+      <c r="A378" s="2">
+        <v>46145.91666666666</v>
+      </c>
+      <c r="B378">
+        <v>1091</v>
+      </c>
+    </row>
+    <row r="379" spans="1:2">
+      <c r="A379" s="2">
+        <v>46145.92708333334</v>
+      </c>
+      <c r="B379">
+        <v>1089</v>
+      </c>
+    </row>
+    <row r="380" spans="1:2">
+      <c r="A380" s="2">
+        <v>46145.9375</v>
+      </c>
+      <c r="B380">
+        <v>1095</v>
+      </c>
+    </row>
+    <row r="381" spans="1:2">
+      <c r="A381" s="2">
+        <v>46145.94791666666</v>
+      </c>
+      <c r="B381">
+        <v>1091</v>
+      </c>
+    </row>
+    <row r="382" spans="1:2">
+      <c r="A382" s="2">
+        <v>46145.95833333334</v>
+      </c>
+      <c r="B382">
+        <v>1129</v>
+      </c>
+    </row>
+    <row r="383" spans="1:2">
+      <c r="A383" s="2">
+        <v>46145.96875</v>
+      </c>
+      <c r="B383">
+        <v>1127</v>
+      </c>
+    </row>
+    <row r="384" spans="1:2">
+      <c r="A384" s="2">
+        <v>46145.97916666666</v>
+      </c>
+      <c r="B384">
+        <v>1124</v>
+      </c>
+    </row>
+    <row r="385" spans="1:2">
+      <c r="A385" s="2">
+        <v>46145.98958333334</v>
+      </c>
+      <c r="B385">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="386" spans="1:2">
+      <c r="A386" s="2">
+        <v>46146</v>
+      </c>
+      <c r="B386">
+        <v>907</v>
+      </c>
+    </row>
+    <row r="387" spans="1:2">
+      <c r="A387" s="2">
+        <v>46146.01041666666</v>
+      </c>
+      <c r="B387">
+        <v>874</v>
+      </c>
+    </row>
+    <row r="388" spans="1:2">
+      <c r="A388" s="2">
+        <v>46146.02083333334</v>
+      </c>
+      <c r="B388">
+        <v>871</v>
+      </c>
+    </row>
+    <row r="389" spans="1:2">
+      <c r="A389" s="2">
+        <v>46146.03125</v>
+      </c>
+      <c r="B389">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="390" spans="1:2">
+      <c r="A390" s="2">
+        <v>46146.04166666666</v>
+      </c>
+      <c r="B390">
+        <v>863</v>
+      </c>
+    </row>
+    <row r="391" spans="1:2">
+      <c r="A391" s="2">
+        <v>46146.05208333334</v>
+      </c>
+      <c r="B391">
+        <v>860</v>
+      </c>
+    </row>
+    <row r="392" spans="1:2">
+      <c r="A392" s="2">
+        <v>46146.0625</v>
+      </c>
+      <c r="B392">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="393" spans="1:2">
+      <c r="A393" s="2">
+        <v>46146.07291666666</v>
+      </c>
+      <c r="B393">
+        <v>862</v>
+      </c>
+    </row>
+    <row r="394" spans="1:2">
+      <c r="A394" s="2">
+        <v>46146.08333333334</v>
+      </c>
+      <c r="B394">
+        <v>794</v>
+      </c>
+    </row>
+    <row r="395" spans="1:2">
+      <c r="A395" s="2">
+        <v>46146.09375</v>
+      </c>
+      <c r="B395">
+        <v>787</v>
+      </c>
+    </row>
+    <row r="396" spans="1:2">
+      <c r="A396" s="2">
+        <v>46146.10416666666</v>
+      </c>
+      <c r="B396">
+        <v>802</v>
+      </c>
+    </row>
+    <row r="397" spans="1:2">
+      <c r="A397" s="2">
+        <v>46146.11458333334</v>
+      </c>
+      <c r="B397">
+        <v>805</v>
+      </c>
+    </row>
+    <row r="398" spans="1:2">
+      <c r="A398" s="2">
+        <v>46146.125</v>
+      </c>
+      <c r="B398">
+        <v>807</v>
+      </c>
+    </row>
+    <row r="399" spans="1:2">
+      <c r="A399" s="2">
+        <v>46146.13541666666</v>
+      </c>
+      <c r="B399">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="400" spans="1:2">
+      <c r="A400" s="2">
+        <v>46146.14583333334</v>
+      </c>
+      <c r="B400">
+        <v>806</v>
+      </c>
+    </row>
+    <row r="401" spans="1:2">
+      <c r="A401" s="2">
+        <v>46146.15625</v>
+      </c>
+      <c r="B401">
+        <v>804</v>
+      </c>
+    </row>
+    <row r="402" spans="1:2">
+      <c r="A402" s="2">
+        <v>46146.16666666666</v>
+      </c>
+      <c r="B402">
+        <v>821</v>
+      </c>
+    </row>
+    <row r="403" spans="1:2">
+      <c r="A403" s="2">
+        <v>46146.17708333334</v>
+      </c>
+      <c r="B403">
+        <v>822</v>
+      </c>
+    </row>
+    <row r="404" spans="1:2">
+      <c r="A404" s="2">
+        <v>46146.1875</v>
+      </c>
+      <c r="B404">
+        <v>823</v>
+      </c>
+    </row>
+    <row r="405" spans="1:2">
+      <c r="A405" s="2">
+        <v>46146.19791666666</v>
+      </c>
+      <c r="B405">
+        <v>825</v>
+      </c>
+    </row>
+    <row r="406" spans="1:2">
+      <c r="A406" s="2">
+        <v>46146.20833333334</v>
+      </c>
+      <c r="B406">
+        <v>828</v>
+      </c>
+    </row>
+    <row r="407" spans="1:2">
+      <c r="A407" s="2">
+        <v>46146.21875</v>
+      </c>
+      <c r="B407">
+        <v>830</v>
+      </c>
+    </row>
+    <row r="408" spans="1:2">
+      <c r="A408" s="2">
+        <v>46146.22916666666</v>
+      </c>
+      <c r="B408">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="409" spans="1:2">
+      <c r="A409" s="2">
+        <v>46146.23958333334</v>
+      </c>
+      <c r="B409">
+        <v>827</v>
+      </c>
+    </row>
+    <row r="410" spans="1:2">
+      <c r="A410" s="2">
+        <v>46146.25</v>
+      </c>
+      <c r="B410">
+        <v>860</v>
+      </c>
+    </row>
+    <row r="411" spans="1:2">
+      <c r="A411" s="2">
+        <v>46146.26041666666</v>
+      </c>
+      <c r="B411">
+        <v>858</v>
+      </c>
+    </row>
+    <row r="412" spans="1:2">
+      <c r="A412" s="2">
+        <v>46146.27083333334</v>
+      </c>
+      <c r="B412">
+        <v>860</v>
+      </c>
+    </row>
+    <row r="413" spans="1:2">
+      <c r="A413" s="2">
+        <v>46146.28125</v>
+      </c>
+      <c r="B413">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="414" spans="1:2">
+      <c r="A414" s="2">
+        <v>46146.29166666666</v>
+      </c>
+      <c r="B414">
+        <v>818</v>
+      </c>
+    </row>
+    <row r="415" spans="1:2">
+      <c r="A415" s="2">
+        <v>46146.30208333334</v>
+      </c>
+      <c r="B415">
+        <v>808</v>
+      </c>
+    </row>
+    <row r="416" spans="1:2">
+      <c r="A416" s="2">
+        <v>46146.3125</v>
+      </c>
+      <c r="B416">
+        <v>807</v>
+      </c>
+    </row>
+    <row r="417" spans="1:2">
+      <c r="A417" s="2">
+        <v>46146.32291666666</v>
+      </c>
+      <c r="B417">
+        <v>804</v>
+      </c>
+    </row>
+    <row r="418" spans="1:2">
+      <c r="A418" s="2">
+        <v>46146.33333333334</v>
+      </c>
+      <c r="B418">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="419" spans="1:2">
+      <c r="A419" s="2">
+        <v>46146.34375</v>
+      </c>
+      <c r="B419">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="420" spans="1:2">
+      <c r="A420" s="2">
+        <v>46146.35416666666</v>
+      </c>
+      <c r="B420">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="421" spans="1:2">
+      <c r="A421" s="2">
+        <v>46146.36458333334</v>
+      </c>
+      <c r="B421">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="422" spans="1:2">
+      <c r="A422" s="2">
+        <v>46146.375</v>
+      </c>
+      <c r="B422">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="423" spans="1:2">
+      <c r="A423" s="2">
+        <v>46146.38541666666</v>
+      </c>
+      <c r="B423">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="424" spans="1:2">
+      <c r="A424" s="2">
+        <v>46146.39583333334</v>
+      </c>
+      <c r="B424">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="425" spans="1:2">
+      <c r="A425" s="2">
+        <v>46146.40625</v>
+      </c>
+      <c r="B425">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="426" spans="1:2">
+      <c r="A426" s="2">
+        <v>46146.41666666666</v>
+      </c>
+      <c r="B426">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="427" spans="1:2">
+      <c r="A427" s="2">
+        <v>46146.42708333334</v>
+      </c>
+      <c r="B427">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="428" spans="1:2">
+      <c r="A428" s="2">
+        <v>46146.4375</v>
+      </c>
+      <c r="B428">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="429" spans="1:2">
+      <c r="A429" s="2">
+        <v>46146.44791666666</v>
+      </c>
+      <c r="B429">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="430" spans="1:2">
+      <c r="A430" s="2">
+        <v>46146.45833333334</v>
+      </c>
+      <c r="B430">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="431" spans="1:2">
+      <c r="A431" s="2">
+        <v>46146.46875</v>
+      </c>
+      <c r="B431">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="432" spans="1:2">
+      <c r="A432" s="2">
+        <v>46146.47916666666</v>
+      </c>
+      <c r="B432">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="433" spans="1:2">
+      <c r="A433" s="2">
+        <v>46146.48958333334</v>
+      </c>
+      <c r="B433">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="434" spans="1:2">
+      <c r="A434" s="2">
+        <v>46146.5</v>
+      </c>
+      <c r="B434">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="435" spans="1:2">
+      <c r="A435" s="2">
+        <v>46146.51041666666</v>
+      </c>
+      <c r="B435">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="436" spans="1:2">
+      <c r="A436" s="2">
+        <v>46146.52083333334</v>
+      </c>
+      <c r="B436">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="437" spans="1:2">
+      <c r="A437" s="2">
+        <v>46146.53125</v>
+      </c>
+      <c r="B437">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="438" spans="1:2">
+      <c r="A438" s="2">
+        <v>46146.54166666666</v>
+      </c>
+      <c r="B438">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="439" spans="1:2">
+      <c r="A439" s="2">
+        <v>46146.55208333334</v>
+      </c>
+      <c r="B439">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="440" spans="1:2">
+      <c r="A440" s="2">
+        <v>46146.5625</v>
+      </c>
+      <c r="B440">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="441" spans="1:2">
+      <c r="A441" s="2">
+        <v>46146.57291666666</v>
+      </c>
+      <c r="B441">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="442" spans="1:2">
+      <c r="A442" s="2">
+        <v>46146.58333333334</v>
+      </c>
+      <c r="B442">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="443" spans="1:2">
+      <c r="A443" s="2">
+        <v>46146.59375</v>
+      </c>
+      <c r="B443">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="444" spans="1:2">
+      <c r="A444" s="2">
+        <v>46146.60416666666</v>
+      </c>
+      <c r="B444">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="445" spans="1:2">
+      <c r="A445" s="2">
+        <v>46146.61458333334</v>
+      </c>
+      <c r="B445">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="446" spans="1:2">
+      <c r="A446" s="2">
+        <v>46146.625</v>
+      </c>
+      <c r="B446">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="447" spans="1:2">
+      <c r="A447" s="2">
+        <v>46146.63541666666</v>
+      </c>
+      <c r="B447">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="448" spans="1:2">
+      <c r="A448" s="2">
+        <v>46146.64583333334</v>
+      </c>
+      <c r="B448">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="449" spans="1:2">
+      <c r="A449" s="2">
+        <v>46146.65625</v>
+      </c>
+      <c r="B449">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="450" spans="1:2">
+      <c r="A450" s="2">
+        <v>46146.66666666666</v>
+      </c>
+      <c r="B450">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="451" spans="1:2">
+      <c r="A451" s="2">
+        <v>46146.67708333334</v>
+      </c>
+      <c r="B451">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="452" spans="1:2">
+      <c r="A452" s="2">
+        <v>46146.6875</v>
+      </c>
+      <c r="B452">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="453" spans="1:2">
+      <c r="A453" s="2">
+        <v>46146.69791666666</v>
+      </c>
+      <c r="B453">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="454" spans="1:2">
+      <c r="A454" s="2">
+        <v>46146.70833333334</v>
+      </c>
+      <c r="B454">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="455" spans="1:2">
+      <c r="A455" s="2">
+        <v>46146.71875</v>
+      </c>
+      <c r="B455">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="456" spans="1:2">
+      <c r="A456" s="2">
+        <v>46146.72916666666</v>
+      </c>
+      <c r="B456">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="457" spans="1:2">
+      <c r="A457" s="2">
+        <v>46146.73958333334</v>
+      </c>
+      <c r="B457">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="458" spans="1:2">
+      <c r="A458" s="2">
+        <v>46146.75</v>
+      </c>
+      <c r="B458">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="459" spans="1:2">
+      <c r="A459" s="2">
+        <v>46146.76041666666</v>
+      </c>
+      <c r="B459">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="460" spans="1:2">
+      <c r="A460" s="2">
+        <v>46146.77083333334</v>
+      </c>
+      <c r="B460">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="461" spans="1:2">
+      <c r="A461" s="2">
+        <v>46146.78125</v>
+      </c>
+      <c r="B461">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="462" spans="1:2">
+      <c r="A462" s="2">
+        <v>46146.79166666666</v>
+      </c>
+      <c r="B462">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="463" spans="1:2">
+      <c r="A463" s="2">
+        <v>46146.80208333334</v>
+      </c>
+      <c r="B463">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="464" spans="1:2">
+      <c r="A464" s="2">
+        <v>46146.8125</v>
+      </c>
+      <c r="B464">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="465" spans="1:2">
+      <c r="A465" s="2">
+        <v>46146.82291666666</v>
+      </c>
+      <c r="B465">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="466" spans="1:2">
+      <c r="A466" s="2">
+        <v>46146.83333333334</v>
+      </c>
+      <c r="B466">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="467" spans="1:2">
+      <c r="A467" s="2">
+        <v>46146.84375</v>
+      </c>
+      <c r="B467">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="468" spans="1:2">
+      <c r="A468" s="2">
+        <v>46146.85416666666</v>
+      </c>
+      <c r="B468">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="469" spans="1:2">
+      <c r="A469" s="2">
+        <v>46146.86458333334</v>
+      </c>
+      <c r="B469">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="470" spans="1:2">
+      <c r="A470" s="2">
+        <v>46146.875</v>
+      </c>
+      <c r="B470">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="471" spans="1:2">
+      <c r="A471" s="2">
+        <v>46146.88541666666</v>
+      </c>
+      <c r="B471">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="472" spans="1:2">
+      <c r="A472" s="2">
+        <v>46146.89583333334</v>
+      </c>
+      <c r="B472">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="473" spans="1:2">
+      <c r="A473" s="2">
+        <v>46146.90625</v>
+      </c>
+      <c r="B473">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="474" spans="1:2">
+      <c r="A474" s="2">
+        <v>46146.91666666666</v>
+      </c>
+      <c r="B474">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="475" spans="1:2">
+      <c r="A475" s="2">
+        <v>46146.92708333334</v>
+      </c>
+      <c r="B475">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="476" spans="1:2">
+      <c r="A476" s="2">
+        <v>46146.9375</v>
+      </c>
+      <c r="B476">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="477" spans="1:2">
+      <c r="A477" s="2">
+        <v>46146.94791666666</v>
+      </c>
+      <c r="B477">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="478" spans="1:2">
+      <c r="A478" s="2">
+        <v>46146.95833333334</v>
+      </c>
+      <c r="B478">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="479" spans="1:2">
+      <c r="A479" s="2">
+        <v>46146.96875</v>
+      </c>
+      <c r="B479">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="480" spans="1:2">
+      <c r="A480" s="2">
+        <v>46146.97916666666</v>
+      </c>
+      <c r="B480">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="481" spans="1:2">
+      <c r="A481" s="2">
+        <v>46146.98958333334</v>
+      </c>
+      <c r="B481">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Updating the model for SunGrowLucia with the April data
</commit_message>
<xml_diff>
--- a/data_fetching/Entsoe/Actual_Production_Hydro_River.xlsx
+++ b/data_fetching/Entsoe/Actual_Production_Hydro_River.xlsx
@@ -394,55 +394,55 @@
     </row>
     <row r="2" spans="1:2">
       <c r="A2" s="2">
-        <v>46147</v>
+        <v>46149</v>
       </c>
       <c r="B2">
-        <v>1017</v>
+        <v>830</v>
       </c>
     </row>
     <row r="3" spans="1:2">
       <c r="A3" s="2">
-        <v>46147.01041666666</v>
+        <v>46149.01041666666</v>
       </c>
       <c r="B3">
-        <v>846</v>
+        <v>826</v>
       </c>
     </row>
     <row r="4" spans="1:2">
       <c r="A4" s="2">
-        <v>46147.02083333334</v>
+        <v>46149.02083333334</v>
       </c>
       <c r="B4">
-        <v>827</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5" spans="1:2">
       <c r="A5" s="2">
-        <v>46147.03125</v>
+        <v>46149.03125</v>
       </c>
       <c r="B5">
-        <v>0</v>
+        <v>824</v>
       </c>
     </row>
     <row r="6" spans="1:2">
       <c r="A6" s="2">
-        <v>46147.04166666666</v>
+        <v>46149.04166666666</v>
       </c>
       <c r="B6">
-        <v>850</v>
+        <v>0</v>
       </c>
     </row>
     <row r="7" spans="1:2">
       <c r="A7" s="2">
-        <v>46147.05208333334</v>
+        <v>46149.05208333334</v>
       </c>
       <c r="B7">
-        <v>847</v>
+        <v>820</v>
       </c>
     </row>
     <row r="8" spans="1:2">
       <c r="A8" s="2">
-        <v>46147.0625</v>
+        <v>46149.0625</v>
       </c>
       <c r="B8">
         <v>0</v>
@@ -450,295 +450,295 @@
     </row>
     <row r="9" spans="1:2">
       <c r="A9" s="2">
-        <v>46147.07291666666</v>
+        <v>46149.07291666666</v>
       </c>
       <c r="B9">
-        <v>849</v>
+        <v>813</v>
       </c>
     </row>
     <row r="10" spans="1:2">
       <c r="A10" s="2">
-        <v>46147.08333333334</v>
+        <v>46149.08333333334</v>
       </c>
       <c r="B10">
-        <v>862</v>
+        <v>807</v>
       </c>
     </row>
     <row r="11" spans="1:2">
       <c r="A11" s="2">
-        <v>46147.09375</v>
+        <v>46149.09375</v>
       </c>
       <c r="B11">
-        <v>863</v>
+        <v>806</v>
       </c>
     </row>
     <row r="12" spans="1:2">
       <c r="A12" s="2">
-        <v>46147.10416666666</v>
+        <v>46149.10416666666</v>
       </c>
       <c r="B12">
-        <v>0</v>
+        <v>805</v>
       </c>
     </row>
     <row r="13" spans="1:2">
       <c r="A13" s="2">
-        <v>46147.11458333334</v>
+        <v>46149.11458333334</v>
       </c>
       <c r="B13">
-        <v>862</v>
+        <v>804</v>
       </c>
     </row>
     <row r="14" spans="1:2">
       <c r="A14" s="2">
-        <v>46147.125</v>
+        <v>46149.125</v>
       </c>
       <c r="B14">
-        <v>863</v>
+        <v>796</v>
       </c>
     </row>
     <row r="15" spans="1:2">
       <c r="A15" s="2">
-        <v>46147.13541666666</v>
+        <v>46149.13541666666</v>
       </c>
       <c r="B15">
-        <v>0</v>
+        <v>795</v>
       </c>
     </row>
     <row r="16" spans="1:2">
       <c r="A16" s="2">
-        <v>46147.14583333334</v>
+        <v>46149.14583333334</v>
       </c>
       <c r="B16">
-        <v>857</v>
+        <v>796</v>
       </c>
     </row>
     <row r="17" spans="1:2">
       <c r="A17" s="2">
-        <v>46147.15625</v>
+        <v>46149.15625</v>
       </c>
       <c r="B17">
-        <v>862</v>
+        <v>797</v>
       </c>
     </row>
     <row r="18" spans="1:2">
       <c r="A18" s="2">
-        <v>46147.16666666666</v>
+        <v>46149.16666666666</v>
       </c>
       <c r="B18">
-        <v>869</v>
+        <v>824</v>
       </c>
     </row>
     <row r="19" spans="1:2">
       <c r="A19" s="2">
-        <v>46147.17708333334</v>
+        <v>46149.17708333334</v>
       </c>
       <c r="B19">
-        <v>908</v>
+        <v>825</v>
       </c>
     </row>
     <row r="20" spans="1:2">
       <c r="A20" s="2">
-        <v>46147.1875</v>
+        <v>46149.1875</v>
       </c>
       <c r="B20">
-        <v>912</v>
+        <v>0</v>
       </c>
     </row>
     <row r="21" spans="1:2">
       <c r="A21" s="2">
-        <v>46147.19791666666</v>
+        <v>46149.19791666666</v>
       </c>
       <c r="B21">
-        <v>914</v>
+        <v>823</v>
       </c>
     </row>
     <row r="22" spans="1:2">
       <c r="A22" s="2">
-        <v>46147.20833333334</v>
+        <v>46149.20833333334</v>
       </c>
       <c r="B22">
-        <v>920</v>
+        <v>840</v>
       </c>
     </row>
     <row r="23" spans="1:2">
       <c r="A23" s="2">
-        <v>46147.21875</v>
+        <v>46149.21875</v>
       </c>
       <c r="B23">
-        <v>0</v>
+        <v>844</v>
       </c>
     </row>
     <row r="24" spans="1:2">
       <c r="A24" s="2">
-        <v>46147.22916666666</v>
+        <v>46149.22916666666</v>
       </c>
       <c r="B24">
-        <v>923</v>
+        <v>850</v>
       </c>
     </row>
     <row r="25" spans="1:2">
       <c r="A25" s="2">
-        <v>46147.23958333334</v>
+        <v>46149.23958333334</v>
       </c>
       <c r="B25">
-        <v>922</v>
+        <v>0</v>
       </c>
     </row>
     <row r="26" spans="1:2">
       <c r="A26" s="2">
-        <v>46147.25</v>
+        <v>46149.25</v>
       </c>
       <c r="B26">
-        <v>937</v>
+        <v>836</v>
       </c>
     </row>
     <row r="27" spans="1:2">
       <c r="A27" s="2">
-        <v>46147.26041666666</v>
+        <v>46149.26041666666</v>
       </c>
       <c r="B27">
-        <v>938</v>
+        <v>839</v>
       </c>
     </row>
     <row r="28" spans="1:2">
       <c r="A28" s="2">
-        <v>46147.27083333334</v>
+        <v>46149.27083333334</v>
       </c>
       <c r="B28">
-        <v>934</v>
+        <v>836</v>
       </c>
     </row>
     <row r="29" spans="1:2">
       <c r="A29" s="2">
-        <v>46147.28125</v>
+        <v>46149.28125</v>
       </c>
       <c r="B29">
-        <v>939</v>
+        <v>840</v>
       </c>
     </row>
     <row r="30" spans="1:2">
       <c r="A30" s="2">
-        <v>46147.29166666666</v>
+        <v>46149.29166666666</v>
       </c>
       <c r="B30">
-        <v>805</v>
+        <v>810</v>
       </c>
     </row>
     <row r="31" spans="1:2">
       <c r="A31" s="2">
-        <v>46147.30208333334</v>
+        <v>46149.30208333334</v>
       </c>
       <c r="B31">
-        <v>767</v>
+        <v>799</v>
       </c>
     </row>
     <row r="32" spans="1:2">
       <c r="A32" s="2">
-        <v>46147.3125</v>
+        <v>46149.3125</v>
       </c>
       <c r="B32">
-        <v>766</v>
+        <v>0</v>
       </c>
     </row>
     <row r="33" spans="1:2">
       <c r="A33" s="2">
-        <v>46147.32291666666</v>
+        <v>46149.32291666666</v>
       </c>
       <c r="B33">
-        <v>768</v>
+        <v>797</v>
       </c>
     </row>
     <row r="34" spans="1:2">
       <c r="A34" s="2">
-        <v>46147.33333333334</v>
+        <v>46149.33333333334</v>
       </c>
       <c r="B34">
-        <v>744</v>
+        <v>790</v>
       </c>
     </row>
     <row r="35" spans="1:2">
       <c r="A35" s="2">
-        <v>46147.34375</v>
+        <v>46149.34375</v>
       </c>
       <c r="B35">
-        <v>746</v>
+        <v>784</v>
       </c>
     </row>
     <row r="36" spans="1:2">
       <c r="A36" s="2">
-        <v>46147.35416666666</v>
+        <v>46149.35416666666</v>
       </c>
       <c r="B36">
-        <v>756</v>
+        <v>786</v>
       </c>
     </row>
     <row r="37" spans="1:2">
       <c r="A37" s="2">
-        <v>46147.36458333334</v>
+        <v>46149.36458333334</v>
       </c>
       <c r="B37">
-        <v>773</v>
+        <v>783</v>
       </c>
     </row>
     <row r="38" spans="1:2">
       <c r="A38" s="2">
-        <v>46147.375</v>
+        <v>46149.375</v>
       </c>
       <c r="B38">
-        <v>867</v>
+        <v>704</v>
       </c>
     </row>
     <row r="39" spans="1:2">
       <c r="A39" s="2">
-        <v>46147.38541666666</v>
+        <v>46149.38541666666</v>
       </c>
       <c r="B39">
-        <v>862</v>
+        <v>684</v>
       </c>
     </row>
     <row r="40" spans="1:2">
       <c r="A40" s="2">
-        <v>46147.39583333334</v>
+        <v>46149.39583333334</v>
       </c>
       <c r="B40">
-        <v>865</v>
+        <v>0</v>
       </c>
     </row>
     <row r="41" spans="1:2">
       <c r="A41" s="2">
-        <v>46147.40625</v>
+        <v>46149.40625</v>
       </c>
       <c r="B41">
-        <v>864</v>
+        <v>691</v>
       </c>
     </row>
     <row r="42" spans="1:2">
       <c r="A42" s="2">
-        <v>46147.41666666666</v>
+        <v>46149.41666666666</v>
       </c>
       <c r="B42">
-        <v>666</v>
+        <v>562</v>
       </c>
     </row>
     <row r="43" spans="1:2">
       <c r="A43" s="2">
-        <v>46147.42708333334</v>
+        <v>46149.42708333334</v>
       </c>
       <c r="B43">
-        <v>651</v>
+        <v>538</v>
       </c>
     </row>
     <row r="44" spans="1:2">
       <c r="A44" s="2">
-        <v>46147.4375</v>
+        <v>46149.4375</v>
       </c>
       <c r="B44">
-        <v>650</v>
+        <v>0</v>
       </c>
     </row>
     <row r="45" spans="1:2">
       <c r="A45" s="2">
-        <v>46147.44791666666</v>
+        <v>46149.44791666666</v>
       </c>
       <c r="B45">
         <v>0</v>
@@ -746,439 +746,439 @@
     </row>
     <row r="46" spans="1:2">
       <c r="A46" s="2">
-        <v>46147.45833333334</v>
+        <v>46149.45833333334</v>
       </c>
       <c r="B46">
-        <v>551</v>
+        <v>539</v>
       </c>
     </row>
     <row r="47" spans="1:2">
       <c r="A47" s="2">
-        <v>46147.46875</v>
+        <v>46149.46875</v>
       </c>
       <c r="B47">
-        <v>543</v>
+        <v>538</v>
       </c>
     </row>
     <row r="48" spans="1:2">
       <c r="A48" s="2">
-        <v>46147.47916666666</v>
+        <v>46149.47916666666</v>
       </c>
       <c r="B48">
-        <v>481</v>
+        <v>537</v>
       </c>
     </row>
     <row r="49" spans="1:2">
       <c r="A49" s="2">
-        <v>46147.48958333334</v>
+        <v>46149.48958333334</v>
       </c>
       <c r="B49">
-        <v>452</v>
+        <v>539</v>
       </c>
     </row>
     <row r="50" spans="1:2">
       <c r="A50" s="2">
-        <v>46147.5</v>
+        <v>46149.5</v>
       </c>
       <c r="B50">
-        <v>473</v>
+        <v>576</v>
       </c>
     </row>
     <row r="51" spans="1:2">
       <c r="A51" s="2">
-        <v>46147.51041666666</v>
+        <v>46149.51041666666</v>
       </c>
       <c r="B51">
-        <v>474</v>
+        <v>0</v>
       </c>
     </row>
     <row r="52" spans="1:2">
       <c r="A52" s="2">
-        <v>46147.52083333334</v>
+        <v>46149.52083333334</v>
       </c>
       <c r="B52">
-        <v>437</v>
+        <v>577</v>
       </c>
     </row>
     <row r="53" spans="1:2">
       <c r="A53" s="2">
-        <v>46147.53125</v>
+        <v>46149.53125</v>
       </c>
       <c r="B53">
-        <v>388</v>
+        <v>575</v>
       </c>
     </row>
     <row r="54" spans="1:2">
       <c r="A54" s="2">
-        <v>46147.54166666666</v>
+        <v>46149.54166666666</v>
       </c>
       <c r="B54">
-        <v>382</v>
+        <v>579</v>
       </c>
     </row>
     <row r="55" spans="1:2">
       <c r="A55" s="2">
-        <v>46147.55208333334</v>
+        <v>46149.55208333334</v>
       </c>
       <c r="B55">
-        <v>380</v>
+        <v>573</v>
       </c>
     </row>
     <row r="56" spans="1:2">
       <c r="A56" s="2">
-        <v>46147.5625</v>
+        <v>46149.5625</v>
       </c>
       <c r="B56">
-        <v>369</v>
+        <v>574</v>
       </c>
     </row>
     <row r="57" spans="1:2">
       <c r="A57" s="2">
-        <v>46147.57291666666</v>
+        <v>46149.57291666666</v>
       </c>
       <c r="B57">
-        <v>360</v>
+        <v>575</v>
       </c>
     </row>
     <row r="58" spans="1:2">
       <c r="A58" s="2">
-        <v>46147.58333333334</v>
+        <v>46149.58333333334</v>
       </c>
       <c r="B58">
-        <v>359</v>
+        <v>600</v>
       </c>
     </row>
     <row r="59" spans="1:2">
       <c r="A59" s="2">
-        <v>46147.59375</v>
+        <v>46149.59375</v>
       </c>
       <c r="B59">
-        <v>360</v>
+        <v>602</v>
       </c>
     </row>
     <row r="60" spans="1:2">
       <c r="A60" s="2">
-        <v>46147.60416666666</v>
+        <v>46149.60416666666</v>
       </c>
       <c r="B60">
-        <v>441</v>
+        <v>0</v>
       </c>
     </row>
     <row r="61" spans="1:2">
       <c r="A61" s="2">
-        <v>46147.61458333334</v>
+        <v>46149.61458333334</v>
       </c>
       <c r="B61">
-        <v>470</v>
+        <v>604</v>
       </c>
     </row>
     <row r="62" spans="1:2">
       <c r="A62" s="2">
-        <v>46147.625</v>
+        <v>46149.625</v>
       </c>
       <c r="B62">
-        <v>538</v>
+        <v>669</v>
       </c>
     </row>
     <row r="63" spans="1:2">
       <c r="A63" s="2">
-        <v>46147.63541666666</v>
+        <v>46149.63541666666</v>
       </c>
       <c r="B63">
-        <v>582</v>
+        <v>702</v>
       </c>
     </row>
     <row r="64" spans="1:2">
       <c r="A64" s="2">
-        <v>46147.64583333334</v>
+        <v>46149.64583333334</v>
       </c>
       <c r="B64">
-        <v>588</v>
+        <v>700</v>
       </c>
     </row>
     <row r="65" spans="1:2">
       <c r="A65" s="2">
-        <v>46147.65625</v>
+        <v>46149.65625</v>
       </c>
       <c r="B65">
-        <v>506</v>
+        <v>658</v>
       </c>
     </row>
     <row r="66" spans="1:2">
       <c r="A66" s="2">
-        <v>46147.66666666666</v>
+        <v>46149.66666666666</v>
       </c>
       <c r="B66">
-        <v>656</v>
+        <v>690</v>
       </c>
     </row>
     <row r="67" spans="1:2">
       <c r="A67" s="2">
-        <v>46147.67708333334</v>
+        <v>46149.67708333334</v>
       </c>
       <c r="B67">
-        <v>721</v>
+        <v>797</v>
       </c>
     </row>
     <row r="68" spans="1:2">
       <c r="A68" s="2">
-        <v>46147.6875</v>
+        <v>46149.6875</v>
       </c>
       <c r="B68">
-        <v>765</v>
+        <v>796</v>
       </c>
     </row>
     <row r="69" spans="1:2">
       <c r="A69" s="2">
-        <v>46147.69791666666</v>
+        <v>46149.69791666666</v>
       </c>
       <c r="B69">
-        <v>771</v>
+        <v>801</v>
       </c>
     </row>
     <row r="70" spans="1:2">
       <c r="A70" s="2">
-        <v>46147.70833333334</v>
+        <v>46149.70833333334</v>
       </c>
       <c r="B70">
-        <v>895</v>
+        <v>877</v>
       </c>
     </row>
     <row r="71" spans="1:2">
       <c r="A71" s="2">
-        <v>46147.71875</v>
+        <v>46149.71875</v>
       </c>
       <c r="B71">
-        <v>916</v>
+        <v>889</v>
       </c>
     </row>
     <row r="72" spans="1:2">
       <c r="A72" s="2">
-        <v>46147.72916666666</v>
+        <v>46149.72916666666</v>
       </c>
       <c r="B72">
-        <v>862</v>
+        <v>884</v>
       </c>
     </row>
     <row r="73" spans="1:2">
       <c r="A73" s="2">
-        <v>46147.73958333334</v>
+        <v>46149.73958333334</v>
       </c>
       <c r="B73">
-        <v>0</v>
+        <v>906</v>
       </c>
     </row>
     <row r="74" spans="1:2">
       <c r="A74" s="2">
-        <v>46147.75</v>
+        <v>46149.75</v>
       </c>
       <c r="B74">
-        <v>980</v>
+        <v>1075</v>
       </c>
     </row>
     <row r="75" spans="1:2">
       <c r="A75" s="2">
-        <v>46147.76041666666</v>
+        <v>46149.76041666666</v>
       </c>
       <c r="B75">
-        <v>1036</v>
+        <v>1086</v>
       </c>
     </row>
     <row r="76" spans="1:2">
       <c r="A76" s="2">
-        <v>46147.77083333334</v>
+        <v>46149.77083333334</v>
       </c>
       <c r="B76">
-        <v>1041</v>
+        <v>1083</v>
       </c>
     </row>
     <row r="77" spans="1:2">
       <c r="A77" s="2">
-        <v>46147.78125</v>
+        <v>46149.78125</v>
       </c>
       <c r="B77">
-        <v>1038</v>
+        <v>1084</v>
       </c>
     </row>
     <row r="78" spans="1:2">
       <c r="A78" s="2">
-        <v>46147.79166666666</v>
+        <v>46149.79166666666</v>
       </c>
       <c r="B78">
-        <v>1073</v>
+        <v>1059</v>
       </c>
     </row>
     <row r="79" spans="1:2">
       <c r="A79" s="2">
-        <v>46147.80208333334</v>
+        <v>46149.80208333334</v>
       </c>
       <c r="B79">
-        <v>1075</v>
+        <v>1060</v>
       </c>
     </row>
     <row r="80" spans="1:2">
       <c r="A80" s="2">
-        <v>46147.8125</v>
+        <v>46149.8125</v>
       </c>
       <c r="B80">
-        <v>1077</v>
+        <v>1061</v>
       </c>
     </row>
     <row r="81" spans="1:2">
       <c r="A81" s="2">
-        <v>46147.82291666666</v>
+        <v>46149.82291666666</v>
       </c>
       <c r="B81">
-        <v>1076</v>
+        <v>1066</v>
       </c>
     </row>
     <row r="82" spans="1:2">
       <c r="A82" s="2">
-        <v>46147.83333333334</v>
+        <v>46149.83333333334</v>
       </c>
       <c r="B82">
-        <v>1080</v>
+        <v>1092</v>
       </c>
     </row>
     <row r="83" spans="1:2">
       <c r="A83" s="2">
-        <v>46147.84375</v>
+        <v>46149.84375</v>
       </c>
       <c r="B83">
-        <v>1075</v>
+        <v>1093</v>
       </c>
     </row>
     <row r="84" spans="1:2">
       <c r="A84" s="2">
-        <v>46147.85416666666</v>
+        <v>46149.85416666666</v>
       </c>
       <c r="B84">
-        <v>1076</v>
+        <v>1092</v>
       </c>
     </row>
     <row r="85" spans="1:2">
       <c r="A85" s="2">
-        <v>46147.86458333334</v>
+        <v>46149.86458333334</v>
       </c>
       <c r="B85">
-        <v>1077</v>
+        <v>1090</v>
       </c>
     </row>
     <row r="86" spans="1:2">
       <c r="A86" s="2">
-        <v>46147.875</v>
+        <v>46149.875</v>
       </c>
       <c r="B86">
-        <v>1093</v>
+        <v>1114</v>
       </c>
     </row>
     <row r="87" spans="1:2">
       <c r="A87" s="2">
-        <v>46147.88541666666</v>
+        <v>46149.88541666666</v>
       </c>
       <c r="B87">
-        <v>1091</v>
+        <v>1110</v>
       </c>
     </row>
     <row r="88" spans="1:2">
       <c r="A88" s="2">
-        <v>46147.89583333334</v>
+        <v>46149.89583333334</v>
       </c>
       <c r="B88">
-        <v>1019</v>
+        <v>0</v>
       </c>
     </row>
     <row r="89" spans="1:2">
       <c r="A89" s="2">
-        <v>46147.90625</v>
+        <v>46149.90625</v>
       </c>
       <c r="B89">
-        <v>1012</v>
+        <v>1105</v>
       </c>
     </row>
     <row r="90" spans="1:2">
       <c r="A90" s="2">
-        <v>46147.91666666666</v>
+        <v>46149.91666666666</v>
       </c>
       <c r="B90">
-        <v>996</v>
+        <v>937</v>
       </c>
     </row>
     <row r="91" spans="1:2">
       <c r="A91" s="2">
-        <v>46147.92708333334</v>
+        <v>46149.92708333334</v>
       </c>
       <c r="B91">
-        <v>977</v>
+        <v>920</v>
       </c>
     </row>
     <row r="92" spans="1:2">
       <c r="A92" s="2">
-        <v>46147.9375</v>
+        <v>46149.9375</v>
       </c>
       <c r="B92">
-        <v>971</v>
+        <v>923</v>
       </c>
     </row>
     <row r="93" spans="1:2">
       <c r="A93" s="2">
-        <v>46147.94791666666</v>
+        <v>46149.94791666666</v>
       </c>
       <c r="B93">
-        <v>988</v>
+        <v>921</v>
       </c>
     </row>
     <row r="94" spans="1:2">
       <c r="A94" s="2">
-        <v>46147.95833333334</v>
+        <v>46149.95833333334</v>
       </c>
       <c r="B94">
-        <v>882</v>
+        <v>906</v>
       </c>
     </row>
     <row r="95" spans="1:2">
       <c r="A95" s="2">
-        <v>46147.96875</v>
+        <v>46149.96875</v>
       </c>
       <c r="B95">
-        <v>868</v>
+        <v>898</v>
       </c>
     </row>
     <row r="96" spans="1:2">
       <c r="A96" s="2">
-        <v>46147.97916666666</v>
+        <v>46149.97916666666</v>
       </c>
       <c r="B96">
-        <v>865</v>
+        <v>899</v>
       </c>
     </row>
     <row r="97" spans="1:2">
       <c r="A97" s="2">
-        <v>46147.98958333334</v>
+        <v>46149.98958333334</v>
       </c>
       <c r="B97">
-        <v>863</v>
+        <v>897</v>
       </c>
     </row>
     <row r="98" spans="1:2">
       <c r="A98" s="2">
-        <v>46148</v>
+        <v>46150</v>
       </c>
       <c r="B98">
-        <v>817</v>
+        <v>928</v>
       </c>
     </row>
     <row r="99" spans="1:2">
       <c r="A99" s="2">
-        <v>46148.01041666666</v>
+        <v>46150.01041666666</v>
       </c>
       <c r="B99">
-        <v>816</v>
+        <v>922</v>
       </c>
     </row>
     <row r="100" spans="1:2">
       <c r="A100" s="2">
-        <v>46148.02083333334</v>
+        <v>46150.02083333334</v>
       </c>
       <c r="B100">
         <v>0</v>
@@ -1186,223 +1186,223 @@
     </row>
     <row r="101" spans="1:2">
       <c r="A101" s="2">
-        <v>46148.03125</v>
+        <v>46150.03125</v>
       </c>
       <c r="B101">
-        <v>0</v>
+        <v>920</v>
       </c>
     </row>
     <row r="102" spans="1:2">
       <c r="A102" s="2">
-        <v>46148.04166666666</v>
+        <v>46150.04166666666</v>
       </c>
       <c r="B102">
-        <v>834</v>
+        <v>894</v>
       </c>
     </row>
     <row r="103" spans="1:2">
       <c r="A103" s="2">
-        <v>46148.05208333334</v>
+        <v>46150.05208333334</v>
       </c>
       <c r="B103">
-        <v>835</v>
+        <v>888</v>
       </c>
     </row>
     <row r="104" spans="1:2">
       <c r="A104" s="2">
-        <v>46148.0625</v>
+        <v>46150.0625</v>
       </c>
       <c r="B104">
-        <v>834</v>
+        <v>889</v>
       </c>
     </row>
     <row r="105" spans="1:2">
       <c r="A105" s="2">
-        <v>46148.07291666666</v>
+        <v>46150.07291666666</v>
       </c>
       <c r="B105">
-        <v>835</v>
+        <v>888</v>
       </c>
     </row>
     <row r="106" spans="1:2">
       <c r="A106" s="2">
-        <v>46148.08333333334</v>
+        <v>46150.08333333334</v>
       </c>
       <c r="B106">
-        <v>839</v>
+        <v>890</v>
       </c>
     </row>
     <row r="107" spans="1:2">
       <c r="A107" s="2">
-        <v>46148.09375</v>
+        <v>46150.09375</v>
       </c>
       <c r="B107">
-        <v>837</v>
+        <v>888</v>
       </c>
     </row>
     <row r="108" spans="1:2">
       <c r="A108" s="2">
-        <v>46148.10416666666</v>
+        <v>46150.10416666666</v>
       </c>
       <c r="B108">
-        <v>836</v>
+        <v>890</v>
       </c>
     </row>
     <row r="109" spans="1:2">
       <c r="A109" s="2">
-        <v>46148.11458333334</v>
+        <v>46150.11458333334</v>
       </c>
       <c r="B109">
-        <v>838</v>
+        <v>0</v>
       </c>
     </row>
     <row r="110" spans="1:2">
       <c r="A110" s="2">
-        <v>46148.125</v>
+        <v>46150.125</v>
       </c>
       <c r="B110">
-        <v>806</v>
+        <v>903</v>
       </c>
     </row>
     <row r="111" spans="1:2">
       <c r="A111" s="2">
-        <v>46148.13541666666</v>
+        <v>46150.13541666666</v>
       </c>
       <c r="B111">
-        <v>805</v>
+        <v>904</v>
       </c>
     </row>
     <row r="112" spans="1:2">
       <c r="A112" s="2">
-        <v>46148.14583333334</v>
+        <v>46150.14583333334</v>
       </c>
       <c r="B112">
-        <v>0</v>
+        <v>903</v>
       </c>
     </row>
     <row r="113" spans="1:2">
       <c r="A113" s="2">
-        <v>46148.15625</v>
+        <v>46150.15625</v>
       </c>
       <c r="B113">
-        <v>807</v>
+        <v>0</v>
       </c>
     </row>
     <row r="114" spans="1:2">
       <c r="A114" s="2">
-        <v>46148.16666666666</v>
+        <v>46150.16666666666</v>
       </c>
       <c r="B114">
-        <v>817</v>
+        <v>907</v>
       </c>
     </row>
     <row r="115" spans="1:2">
       <c r="A115" s="2">
-        <v>46148.17708333334</v>
+        <v>46150.17708333334</v>
       </c>
       <c r="B115">
-        <v>0</v>
+        <v>906</v>
       </c>
     </row>
     <row r="116" spans="1:2">
       <c r="A116" s="2">
-        <v>46148.1875</v>
+        <v>46150.1875</v>
       </c>
       <c r="B116">
-        <v>0</v>
+        <v>905</v>
       </c>
     </row>
     <row r="117" spans="1:2">
       <c r="A117" s="2">
-        <v>46148.19791666666</v>
+        <v>46150.19791666666</v>
       </c>
       <c r="B117">
-        <v>820</v>
+        <v>903</v>
       </c>
     </row>
     <row r="118" spans="1:2">
       <c r="A118" s="2">
-        <v>46148.20833333334</v>
+        <v>46150.20833333334</v>
       </c>
       <c r="B118">
-        <v>809</v>
+        <v>925</v>
       </c>
     </row>
     <row r="119" spans="1:2">
       <c r="A119" s="2">
-        <v>46148.21875</v>
+        <v>46150.21875</v>
       </c>
       <c r="B119">
-        <v>810</v>
+        <v>928</v>
       </c>
     </row>
     <row r="120" spans="1:2">
       <c r="A120" s="2">
-        <v>46148.22916666666</v>
+        <v>46150.22916666666</v>
       </c>
       <c r="B120">
-        <v>809</v>
+        <v>0</v>
       </c>
     </row>
     <row r="121" spans="1:2">
       <c r="A121" s="2">
-        <v>46148.23958333334</v>
+        <v>46150.23958333334</v>
       </c>
       <c r="B121">
-        <v>807</v>
+        <v>0</v>
       </c>
     </row>
     <row r="122" spans="1:2">
       <c r="A122" s="2">
-        <v>46148.25</v>
+        <v>46150.25</v>
       </c>
       <c r="B122">
-        <v>835</v>
+        <v>950</v>
       </c>
     </row>
     <row r="123" spans="1:2">
       <c r="A123" s="2">
-        <v>46148.26041666666</v>
+        <v>46150.26041666666</v>
       </c>
       <c r="B123">
-        <v>0</v>
+        <v>947</v>
       </c>
     </row>
     <row r="124" spans="1:2">
       <c r="A124" s="2">
-        <v>46148.27083333334</v>
+        <v>46150.27083333334</v>
       </c>
       <c r="B124">
-        <v>834</v>
+        <v>948</v>
       </c>
     </row>
     <row r="125" spans="1:2">
       <c r="A125" s="2">
-        <v>46148.28125</v>
+        <v>46150.28125</v>
       </c>
       <c r="B125">
-        <v>835</v>
+        <v>953</v>
       </c>
     </row>
     <row r="126" spans="1:2">
       <c r="A126" s="2">
-        <v>46148.29166666666</v>
+        <v>46150.29166666666</v>
       </c>
       <c r="B126">
-        <v>821</v>
+        <v>939</v>
       </c>
     </row>
     <row r="127" spans="1:2">
       <c r="A127" s="2">
-        <v>46148.30208333334</v>
+        <v>46150.30208333334</v>
       </c>
       <c r="B127">
-        <v>815</v>
+        <v>935</v>
       </c>
     </row>
     <row r="128" spans="1:2">
       <c r="A128" s="2">
-        <v>46148.3125</v>
+        <v>46150.3125</v>
       </c>
       <c r="B128">
         <v>0</v>
@@ -1410,7 +1410,7 @@
     </row>
     <row r="129" spans="1:2">
       <c r="A129" s="2">
-        <v>46148.32291666666</v>
+        <v>46150.32291666666</v>
       </c>
       <c r="B129">
         <v>0</v>
@@ -1418,7 +1418,7 @@
     </row>
     <row r="130" spans="1:2">
       <c r="A130" s="2">
-        <v>46148.33333333334</v>
+        <v>46150.33333333334</v>
       </c>
       <c r="B130">
         <v>0</v>
@@ -1426,7 +1426,7 @@
     </row>
     <row r="131" spans="1:2">
       <c r="A131" s="2">
-        <v>46148.34375</v>
+        <v>46150.34375</v>
       </c>
       <c r="B131">
         <v>0</v>
@@ -1434,7 +1434,7 @@
     </row>
     <row r="132" spans="1:2">
       <c r="A132" s="2">
-        <v>46148.35416666666</v>
+        <v>46150.35416666666</v>
       </c>
       <c r="B132">
         <v>0</v>
@@ -1442,7 +1442,7 @@
     </row>
     <row r="133" spans="1:2">
       <c r="A133" s="2">
-        <v>46148.36458333334</v>
+        <v>46150.36458333334</v>
       </c>
       <c r="B133">
         <v>0</v>
@@ -1450,7 +1450,7 @@
     </row>
     <row r="134" spans="1:2">
       <c r="A134" s="2">
-        <v>46148.375</v>
+        <v>46150.375</v>
       </c>
       <c r="B134">
         <v>0</v>
@@ -1458,7 +1458,7 @@
     </row>
     <row r="135" spans="1:2">
       <c r="A135" s="2">
-        <v>46148.38541666666</v>
+        <v>46150.38541666666</v>
       </c>
       <c r="B135">
         <v>0</v>
@@ -1466,7 +1466,7 @@
     </row>
     <row r="136" spans="1:2">
       <c r="A136" s="2">
-        <v>46148.39583333334</v>
+        <v>46150.39583333334</v>
       </c>
       <c r="B136">
         <v>0</v>
@@ -1474,7 +1474,7 @@
     </row>
     <row r="137" spans="1:2">
       <c r="A137" s="2">
-        <v>46148.40625</v>
+        <v>46150.40625</v>
       </c>
       <c r="B137">
         <v>0</v>
@@ -1482,7 +1482,7 @@
     </row>
     <row r="138" spans="1:2">
       <c r="A138" s="2">
-        <v>46148.41666666666</v>
+        <v>46150.41666666666</v>
       </c>
       <c r="B138">
         <v>0</v>
@@ -1490,7 +1490,7 @@
     </row>
     <row r="139" spans="1:2">
       <c r="A139" s="2">
-        <v>46148.42708333334</v>
+        <v>46150.42708333334</v>
       </c>
       <c r="B139">
         <v>0</v>
@@ -1498,7 +1498,7 @@
     </row>
     <row r="140" spans="1:2">
       <c r="A140" s="2">
-        <v>46148.4375</v>
+        <v>46150.4375</v>
       </c>
       <c r="B140">
         <v>0</v>
@@ -1506,7 +1506,7 @@
     </row>
     <row r="141" spans="1:2">
       <c r="A141" s="2">
-        <v>46148.44791666666</v>
+        <v>46150.44791666666</v>
       </c>
       <c r="B141">
         <v>0</v>
@@ -1514,7 +1514,7 @@
     </row>
     <row r="142" spans="1:2">
       <c r="A142" s="2">
-        <v>46148.45833333334</v>
+        <v>46150.45833333334</v>
       </c>
       <c r="B142">
         <v>0</v>
@@ -1522,7 +1522,7 @@
     </row>
     <row r="143" spans="1:2">
       <c r="A143" s="2">
-        <v>46148.46875</v>
+        <v>46150.46875</v>
       </c>
       <c r="B143">
         <v>0</v>
@@ -1530,7 +1530,7 @@
     </row>
     <row r="144" spans="1:2">
       <c r="A144" s="2">
-        <v>46148.47916666666</v>
+        <v>46150.47916666666</v>
       </c>
       <c r="B144">
         <v>0</v>
@@ -1538,7 +1538,7 @@
     </row>
     <row r="145" spans="1:2">
       <c r="A145" s="2">
-        <v>46148.48958333334</v>
+        <v>46150.48958333334</v>
       </c>
       <c r="B145">
         <v>0</v>
@@ -1546,7 +1546,7 @@
     </row>
     <row r="146" spans="1:2">
       <c r="A146" s="2">
-        <v>46148.5</v>
+        <v>46150.5</v>
       </c>
       <c r="B146">
         <v>0</v>
@@ -1554,7 +1554,7 @@
     </row>
     <row r="147" spans="1:2">
       <c r="A147" s="2">
-        <v>46148.51041666666</v>
+        <v>46150.51041666666</v>
       </c>
       <c r="B147">
         <v>0</v>
@@ -1562,7 +1562,7 @@
     </row>
     <row r="148" spans="1:2">
       <c r="A148" s="2">
-        <v>46148.52083333334</v>
+        <v>46150.52083333334</v>
       </c>
       <c r="B148">
         <v>0</v>
@@ -1570,7 +1570,7 @@
     </row>
     <row r="149" spans="1:2">
       <c r="A149" s="2">
-        <v>46148.53125</v>
+        <v>46150.53125</v>
       </c>
       <c r="B149">
         <v>0</v>
@@ -1578,7 +1578,7 @@
     </row>
     <row r="150" spans="1:2">
       <c r="A150" s="2">
-        <v>46148.54166666666</v>
+        <v>46150.54166666666</v>
       </c>
       <c r="B150">
         <v>0</v>
@@ -1586,7 +1586,7 @@
     </row>
     <row r="151" spans="1:2">
       <c r="A151" s="2">
-        <v>46148.55208333334</v>
+        <v>46150.55208333334</v>
       </c>
       <c r="B151">
         <v>0</v>
@@ -1594,7 +1594,7 @@
     </row>
     <row r="152" spans="1:2">
       <c r="A152" s="2">
-        <v>46148.5625</v>
+        <v>46150.5625</v>
       </c>
       <c r="B152">
         <v>0</v>
@@ -1602,7 +1602,7 @@
     </row>
     <row r="153" spans="1:2">
       <c r="A153" s="2">
-        <v>46148.57291666666</v>
+        <v>46150.57291666666</v>
       </c>
       <c r="B153">
         <v>0</v>
@@ -1610,7 +1610,7 @@
     </row>
     <row r="154" spans="1:2">
       <c r="A154" s="2">
-        <v>46148.58333333334</v>
+        <v>46150.58333333334</v>
       </c>
       <c r="B154">
         <v>0</v>
@@ -1618,7 +1618,7 @@
     </row>
     <row r="155" spans="1:2">
       <c r="A155" s="2">
-        <v>46148.59375</v>
+        <v>46150.59375</v>
       </c>
       <c r="B155">
         <v>0</v>
@@ -1626,7 +1626,7 @@
     </row>
     <row r="156" spans="1:2">
       <c r="A156" s="2">
-        <v>46148.60416666666</v>
+        <v>46150.60416666666</v>
       </c>
       <c r="B156">
         <v>0</v>
@@ -1634,7 +1634,7 @@
     </row>
     <row r="157" spans="1:2">
       <c r="A157" s="2">
-        <v>46148.61458333334</v>
+        <v>46150.61458333334</v>
       </c>
       <c r="B157">
         <v>0</v>
@@ -1642,7 +1642,7 @@
     </row>
     <row r="158" spans="1:2">
       <c r="A158" s="2">
-        <v>46148.625</v>
+        <v>46150.625</v>
       </c>
       <c r="B158">
         <v>0</v>
@@ -1650,7 +1650,7 @@
     </row>
     <row r="159" spans="1:2">
       <c r="A159" s="2">
-        <v>46148.63541666666</v>
+        <v>46150.63541666666</v>
       </c>
       <c r="B159">
         <v>0</v>
@@ -1658,7 +1658,7 @@
     </row>
     <row r="160" spans="1:2">
       <c r="A160" s="2">
-        <v>46148.64583333334</v>
+        <v>46150.64583333334</v>
       </c>
       <c r="B160">
         <v>0</v>
@@ -1666,7 +1666,7 @@
     </row>
     <row r="161" spans="1:2">
       <c r="A161" s="2">
-        <v>46148.65625</v>
+        <v>46150.65625</v>
       </c>
       <c r="B161">
         <v>0</v>
@@ -1674,7 +1674,7 @@
     </row>
     <row r="162" spans="1:2">
       <c r="A162" s="2">
-        <v>46148.66666666666</v>
+        <v>46150.66666666666</v>
       </c>
       <c r="B162">
         <v>0</v>
@@ -1682,7 +1682,7 @@
     </row>
     <row r="163" spans="1:2">
       <c r="A163" s="2">
-        <v>46148.67708333334</v>
+        <v>46150.67708333334</v>
       </c>
       <c r="B163">
         <v>0</v>
@@ -1690,7 +1690,7 @@
     </row>
     <row r="164" spans="1:2">
       <c r="A164" s="2">
-        <v>46148.6875</v>
+        <v>46150.6875</v>
       </c>
       <c r="B164">
         <v>0</v>
@@ -1698,7 +1698,7 @@
     </row>
     <row r="165" spans="1:2">
       <c r="A165" s="2">
-        <v>46148.69791666666</v>
+        <v>46150.69791666666</v>
       </c>
       <c r="B165">
         <v>0</v>
@@ -1706,7 +1706,7 @@
     </row>
     <row r="166" spans="1:2">
       <c r="A166" s="2">
-        <v>46148.70833333334</v>
+        <v>46150.70833333334</v>
       </c>
       <c r="B166">
         <v>0</v>
@@ -1714,7 +1714,7 @@
     </row>
     <row r="167" spans="1:2">
       <c r="A167" s="2">
-        <v>46148.71875</v>
+        <v>46150.71875</v>
       </c>
       <c r="B167">
         <v>0</v>
@@ -1722,7 +1722,7 @@
     </row>
     <row r="168" spans="1:2">
       <c r="A168" s="2">
-        <v>46148.72916666666</v>
+        <v>46150.72916666666</v>
       </c>
       <c r="B168">
         <v>0</v>
@@ -1730,7 +1730,7 @@
     </row>
     <row r="169" spans="1:2">
       <c r="A169" s="2">
-        <v>46148.73958333334</v>
+        <v>46150.73958333334</v>
       </c>
       <c r="B169">
         <v>0</v>
@@ -1738,7 +1738,7 @@
     </row>
     <row r="170" spans="1:2">
       <c r="A170" s="2">
-        <v>46148.75</v>
+        <v>46150.75</v>
       </c>
       <c r="B170">
         <v>0</v>
@@ -1746,7 +1746,7 @@
     </row>
     <row r="171" spans="1:2">
       <c r="A171" s="2">
-        <v>46148.76041666666</v>
+        <v>46150.76041666666</v>
       </c>
       <c r="B171">
         <v>0</v>
@@ -1754,7 +1754,7 @@
     </row>
     <row r="172" spans="1:2">
       <c r="A172" s="2">
-        <v>46148.77083333334</v>
+        <v>46150.77083333334</v>
       </c>
       <c r="B172">
         <v>0</v>
@@ -1762,7 +1762,7 @@
     </row>
     <row r="173" spans="1:2">
       <c r="A173" s="2">
-        <v>46148.78125</v>
+        <v>46150.78125</v>
       </c>
       <c r="B173">
         <v>0</v>
@@ -1770,7 +1770,7 @@
     </row>
     <row r="174" spans="1:2">
       <c r="A174" s="2">
-        <v>46148.79166666666</v>
+        <v>46150.79166666666</v>
       </c>
       <c r="B174">
         <v>0</v>
@@ -1778,7 +1778,7 @@
     </row>
     <row r="175" spans="1:2">
       <c r="A175" s="2">
-        <v>46148.80208333334</v>
+        <v>46150.80208333334</v>
       </c>
       <c r="B175">
         <v>0</v>
@@ -1786,7 +1786,7 @@
     </row>
     <row r="176" spans="1:2">
       <c r="A176" s="2">
-        <v>46148.8125</v>
+        <v>46150.8125</v>
       </c>
       <c r="B176">
         <v>0</v>
@@ -1794,7 +1794,7 @@
     </row>
     <row r="177" spans="1:2">
       <c r="A177" s="2">
-        <v>46148.82291666666</v>
+        <v>46150.82291666666</v>
       </c>
       <c r="B177">
         <v>0</v>
@@ -1802,7 +1802,7 @@
     </row>
     <row r="178" spans="1:2">
       <c r="A178" s="2">
-        <v>46148.83333333334</v>
+        <v>46150.83333333334</v>
       </c>
       <c r="B178">
         <v>0</v>
@@ -1810,7 +1810,7 @@
     </row>
     <row r="179" spans="1:2">
       <c r="A179" s="2">
-        <v>46148.84375</v>
+        <v>46150.84375</v>
       </c>
       <c r="B179">
         <v>0</v>
@@ -1818,7 +1818,7 @@
     </row>
     <row r="180" spans="1:2">
       <c r="A180" s="2">
-        <v>46148.85416666666</v>
+        <v>46150.85416666666</v>
       </c>
       <c r="B180">
         <v>0</v>
@@ -1826,7 +1826,7 @@
     </row>
     <row r="181" spans="1:2">
       <c r="A181" s="2">
-        <v>46148.86458333334</v>
+        <v>46150.86458333334</v>
       </c>
       <c r="B181">
         <v>0</v>
@@ -1834,7 +1834,7 @@
     </row>
     <row r="182" spans="1:2">
       <c r="A182" s="2">
-        <v>46148.875</v>
+        <v>46150.875</v>
       </c>
       <c r="B182">
         <v>0</v>
@@ -1842,7 +1842,7 @@
     </row>
     <row r="183" spans="1:2">
       <c r="A183" s="2">
-        <v>46148.88541666666</v>
+        <v>46150.88541666666</v>
       </c>
       <c r="B183">
         <v>0</v>
@@ -1850,7 +1850,7 @@
     </row>
     <row r="184" spans="1:2">
       <c r="A184" s="2">
-        <v>46148.89583333334</v>
+        <v>46150.89583333334</v>
       </c>
       <c r="B184">
         <v>0</v>
@@ -1858,7 +1858,7 @@
     </row>
     <row r="185" spans="1:2">
       <c r="A185" s="2">
-        <v>46148.90625</v>
+        <v>46150.90625</v>
       </c>
       <c r="B185">
         <v>0</v>
@@ -1866,7 +1866,7 @@
     </row>
     <row r="186" spans="1:2">
       <c r="A186" s="2">
-        <v>46148.91666666666</v>
+        <v>46150.91666666666</v>
       </c>
       <c r="B186">
         <v>0</v>
@@ -1874,7 +1874,7 @@
     </row>
     <row r="187" spans="1:2">
       <c r="A187" s="2">
-        <v>46148.92708333334</v>
+        <v>46150.92708333334</v>
       </c>
       <c r="B187">
         <v>0</v>
@@ -1882,7 +1882,7 @@
     </row>
     <row r="188" spans="1:2">
       <c r="A188" s="2">
-        <v>46148.9375</v>
+        <v>46150.9375</v>
       </c>
       <c r="B188">
         <v>0</v>
@@ -1890,7 +1890,7 @@
     </row>
     <row r="189" spans="1:2">
       <c r="A189" s="2">
-        <v>46148.94791666666</v>
+        <v>46150.94791666666</v>
       </c>
       <c r="B189">
         <v>0</v>
@@ -1898,7 +1898,7 @@
     </row>
     <row r="190" spans="1:2">
       <c r="A190" s="2">
-        <v>46148.95833333334</v>
+        <v>46150.95833333334</v>
       </c>
       <c r="B190">
         <v>0</v>
@@ -1906,7 +1906,7 @@
     </row>
     <row r="191" spans="1:2">
       <c r="A191" s="2">
-        <v>46148.96875</v>
+        <v>46150.96875</v>
       </c>
       <c r="B191">
         <v>0</v>
@@ -1914,7 +1914,7 @@
     </row>
     <row r="192" spans="1:2">
       <c r="A192" s="2">
-        <v>46148.97916666666</v>
+        <v>46150.97916666666</v>
       </c>
       <c r="B192">
         <v>0</v>
@@ -1922,7 +1922,7 @@
     </row>
     <row r="193" spans="1:2">
       <c r="A193" s="2">
-        <v>46148.98958333334</v>
+        <v>46150.98958333334</v>
       </c>
       <c r="B193">
         <v>0</v>

</xml_diff>

<commit_message>
Updating the model for Motif
</commit_message>
<xml_diff>
--- a/data_fetching/Entsoe/Actual_Production_Hydro_River.xlsx
+++ b/data_fetching/Entsoe/Actual_Production_Hydro_River.xlsx
@@ -394,895 +394,895 @@
     </row>
     <row r="2" spans="1:2">
       <c r="A2" s="2">
-        <v>46149</v>
+        <v>46153</v>
       </c>
       <c r="B2">
-        <v>830</v>
+        <v>1033</v>
       </c>
     </row>
     <row r="3" spans="1:2">
       <c r="A3" s="2">
-        <v>46149.01041666666</v>
+        <v>46153.01041666666</v>
       </c>
       <c r="B3">
-        <v>826</v>
+        <v>1032</v>
       </c>
     </row>
     <row r="4" spans="1:2">
       <c r="A4" s="2">
-        <v>46149.02083333334</v>
+        <v>46153.02083333334</v>
       </c>
       <c r="B4">
-        <v>0</v>
+        <v>1030</v>
       </c>
     </row>
     <row r="5" spans="1:2">
       <c r="A5" s="2">
-        <v>46149.03125</v>
+        <v>46153.03125</v>
       </c>
       <c r="B5">
-        <v>824</v>
+        <v>1028</v>
       </c>
     </row>
     <row r="6" spans="1:2">
       <c r="A6" s="2">
-        <v>46149.04166666666</v>
+        <v>46153.04166666666</v>
       </c>
       <c r="B6">
-        <v>0</v>
+        <v>1032</v>
       </c>
     </row>
     <row r="7" spans="1:2">
       <c r="A7" s="2">
-        <v>46149.05208333334</v>
+        <v>46153.05208333334</v>
       </c>
       <c r="B7">
-        <v>820</v>
+        <v>1029</v>
       </c>
     </row>
     <row r="8" spans="1:2">
       <c r="A8" s="2">
-        <v>46149.0625</v>
+        <v>46153.0625</v>
       </c>
       <c r="B8">
-        <v>0</v>
+        <v>1027</v>
       </c>
     </row>
     <row r="9" spans="1:2">
       <c r="A9" s="2">
-        <v>46149.07291666666</v>
+        <v>46153.07291666666</v>
       </c>
       <c r="B9">
-        <v>813</v>
+        <v>1031</v>
       </c>
     </row>
     <row r="10" spans="1:2">
       <c r="A10" s="2">
-        <v>46149.08333333334</v>
+        <v>46153.08333333334</v>
       </c>
       <c r="B10">
-        <v>807</v>
+        <v>1036</v>
       </c>
     </row>
     <row r="11" spans="1:2">
       <c r="A11" s="2">
-        <v>46149.09375</v>
+        <v>46153.09375</v>
       </c>
       <c r="B11">
-        <v>806</v>
+        <v>1033</v>
       </c>
     </row>
     <row r="12" spans="1:2">
       <c r="A12" s="2">
-        <v>46149.10416666666</v>
+        <v>46153.10416666666</v>
       </c>
       <c r="B12">
-        <v>805</v>
+        <v>1035</v>
       </c>
     </row>
     <row r="13" spans="1:2">
       <c r="A13" s="2">
-        <v>46149.11458333334</v>
+        <v>46153.11458333334</v>
       </c>
       <c r="B13">
-        <v>804</v>
+        <v>1036</v>
       </c>
     </row>
     <row r="14" spans="1:2">
       <c r="A14" s="2">
-        <v>46149.125</v>
+        <v>46153.125</v>
       </c>
       <c r="B14">
-        <v>796</v>
+        <v>1039</v>
       </c>
     </row>
     <row r="15" spans="1:2">
       <c r="A15" s="2">
-        <v>46149.13541666666</v>
+        <v>46153.13541666666</v>
       </c>
       <c r="B15">
-        <v>795</v>
+        <v>1040</v>
       </c>
     </row>
     <row r="16" spans="1:2">
       <c r="A16" s="2">
-        <v>46149.14583333334</v>
+        <v>46153.14583333334</v>
       </c>
       <c r="B16">
-        <v>796</v>
+        <v>0</v>
       </c>
     </row>
     <row r="17" spans="1:2">
       <c r="A17" s="2">
-        <v>46149.15625</v>
+        <v>46153.15625</v>
       </c>
       <c r="B17">
-        <v>797</v>
+        <v>1038</v>
       </c>
     </row>
     <row r="18" spans="1:2">
       <c r="A18" s="2">
-        <v>46149.16666666666</v>
+        <v>46153.16666666666</v>
       </c>
       <c r="B18">
-        <v>824</v>
+        <v>1048</v>
       </c>
     </row>
     <row r="19" spans="1:2">
       <c r="A19" s="2">
-        <v>46149.17708333334</v>
+        <v>46153.17708333334</v>
       </c>
       <c r="B19">
-        <v>825</v>
+        <v>0</v>
       </c>
     </row>
     <row r="20" spans="1:2">
       <c r="A20" s="2">
-        <v>46149.1875</v>
+        <v>46153.1875</v>
       </c>
       <c r="B20">
-        <v>0</v>
+        <v>1047</v>
       </c>
     </row>
     <row r="21" spans="1:2">
       <c r="A21" s="2">
-        <v>46149.19791666666</v>
+        <v>46153.19791666666</v>
       </c>
       <c r="B21">
-        <v>823</v>
+        <v>1049</v>
       </c>
     </row>
     <row r="22" spans="1:2">
       <c r="A22" s="2">
-        <v>46149.20833333334</v>
+        <v>46153.20833333334</v>
       </c>
       <c r="B22">
-        <v>840</v>
+        <v>1051</v>
       </c>
     </row>
     <row r="23" spans="1:2">
       <c r="A23" s="2">
-        <v>46149.21875</v>
+        <v>46153.21875</v>
       </c>
       <c r="B23">
-        <v>844</v>
+        <v>1053</v>
       </c>
     </row>
     <row r="24" spans="1:2">
       <c r="A24" s="2">
-        <v>46149.22916666666</v>
+        <v>46153.22916666666</v>
       </c>
       <c r="B24">
-        <v>850</v>
+        <v>1050</v>
       </c>
     </row>
     <row r="25" spans="1:2">
       <c r="A25" s="2">
-        <v>46149.23958333334</v>
+        <v>46153.23958333334</v>
       </c>
       <c r="B25">
-        <v>0</v>
+        <v>1053</v>
       </c>
     </row>
     <row r="26" spans="1:2">
       <c r="A26" s="2">
-        <v>46149.25</v>
+        <v>46153.25</v>
       </c>
       <c r="B26">
-        <v>836</v>
+        <v>1049</v>
       </c>
     </row>
     <row r="27" spans="1:2">
       <c r="A27" s="2">
-        <v>46149.26041666666</v>
+        <v>46153.26041666666</v>
       </c>
       <c r="B27">
-        <v>839</v>
+        <v>1043</v>
       </c>
     </row>
     <row r="28" spans="1:2">
       <c r="A28" s="2">
-        <v>46149.27083333334</v>
+        <v>46153.27083333334</v>
       </c>
       <c r="B28">
-        <v>836</v>
+        <v>1045</v>
       </c>
     </row>
     <row r="29" spans="1:2">
       <c r="A29" s="2">
-        <v>46149.28125</v>
+        <v>46153.28125</v>
       </c>
       <c r="B29">
-        <v>840</v>
+        <v>1013</v>
       </c>
     </row>
     <row r="30" spans="1:2">
       <c r="A30" s="2">
-        <v>46149.29166666666</v>
+        <v>46153.29166666666</v>
       </c>
       <c r="B30">
-        <v>810</v>
+        <v>985</v>
       </c>
     </row>
     <row r="31" spans="1:2">
       <c r="A31" s="2">
-        <v>46149.30208333334</v>
+        <v>46153.30208333334</v>
       </c>
       <c r="B31">
-        <v>799</v>
+        <v>980</v>
       </c>
     </row>
     <row r="32" spans="1:2">
       <c r="A32" s="2">
-        <v>46149.3125</v>
+        <v>46153.3125</v>
       </c>
       <c r="B32">
-        <v>0</v>
+        <v>981</v>
       </c>
     </row>
     <row r="33" spans="1:2">
       <c r="A33" s="2">
-        <v>46149.32291666666</v>
+        <v>46153.32291666666</v>
       </c>
       <c r="B33">
-        <v>797</v>
+        <v>983</v>
       </c>
     </row>
     <row r="34" spans="1:2">
       <c r="A34" s="2">
-        <v>46149.33333333334</v>
+        <v>46153.33333333334</v>
       </c>
       <c r="B34">
-        <v>790</v>
+        <v>967</v>
       </c>
     </row>
     <row r="35" spans="1:2">
       <c r="A35" s="2">
-        <v>46149.34375</v>
+        <v>46153.34375</v>
       </c>
       <c r="B35">
-        <v>784</v>
+        <v>964</v>
       </c>
     </row>
     <row r="36" spans="1:2">
       <c r="A36" s="2">
-        <v>46149.35416666666</v>
+        <v>46153.35416666666</v>
       </c>
       <c r="B36">
-        <v>786</v>
+        <v>969</v>
       </c>
     </row>
     <row r="37" spans="1:2">
       <c r="A37" s="2">
-        <v>46149.36458333334</v>
+        <v>46153.36458333334</v>
       </c>
       <c r="B37">
-        <v>783</v>
+        <v>965</v>
       </c>
     </row>
     <row r="38" spans="1:2">
       <c r="A38" s="2">
-        <v>46149.375</v>
+        <v>46153.375</v>
       </c>
       <c r="B38">
-        <v>704</v>
+        <v>893</v>
       </c>
     </row>
     <row r="39" spans="1:2">
       <c r="A39" s="2">
-        <v>46149.38541666666</v>
+        <v>46153.38541666666</v>
       </c>
       <c r="B39">
-        <v>684</v>
+        <v>883</v>
       </c>
     </row>
     <row r="40" spans="1:2">
       <c r="A40" s="2">
-        <v>46149.39583333334</v>
+        <v>46153.39583333334</v>
       </c>
       <c r="B40">
-        <v>0</v>
+        <v>886</v>
       </c>
     </row>
     <row r="41" spans="1:2">
       <c r="A41" s="2">
-        <v>46149.40625</v>
+        <v>46153.40625</v>
       </c>
       <c r="B41">
-        <v>691</v>
+        <v>882</v>
       </c>
     </row>
     <row r="42" spans="1:2">
       <c r="A42" s="2">
-        <v>46149.41666666666</v>
+        <v>46153.41666666666</v>
       </c>
       <c r="B42">
-        <v>562</v>
+        <v>0</v>
       </c>
     </row>
     <row r="43" spans="1:2">
       <c r="A43" s="2">
-        <v>46149.42708333334</v>
+        <v>46153.42708333334</v>
       </c>
       <c r="B43">
-        <v>538</v>
+        <v>881</v>
       </c>
     </row>
     <row r="44" spans="1:2">
       <c r="A44" s="2">
-        <v>46149.4375</v>
+        <v>46153.4375</v>
       </c>
       <c r="B44">
-        <v>0</v>
+        <v>964</v>
       </c>
     </row>
     <row r="45" spans="1:2">
       <c r="A45" s="2">
-        <v>46149.44791666666</v>
+        <v>46153.44791666666</v>
       </c>
       <c r="B45">
-        <v>0</v>
+        <v>968</v>
       </c>
     </row>
     <row r="46" spans="1:2">
       <c r="A46" s="2">
-        <v>46149.45833333334</v>
+        <v>46153.45833333334</v>
       </c>
       <c r="B46">
-        <v>539</v>
+        <v>893</v>
       </c>
     </row>
     <row r="47" spans="1:2">
       <c r="A47" s="2">
-        <v>46149.46875</v>
+        <v>46153.46875</v>
       </c>
       <c r="B47">
-        <v>538</v>
+        <v>886</v>
       </c>
     </row>
     <row r="48" spans="1:2">
       <c r="A48" s="2">
-        <v>46149.47916666666</v>
+        <v>46153.47916666666</v>
       </c>
       <c r="B48">
-        <v>537</v>
+        <v>927</v>
       </c>
     </row>
     <row r="49" spans="1:2">
       <c r="A49" s="2">
-        <v>46149.48958333334</v>
+        <v>46153.48958333334</v>
       </c>
       <c r="B49">
-        <v>539</v>
+        <v>928</v>
       </c>
     </row>
     <row r="50" spans="1:2">
       <c r="A50" s="2">
-        <v>46149.5</v>
+        <v>46153.5</v>
       </c>
       <c r="B50">
-        <v>576</v>
+        <v>927</v>
       </c>
     </row>
     <row r="51" spans="1:2">
       <c r="A51" s="2">
-        <v>46149.51041666666</v>
+        <v>46153.51041666666</v>
       </c>
       <c r="B51">
-        <v>0</v>
+        <v>925</v>
       </c>
     </row>
     <row r="52" spans="1:2">
       <c r="A52" s="2">
-        <v>46149.52083333334</v>
+        <v>46153.52083333334</v>
       </c>
       <c r="B52">
-        <v>577</v>
+        <v>928</v>
       </c>
     </row>
     <row r="53" spans="1:2">
       <c r="A53" s="2">
-        <v>46149.53125</v>
+        <v>46153.53125</v>
       </c>
       <c r="B53">
-        <v>575</v>
+        <v>934</v>
       </c>
     </row>
     <row r="54" spans="1:2">
       <c r="A54" s="2">
-        <v>46149.54166666666</v>
+        <v>46153.54166666666</v>
       </c>
       <c r="B54">
-        <v>579</v>
+        <v>972</v>
       </c>
     </row>
     <row r="55" spans="1:2">
       <c r="A55" s="2">
-        <v>46149.55208333334</v>
+        <v>46153.55208333334</v>
       </c>
       <c r="B55">
-        <v>573</v>
+        <v>973</v>
       </c>
     </row>
     <row r="56" spans="1:2">
       <c r="A56" s="2">
-        <v>46149.5625</v>
+        <v>46153.5625</v>
       </c>
       <c r="B56">
-        <v>574</v>
+        <v>972</v>
       </c>
     </row>
     <row r="57" spans="1:2">
       <c r="A57" s="2">
-        <v>46149.57291666666</v>
+        <v>46153.57291666666</v>
       </c>
       <c r="B57">
-        <v>575</v>
+        <v>970</v>
       </c>
     </row>
     <row r="58" spans="1:2">
       <c r="A58" s="2">
-        <v>46149.58333333334</v>
+        <v>46153.58333333334</v>
       </c>
       <c r="B58">
-        <v>600</v>
+        <v>979</v>
       </c>
     </row>
     <row r="59" spans="1:2">
       <c r="A59" s="2">
-        <v>46149.59375</v>
+        <v>46153.59375</v>
       </c>
       <c r="B59">
-        <v>602</v>
+        <v>983</v>
       </c>
     </row>
     <row r="60" spans="1:2">
       <c r="A60" s="2">
-        <v>46149.60416666666</v>
+        <v>46153.60416666666</v>
       </c>
       <c r="B60">
-        <v>0</v>
+        <v>916</v>
       </c>
     </row>
     <row r="61" spans="1:2">
       <c r="A61" s="2">
-        <v>46149.61458333334</v>
+        <v>46153.61458333334</v>
       </c>
       <c r="B61">
-        <v>604</v>
+        <v>914</v>
       </c>
     </row>
     <row r="62" spans="1:2">
       <c r="A62" s="2">
-        <v>46149.625</v>
+        <v>46153.625</v>
       </c>
       <c r="B62">
-        <v>669</v>
+        <v>923</v>
       </c>
     </row>
     <row r="63" spans="1:2">
       <c r="A63" s="2">
-        <v>46149.63541666666</v>
+        <v>46153.63541666666</v>
       </c>
       <c r="B63">
-        <v>702</v>
+        <v>912</v>
       </c>
     </row>
     <row r="64" spans="1:2">
       <c r="A64" s="2">
-        <v>46149.64583333334</v>
+        <v>46153.64583333334</v>
       </c>
       <c r="B64">
-        <v>700</v>
+        <v>902</v>
       </c>
     </row>
     <row r="65" spans="1:2">
       <c r="A65" s="2">
-        <v>46149.65625</v>
+        <v>46153.65625</v>
       </c>
       <c r="B65">
-        <v>658</v>
+        <v>901</v>
       </c>
     </row>
     <row r="66" spans="1:2">
       <c r="A66" s="2">
-        <v>46149.66666666666</v>
+        <v>46153.66666666666</v>
       </c>
       <c r="B66">
-        <v>690</v>
+        <v>934</v>
       </c>
     </row>
     <row r="67" spans="1:2">
       <c r="A67" s="2">
-        <v>46149.67708333334</v>
+        <v>46153.67708333334</v>
       </c>
       <c r="B67">
-        <v>797</v>
+        <v>940</v>
       </c>
     </row>
     <row r="68" spans="1:2">
       <c r="A68" s="2">
-        <v>46149.6875</v>
+        <v>46153.6875</v>
       </c>
       <c r="B68">
-        <v>796</v>
+        <v>941</v>
       </c>
     </row>
     <row r="69" spans="1:2">
       <c r="A69" s="2">
-        <v>46149.69791666666</v>
+        <v>46153.69791666666</v>
       </c>
       <c r="B69">
-        <v>801</v>
+        <v>950</v>
       </c>
     </row>
     <row r="70" spans="1:2">
       <c r="A70" s="2">
-        <v>46149.70833333334</v>
+        <v>46153.70833333334</v>
       </c>
       <c r="B70">
-        <v>877</v>
+        <v>1060</v>
       </c>
     </row>
     <row r="71" spans="1:2">
       <c r="A71" s="2">
-        <v>46149.71875</v>
+        <v>46153.71875</v>
       </c>
       <c r="B71">
-        <v>889</v>
+        <v>1070</v>
       </c>
     </row>
     <row r="72" spans="1:2">
       <c r="A72" s="2">
-        <v>46149.72916666666</v>
+        <v>46153.72916666666</v>
       </c>
       <c r="B72">
-        <v>884</v>
+        <v>1101</v>
       </c>
     </row>
     <row r="73" spans="1:2">
       <c r="A73" s="2">
-        <v>46149.73958333334</v>
+        <v>46153.73958333334</v>
       </c>
       <c r="B73">
-        <v>906</v>
+        <v>1109</v>
       </c>
     </row>
     <row r="74" spans="1:2">
       <c r="A74" s="2">
-        <v>46149.75</v>
+        <v>46153.75</v>
       </c>
       <c r="B74">
-        <v>1075</v>
+        <v>1244</v>
       </c>
     </row>
     <row r="75" spans="1:2">
       <c r="A75" s="2">
-        <v>46149.76041666666</v>
+        <v>46153.76041666666</v>
       </c>
       <c r="B75">
-        <v>1086</v>
+        <v>1252</v>
       </c>
     </row>
     <row r="76" spans="1:2">
       <c r="A76" s="2">
-        <v>46149.77083333334</v>
+        <v>46153.77083333334</v>
       </c>
       <c r="B76">
-        <v>1083</v>
+        <v>1257</v>
       </c>
     </row>
     <row r="77" spans="1:2">
       <c r="A77" s="2">
-        <v>46149.78125</v>
+        <v>46153.78125</v>
       </c>
       <c r="B77">
-        <v>1084</v>
+        <v>1259</v>
       </c>
     </row>
     <row r="78" spans="1:2">
       <c r="A78" s="2">
-        <v>46149.79166666666</v>
+        <v>46153.79166666666</v>
       </c>
       <c r="B78">
-        <v>1059</v>
+        <v>1250</v>
       </c>
     </row>
     <row r="79" spans="1:2">
       <c r="A79" s="2">
-        <v>46149.80208333334</v>
+        <v>46153.80208333334</v>
       </c>
       <c r="B79">
-        <v>1060</v>
+        <v>1258</v>
       </c>
     </row>
     <row r="80" spans="1:2">
       <c r="A80" s="2">
-        <v>46149.8125</v>
+        <v>46153.8125</v>
       </c>
       <c r="B80">
-        <v>1061</v>
+        <v>1254</v>
       </c>
     </row>
     <row r="81" spans="1:2">
       <c r="A81" s="2">
-        <v>46149.82291666666</v>
+        <v>46153.82291666666</v>
       </c>
       <c r="B81">
-        <v>1066</v>
+        <v>0</v>
       </c>
     </row>
     <row r="82" spans="1:2">
       <c r="A82" s="2">
-        <v>46149.83333333334</v>
+        <v>46153.83333333334</v>
       </c>
       <c r="B82">
-        <v>1092</v>
+        <v>1252</v>
       </c>
     </row>
     <row r="83" spans="1:2">
       <c r="A83" s="2">
-        <v>46149.84375</v>
+        <v>46153.84375</v>
       </c>
       <c r="B83">
-        <v>1093</v>
+        <v>1254</v>
       </c>
     </row>
     <row r="84" spans="1:2">
       <c r="A84" s="2">
-        <v>46149.85416666666</v>
+        <v>46153.85416666666</v>
       </c>
       <c r="B84">
-        <v>1092</v>
+        <v>1253</v>
       </c>
     </row>
     <row r="85" spans="1:2">
       <c r="A85" s="2">
-        <v>46149.86458333334</v>
+        <v>46153.86458333334</v>
       </c>
       <c r="B85">
-        <v>1090</v>
+        <v>0</v>
       </c>
     </row>
     <row r="86" spans="1:2">
       <c r="A86" s="2">
-        <v>46149.875</v>
+        <v>46153.875</v>
       </c>
       <c r="B86">
-        <v>1114</v>
+        <v>1235</v>
       </c>
     </row>
     <row r="87" spans="1:2">
       <c r="A87" s="2">
-        <v>46149.88541666666</v>
+        <v>46153.88541666666</v>
       </c>
       <c r="B87">
-        <v>1110</v>
+        <v>0</v>
       </c>
     </row>
     <row r="88" spans="1:2">
       <c r="A88" s="2">
-        <v>46149.89583333334</v>
+        <v>46153.89583333334</v>
       </c>
       <c r="B88">
-        <v>0</v>
+        <v>1234</v>
       </c>
     </row>
     <row r="89" spans="1:2">
       <c r="A89" s="2">
-        <v>46149.90625</v>
+        <v>46153.90625</v>
       </c>
       <c r="B89">
-        <v>1105</v>
+        <v>1230</v>
       </c>
     </row>
     <row r="90" spans="1:2">
       <c r="A90" s="2">
-        <v>46149.91666666666</v>
+        <v>46153.91666666666</v>
       </c>
       <c r="B90">
-        <v>937</v>
+        <v>1106</v>
       </c>
     </row>
     <row r="91" spans="1:2">
       <c r="A91" s="2">
-        <v>46149.92708333334</v>
+        <v>46153.92708333334</v>
       </c>
       <c r="B91">
-        <v>920</v>
+        <v>1079</v>
       </c>
     </row>
     <row r="92" spans="1:2">
       <c r="A92" s="2">
-        <v>46149.9375</v>
+        <v>46153.9375</v>
       </c>
       <c r="B92">
-        <v>923</v>
+        <v>0</v>
       </c>
     </row>
     <row r="93" spans="1:2">
       <c r="A93" s="2">
-        <v>46149.94791666666</v>
+        <v>46153.94791666666</v>
       </c>
       <c r="B93">
-        <v>921</v>
+        <v>1080</v>
       </c>
     </row>
     <row r="94" spans="1:2">
       <c r="A94" s="2">
-        <v>46149.95833333334</v>
+        <v>46153.95833333334</v>
       </c>
       <c r="B94">
-        <v>906</v>
+        <v>972</v>
       </c>
     </row>
     <row r="95" spans="1:2">
       <c r="A95" s="2">
-        <v>46149.96875</v>
+        <v>46153.96875</v>
       </c>
       <c r="B95">
-        <v>898</v>
+        <v>964</v>
       </c>
     </row>
     <row r="96" spans="1:2">
       <c r="A96" s="2">
-        <v>46149.97916666666</v>
+        <v>46153.97916666666</v>
       </c>
       <c r="B96">
-        <v>899</v>
+        <v>965</v>
       </c>
     </row>
     <row r="97" spans="1:2">
       <c r="A97" s="2">
-        <v>46149.98958333334</v>
+        <v>46153.98958333334</v>
       </c>
       <c r="B97">
-        <v>897</v>
+        <v>953</v>
       </c>
     </row>
     <row r="98" spans="1:2">
       <c r="A98" s="2">
-        <v>46150</v>
+        <v>46154</v>
       </c>
       <c r="B98">
-        <v>928</v>
+        <v>965</v>
       </c>
     </row>
     <row r="99" spans="1:2">
       <c r="A99" s="2">
-        <v>46150.01041666666</v>
+        <v>46154.01041666666</v>
       </c>
       <c r="B99">
-        <v>922</v>
+        <v>964</v>
       </c>
     </row>
     <row r="100" spans="1:2">
       <c r="A100" s="2">
-        <v>46150.02083333334</v>
+        <v>46154.02083333334</v>
       </c>
       <c r="B100">
-        <v>0</v>
+        <v>961</v>
       </c>
     </row>
     <row r="101" spans="1:2">
       <c r="A101" s="2">
-        <v>46150.03125</v>
+        <v>46154.03125</v>
       </c>
       <c r="B101">
-        <v>920</v>
+        <v>0</v>
       </c>
     </row>
     <row r="102" spans="1:2">
       <c r="A102" s="2">
-        <v>46150.04166666666</v>
+        <v>46154.04166666666</v>
       </c>
       <c r="B102">
-        <v>894</v>
+        <v>964</v>
       </c>
     </row>
     <row r="103" spans="1:2">
       <c r="A103" s="2">
-        <v>46150.05208333334</v>
+        <v>46154.05208333334</v>
       </c>
       <c r="B103">
-        <v>888</v>
+        <v>960</v>
       </c>
     </row>
     <row r="104" spans="1:2">
       <c r="A104" s="2">
-        <v>46150.0625</v>
+        <v>46154.0625</v>
       </c>
       <c r="B104">
-        <v>889</v>
+        <v>961</v>
       </c>
     </row>
     <row r="105" spans="1:2">
       <c r="A105" s="2">
-        <v>46150.07291666666</v>
+        <v>46154.07291666666</v>
       </c>
       <c r="B105">
-        <v>888</v>
+        <v>0</v>
       </c>
     </row>
     <row r="106" spans="1:2">
       <c r="A106" s="2">
-        <v>46150.08333333334</v>
+        <v>46154.08333333334</v>
       </c>
       <c r="B106">
-        <v>890</v>
+        <v>957</v>
       </c>
     </row>
     <row r="107" spans="1:2">
       <c r="A107" s="2">
-        <v>46150.09375</v>
+        <v>46154.09375</v>
       </c>
       <c r="B107">
-        <v>888</v>
+        <v>954</v>
       </c>
     </row>
     <row r="108" spans="1:2">
       <c r="A108" s="2">
-        <v>46150.10416666666</v>
+        <v>46154.10416666666</v>
       </c>
       <c r="B108">
-        <v>890</v>
+        <v>956</v>
       </c>
     </row>
     <row r="109" spans="1:2">
       <c r="A109" s="2">
-        <v>46150.11458333334</v>
+        <v>46154.11458333334</v>
       </c>
       <c r="B109">
-        <v>0</v>
+        <v>918</v>
       </c>
     </row>
     <row r="110" spans="1:2">
       <c r="A110" s="2">
-        <v>46150.125</v>
+        <v>46154.125</v>
       </c>
       <c r="B110">
-        <v>903</v>
+        <v>945</v>
       </c>
     </row>
     <row r="111" spans="1:2">
       <c r="A111" s="2">
-        <v>46150.13541666666</v>
+        <v>46154.13541666666</v>
       </c>
       <c r="B111">
-        <v>904</v>
+        <v>0</v>
       </c>
     </row>
     <row r="112" spans="1:2">
       <c r="A112" s="2">
-        <v>46150.14583333334</v>
+        <v>46154.14583333334</v>
       </c>
       <c r="B112">
-        <v>903</v>
+        <v>967</v>
       </c>
     </row>
     <row r="113" spans="1:2">
       <c r="A113" s="2">
-        <v>46150.15625</v>
+        <v>46154.15625</v>
       </c>
       <c r="B113">
         <v>0</v>
@@ -1290,215 +1290,215 @@
     </row>
     <row r="114" spans="1:2">
       <c r="A114" s="2">
-        <v>46150.16666666666</v>
+        <v>46154.16666666666</v>
       </c>
       <c r="B114">
-        <v>907</v>
+        <v>0</v>
       </c>
     </row>
     <row r="115" spans="1:2">
       <c r="A115" s="2">
-        <v>46150.17708333334</v>
+        <v>46154.17708333334</v>
       </c>
       <c r="B115">
-        <v>906</v>
+        <v>997</v>
       </c>
     </row>
     <row r="116" spans="1:2">
       <c r="A116" s="2">
-        <v>46150.1875</v>
+        <v>46154.1875</v>
       </c>
       <c r="B116">
-        <v>905</v>
+        <v>1022</v>
       </c>
     </row>
     <row r="117" spans="1:2">
       <c r="A117" s="2">
-        <v>46150.19791666666</v>
+        <v>46154.19791666666</v>
       </c>
       <c r="B117">
-        <v>903</v>
+        <v>1025</v>
       </c>
     </row>
     <row r="118" spans="1:2">
       <c r="A118" s="2">
-        <v>46150.20833333334</v>
+        <v>46154.20833333334</v>
       </c>
       <c r="B118">
-        <v>925</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="119" spans="1:2">
       <c r="A119" s="2">
-        <v>46150.21875</v>
+        <v>46154.21875</v>
       </c>
       <c r="B119">
-        <v>928</v>
+        <v>1033</v>
       </c>
     </row>
     <row r="120" spans="1:2">
       <c r="A120" s="2">
-        <v>46150.22916666666</v>
+        <v>46154.22916666666</v>
       </c>
       <c r="B120">
-        <v>0</v>
+        <v>1042</v>
       </c>
     </row>
     <row r="121" spans="1:2">
       <c r="A121" s="2">
-        <v>46150.23958333334</v>
+        <v>46154.23958333334</v>
       </c>
       <c r="B121">
-        <v>0</v>
+        <v>1043</v>
       </c>
     </row>
     <row r="122" spans="1:2">
       <c r="A122" s="2">
-        <v>46150.25</v>
+        <v>46154.25</v>
       </c>
       <c r="B122">
-        <v>950</v>
+        <v>1045</v>
       </c>
     </row>
     <row r="123" spans="1:2">
       <c r="A123" s="2">
-        <v>46150.26041666666</v>
+        <v>46154.26041666666</v>
       </c>
       <c r="B123">
-        <v>947</v>
+        <v>0</v>
       </c>
     </row>
     <row r="124" spans="1:2">
       <c r="A124" s="2">
-        <v>46150.27083333334</v>
+        <v>46154.27083333334</v>
       </c>
       <c r="B124">
-        <v>948</v>
+        <v>1053</v>
       </c>
     </row>
     <row r="125" spans="1:2">
       <c r="A125" s="2">
-        <v>46150.28125</v>
+        <v>46154.28125</v>
       </c>
       <c r="B125">
-        <v>953</v>
+        <v>1054</v>
       </c>
     </row>
     <row r="126" spans="1:2">
       <c r="A126" s="2">
-        <v>46150.29166666666</v>
+        <v>46154.29166666666</v>
       </c>
       <c r="B126">
-        <v>939</v>
+        <v>1022</v>
       </c>
     </row>
     <row r="127" spans="1:2">
       <c r="A127" s="2">
-        <v>46150.30208333334</v>
+        <v>46154.30208333334</v>
       </c>
       <c r="B127">
-        <v>935</v>
+        <v>1014</v>
       </c>
     </row>
     <row r="128" spans="1:2">
       <c r="A128" s="2">
-        <v>46150.3125</v>
+        <v>46154.3125</v>
       </c>
       <c r="B128">
-        <v>0</v>
+        <v>1023</v>
       </c>
     </row>
     <row r="129" spans="1:2">
       <c r="A129" s="2">
-        <v>46150.32291666666</v>
+        <v>46154.32291666666</v>
       </c>
       <c r="B129">
-        <v>0</v>
+        <v>974</v>
       </c>
     </row>
     <row r="130" spans="1:2">
       <c r="A130" s="2">
-        <v>46150.33333333334</v>
+        <v>46154.33333333334</v>
       </c>
       <c r="B130">
-        <v>0</v>
+        <v>863</v>
       </c>
     </row>
     <row r="131" spans="1:2">
       <c r="A131" s="2">
-        <v>46150.34375</v>
+        <v>46154.34375</v>
       </c>
       <c r="B131">
-        <v>0</v>
+        <v>852</v>
       </c>
     </row>
     <row r="132" spans="1:2">
       <c r="A132" s="2">
-        <v>46150.35416666666</v>
+        <v>46154.35416666666</v>
       </c>
       <c r="B132">
-        <v>0</v>
+        <v>952</v>
       </c>
     </row>
     <row r="133" spans="1:2">
       <c r="A133" s="2">
-        <v>46150.36458333334</v>
+        <v>46154.36458333334</v>
       </c>
       <c r="B133">
-        <v>0</v>
+        <v>975</v>
       </c>
     </row>
     <row r="134" spans="1:2">
       <c r="A134" s="2">
-        <v>46150.375</v>
+        <v>46154.375</v>
       </c>
       <c r="B134">
-        <v>0</v>
+        <v>1013</v>
       </c>
     </row>
     <row r="135" spans="1:2">
       <c r="A135" s="2">
-        <v>46150.38541666666</v>
+        <v>46154.38541666666</v>
       </c>
       <c r="B135">
-        <v>0</v>
+        <v>1222</v>
       </c>
     </row>
     <row r="136" spans="1:2">
       <c r="A136" s="2">
-        <v>46150.39583333334</v>
+        <v>46154.39583333334</v>
       </c>
       <c r="B136">
-        <v>0</v>
+        <v>1329</v>
       </c>
     </row>
     <row r="137" spans="1:2">
       <c r="A137" s="2">
-        <v>46150.40625</v>
+        <v>46154.40625</v>
       </c>
       <c r="B137">
-        <v>0</v>
+        <v>1342</v>
       </c>
     </row>
     <row r="138" spans="1:2">
       <c r="A138" s="2">
-        <v>46150.41666666666</v>
+        <v>46154.41666666666</v>
       </c>
       <c r="B138">
-        <v>0</v>
+        <v>1170</v>
       </c>
     </row>
     <row r="139" spans="1:2">
       <c r="A139" s="2">
-        <v>46150.42708333334</v>
+        <v>46154.42708333334</v>
       </c>
       <c r="B139">
-        <v>0</v>
+        <v>948</v>
       </c>
     </row>
     <row r="140" spans="1:2">
       <c r="A140" s="2">
-        <v>46150.4375</v>
+        <v>46154.4375</v>
       </c>
       <c r="B140">
         <v>0</v>
@@ -1506,7 +1506,7 @@
     </row>
     <row r="141" spans="1:2">
       <c r="A141" s="2">
-        <v>46150.44791666666</v>
+        <v>46154.44791666666</v>
       </c>
       <c r="B141">
         <v>0</v>
@@ -1514,7 +1514,7 @@
     </row>
     <row r="142" spans="1:2">
       <c r="A142" s="2">
-        <v>46150.45833333334</v>
+        <v>46154.45833333334</v>
       </c>
       <c r="B142">
         <v>0</v>
@@ -1522,7 +1522,7 @@
     </row>
     <row r="143" spans="1:2">
       <c r="A143" s="2">
-        <v>46150.46875</v>
+        <v>46154.46875</v>
       </c>
       <c r="B143">
         <v>0</v>
@@ -1530,7 +1530,7 @@
     </row>
     <row r="144" spans="1:2">
       <c r="A144" s="2">
-        <v>46150.47916666666</v>
+        <v>46154.47916666666</v>
       </c>
       <c r="B144">
         <v>0</v>
@@ -1538,7 +1538,7 @@
     </row>
     <row r="145" spans="1:2">
       <c r="A145" s="2">
-        <v>46150.48958333334</v>
+        <v>46154.48958333334</v>
       </c>
       <c r="B145">
         <v>0</v>
@@ -1546,7 +1546,7 @@
     </row>
     <row r="146" spans="1:2">
       <c r="A146" s="2">
-        <v>46150.5</v>
+        <v>46154.5</v>
       </c>
       <c r="B146">
         <v>0</v>
@@ -1554,7 +1554,7 @@
     </row>
     <row r="147" spans="1:2">
       <c r="A147" s="2">
-        <v>46150.51041666666</v>
+        <v>46154.51041666666</v>
       </c>
       <c r="B147">
         <v>0</v>
@@ -1562,7 +1562,7 @@
     </row>
     <row r="148" spans="1:2">
       <c r="A148" s="2">
-        <v>46150.52083333334</v>
+        <v>46154.52083333334</v>
       </c>
       <c r="B148">
         <v>0</v>
@@ -1570,7 +1570,7 @@
     </row>
     <row r="149" spans="1:2">
       <c r="A149" s="2">
-        <v>46150.53125</v>
+        <v>46154.53125</v>
       </c>
       <c r="B149">
         <v>0</v>
@@ -1578,7 +1578,7 @@
     </row>
     <row r="150" spans="1:2">
       <c r="A150" s="2">
-        <v>46150.54166666666</v>
+        <v>46154.54166666666</v>
       </c>
       <c r="B150">
         <v>0</v>
@@ -1586,7 +1586,7 @@
     </row>
     <row r="151" spans="1:2">
       <c r="A151" s="2">
-        <v>46150.55208333334</v>
+        <v>46154.55208333334</v>
       </c>
       <c r="B151">
         <v>0</v>
@@ -1594,7 +1594,7 @@
     </row>
     <row r="152" spans="1:2">
       <c r="A152" s="2">
-        <v>46150.5625</v>
+        <v>46154.5625</v>
       </c>
       <c r="B152">
         <v>0</v>
@@ -1602,7 +1602,7 @@
     </row>
     <row r="153" spans="1:2">
       <c r="A153" s="2">
-        <v>46150.57291666666</v>
+        <v>46154.57291666666</v>
       </c>
       <c r="B153">
         <v>0</v>
@@ -1610,7 +1610,7 @@
     </row>
     <row r="154" spans="1:2">
       <c r="A154" s="2">
-        <v>46150.58333333334</v>
+        <v>46154.58333333334</v>
       </c>
       <c r="B154">
         <v>0</v>
@@ -1618,7 +1618,7 @@
     </row>
     <row r="155" spans="1:2">
       <c r="A155" s="2">
-        <v>46150.59375</v>
+        <v>46154.59375</v>
       </c>
       <c r="B155">
         <v>0</v>
@@ -1626,7 +1626,7 @@
     </row>
     <row r="156" spans="1:2">
       <c r="A156" s="2">
-        <v>46150.60416666666</v>
+        <v>46154.60416666666</v>
       </c>
       <c r="B156">
         <v>0</v>
@@ -1634,7 +1634,7 @@
     </row>
     <row r="157" spans="1:2">
       <c r="A157" s="2">
-        <v>46150.61458333334</v>
+        <v>46154.61458333334</v>
       </c>
       <c r="B157">
         <v>0</v>
@@ -1642,7 +1642,7 @@
     </row>
     <row r="158" spans="1:2">
       <c r="A158" s="2">
-        <v>46150.625</v>
+        <v>46154.625</v>
       </c>
       <c r="B158">
         <v>0</v>
@@ -1650,7 +1650,7 @@
     </row>
     <row r="159" spans="1:2">
       <c r="A159" s="2">
-        <v>46150.63541666666</v>
+        <v>46154.63541666666</v>
       </c>
       <c r="B159">
         <v>0</v>
@@ -1658,7 +1658,7 @@
     </row>
     <row r="160" spans="1:2">
       <c r="A160" s="2">
-        <v>46150.64583333334</v>
+        <v>46154.64583333334</v>
       </c>
       <c r="B160">
         <v>0</v>
@@ -1666,7 +1666,7 @@
     </row>
     <row r="161" spans="1:2">
       <c r="A161" s="2">
-        <v>46150.65625</v>
+        <v>46154.65625</v>
       </c>
       <c r="B161">
         <v>0</v>
@@ -1674,7 +1674,7 @@
     </row>
     <row r="162" spans="1:2">
       <c r="A162" s="2">
-        <v>46150.66666666666</v>
+        <v>46154.66666666666</v>
       </c>
       <c r="B162">
         <v>0</v>
@@ -1682,7 +1682,7 @@
     </row>
     <row r="163" spans="1:2">
       <c r="A163" s="2">
-        <v>46150.67708333334</v>
+        <v>46154.67708333334</v>
       </c>
       <c r="B163">
         <v>0</v>
@@ -1690,7 +1690,7 @@
     </row>
     <row r="164" spans="1:2">
       <c r="A164" s="2">
-        <v>46150.6875</v>
+        <v>46154.6875</v>
       </c>
       <c r="B164">
         <v>0</v>
@@ -1698,7 +1698,7 @@
     </row>
     <row r="165" spans="1:2">
       <c r="A165" s="2">
-        <v>46150.69791666666</v>
+        <v>46154.69791666666</v>
       </c>
       <c r="B165">
         <v>0</v>
@@ -1706,7 +1706,7 @@
     </row>
     <row r="166" spans="1:2">
       <c r="A166" s="2">
-        <v>46150.70833333334</v>
+        <v>46154.70833333334</v>
       </c>
       <c r="B166">
         <v>0</v>
@@ -1714,7 +1714,7 @@
     </row>
     <row r="167" spans="1:2">
       <c r="A167" s="2">
-        <v>46150.71875</v>
+        <v>46154.71875</v>
       </c>
       <c r="B167">
         <v>0</v>
@@ -1722,7 +1722,7 @@
     </row>
     <row r="168" spans="1:2">
       <c r="A168" s="2">
-        <v>46150.72916666666</v>
+        <v>46154.72916666666</v>
       </c>
       <c r="B168">
         <v>0</v>
@@ -1730,7 +1730,7 @@
     </row>
     <row r="169" spans="1:2">
       <c r="A169" s="2">
-        <v>46150.73958333334</v>
+        <v>46154.73958333334</v>
       </c>
       <c r="B169">
         <v>0</v>
@@ -1738,7 +1738,7 @@
     </row>
     <row r="170" spans="1:2">
       <c r="A170" s="2">
-        <v>46150.75</v>
+        <v>46154.75</v>
       </c>
       <c r="B170">
         <v>0</v>
@@ -1746,7 +1746,7 @@
     </row>
     <row r="171" spans="1:2">
       <c r="A171" s="2">
-        <v>46150.76041666666</v>
+        <v>46154.76041666666</v>
       </c>
       <c r="B171">
         <v>0</v>
@@ -1754,7 +1754,7 @@
     </row>
     <row r="172" spans="1:2">
       <c r="A172" s="2">
-        <v>46150.77083333334</v>
+        <v>46154.77083333334</v>
       </c>
       <c r="B172">
         <v>0</v>
@@ -1762,7 +1762,7 @@
     </row>
     <row r="173" spans="1:2">
       <c r="A173" s="2">
-        <v>46150.78125</v>
+        <v>46154.78125</v>
       </c>
       <c r="B173">
         <v>0</v>
@@ -1770,7 +1770,7 @@
     </row>
     <row r="174" spans="1:2">
       <c r="A174" s="2">
-        <v>46150.79166666666</v>
+        <v>46154.79166666666</v>
       </c>
       <c r="B174">
         <v>0</v>
@@ -1778,7 +1778,7 @@
     </row>
     <row r="175" spans="1:2">
       <c r="A175" s="2">
-        <v>46150.80208333334</v>
+        <v>46154.80208333334</v>
       </c>
       <c r="B175">
         <v>0</v>
@@ -1786,7 +1786,7 @@
     </row>
     <row r="176" spans="1:2">
       <c r="A176" s="2">
-        <v>46150.8125</v>
+        <v>46154.8125</v>
       </c>
       <c r="B176">
         <v>0</v>
@@ -1794,7 +1794,7 @@
     </row>
     <row r="177" spans="1:2">
       <c r="A177" s="2">
-        <v>46150.82291666666</v>
+        <v>46154.82291666666</v>
       </c>
       <c r="B177">
         <v>0</v>
@@ -1802,7 +1802,7 @@
     </row>
     <row r="178" spans="1:2">
       <c r="A178" s="2">
-        <v>46150.83333333334</v>
+        <v>46154.83333333334</v>
       </c>
       <c r="B178">
         <v>0</v>
@@ -1810,7 +1810,7 @@
     </row>
     <row r="179" spans="1:2">
       <c r="A179" s="2">
-        <v>46150.84375</v>
+        <v>46154.84375</v>
       </c>
       <c r="B179">
         <v>0</v>
@@ -1818,7 +1818,7 @@
     </row>
     <row r="180" spans="1:2">
       <c r="A180" s="2">
-        <v>46150.85416666666</v>
+        <v>46154.85416666666</v>
       </c>
       <c r="B180">
         <v>0</v>
@@ -1826,7 +1826,7 @@
     </row>
     <row r="181" spans="1:2">
       <c r="A181" s="2">
-        <v>46150.86458333334</v>
+        <v>46154.86458333334</v>
       </c>
       <c r="B181">
         <v>0</v>
@@ -1834,7 +1834,7 @@
     </row>
     <row r="182" spans="1:2">
       <c r="A182" s="2">
-        <v>46150.875</v>
+        <v>46154.875</v>
       </c>
       <c r="B182">
         <v>0</v>
@@ -1842,7 +1842,7 @@
     </row>
     <row r="183" spans="1:2">
       <c r="A183" s="2">
-        <v>46150.88541666666</v>
+        <v>46154.88541666666</v>
       </c>
       <c r="B183">
         <v>0</v>
@@ -1850,7 +1850,7 @@
     </row>
     <row r="184" spans="1:2">
       <c r="A184" s="2">
-        <v>46150.89583333334</v>
+        <v>46154.89583333334</v>
       </c>
       <c r="B184">
         <v>0</v>
@@ -1858,7 +1858,7 @@
     </row>
     <row r="185" spans="1:2">
       <c r="A185" s="2">
-        <v>46150.90625</v>
+        <v>46154.90625</v>
       </c>
       <c r="B185">
         <v>0</v>
@@ -1866,7 +1866,7 @@
     </row>
     <row r="186" spans="1:2">
       <c r="A186" s="2">
-        <v>46150.91666666666</v>
+        <v>46154.91666666666</v>
       </c>
       <c r="B186">
         <v>0</v>
@@ -1874,7 +1874,7 @@
     </row>
     <row r="187" spans="1:2">
       <c r="A187" s="2">
-        <v>46150.92708333334</v>
+        <v>46154.92708333334</v>
       </c>
       <c r="B187">
         <v>0</v>
@@ -1882,7 +1882,7 @@
     </row>
     <row r="188" spans="1:2">
       <c r="A188" s="2">
-        <v>46150.9375</v>
+        <v>46154.9375</v>
       </c>
       <c r="B188">
         <v>0</v>
@@ -1890,7 +1890,7 @@
     </row>
     <row r="189" spans="1:2">
       <c r="A189" s="2">
-        <v>46150.94791666666</v>
+        <v>46154.94791666666</v>
       </c>
       <c r="B189">
         <v>0</v>
@@ -1898,7 +1898,7 @@
     </row>
     <row r="190" spans="1:2">
       <c r="A190" s="2">
-        <v>46150.95833333334</v>
+        <v>46154.95833333334</v>
       </c>
       <c r="B190">
         <v>0</v>
@@ -1906,7 +1906,7 @@
     </row>
     <row r="191" spans="1:2">
       <c r="A191" s="2">
-        <v>46150.96875</v>
+        <v>46154.96875</v>
       </c>
       <c r="B191">
         <v>0</v>
@@ -1914,7 +1914,7 @@
     </row>
     <row r="192" spans="1:2">
       <c r="A192" s="2">
-        <v>46150.97916666666</v>
+        <v>46154.97916666666</v>
       </c>
       <c r="B192">
         <v>0</v>
@@ -1922,7 +1922,7 @@
     </row>
     <row r="193" spans="1:2">
       <c r="A193" s="2">
-        <v>46150.98958333334</v>
+        <v>46154.98958333334</v>
       </c>
       <c r="B193">
         <v>0</v>

</xml_diff>

<commit_message>
Updating the models for Adrem and MM&MV)
</commit_message>
<xml_diff>
--- a/data_fetching/Entsoe/Actual_Production_Hydro_River.xlsx
+++ b/data_fetching/Entsoe/Actual_Production_Hydro_River.xlsx
@@ -381,7 +381,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B141"/>
+  <dimension ref="A1:B340"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:2">
@@ -394,87 +394,87 @@
     </row>
     <row r="2" spans="1:2">
       <c r="A2" s="2">
-        <v>46212</v>
+        <v>46213</v>
       </c>
       <c r="B2">
-        <v>589</v>
+        <v>625</v>
       </c>
     </row>
     <row r="3" spans="1:2">
       <c r="A3" s="2">
-        <v>46212.01041666666</v>
+        <v>46213.01041666666</v>
       </c>
       <c r="B3">
-        <v>587</v>
+        <v>617</v>
       </c>
     </row>
     <row r="4" spans="1:2">
       <c r="A4" s="2">
-        <v>46212.02083333334</v>
+        <v>46213.02083333334</v>
       </c>
       <c r="B4">
-        <v>587</v>
+        <v>616</v>
       </c>
     </row>
     <row r="5" spans="1:2">
       <c r="A5" s="2">
-        <v>46212.03125</v>
+        <v>46213.03125</v>
       </c>
       <c r="B5">
-        <v>586</v>
+        <v>615</v>
       </c>
     </row>
     <row r="6" spans="1:2">
       <c r="A6" s="2">
-        <v>46212.04166666666</v>
+        <v>46213.04166666666</v>
       </c>
       <c r="B6">
-        <v>557</v>
+        <v>536</v>
       </c>
     </row>
     <row r="7" spans="1:2">
       <c r="A7" s="2">
-        <v>46212.05208333334</v>
+        <v>46213.05208333334</v>
       </c>
       <c r="B7">
-        <v>554</v>
+        <v>532</v>
       </c>
     </row>
     <row r="8" spans="1:2">
       <c r="A8" s="2">
-        <v>46212.0625</v>
+        <v>46213.0625</v>
       </c>
       <c r="B8">
-        <v>554</v>
+        <v>532</v>
       </c>
     </row>
     <row r="9" spans="1:2">
       <c r="A9" s="2">
-        <v>46212.07291666666</v>
+        <v>46213.07291666666</v>
       </c>
       <c r="B9">
-        <v>554</v>
+        <v>510</v>
       </c>
     </row>
     <row r="10" spans="1:2">
       <c r="A10" s="2">
-        <v>46212.08333333334</v>
+        <v>46213.08333333334</v>
       </c>
       <c r="B10">
-        <v>499</v>
+        <v>491</v>
       </c>
     </row>
     <row r="11" spans="1:2">
       <c r="A11" s="2">
-        <v>46212.09375</v>
+        <v>46213.09375</v>
       </c>
       <c r="B11">
-        <v>494</v>
+        <v>493</v>
       </c>
     </row>
     <row r="12" spans="1:2">
       <c r="A12" s="2">
-        <v>46212.10416666666</v>
+        <v>46213.10416666666</v>
       </c>
       <c r="B12">
         <v>493</v>
@@ -482,7 +482,7 @@
     </row>
     <row r="13" spans="1:2">
       <c r="A13" s="2">
-        <v>46212.11458333334</v>
+        <v>46213.11458333334</v>
       </c>
       <c r="B13">
         <v>493</v>
@@ -490,1026 +490,2618 @@
     </row>
     <row r="14" spans="1:2">
       <c r="A14" s="2">
-        <v>46212.125</v>
+        <v>46213.125</v>
       </c>
       <c r="B14">
-        <v>464</v>
+        <v>478</v>
       </c>
     </row>
     <row r="15" spans="1:2">
       <c r="A15" s="2">
-        <v>46212.13541666666</v>
+        <v>46213.13541666666</v>
       </c>
       <c r="B15">
-        <v>473</v>
+        <v>478</v>
       </c>
     </row>
     <row r="16" spans="1:2">
       <c r="A16" s="2">
-        <v>46212.14583333334</v>
+        <v>46213.14583333334</v>
       </c>
       <c r="B16">
-        <v>472</v>
+        <v>478</v>
       </c>
     </row>
     <row r="17" spans="1:2">
       <c r="A17" s="2">
-        <v>46212.15625</v>
+        <v>46213.15625</v>
       </c>
       <c r="B17">
-        <v>473</v>
+        <v>478</v>
       </c>
     </row>
     <row r="18" spans="1:2">
       <c r="A18" s="2">
-        <v>46212.16666666666</v>
+        <v>46213.16666666666</v>
       </c>
       <c r="B18">
-        <v>512</v>
+        <v>505</v>
       </c>
     </row>
     <row r="19" spans="1:2">
       <c r="A19" s="2">
-        <v>46212.17708333334</v>
+        <v>46213.17708333334</v>
       </c>
       <c r="B19">
-        <v>514</v>
+        <v>509</v>
       </c>
     </row>
     <row r="20" spans="1:2">
       <c r="A20" s="2">
-        <v>46212.1875</v>
+        <v>46213.1875</v>
       </c>
       <c r="B20">
-        <v>513</v>
+        <v>509</v>
       </c>
     </row>
     <row r="21" spans="1:2">
       <c r="A21" s="2">
-        <v>46212.19791666666</v>
+        <v>46213.19791666666</v>
       </c>
       <c r="B21">
-        <v>516</v>
+        <v>513</v>
       </c>
     </row>
     <row r="22" spans="1:2">
       <c r="A22" s="2">
-        <v>46212.20833333334</v>
+        <v>46213.20833333334</v>
       </c>
       <c r="B22">
-        <v>584</v>
+        <v>604</v>
       </c>
     </row>
     <row r="23" spans="1:2">
       <c r="A23" s="2">
-        <v>46212.21875</v>
+        <v>46213.21875</v>
       </c>
       <c r="B23">
-        <v>592</v>
+        <v>613</v>
       </c>
     </row>
     <row r="24" spans="1:2">
       <c r="A24" s="2">
-        <v>46212.22916666666</v>
+        <v>46213.22916666666</v>
       </c>
       <c r="B24">
-        <v>600</v>
+        <v>609</v>
       </c>
     </row>
     <row r="25" spans="1:2">
       <c r="A25" s="2">
-        <v>46212.23958333334</v>
+        <v>46213.23958333334</v>
       </c>
       <c r="B25">
-        <v>602</v>
+        <v>615</v>
       </c>
     </row>
     <row r="26" spans="1:2">
       <c r="A26" s="2">
-        <v>46212.25</v>
+        <v>46213.25</v>
       </c>
       <c r="B26">
-        <v>724</v>
+        <v>788</v>
       </c>
     </row>
     <row r="27" spans="1:2">
       <c r="A27" s="2">
-        <v>46212.26041666666</v>
+        <v>46213.26041666666</v>
       </c>
       <c r="B27">
-        <v>729</v>
+        <v>810</v>
       </c>
     </row>
     <row r="28" spans="1:2">
       <c r="A28" s="2">
-        <v>46212.27083333334</v>
+        <v>46213.27083333334</v>
       </c>
       <c r="B28">
-        <v>729</v>
+        <v>812</v>
       </c>
     </row>
     <row r="29" spans="1:2">
       <c r="A29" s="2">
-        <v>46212.28125</v>
+        <v>46213.28125</v>
       </c>
       <c r="B29">
-        <v>729</v>
+        <v>812</v>
       </c>
     </row>
     <row r="30" spans="1:2">
       <c r="A30" s="2">
-        <v>46212.29166666666</v>
+        <v>46213.29166666666</v>
       </c>
       <c r="B30">
-        <v>712</v>
+        <v>840</v>
       </c>
     </row>
     <row r="31" spans="1:2">
       <c r="A31" s="2">
-        <v>46212.30208333334</v>
+        <v>46213.30208333334</v>
       </c>
       <c r="B31">
-        <v>711</v>
+        <v>841</v>
       </c>
     </row>
     <row r="32" spans="1:2">
       <c r="A32" s="2">
-        <v>46212.3125</v>
+        <v>46213.3125</v>
       </c>
       <c r="B32">
-        <v>703</v>
+        <v>852</v>
       </c>
     </row>
     <row r="33" spans="1:2">
       <c r="A33" s="2">
-        <v>46212.32291666666</v>
+        <v>46213.32291666666</v>
       </c>
       <c r="B33">
-        <v>701</v>
+        <v>848</v>
       </c>
     </row>
     <row r="34" spans="1:2">
       <c r="A34" s="2">
-        <v>46212.33333333334</v>
+        <v>46213.33333333334</v>
       </c>
       <c r="B34">
-        <v>717</v>
+        <v>812</v>
       </c>
     </row>
     <row r="35" spans="1:2">
       <c r="A35" s="2">
-        <v>46212.34375</v>
+        <v>46213.34375</v>
       </c>
       <c r="B35">
-        <v>718</v>
+        <v>813</v>
       </c>
     </row>
     <row r="36" spans="1:2">
       <c r="A36" s="2">
-        <v>46212.35416666666</v>
+        <v>46213.35416666666</v>
       </c>
       <c r="B36">
-        <v>706</v>
+        <v>807</v>
       </c>
     </row>
     <row r="37" spans="1:2">
       <c r="A37" s="2">
-        <v>46212.36458333334</v>
+        <v>46213.36458333334</v>
       </c>
       <c r="B37">
-        <v>705</v>
+        <v>811</v>
       </c>
     </row>
     <row r="38" spans="1:2">
       <c r="A38" s="2">
-        <v>46212.375</v>
+        <v>46213.375</v>
       </c>
       <c r="B38">
-        <v>713</v>
+        <v>669</v>
       </c>
     </row>
     <row r="39" spans="1:2">
       <c r="A39" s="2">
-        <v>46212.38541666666</v>
+        <v>46213.38541666666</v>
       </c>
       <c r="B39">
-        <v>686</v>
+        <v>661</v>
       </c>
     </row>
     <row r="40" spans="1:2">
       <c r="A40" s="2">
-        <v>46212.39583333334</v>
+        <v>46213.39583333334</v>
       </c>
       <c r="B40">
-        <v>729</v>
+        <v>660</v>
       </c>
     </row>
     <row r="41" spans="1:2">
       <c r="A41" s="2">
-        <v>46212.40625</v>
+        <v>46213.40625</v>
       </c>
       <c r="B41">
-        <v>734</v>
+        <v>661</v>
       </c>
     </row>
     <row r="42" spans="1:2">
       <c r="A42" s="2">
-        <v>46212.41666666666</v>
+        <v>46213.41666666666</v>
       </c>
       <c r="B42">
-        <v>579</v>
+        <v>652</v>
       </c>
     </row>
     <row r="43" spans="1:2">
       <c r="A43" s="2">
-        <v>46212.42708333334</v>
+        <v>46213.42708333334</v>
       </c>
       <c r="B43">
-        <v>603</v>
+        <v>614</v>
       </c>
     </row>
     <row r="44" spans="1:2">
       <c r="A44" s="2">
-        <v>46212.4375</v>
+        <v>46213.4375</v>
       </c>
       <c r="B44">
-        <v>614</v>
+        <v>618</v>
       </c>
     </row>
     <row r="45" spans="1:2">
       <c r="A45" s="2">
-        <v>46212.44791666666</v>
+        <v>46213.44791666666</v>
       </c>
       <c r="B45">
-        <v>611</v>
+        <v>615</v>
       </c>
     </row>
     <row r="46" spans="1:2">
       <c r="A46" s="2">
-        <v>46212.45833333334</v>
+        <v>46213.45833333334</v>
       </c>
       <c r="B46">
-        <v>653</v>
+        <v>561</v>
       </c>
     </row>
     <row r="47" spans="1:2">
       <c r="A47" s="2">
-        <v>46212.46875</v>
+        <v>46213.46875</v>
       </c>
       <c r="B47">
-        <v>640</v>
+        <v>609</v>
       </c>
     </row>
     <row r="48" spans="1:2">
       <c r="A48" s="2">
-        <v>46212.47916666666</v>
+        <v>46213.47916666666</v>
       </c>
       <c r="B48">
-        <v>630</v>
+        <v>613</v>
       </c>
     </row>
     <row r="49" spans="1:2">
       <c r="A49" s="2">
-        <v>46212.48958333334</v>
+        <v>46213.48958333334</v>
       </c>
       <c r="B49">
-        <v>643</v>
+        <v>604</v>
       </c>
     </row>
     <row r="50" spans="1:2">
       <c r="A50" s="2">
-        <v>46212.5</v>
+        <v>46213.5</v>
       </c>
       <c r="B50">
-        <v>551</v>
+        <v>389</v>
       </c>
     </row>
     <row r="51" spans="1:2">
       <c r="A51" s="2">
-        <v>46212.51041666666</v>
+        <v>46213.51041666666</v>
       </c>
       <c r="B51">
-        <v>545</v>
+        <v>376</v>
       </c>
     </row>
     <row r="52" spans="1:2">
       <c r="A52" s="2">
-        <v>46212.52083333334</v>
+        <v>46213.52083333334</v>
       </c>
       <c r="B52">
-        <v>536</v>
+        <v>439</v>
       </c>
     </row>
     <row r="53" spans="1:2">
       <c r="A53" s="2">
-        <v>46212.53125</v>
+        <v>46213.53125</v>
       </c>
       <c r="B53">
-        <v>541</v>
+        <v>443</v>
       </c>
     </row>
     <row r="54" spans="1:2">
       <c r="A54" s="2">
-        <v>46212.54166666666</v>
+        <v>46213.54166666666</v>
       </c>
       <c r="B54">
-        <v>362</v>
+        <v>439</v>
       </c>
     </row>
     <row r="55" spans="1:2">
       <c r="A55" s="2">
-        <v>46212.55208333334</v>
+        <v>46213.55208333334</v>
       </c>
       <c r="B55">
-        <v>350</v>
+        <v>448</v>
       </c>
     </row>
     <row r="56" spans="1:2">
       <c r="A56" s="2">
-        <v>46212.5625</v>
+        <v>46213.5625</v>
       </c>
       <c r="B56">
-        <v>350</v>
+        <v>518</v>
       </c>
     </row>
     <row r="57" spans="1:2">
       <c r="A57" s="2">
-        <v>46212.57291666666</v>
+        <v>46213.57291666666</v>
       </c>
       <c r="B57">
-        <v>356</v>
+        <v>529</v>
       </c>
     </row>
     <row r="58" spans="1:2">
       <c r="A58" s="2">
-        <v>46212.58333333334</v>
+        <v>46213.58333333334</v>
       </c>
       <c r="B58">
-        <v>367</v>
+        <v>632</v>
       </c>
     </row>
     <row r="59" spans="1:2">
       <c r="A59" s="2">
-        <v>46212.59375</v>
+        <v>46213.59375</v>
       </c>
       <c r="B59">
-        <v>367</v>
+        <v>619</v>
       </c>
     </row>
     <row r="60" spans="1:2">
       <c r="A60" s="2">
-        <v>46212.60416666666</v>
+        <v>46213.60416666666</v>
       </c>
       <c r="B60">
-        <v>367</v>
+        <v>451</v>
       </c>
     </row>
     <row r="61" spans="1:2">
       <c r="A61" s="2">
-        <v>46212.61458333334</v>
+        <v>46213.61458333334</v>
       </c>
       <c r="B61">
-        <v>376</v>
+        <v>422</v>
       </c>
     </row>
     <row r="62" spans="1:2">
       <c r="A62" s="2">
-        <v>46212.625</v>
+        <v>46213.625</v>
       </c>
       <c r="B62">
-        <v>574</v>
+        <v>504</v>
       </c>
     </row>
     <row r="63" spans="1:2">
       <c r="A63" s="2">
-        <v>46212.63541666666</v>
+        <v>46213.63541666666</v>
       </c>
       <c r="B63">
-        <v>578</v>
+        <v>511</v>
       </c>
     </row>
     <row r="64" spans="1:2">
       <c r="A64" s="2">
-        <v>46212.64583333334</v>
+        <v>46213.64583333334</v>
       </c>
       <c r="B64">
-        <v>582</v>
+        <v>511</v>
       </c>
     </row>
     <row r="65" spans="1:2">
       <c r="A65" s="2">
-        <v>46212.65625</v>
+        <v>46213.65625</v>
       </c>
       <c r="B65">
-        <v>583</v>
+        <v>514</v>
       </c>
     </row>
     <row r="66" spans="1:2">
       <c r="A66" s="2">
-        <v>46212.66666666666</v>
+        <v>46213.66666666666</v>
       </c>
       <c r="B66">
-        <v>751</v>
+        <v>662</v>
       </c>
     </row>
     <row r="67" spans="1:2">
       <c r="A67" s="2">
-        <v>46212.67708333334</v>
+        <v>46213.67708333334</v>
       </c>
       <c r="B67">
-        <v>810</v>
+        <v>693</v>
       </c>
     </row>
     <row r="68" spans="1:2">
       <c r="A68" s="2">
-        <v>46212.6875</v>
+        <v>46213.6875</v>
       </c>
       <c r="B68">
-        <v>798</v>
+        <v>692</v>
       </c>
     </row>
     <row r="69" spans="1:2">
       <c r="A69" s="2">
-        <v>46212.69791666666</v>
+        <v>46213.69791666666</v>
       </c>
       <c r="B69">
-        <v>816</v>
+        <v>691</v>
       </c>
     </row>
     <row r="70" spans="1:2">
       <c r="A70" s="2">
-        <v>46212.70833333334</v>
+        <v>46213.70833333334</v>
       </c>
       <c r="B70">
-        <v>847</v>
+        <v>771</v>
       </c>
     </row>
     <row r="71" spans="1:2">
       <c r="A71" s="2">
-        <v>46212.71875</v>
+        <v>46213.71875</v>
       </c>
       <c r="B71">
-        <v>891</v>
+        <v>787</v>
       </c>
     </row>
     <row r="72" spans="1:2">
       <c r="A72" s="2">
-        <v>46212.72916666666</v>
+        <v>46213.72916666666</v>
       </c>
       <c r="B72">
-        <v>915</v>
+        <v>786</v>
       </c>
     </row>
     <row r="73" spans="1:2">
       <c r="A73" s="2">
-        <v>46212.73958333334</v>
+        <v>46213.73958333334</v>
       </c>
       <c r="B73">
-        <v>915</v>
+        <v>787</v>
       </c>
     </row>
     <row r="74" spans="1:2">
       <c r="A74" s="2">
-        <v>46212.75</v>
+        <v>46213.75</v>
       </c>
       <c r="B74">
-        <v>917</v>
+        <v>807</v>
       </c>
     </row>
     <row r="75" spans="1:2">
       <c r="A75" s="2">
-        <v>46212.76041666666</v>
+        <v>46213.76041666666</v>
       </c>
       <c r="B75">
-        <v>896</v>
+        <v>815</v>
       </c>
     </row>
     <row r="76" spans="1:2">
       <c r="A76" s="2">
-        <v>46212.77083333334</v>
+        <v>46213.77083333334</v>
       </c>
       <c r="B76">
-        <v>895</v>
+        <v>814</v>
       </c>
     </row>
     <row r="77" spans="1:2">
       <c r="A77" s="2">
-        <v>46212.78125</v>
+        <v>46213.78125</v>
       </c>
       <c r="B77">
-        <v>898</v>
+        <v>810</v>
       </c>
     </row>
     <row r="78" spans="1:2">
       <c r="A78" s="2">
-        <v>46212.79166666666</v>
+        <v>46213.79166666666</v>
       </c>
       <c r="B78">
-        <v>802</v>
+        <v>806</v>
       </c>
     </row>
     <row r="79" spans="1:2">
       <c r="A79" s="2">
-        <v>46212.80208333334</v>
+        <v>46213.80208333334</v>
       </c>
       <c r="B79">
-        <v>797</v>
+        <v>807</v>
       </c>
     </row>
     <row r="80" spans="1:2">
       <c r="A80" s="2">
-        <v>46212.8125</v>
+        <v>46213.8125</v>
       </c>
       <c r="B80">
-        <v>802</v>
+        <v>809</v>
       </c>
     </row>
     <row r="81" spans="1:2">
       <c r="A81" s="2">
-        <v>46212.82291666666</v>
+        <v>46213.82291666666</v>
       </c>
       <c r="B81">
-        <v>803</v>
+        <v>812</v>
       </c>
     </row>
     <row r="82" spans="1:2">
       <c r="A82" s="2">
-        <v>46212.83333333334</v>
+        <v>46213.83333333334</v>
       </c>
       <c r="B82">
-        <v>794</v>
+        <v>814</v>
       </c>
     </row>
     <row r="83" spans="1:2">
       <c r="A83" s="2">
-        <v>46212.84375</v>
+        <v>46213.84375</v>
       </c>
       <c r="B83">
-        <v>794</v>
+        <v>814</v>
       </c>
     </row>
     <row r="84" spans="1:2">
       <c r="A84" s="2">
-        <v>46212.85416666666</v>
+        <v>46213.85416666666</v>
       </c>
       <c r="B84">
-        <v>791</v>
+        <v>817</v>
       </c>
     </row>
     <row r="85" spans="1:2">
       <c r="A85" s="2">
-        <v>46212.86458333334</v>
+        <v>46213.86458333334</v>
       </c>
       <c r="B85">
-        <v>788</v>
+        <v>819</v>
       </c>
     </row>
     <row r="86" spans="1:2">
       <c r="A86" s="2">
-        <v>46212.875</v>
+        <v>46213.875</v>
       </c>
       <c r="B86">
-        <v>758</v>
+        <v>822</v>
       </c>
     </row>
     <row r="87" spans="1:2">
       <c r="A87" s="2">
-        <v>46212.88541666666</v>
+        <v>46213.88541666666</v>
       </c>
       <c r="B87">
-        <v>786</v>
+        <v>820</v>
       </c>
     </row>
     <row r="88" spans="1:2">
       <c r="A88" s="2">
-        <v>46212.89583333334</v>
+        <v>46213.89583333334</v>
       </c>
       <c r="B88">
-        <v>806</v>
+        <v>832</v>
       </c>
     </row>
     <row r="89" spans="1:2">
       <c r="A89" s="2">
-        <v>46212.90625</v>
+        <v>46213.90625</v>
       </c>
       <c r="B89">
-        <v>791</v>
+        <v>834</v>
       </c>
     </row>
     <row r="90" spans="1:2">
       <c r="A90" s="2">
-        <v>46212.91666666666</v>
+        <v>46213.91666666666</v>
       </c>
       <c r="B90">
-        <v>771</v>
+        <v>814</v>
       </c>
     </row>
     <row r="91" spans="1:2">
       <c r="A91" s="2">
-        <v>46212.92708333334</v>
+        <v>46213.92708333334</v>
       </c>
       <c r="B91">
-        <v>780</v>
+        <v>807</v>
       </c>
     </row>
     <row r="92" spans="1:2">
       <c r="A92" s="2">
-        <v>46212.9375</v>
+        <v>46213.9375</v>
       </c>
       <c r="B92">
-        <v>777</v>
+        <v>808</v>
       </c>
     </row>
     <row r="93" spans="1:2">
       <c r="A93" s="2">
-        <v>46212.94791666666</v>
+        <v>46213.94791666666</v>
       </c>
       <c r="B93">
-        <v>780</v>
+        <v>808</v>
       </c>
     </row>
     <row r="94" spans="1:2">
       <c r="A94" s="2">
-        <v>46212.95833333334</v>
+        <v>46213.95833333334</v>
       </c>
       <c r="B94">
-        <v>744</v>
+        <v>816</v>
       </c>
     </row>
     <row r="95" spans="1:2">
       <c r="A95" s="2">
-        <v>46212.96875</v>
+        <v>46213.96875</v>
       </c>
       <c r="B95">
-        <v>746</v>
+        <v>817</v>
       </c>
     </row>
     <row r="96" spans="1:2">
       <c r="A96" s="2">
-        <v>46212.97916666666</v>
+        <v>46213.97916666666</v>
       </c>
       <c r="B96">
-        <v>753</v>
+        <v>818</v>
       </c>
     </row>
     <row r="97" spans="1:2">
       <c r="A97" s="2">
-        <v>46212.98958333334</v>
+        <v>46213.98958333334</v>
       </c>
       <c r="B97">
-        <v>755</v>
+        <v>815</v>
       </c>
     </row>
     <row r="98" spans="1:2">
       <c r="A98" s="2">
-        <v>46213</v>
+        <v>46214</v>
       </c>
       <c r="B98">
-        <v>625</v>
+        <v>810</v>
       </c>
     </row>
     <row r="99" spans="1:2">
       <c r="A99" s="2">
-        <v>46213.01041666666</v>
+        <v>46214.01041666666</v>
       </c>
       <c r="B99">
-        <v>617</v>
+        <v>807</v>
       </c>
     </row>
     <row r="100" spans="1:2">
       <c r="A100" s="2">
-        <v>46213.02083333334</v>
+        <v>46214.02083333334</v>
       </c>
       <c r="B100">
-        <v>616</v>
+        <v>806</v>
       </c>
     </row>
     <row r="101" spans="1:2">
       <c r="A101" s="2">
-        <v>46213.03125</v>
+        <v>46214.03125</v>
       </c>
       <c r="B101">
-        <v>615</v>
+        <v>805</v>
       </c>
     </row>
     <row r="102" spans="1:2">
       <c r="A102" s="2">
-        <v>46213.04166666666</v>
+        <v>46214.04166666666</v>
       </c>
       <c r="B102">
-        <v>536</v>
+        <v>810</v>
       </c>
     </row>
     <row r="103" spans="1:2">
       <c r="A103" s="2">
-        <v>46213.05208333334</v>
+        <v>46214.05208333334</v>
       </c>
       <c r="B103">
-        <v>532</v>
+        <v>806</v>
       </c>
     </row>
     <row r="104" spans="1:2">
       <c r="A104" s="2">
-        <v>46213.0625</v>
+        <v>46214.0625</v>
       </c>
       <c r="B104">
-        <v>532</v>
+        <v>805</v>
       </c>
     </row>
     <row r="105" spans="1:2">
       <c r="A105" s="2">
-        <v>46213.07291666666</v>
+        <v>46214.07291666666</v>
       </c>
       <c r="B105">
-        <v>510</v>
+        <v>805</v>
       </c>
     </row>
     <row r="106" spans="1:2">
       <c r="A106" s="2">
-        <v>46213.08333333334</v>
+        <v>46214.08333333334</v>
       </c>
       <c r="B106">
-        <v>491</v>
+        <v>775</v>
       </c>
     </row>
     <row r="107" spans="1:2">
       <c r="A107" s="2">
-        <v>46213.09375</v>
+        <v>46214.09375</v>
       </c>
       <c r="B107">
-        <v>493</v>
+        <v>771</v>
       </c>
     </row>
     <row r="108" spans="1:2">
       <c r="A108" s="2">
-        <v>46213.10416666666</v>
+        <v>46214.10416666666</v>
       </c>
       <c r="B108">
-        <v>493</v>
+        <v>767</v>
       </c>
     </row>
     <row r="109" spans="1:2">
       <c r="A109" s="2">
-        <v>46213.11458333334</v>
+        <v>46214.11458333334</v>
       </c>
       <c r="B109">
-        <v>493</v>
+        <v>768</v>
       </c>
     </row>
     <row r="110" spans="1:2">
       <c r="A110" s="2">
-        <v>46213.125</v>
+        <v>46214.125</v>
       </c>
       <c r="B110">
-        <v>478</v>
+        <v>770</v>
       </c>
     </row>
     <row r="111" spans="1:2">
       <c r="A111" s="2">
-        <v>46213.13541666666</v>
+        <v>46214.13541666666</v>
       </c>
       <c r="B111">
-        <v>478</v>
+        <v>767</v>
       </c>
     </row>
     <row r="112" spans="1:2">
       <c r="A112" s="2">
-        <v>46213.14583333334</v>
+        <v>46214.14583333334</v>
       </c>
       <c r="B112">
-        <v>478</v>
+        <v>767</v>
       </c>
     </row>
     <row r="113" spans="1:2">
       <c r="A113" s="2">
-        <v>46213.15625</v>
+        <v>46214.15625</v>
       </c>
       <c r="B113">
-        <v>478</v>
+        <v>768</v>
       </c>
     </row>
     <row r="114" spans="1:2">
       <c r="A114" s="2">
-        <v>46213.16666666666</v>
+        <v>46214.16666666666</v>
       </c>
       <c r="B114">
-        <v>505</v>
+        <v>771</v>
       </c>
     </row>
     <row r="115" spans="1:2">
       <c r="A115" s="2">
-        <v>46213.17708333334</v>
+        <v>46214.17708333334</v>
       </c>
       <c r="B115">
-        <v>509</v>
+        <v>771</v>
       </c>
     </row>
     <row r="116" spans="1:2">
       <c r="A116" s="2">
-        <v>46213.1875</v>
+        <v>46214.1875</v>
       </c>
       <c r="B116">
-        <v>509</v>
+        <v>772</v>
       </c>
     </row>
     <row r="117" spans="1:2">
       <c r="A117" s="2">
-        <v>46213.19791666666</v>
+        <v>46214.19791666666</v>
       </c>
       <c r="B117">
-        <v>513</v>
+        <v>780</v>
       </c>
     </row>
     <row r="118" spans="1:2">
       <c r="A118" s="2">
-        <v>46213.20833333334</v>
+        <v>46214.20833333334</v>
       </c>
       <c r="B118">
-        <v>604</v>
+        <v>806</v>
       </c>
     </row>
     <row r="119" spans="1:2">
       <c r="A119" s="2">
-        <v>46213.21875</v>
+        <v>46214.21875</v>
       </c>
       <c r="B119">
-        <v>613</v>
+        <v>808</v>
       </c>
     </row>
     <row r="120" spans="1:2">
       <c r="A120" s="2">
-        <v>46213.22916666666</v>
+        <v>46214.22916666666</v>
       </c>
       <c r="B120">
-        <v>609</v>
+        <v>807</v>
       </c>
     </row>
     <row r="121" spans="1:2">
       <c r="A121" s="2">
-        <v>46213.23958333334</v>
+        <v>46214.23958333334</v>
       </c>
       <c r="B121">
-        <v>615</v>
+        <v>809</v>
       </c>
     </row>
     <row r="122" spans="1:2">
       <c r="A122" s="2">
-        <v>46213.25</v>
+        <v>46214.25</v>
       </c>
       <c r="B122">
-        <v>788</v>
+        <v>910</v>
       </c>
     </row>
     <row r="123" spans="1:2">
       <c r="A123" s="2">
-        <v>46213.26041666666</v>
+        <v>46214.26041666666</v>
       </c>
       <c r="B123">
-        <v>810</v>
+        <v>910</v>
       </c>
     </row>
     <row r="124" spans="1:2">
       <c r="A124" s="2">
-        <v>46213.27083333334</v>
+        <v>46214.27083333334</v>
       </c>
       <c r="B124">
-        <v>812</v>
+        <v>908</v>
       </c>
     </row>
     <row r="125" spans="1:2">
       <c r="A125" s="2">
-        <v>46213.28125</v>
+        <v>46214.28125</v>
       </c>
       <c r="B125">
-        <v>812</v>
+        <v>917</v>
       </c>
     </row>
     <row r="126" spans="1:2">
       <c r="A126" s="2">
-        <v>46213.29166666666</v>
+        <v>46214.29166666666</v>
       </c>
       <c r="B126">
-        <v>840</v>
+        <v>891</v>
       </c>
     </row>
     <row r="127" spans="1:2">
       <c r="A127" s="2">
-        <v>46213.30208333334</v>
+        <v>46214.30208333334</v>
       </c>
       <c r="B127">
-        <v>841</v>
+        <v>888</v>
       </c>
     </row>
     <row r="128" spans="1:2">
       <c r="A128" s="2">
-        <v>46213.3125</v>
+        <v>46214.3125</v>
       </c>
       <c r="B128">
-        <v>852</v>
+        <v>885</v>
       </c>
     </row>
     <row r="129" spans="1:2">
       <c r="A129" s="2">
-        <v>46213.32291666666</v>
+        <v>46214.32291666666</v>
       </c>
       <c r="B129">
-        <v>848</v>
+        <v>886</v>
       </c>
     </row>
     <row r="130" spans="1:2">
       <c r="A130" s="2">
-        <v>46213.33333333334</v>
+        <v>46214.33333333334</v>
       </c>
       <c r="B130">
-        <v>812</v>
+        <v>887</v>
       </c>
     </row>
     <row r="131" spans="1:2">
       <c r="A131" s="2">
-        <v>46213.34375</v>
+        <v>46214.34375</v>
       </c>
       <c r="B131">
-        <v>813</v>
+        <v>885</v>
       </c>
     </row>
     <row r="132" spans="1:2">
       <c r="A132" s="2">
-        <v>46213.35416666666</v>
+        <v>46214.35416666666</v>
       </c>
       <c r="B132">
-        <v>807</v>
+        <v>881</v>
       </c>
     </row>
     <row r="133" spans="1:2">
       <c r="A133" s="2">
-        <v>46213.36458333334</v>
+        <v>46214.36458333334</v>
       </c>
       <c r="B133">
-        <v>811</v>
+        <v>882</v>
       </c>
     </row>
     <row r="134" spans="1:2">
       <c r="A134" s="2">
-        <v>46213.375</v>
+        <v>46214.375</v>
       </c>
       <c r="B134">
-        <v>669</v>
+        <v>708</v>
       </c>
     </row>
     <row r="135" spans="1:2">
       <c r="A135" s="2">
-        <v>46213.38541666666</v>
+        <v>46214.38541666666</v>
       </c>
       <c r="B135">
-        <v>661</v>
+        <v>674</v>
       </c>
     </row>
     <row r="136" spans="1:2">
       <c r="A136" s="2">
-        <v>46213.39583333334</v>
+        <v>46214.39583333334</v>
       </c>
       <c r="B136">
-        <v>660</v>
+        <v>673</v>
       </c>
     </row>
     <row r="137" spans="1:2">
       <c r="A137" s="2">
-        <v>46213.40625</v>
+        <v>46214.40625</v>
       </c>
       <c r="B137">
-        <v>661</v>
+        <v>674</v>
       </c>
     </row>
     <row r="138" spans="1:2">
       <c r="A138" s="2">
-        <v>46213.41666666666</v>
+        <v>46214.41666666666</v>
       </c>
       <c r="B138">
-        <v>652</v>
+        <v>426</v>
       </c>
     </row>
     <row r="139" spans="1:2">
       <c r="A139" s="2">
-        <v>46213.42708333334</v>
+        <v>46214.42708333334</v>
       </c>
       <c r="B139">
-        <v>614</v>
+        <v>383</v>
       </c>
     </row>
     <row r="140" spans="1:2">
       <c r="A140" s="2">
-        <v>46213.4375</v>
+        <v>46214.4375</v>
       </c>
       <c r="B140">
-        <v>618</v>
+        <v>382</v>
       </c>
     </row>
     <row r="141" spans="1:2">
       <c r="A141" s="2">
-        <v>46213.44791666666</v>
+        <v>46214.44791666666</v>
       </c>
       <c r="B141">
-        <v>615</v>
+        <v>384</v>
+      </c>
+    </row>
+    <row r="142" spans="1:2">
+      <c r="A142" s="2">
+        <v>46214.45833333334</v>
+      </c>
+      <c r="B142">
+        <v>377</v>
+      </c>
+    </row>
+    <row r="143" spans="1:2">
+      <c r="A143" s="2">
+        <v>46214.46875</v>
+      </c>
+      <c r="B143">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="144" spans="1:2">
+      <c r="A144" s="2">
+        <v>46214.47916666666</v>
+      </c>
+      <c r="B144">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="145" spans="1:2">
+      <c r="A145" s="2">
+        <v>46214.48958333334</v>
+      </c>
+      <c r="B145">
+        <v>376</v>
+      </c>
+    </row>
+    <row r="146" spans="1:2">
+      <c r="A146" s="2">
+        <v>46214.5</v>
+      </c>
+      <c r="B146">
+        <v>381</v>
+      </c>
+    </row>
+    <row r="147" spans="1:2">
+      <c r="A147" s="2">
+        <v>46214.51041666666</v>
+      </c>
+      <c r="B147">
+        <v>380</v>
+      </c>
+    </row>
+    <row r="148" spans="1:2">
+      <c r="A148" s="2">
+        <v>46214.52083333334</v>
+      </c>
+      <c r="B148">
+        <v>381</v>
+      </c>
+    </row>
+    <row r="149" spans="1:2">
+      <c r="A149" s="2">
+        <v>46214.53125</v>
+      </c>
+      <c r="B149">
+        <v>382</v>
+      </c>
+    </row>
+    <row r="150" spans="1:2">
+      <c r="A150" s="2">
+        <v>46214.54166666666</v>
+      </c>
+      <c r="B150">
+        <v>391</v>
+      </c>
+    </row>
+    <row r="151" spans="1:2">
+      <c r="A151" s="2">
+        <v>46214.55208333334</v>
+      </c>
+      <c r="B151">
+        <v>378</v>
+      </c>
+    </row>
+    <row r="152" spans="1:2">
+      <c r="A152" s="2">
+        <v>46214.5625</v>
+      </c>
+      <c r="B152">
+        <v>359</v>
+      </c>
+    </row>
+    <row r="153" spans="1:2">
+      <c r="A153" s="2">
+        <v>46214.57291666666</v>
+      </c>
+      <c r="B153">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="154" spans="1:2">
+      <c r="A154" s="2">
+        <v>46214.58333333334</v>
+      </c>
+      <c r="B154">
+        <v>369</v>
+      </c>
+    </row>
+    <row r="155" spans="1:2">
+      <c r="A155" s="2">
+        <v>46214.59375</v>
+      </c>
+      <c r="B155">
+        <v>370</v>
+      </c>
+    </row>
+    <row r="156" spans="1:2">
+      <c r="A156" s="2">
+        <v>46214.60416666666</v>
+      </c>
+      <c r="B156">
+        <v>370</v>
+      </c>
+    </row>
+    <row r="157" spans="1:2">
+      <c r="A157" s="2">
+        <v>46214.61458333334</v>
+      </c>
+      <c r="B157">
+        <v>370</v>
+      </c>
+    </row>
+    <row r="158" spans="1:2">
+      <c r="A158" s="2">
+        <v>46214.625</v>
+      </c>
+      <c r="B158">
+        <v>355</v>
+      </c>
+    </row>
+    <row r="159" spans="1:2">
+      <c r="A159" s="2">
+        <v>46214.63541666666</v>
+      </c>
+      <c r="B159">
+        <v>354</v>
+      </c>
+    </row>
+    <row r="160" spans="1:2">
+      <c r="A160" s="2">
+        <v>46214.64583333334</v>
+      </c>
+      <c r="B160">
+        <v>351</v>
+      </c>
+    </row>
+    <row r="161" spans="1:2">
+      <c r="A161" s="2">
+        <v>46214.65625</v>
+      </c>
+      <c r="B161">
+        <v>351</v>
+      </c>
+    </row>
+    <row r="162" spans="1:2">
+      <c r="A162" s="2">
+        <v>46214.66666666666</v>
+      </c>
+      <c r="B162">
+        <v>349</v>
+      </c>
+    </row>
+    <row r="163" spans="1:2">
+      <c r="A163" s="2">
+        <v>46214.67708333334</v>
+      </c>
+      <c r="B163">
+        <v>352</v>
+      </c>
+    </row>
+    <row r="164" spans="1:2">
+      <c r="A164" s="2">
+        <v>46214.6875</v>
+      </c>
+      <c r="B164">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="165" spans="1:2">
+      <c r="A165" s="2">
+        <v>46214.69791666666</v>
+      </c>
+      <c r="B165">
+        <v>378</v>
+      </c>
+    </row>
+    <row r="166" spans="1:2">
+      <c r="A166" s="2">
+        <v>46214.70833333334</v>
+      </c>
+      <c r="B166">
+        <v>778</v>
+      </c>
+    </row>
+    <row r="167" spans="1:2">
+      <c r="A167" s="2">
+        <v>46214.71875</v>
+      </c>
+      <c r="B167">
+        <v>795</v>
+      </c>
+    </row>
+    <row r="168" spans="1:2">
+      <c r="A168" s="2">
+        <v>46214.72916666666</v>
+      </c>
+      <c r="B168">
+        <v>811</v>
+      </c>
+    </row>
+    <row r="169" spans="1:2">
+      <c r="A169" s="2">
+        <v>46214.73958333334</v>
+      </c>
+      <c r="B169">
+        <v>846</v>
+      </c>
+    </row>
+    <row r="170" spans="1:2">
+      <c r="A170" s="2">
+        <v>46214.75</v>
+      </c>
+      <c r="B170">
+        <v>850</v>
+      </c>
+    </row>
+    <row r="171" spans="1:2">
+      <c r="A171" s="2">
+        <v>46214.76041666666</v>
+      </c>
+      <c r="B171">
+        <v>852</v>
+      </c>
+    </row>
+    <row r="172" spans="1:2">
+      <c r="A172" s="2">
+        <v>46214.77083333334</v>
+      </c>
+      <c r="B172">
+        <v>852</v>
+      </c>
+    </row>
+    <row r="173" spans="1:2">
+      <c r="A173" s="2">
+        <v>46214.78125</v>
+      </c>
+      <c r="B173">
+        <v>850</v>
+      </c>
+    </row>
+    <row r="174" spans="1:2">
+      <c r="A174" s="2">
+        <v>46214.79166666666</v>
+      </c>
+      <c r="B174">
+        <v>839</v>
+      </c>
+    </row>
+    <row r="175" spans="1:2">
+      <c r="A175" s="2">
+        <v>46214.80208333334</v>
+      </c>
+      <c r="B175">
+        <v>838</v>
+      </c>
+    </row>
+    <row r="176" spans="1:2">
+      <c r="A176" s="2">
+        <v>46214.8125</v>
+      </c>
+      <c r="B176">
+        <v>829</v>
+      </c>
+    </row>
+    <row r="177" spans="1:2">
+      <c r="A177" s="2">
+        <v>46214.82291666666</v>
+      </c>
+      <c r="B177">
+        <v>835</v>
+      </c>
+    </row>
+    <row r="178" spans="1:2">
+      <c r="A178" s="2">
+        <v>46214.83333333334</v>
+      </c>
+      <c r="B178">
+        <v>819</v>
+      </c>
+    </row>
+    <row r="179" spans="1:2">
+      <c r="A179" s="2">
+        <v>46214.84375</v>
+      </c>
+      <c r="B179">
+        <v>817</v>
+      </c>
+    </row>
+    <row r="180" spans="1:2">
+      <c r="A180" s="2">
+        <v>46214.85416666666</v>
+      </c>
+      <c r="B180">
+        <v>818</v>
+      </c>
+    </row>
+    <row r="181" spans="1:2">
+      <c r="A181" s="2">
+        <v>46214.86458333334</v>
+      </c>
+      <c r="B181">
+        <v>816</v>
+      </c>
+    </row>
+    <row r="182" spans="1:2">
+      <c r="A182" s="2">
+        <v>46214.875</v>
+      </c>
+      <c r="B182">
+        <v>817</v>
+      </c>
+    </row>
+    <row r="183" spans="1:2">
+      <c r="A183" s="2">
+        <v>46214.88541666666</v>
+      </c>
+      <c r="B183">
+        <v>817</v>
+      </c>
+    </row>
+    <row r="184" spans="1:2">
+      <c r="A184" s="2">
+        <v>46214.89583333334</v>
+      </c>
+      <c r="B184">
+        <v>814</v>
+      </c>
+    </row>
+    <row r="185" spans="1:2">
+      <c r="A185" s="2">
+        <v>46214.90625</v>
+      </c>
+      <c r="B185">
+        <v>814</v>
+      </c>
+    </row>
+    <row r="186" spans="1:2">
+      <c r="A186" s="2">
+        <v>46214.91666666666</v>
+      </c>
+      <c r="B186">
+        <v>812</v>
+      </c>
+    </row>
+    <row r="187" spans="1:2">
+      <c r="A187" s="2">
+        <v>46214.92708333334</v>
+      </c>
+      <c r="B187">
+        <v>807</v>
+      </c>
+    </row>
+    <row r="188" spans="1:2">
+      <c r="A188" s="2">
+        <v>46214.9375</v>
+      </c>
+      <c r="B188">
+        <v>806</v>
+      </c>
+    </row>
+    <row r="189" spans="1:2">
+      <c r="A189" s="2">
+        <v>46214.94791666666</v>
+      </c>
+      <c r="B189">
+        <v>810</v>
+      </c>
+    </row>
+    <row r="190" spans="1:2">
+      <c r="A190" s="2">
+        <v>46214.95833333334</v>
+      </c>
+      <c r="B190">
+        <v>759</v>
+      </c>
+    </row>
+    <row r="191" spans="1:2">
+      <c r="A191" s="2">
+        <v>46214.96875</v>
+      </c>
+      <c r="B191">
+        <v>754</v>
+      </c>
+    </row>
+    <row r="192" spans="1:2">
+      <c r="A192" s="2">
+        <v>46214.97916666666</v>
+      </c>
+      <c r="B192">
+        <v>750</v>
+      </c>
+    </row>
+    <row r="193" spans="1:2">
+      <c r="A193" s="2">
+        <v>46214.98958333334</v>
+      </c>
+      <c r="B193">
+        <v>745</v>
+      </c>
+    </row>
+    <row r="194" spans="1:2">
+      <c r="A194" s="2">
+        <v>46215</v>
+      </c>
+      <c r="B194">
+        <v>748</v>
+      </c>
+    </row>
+    <row r="195" spans="1:2">
+      <c r="A195" s="2">
+        <v>46215.01041666666</v>
+      </c>
+      <c r="B195">
+        <v>742</v>
+      </c>
+    </row>
+    <row r="196" spans="1:2">
+      <c r="A196" s="2">
+        <v>46215.02083333334</v>
+      </c>
+      <c r="B196">
+        <v>742</v>
+      </c>
+    </row>
+    <row r="197" spans="1:2">
+      <c r="A197" s="2">
+        <v>46215.03125</v>
+      </c>
+      <c r="B197">
+        <v>740</v>
+      </c>
+    </row>
+    <row r="198" spans="1:2">
+      <c r="A198" s="2">
+        <v>46215.04166666666</v>
+      </c>
+      <c r="B198">
+        <v>742</v>
+      </c>
+    </row>
+    <row r="199" spans="1:2">
+      <c r="A199" s="2">
+        <v>46215.05208333334</v>
+      </c>
+      <c r="B199">
+        <v>743</v>
+      </c>
+    </row>
+    <row r="200" spans="1:2">
+      <c r="A200" s="2">
+        <v>46215.0625</v>
+      </c>
+      <c r="B200">
+        <v>740</v>
+      </c>
+    </row>
+    <row r="201" spans="1:2">
+      <c r="A201" s="2">
+        <v>46215.07291666666</v>
+      </c>
+      <c r="B201">
+        <v>738</v>
+      </c>
+    </row>
+    <row r="202" spans="1:2">
+      <c r="A202" s="2">
+        <v>46215.08333333334</v>
+      </c>
+      <c r="B202">
+        <v>795</v>
+      </c>
+    </row>
+    <row r="203" spans="1:2">
+      <c r="A203" s="2">
+        <v>46215.09375</v>
+      </c>
+      <c r="B203">
+        <v>799</v>
+      </c>
+    </row>
+    <row r="204" spans="1:2">
+      <c r="A204" s="2">
+        <v>46215.10416666666</v>
+      </c>
+      <c r="B204">
+        <v>799</v>
+      </c>
+    </row>
+    <row r="205" spans="1:2">
+      <c r="A205" s="2">
+        <v>46215.11458333334</v>
+      </c>
+      <c r="B205">
+        <v>800</v>
+      </c>
+    </row>
+    <row r="206" spans="1:2">
+      <c r="A206" s="2">
+        <v>46215.125</v>
+      </c>
+      <c r="B206">
+        <v>801</v>
+      </c>
+    </row>
+    <row r="207" spans="1:2">
+      <c r="A207" s="2">
+        <v>46215.13541666666</v>
+      </c>
+      <c r="B207">
+        <v>800</v>
+      </c>
+    </row>
+    <row r="208" spans="1:2">
+      <c r="A208" s="2">
+        <v>46215.14583333334</v>
+      </c>
+      <c r="B208">
+        <v>799</v>
+      </c>
+    </row>
+    <row r="209" spans="1:2">
+      <c r="A209" s="2">
+        <v>46215.15625</v>
+      </c>
+      <c r="B209">
+        <v>800</v>
+      </c>
+    </row>
+    <row r="210" spans="1:2">
+      <c r="A210" s="2">
+        <v>46215.16666666666</v>
+      </c>
+      <c r="B210">
+        <v>797</v>
+      </c>
+    </row>
+    <row r="211" spans="1:2">
+      <c r="A211" s="2">
+        <v>46215.17708333334</v>
+      </c>
+      <c r="B211">
+        <v>770</v>
+      </c>
+    </row>
+    <row r="212" spans="1:2">
+      <c r="A212" s="2">
+        <v>46215.1875</v>
+      </c>
+      <c r="B212">
+        <v>768</v>
+      </c>
+    </row>
+    <row r="213" spans="1:2">
+      <c r="A213" s="2">
+        <v>46215.19791666666</v>
+      </c>
+      <c r="B213">
+        <v>743</v>
+      </c>
+    </row>
+    <row r="214" spans="1:2">
+      <c r="A214" s="2">
+        <v>46215.20833333334</v>
+      </c>
+      <c r="B214">
+        <v>774</v>
+      </c>
+    </row>
+    <row r="215" spans="1:2">
+      <c r="A215" s="2">
+        <v>46215.21875</v>
+      </c>
+      <c r="B215">
+        <v>775</v>
+      </c>
+    </row>
+    <row r="216" spans="1:2">
+      <c r="A216" s="2">
+        <v>46215.22916666666</v>
+      </c>
+      <c r="B216">
+        <v>775</v>
+      </c>
+    </row>
+    <row r="217" spans="1:2">
+      <c r="A217" s="2">
+        <v>46215.23958333334</v>
+      </c>
+      <c r="B217">
+        <v>775</v>
+      </c>
+    </row>
+    <row r="218" spans="1:2">
+      <c r="A218" s="2">
+        <v>46215.25</v>
+      </c>
+      <c r="B218">
+        <v>792</v>
+      </c>
+    </row>
+    <row r="219" spans="1:2">
+      <c r="A219" s="2">
+        <v>46215.26041666666</v>
+      </c>
+      <c r="B219">
+        <v>792</v>
+      </c>
+    </row>
+    <row r="220" spans="1:2">
+      <c r="A220" s="2">
+        <v>46215.27083333334</v>
+      </c>
+      <c r="B220">
+        <v>801</v>
+      </c>
+    </row>
+    <row r="221" spans="1:2">
+      <c r="A221" s="2">
+        <v>46215.28125</v>
+      </c>
+      <c r="B221">
+        <v>815</v>
+      </c>
+    </row>
+    <row r="222" spans="1:2">
+      <c r="A222" s="2">
+        <v>46215.29166666666</v>
+      </c>
+      <c r="B222">
+        <v>791</v>
+      </c>
+    </row>
+    <row r="223" spans="1:2">
+      <c r="A223" s="2">
+        <v>46215.30208333334</v>
+      </c>
+      <c r="B223">
+        <v>787</v>
+      </c>
+    </row>
+    <row r="224" spans="1:2">
+      <c r="A224" s="2">
+        <v>46215.3125</v>
+      </c>
+      <c r="B224">
+        <v>860</v>
+      </c>
+    </row>
+    <row r="225" spans="1:2">
+      <c r="A225" s="2">
+        <v>46215.32291666666</v>
+      </c>
+      <c r="B225">
+        <v>864</v>
+      </c>
+    </row>
+    <row r="226" spans="1:2">
+      <c r="A226" s="2">
+        <v>46215.33333333334</v>
+      </c>
+      <c r="B226">
+        <v>773</v>
+      </c>
+    </row>
+    <row r="227" spans="1:2">
+      <c r="A227" s="2">
+        <v>46215.34375</v>
+      </c>
+      <c r="B227">
+        <v>761</v>
+      </c>
+    </row>
+    <row r="228" spans="1:2">
+      <c r="A228" s="2">
+        <v>46215.35416666666</v>
+      </c>
+      <c r="B228">
+        <v>761</v>
+      </c>
+    </row>
+    <row r="229" spans="1:2">
+      <c r="A229" s="2">
+        <v>46215.36458333334</v>
+      </c>
+      <c r="B229">
+        <v>755</v>
+      </c>
+    </row>
+    <row r="230" spans="1:2">
+      <c r="A230" s="2">
+        <v>46215.375</v>
+      </c>
+      <c r="B230">
+        <v>388</v>
+      </c>
+    </row>
+    <row r="231" spans="1:2">
+      <c r="A231" s="2">
+        <v>46215.38541666666</v>
+      </c>
+      <c r="B231">
+        <v>346</v>
+      </c>
+    </row>
+    <row r="232" spans="1:2">
+      <c r="A232" s="2">
+        <v>46215.39583333334</v>
+      </c>
+      <c r="B232">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="233" spans="1:2">
+      <c r="A233" s="2">
+        <v>46215.40625</v>
+      </c>
+      <c r="B233">
+        <v>348</v>
+      </c>
+    </row>
+    <row r="234" spans="1:2">
+      <c r="A234" s="2">
+        <v>46215.41666666666</v>
+      </c>
+      <c r="B234">
+        <v>342</v>
+      </c>
+    </row>
+    <row r="235" spans="1:2">
+      <c r="A235" s="2">
+        <v>46215.42708333334</v>
+      </c>
+      <c r="B235">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="236" spans="1:2">
+      <c r="A236" s="2">
+        <v>46215.4375</v>
+      </c>
+      <c r="B236">
+        <v>338</v>
+      </c>
+    </row>
+    <row r="237" spans="1:2">
+      <c r="A237" s="2">
+        <v>46215.44791666666</v>
+      </c>
+      <c r="B237">
+        <v>339</v>
+      </c>
+    </row>
+    <row r="238" spans="1:2">
+      <c r="A238" s="2">
+        <v>46215.45833333334</v>
+      </c>
+      <c r="B238">
+        <v>335</v>
+      </c>
+    </row>
+    <row r="239" spans="1:2">
+      <c r="A239" s="2">
+        <v>46215.46875</v>
+      </c>
+      <c r="B239">
+        <v>334</v>
+      </c>
+    </row>
+    <row r="240" spans="1:2">
+      <c r="A240" s="2">
+        <v>46215.47916666666</v>
+      </c>
+      <c r="B240">
+        <v>333</v>
+      </c>
+    </row>
+    <row r="241" spans="1:2">
+      <c r="A241" s="2">
+        <v>46215.48958333334</v>
+      </c>
+      <c r="B241">
+        <v>333</v>
+      </c>
+    </row>
+    <row r="242" spans="1:2">
+      <c r="A242" s="2">
+        <v>46215.5</v>
+      </c>
+      <c r="B242">
+        <v>324</v>
+      </c>
+    </row>
+    <row r="243" spans="1:2">
+      <c r="A243" s="2">
+        <v>46215.51041666666</v>
+      </c>
+      <c r="B243">
+        <v>325</v>
+      </c>
+    </row>
+    <row r="244" spans="1:2">
+      <c r="A244" s="2">
+        <v>46215.52083333334</v>
+      </c>
+      <c r="B244">
+        <v>324</v>
+      </c>
+    </row>
+    <row r="245" spans="1:2">
+      <c r="A245" s="2">
+        <v>46215.53125</v>
+      </c>
+      <c r="B245">
+        <v>324</v>
+      </c>
+    </row>
+    <row r="246" spans="1:2">
+      <c r="A246" s="2">
+        <v>46215.54166666666</v>
+      </c>
+      <c r="B246">
+        <v>334</v>
+      </c>
+    </row>
+    <row r="247" spans="1:2">
+      <c r="A247" s="2">
+        <v>46215.55208333334</v>
+      </c>
+      <c r="B247">
+        <v>335</v>
+      </c>
+    </row>
+    <row r="248" spans="1:2">
+      <c r="A248" s="2">
+        <v>46215.5625</v>
+      </c>
+      <c r="B248">
+        <v>328</v>
+      </c>
+    </row>
+    <row r="249" spans="1:2">
+      <c r="A249" s="2">
+        <v>46215.57291666666</v>
+      </c>
+      <c r="B249">
+        <v>324</v>
+      </c>
+    </row>
+    <row r="250" spans="1:2">
+      <c r="A250" s="2">
+        <v>46215.58333333334</v>
+      </c>
+      <c r="B250">
+        <v>302</v>
+      </c>
+    </row>
+    <row r="251" spans="1:2">
+      <c r="A251" s="2">
+        <v>46215.59375</v>
+      </c>
+      <c r="B251">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="252" spans="1:2">
+      <c r="A252" s="2">
+        <v>46215.60416666666</v>
+      </c>
+      <c r="B252">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="253" spans="1:2">
+      <c r="A253" s="2">
+        <v>46215.61458333334</v>
+      </c>
+      <c r="B253">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="254" spans="1:2">
+      <c r="A254" s="2">
+        <v>46215.625</v>
+      </c>
+      <c r="B254">
+        <v>287</v>
+      </c>
+    </row>
+    <row r="255" spans="1:2">
+      <c r="A255" s="2">
+        <v>46215.63541666666</v>
+      </c>
+      <c r="B255">
+        <v>285</v>
+      </c>
+    </row>
+    <row r="256" spans="1:2">
+      <c r="A256" s="2">
+        <v>46215.64583333334</v>
+      </c>
+      <c r="B256">
+        <v>285</v>
+      </c>
+    </row>
+    <row r="257" spans="1:2">
+      <c r="A257" s="2">
+        <v>46215.65625</v>
+      </c>
+      <c r="B257">
+        <v>285</v>
+      </c>
+    </row>
+    <row r="258" spans="1:2">
+      <c r="A258" s="2">
+        <v>46215.66666666666</v>
+      </c>
+      <c r="B258">
+        <v>316</v>
+      </c>
+    </row>
+    <row r="259" spans="1:2">
+      <c r="A259" s="2">
+        <v>46215.67708333334</v>
+      </c>
+      <c r="B259">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="260" spans="1:2">
+      <c r="A260" s="2">
+        <v>46215.6875</v>
+      </c>
+      <c r="B260">
+        <v>408</v>
+      </c>
+    </row>
+    <row r="261" spans="1:2">
+      <c r="A261" s="2">
+        <v>46215.69791666666</v>
+      </c>
+      <c r="B261">
+        <v>433</v>
+      </c>
+    </row>
+    <row r="262" spans="1:2">
+      <c r="A262" s="2">
+        <v>46215.70833333334</v>
+      </c>
+      <c r="B262">
+        <v>881</v>
+      </c>
+    </row>
+    <row r="263" spans="1:2">
+      <c r="A263" s="2">
+        <v>46215.71875</v>
+      </c>
+      <c r="B263">
+        <v>901</v>
+      </c>
+    </row>
+    <row r="264" spans="1:2">
+      <c r="A264" s="2">
+        <v>46215.72916666666</v>
+      </c>
+      <c r="B264">
+        <v>909</v>
+      </c>
+    </row>
+    <row r="265" spans="1:2">
+      <c r="A265" s="2">
+        <v>46215.73958333334</v>
+      </c>
+      <c r="B265">
+        <v>905</v>
+      </c>
+    </row>
+    <row r="266" spans="1:2">
+      <c r="A266" s="2">
+        <v>46215.75</v>
+      </c>
+      <c r="B266">
+        <v>950</v>
+      </c>
+    </row>
+    <row r="267" spans="1:2">
+      <c r="A267" s="2">
+        <v>46215.76041666666</v>
+      </c>
+      <c r="B267">
+        <v>901</v>
+      </c>
+    </row>
+    <row r="268" spans="1:2">
+      <c r="A268" s="2">
+        <v>46215.77083333334</v>
+      </c>
+      <c r="B268">
+        <v>887</v>
+      </c>
+    </row>
+    <row r="269" spans="1:2">
+      <c r="A269" s="2">
+        <v>46215.78125</v>
+      </c>
+      <c r="B269">
+        <v>888</v>
+      </c>
+    </row>
+    <row r="270" spans="1:2">
+      <c r="A270" s="2">
+        <v>46215.79166666666</v>
+      </c>
+      <c r="B270">
+        <v>938</v>
+      </c>
+    </row>
+    <row r="271" spans="1:2">
+      <c r="A271" s="2">
+        <v>46215.80208333334</v>
+      </c>
+      <c r="B271">
+        <v>940</v>
+      </c>
+    </row>
+    <row r="272" spans="1:2">
+      <c r="A272" s="2">
+        <v>46215.8125</v>
+      </c>
+      <c r="B272">
+        <v>944</v>
+      </c>
+    </row>
+    <row r="273" spans="1:2">
+      <c r="A273" s="2">
+        <v>46215.82291666666</v>
+      </c>
+      <c r="B273">
+        <v>937</v>
+      </c>
+    </row>
+    <row r="274" spans="1:2">
+      <c r="A274" s="2">
+        <v>46215.83333333334</v>
+      </c>
+      <c r="B274">
+        <v>935</v>
+      </c>
+    </row>
+    <row r="275" spans="1:2">
+      <c r="A275" s="2">
+        <v>46215.84375</v>
+      </c>
+      <c r="B275">
+        <v>936</v>
+      </c>
+    </row>
+    <row r="276" spans="1:2">
+      <c r="A276" s="2">
+        <v>46215.85416666666</v>
+      </c>
+      <c r="B276">
+        <v>934</v>
+      </c>
+    </row>
+    <row r="277" spans="1:2">
+      <c r="A277" s="2">
+        <v>46215.86458333334</v>
+      </c>
+      <c r="B277">
+        <v>930</v>
+      </c>
+    </row>
+    <row r="278" spans="1:2">
+      <c r="A278" s="2">
+        <v>46215.875</v>
+      </c>
+      <c r="B278">
+        <v>908</v>
+      </c>
+    </row>
+    <row r="279" spans="1:2">
+      <c r="A279" s="2">
+        <v>46215.88541666666</v>
+      </c>
+      <c r="B279">
+        <v>909</v>
+      </c>
+    </row>
+    <row r="280" spans="1:2">
+      <c r="A280" s="2">
+        <v>46215.89583333334</v>
+      </c>
+      <c r="B280">
+        <v>913</v>
+      </c>
+    </row>
+    <row r="281" spans="1:2">
+      <c r="A281" s="2">
+        <v>46215.90625</v>
+      </c>
+      <c r="B281">
+        <v>876</v>
+      </c>
+    </row>
+    <row r="282" spans="1:2">
+      <c r="A282" s="2">
+        <v>46215.91666666666</v>
+      </c>
+      <c r="B282">
+        <v>910</v>
+      </c>
+    </row>
+    <row r="283" spans="1:2">
+      <c r="A283" s="2">
+        <v>46215.92708333334</v>
+      </c>
+      <c r="B283">
+        <v>912</v>
+      </c>
+    </row>
+    <row r="284" spans="1:2">
+      <c r="A284" s="2">
+        <v>46215.9375</v>
+      </c>
+      <c r="B284">
+        <v>913</v>
+      </c>
+    </row>
+    <row r="285" spans="1:2">
+      <c r="A285" s="2">
+        <v>46215.94791666666</v>
+      </c>
+      <c r="B285">
+        <v>912</v>
+      </c>
+    </row>
+    <row r="286" spans="1:2">
+      <c r="A286" s="2">
+        <v>46215.95833333334</v>
+      </c>
+      <c r="B286">
+        <v>757</v>
+      </c>
+    </row>
+    <row r="287" spans="1:2">
+      <c r="A287" s="2">
+        <v>46215.96875</v>
+      </c>
+      <c r="B287">
+        <v>744</v>
+      </c>
+    </row>
+    <row r="288" spans="1:2">
+      <c r="A288" s="2">
+        <v>46215.97916666666</v>
+      </c>
+      <c r="B288">
+        <v>750</v>
+      </c>
+    </row>
+    <row r="289" spans="1:2">
+      <c r="A289" s="2">
+        <v>46215.98958333334</v>
+      </c>
+      <c r="B289">
+        <v>750</v>
+      </c>
+    </row>
+    <row r="290" spans="1:2">
+      <c r="A290" s="2">
+        <v>46216</v>
+      </c>
+      <c r="B290">
+        <v>692</v>
+      </c>
+    </row>
+    <row r="291" spans="1:2">
+      <c r="A291" s="2">
+        <v>46216.01041666666</v>
+      </c>
+      <c r="B291">
+        <v>681</v>
+      </c>
+    </row>
+    <row r="292" spans="1:2">
+      <c r="A292" s="2">
+        <v>46216.02083333334</v>
+      </c>
+      <c r="B292">
+        <v>681</v>
+      </c>
+    </row>
+    <row r="293" spans="1:2">
+      <c r="A293" s="2">
+        <v>46216.03125</v>
+      </c>
+      <c r="B293">
+        <v>682</v>
+      </c>
+    </row>
+    <row r="294" spans="1:2">
+      <c r="A294" s="2">
+        <v>46216.04166666666</v>
+      </c>
+      <c r="B294">
+        <v>654</v>
+      </c>
+    </row>
+    <row r="295" spans="1:2">
+      <c r="A295" s="2">
+        <v>46216.05208333334</v>
+      </c>
+      <c r="B295">
+        <v>635</v>
+      </c>
+    </row>
+    <row r="296" spans="1:2">
+      <c r="A296" s="2">
+        <v>46216.0625</v>
+      </c>
+      <c r="B296">
+        <v>635</v>
+      </c>
+    </row>
+    <row r="297" spans="1:2">
+      <c r="A297" s="2">
+        <v>46216.07291666666</v>
+      </c>
+      <c r="B297">
+        <v>635</v>
+      </c>
+    </row>
+    <row r="298" spans="1:2">
+      <c r="A298" s="2">
+        <v>46216.08333333334</v>
+      </c>
+      <c r="B298">
+        <v>604</v>
+      </c>
+    </row>
+    <row r="299" spans="1:2">
+      <c r="A299" s="2">
+        <v>46216.09375</v>
+      </c>
+      <c r="B299">
+        <v>641</v>
+      </c>
+    </row>
+    <row r="300" spans="1:2">
+      <c r="A300" s="2">
+        <v>46216.10416666666</v>
+      </c>
+      <c r="B300">
+        <v>642</v>
+      </c>
+    </row>
+    <row r="301" spans="1:2">
+      <c r="A301" s="2">
+        <v>46216.11458333334</v>
+      </c>
+      <c r="B301">
+        <v>643</v>
+      </c>
+    </row>
+    <row r="302" spans="1:2">
+      <c r="A302" s="2">
+        <v>46216.125</v>
+      </c>
+      <c r="B302">
+        <v>644</v>
+      </c>
+    </row>
+    <row r="303" spans="1:2">
+      <c r="A303" s="2">
+        <v>46216.13541666666</v>
+      </c>
+      <c r="B303">
+        <v>644</v>
+      </c>
+    </row>
+    <row r="304" spans="1:2">
+      <c r="A304" s="2">
+        <v>46216.14583333334</v>
+      </c>
+      <c r="B304">
+        <v>642</v>
+      </c>
+    </row>
+    <row r="305" spans="1:2">
+      <c r="A305" s="2">
+        <v>46216.15625</v>
+      </c>
+      <c r="B305">
+        <v>644</v>
+      </c>
+    </row>
+    <row r="306" spans="1:2">
+      <c r="A306" s="2">
+        <v>46216.16666666666</v>
+      </c>
+      <c r="B306">
+        <v>676</v>
+      </c>
+    </row>
+    <row r="307" spans="1:2">
+      <c r="A307" s="2">
+        <v>46216.17708333334</v>
+      </c>
+      <c r="B307">
+        <v>677</v>
+      </c>
+    </row>
+    <row r="308" spans="1:2">
+      <c r="A308" s="2">
+        <v>46216.1875</v>
+      </c>
+      <c r="B308">
+        <v>679</v>
+      </c>
+    </row>
+    <row r="309" spans="1:2">
+      <c r="A309" s="2">
+        <v>46216.19791666666</v>
+      </c>
+      <c r="B309">
+        <v>683</v>
+      </c>
+    </row>
+    <row r="310" spans="1:2">
+      <c r="A310" s="2">
+        <v>46216.20833333334</v>
+      </c>
+      <c r="B310">
+        <v>768</v>
+      </c>
+    </row>
+    <row r="311" spans="1:2">
+      <c r="A311" s="2">
+        <v>46216.21875</v>
+      </c>
+      <c r="B311">
+        <v>770</v>
+      </c>
+    </row>
+    <row r="312" spans="1:2">
+      <c r="A312" s="2">
+        <v>46216.22916666666</v>
+      </c>
+      <c r="B312">
+        <v>771</v>
+      </c>
+    </row>
+    <row r="313" spans="1:2">
+      <c r="A313" s="2">
+        <v>46216.23958333334</v>
+      </c>
+      <c r="B313">
+        <v>758</v>
+      </c>
+    </row>
+    <row r="314" spans="1:2">
+      <c r="A314" s="2">
+        <v>46216.25</v>
+      </c>
+      <c r="B314">
+        <v>730</v>
+      </c>
+    </row>
+    <row r="315" spans="1:2">
+      <c r="A315" s="2">
+        <v>46216.26041666666</v>
+      </c>
+      <c r="B315">
+        <v>724</v>
+      </c>
+    </row>
+    <row r="316" spans="1:2">
+      <c r="A316" s="2">
+        <v>46216.27083333334</v>
+      </c>
+      <c r="B316">
+        <v>724</v>
+      </c>
+    </row>
+    <row r="317" spans="1:2">
+      <c r="A317" s="2">
+        <v>46216.28125</v>
+      </c>
+      <c r="B317">
+        <v>727</v>
+      </c>
+    </row>
+    <row r="318" spans="1:2">
+      <c r="A318" s="2">
+        <v>46216.29166666666</v>
+      </c>
+      <c r="B318">
+        <v>739</v>
+      </c>
+    </row>
+    <row r="319" spans="1:2">
+      <c r="A319" s="2">
+        <v>46216.30208333334</v>
+      </c>
+      <c r="B319">
+        <v>739</v>
+      </c>
+    </row>
+    <row r="320" spans="1:2">
+      <c r="A320" s="2">
+        <v>46216.3125</v>
+      </c>
+      <c r="B320">
+        <v>749</v>
+      </c>
+    </row>
+    <row r="321" spans="1:2">
+      <c r="A321" s="2">
+        <v>46216.32291666666</v>
+      </c>
+      <c r="B321">
+        <v>740</v>
+      </c>
+    </row>
+    <row r="322" spans="1:2">
+      <c r="A322" s="2">
+        <v>46216.33333333334</v>
+      </c>
+      <c r="B322">
+        <v>684</v>
+      </c>
+    </row>
+    <row r="323" spans="1:2">
+      <c r="A323" s="2">
+        <v>46216.34375</v>
+      </c>
+      <c r="B323">
+        <v>676</v>
+      </c>
+    </row>
+    <row r="324" spans="1:2">
+      <c r="A324" s="2">
+        <v>46216.35416666666</v>
+      </c>
+      <c r="B324">
+        <v>675</v>
+      </c>
+    </row>
+    <row r="325" spans="1:2">
+      <c r="A325" s="2">
+        <v>46216.36458333334</v>
+      </c>
+      <c r="B325">
+        <v>675</v>
+      </c>
+    </row>
+    <row r="326" spans="1:2">
+      <c r="A326" s="2">
+        <v>46216.375</v>
+      </c>
+      <c r="B326">
+        <v>464</v>
+      </c>
+    </row>
+    <row r="327" spans="1:2">
+      <c r="A327" s="2">
+        <v>46216.38541666666</v>
+      </c>
+      <c r="B327">
+        <v>427</v>
+      </c>
+    </row>
+    <row r="328" spans="1:2">
+      <c r="A328" s="2">
+        <v>46216.39583333334</v>
+      </c>
+      <c r="B328">
+        <v>426</v>
+      </c>
+    </row>
+    <row r="329" spans="1:2">
+      <c r="A329" s="2">
+        <v>46216.40625</v>
+      </c>
+      <c r="B329">
+        <v>425</v>
+      </c>
+    </row>
+    <row r="330" spans="1:2">
+      <c r="A330" s="2">
+        <v>46216.41666666666</v>
+      </c>
+      <c r="B330">
+        <v>316</v>
+      </c>
+    </row>
+    <row r="331" spans="1:2">
+      <c r="A331" s="2">
+        <v>46216.42708333334</v>
+      </c>
+      <c r="B331">
+        <v>302</v>
+      </c>
+    </row>
+    <row r="332" spans="1:2">
+      <c r="A332" s="2">
+        <v>46216.4375</v>
+      </c>
+      <c r="B332">
+        <v>302</v>
+      </c>
+    </row>
+    <row r="333" spans="1:2">
+      <c r="A333" s="2">
+        <v>46216.44791666666</v>
+      </c>
+      <c r="B333">
+        <v>303</v>
+      </c>
+    </row>
+    <row r="334" spans="1:2">
+      <c r="A334" s="2">
+        <v>46216.45833333334</v>
+      </c>
+      <c r="B334">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="335" spans="1:2">
+      <c r="A335" s="2">
+        <v>46216.46875</v>
+      </c>
+      <c r="B335">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="336" spans="1:2">
+      <c r="A336" s="2">
+        <v>46216.47916666666</v>
+      </c>
+      <c r="B336">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="337" spans="1:2">
+      <c r="A337" s="2">
+        <v>46216.48958333334</v>
+      </c>
+      <c r="B337">
+        <v>359</v>
+      </c>
+    </row>
+    <row r="338" spans="1:2">
+      <c r="A338" s="2">
+        <v>46216.5</v>
+      </c>
+      <c r="B338">
+        <v>385</v>
+      </c>
+    </row>
+    <row r="339" spans="1:2">
+      <c r="A339" s="2">
+        <v>46216.51041666666</v>
+      </c>
+      <c r="B339">
+        <v>383</v>
+      </c>
+    </row>
+    <row r="340" spans="1:2">
+      <c r="A340" s="2">
+        <v>46216.52083333334</v>
+      </c>
+      <c r="B340">
+        <v>387</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Updating the model for Ferma Frumusica
</commit_message>
<xml_diff>
--- a/data_fetching/Entsoe/Actual_Production_Hydro_River.xlsx
+++ b/data_fetching/Entsoe/Actual_Production_Hydro_River.xlsx
@@ -381,7 +381,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B139"/>
+  <dimension ref="A1:B320"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:2">
@@ -394,495 +394,495 @@
     </row>
     <row r="2" spans="1:2">
       <c r="A2" s="2">
-        <v>46218</v>
+        <v>46220</v>
       </c>
       <c r="B2">
-        <v>530</v>
+        <v>585</v>
       </c>
     </row>
     <row r="3" spans="1:2">
       <c r="A3" s="2">
-        <v>46218.01041666666</v>
+        <v>46220.01041666666</v>
       </c>
       <c r="B3">
-        <v>527</v>
+        <v>582</v>
       </c>
     </row>
     <row r="4" spans="1:2">
       <c r="A4" s="2">
-        <v>46218.02083333334</v>
+        <v>46220.02083333334</v>
       </c>
       <c r="B4">
-        <v>526</v>
+        <v>580</v>
       </c>
     </row>
     <row r="5" spans="1:2">
       <c r="A5" s="2">
-        <v>46218.03125</v>
+        <v>46220.03125</v>
       </c>
       <c r="B5">
-        <v>525</v>
+        <v>580</v>
       </c>
     </row>
     <row r="6" spans="1:2">
       <c r="A6" s="2">
-        <v>46218.04166666666</v>
+        <v>46220.04166666666</v>
       </c>
       <c r="B6">
-        <v>503</v>
+        <v>560</v>
       </c>
     </row>
     <row r="7" spans="1:2">
       <c r="A7" s="2">
-        <v>46218.05208333334</v>
+        <v>46220.05208333334</v>
       </c>
       <c r="B7">
-        <v>499</v>
+        <v>558</v>
       </c>
     </row>
     <row r="8" spans="1:2">
       <c r="A8" s="2">
-        <v>46218.0625</v>
+        <v>46220.0625</v>
       </c>
       <c r="B8">
-        <v>499</v>
+        <v>559</v>
       </c>
     </row>
     <row r="9" spans="1:2">
       <c r="A9" s="2">
-        <v>46218.07291666666</v>
+        <v>46220.07291666666</v>
       </c>
       <c r="B9">
-        <v>499</v>
+        <v>558</v>
       </c>
     </row>
     <row r="10" spans="1:2">
       <c r="A10" s="2">
-        <v>46218.08333333334</v>
+        <v>46220.08333333334</v>
       </c>
       <c r="B10">
-        <v>448</v>
+        <v>538</v>
       </c>
     </row>
     <row r="11" spans="1:2">
       <c r="A11" s="2">
-        <v>46218.09375</v>
+        <v>46220.09375</v>
       </c>
       <c r="B11">
-        <v>445</v>
+        <v>537</v>
       </c>
     </row>
     <row r="12" spans="1:2">
       <c r="A12" s="2">
-        <v>46218.10416666666</v>
+        <v>46220.10416666666</v>
       </c>
       <c r="B12">
-        <v>445</v>
+        <v>538</v>
       </c>
     </row>
     <row r="13" spans="1:2">
       <c r="A13" s="2">
-        <v>46218.11458333334</v>
+        <v>46220.11458333334</v>
       </c>
       <c r="B13">
-        <v>440</v>
+        <v>537</v>
       </c>
     </row>
     <row r="14" spans="1:2">
       <c r="A14" s="2">
-        <v>46218.125</v>
+        <v>46220.125</v>
       </c>
       <c r="B14">
-        <v>442</v>
+        <v>525</v>
       </c>
     </row>
     <row r="15" spans="1:2">
       <c r="A15" s="2">
-        <v>46218.13541666666</v>
+        <v>46220.13541666666</v>
       </c>
       <c r="B15">
-        <v>444</v>
+        <v>535</v>
       </c>
     </row>
     <row r="16" spans="1:2">
       <c r="A16" s="2">
-        <v>46218.14583333334</v>
+        <v>46220.14583333334</v>
       </c>
       <c r="B16">
-        <v>463</v>
+        <v>535</v>
       </c>
     </row>
     <row r="17" spans="1:2">
       <c r="A17" s="2">
-        <v>46218.15625</v>
+        <v>46220.15625</v>
       </c>
       <c r="B17">
-        <v>471</v>
+        <v>535</v>
       </c>
     </row>
     <row r="18" spans="1:2">
       <c r="A18" s="2">
-        <v>46218.16666666666</v>
+        <v>46220.16666666666</v>
       </c>
       <c r="B18">
-        <v>470</v>
+        <v>537</v>
       </c>
     </row>
     <row r="19" spans="1:2">
       <c r="A19" s="2">
-        <v>46218.17708333334</v>
+        <v>46220.17708333334</v>
       </c>
       <c r="B19">
-        <v>470</v>
+        <v>537</v>
       </c>
     </row>
     <row r="20" spans="1:2">
       <c r="A20" s="2">
-        <v>46218.1875</v>
+        <v>46220.1875</v>
       </c>
       <c r="B20">
-        <v>470</v>
+        <v>537</v>
       </c>
     </row>
     <row r="21" spans="1:2">
       <c r="A21" s="2">
-        <v>46218.19791666666</v>
+        <v>46220.19791666666</v>
       </c>
       <c r="B21">
-        <v>471</v>
+        <v>538</v>
       </c>
     </row>
     <row r="22" spans="1:2">
       <c r="A22" s="2">
-        <v>46218.20833333334</v>
+        <v>46220.20833333334</v>
       </c>
       <c r="B22">
-        <v>487</v>
+        <v>535</v>
       </c>
     </row>
     <row r="23" spans="1:2">
       <c r="A23" s="2">
-        <v>46218.21875</v>
+        <v>46220.21875</v>
       </c>
       <c r="B23">
-        <v>488</v>
+        <v>531</v>
       </c>
     </row>
     <row r="24" spans="1:2">
       <c r="A24" s="2">
-        <v>46218.22916666666</v>
+        <v>46220.22916666666</v>
       </c>
       <c r="B24">
-        <v>488</v>
+        <v>519</v>
       </c>
     </row>
     <row r="25" spans="1:2">
       <c r="A25" s="2">
-        <v>46218.23958333334</v>
+        <v>46220.23958333334</v>
       </c>
       <c r="B25">
-        <v>495</v>
+        <v>520</v>
       </c>
     </row>
     <row r="26" spans="1:2">
       <c r="A26" s="2">
-        <v>46218.25</v>
+        <v>46220.25</v>
       </c>
       <c r="B26">
-        <v>473</v>
+        <v>591</v>
       </c>
     </row>
     <row r="27" spans="1:2">
       <c r="A27" s="2">
-        <v>46218.26041666666</v>
+        <v>46220.26041666666</v>
       </c>
       <c r="B27">
-        <v>454</v>
+        <v>597</v>
       </c>
     </row>
     <row r="28" spans="1:2">
       <c r="A28" s="2">
-        <v>46218.27083333334</v>
+        <v>46220.27083333334</v>
       </c>
       <c r="B28">
-        <v>454</v>
+        <v>597</v>
       </c>
     </row>
     <row r="29" spans="1:2">
       <c r="A29" s="2">
-        <v>46218.28125</v>
+        <v>46220.28125</v>
       </c>
       <c r="B29">
-        <v>455</v>
+        <v>597</v>
       </c>
     </row>
     <row r="30" spans="1:2">
       <c r="A30" s="2">
-        <v>46218.29166666666</v>
+        <v>46220.29166666666</v>
       </c>
       <c r="B30">
-        <v>487</v>
+        <v>579</v>
       </c>
     </row>
     <row r="31" spans="1:2">
       <c r="A31" s="2">
-        <v>46218.30208333334</v>
+        <v>46220.30208333334</v>
       </c>
       <c r="B31">
-        <v>488</v>
+        <v>578</v>
       </c>
     </row>
     <row r="32" spans="1:2">
       <c r="A32" s="2">
-        <v>46218.3125</v>
+        <v>46220.3125</v>
       </c>
       <c r="B32">
-        <v>489</v>
+        <v>578</v>
       </c>
     </row>
     <row r="33" spans="1:2">
       <c r="A33" s="2">
-        <v>46218.32291666666</v>
+        <v>46220.32291666666</v>
       </c>
       <c r="B33">
-        <v>508</v>
+        <v>576</v>
       </c>
     </row>
     <row r="34" spans="1:2">
       <c r="A34" s="2">
-        <v>46218.33333333334</v>
+        <v>46220.33333333334</v>
       </c>
       <c r="B34">
-        <v>540</v>
+        <v>557</v>
       </c>
     </row>
     <row r="35" spans="1:2">
       <c r="A35" s="2">
-        <v>46218.34375</v>
+        <v>46220.34375</v>
       </c>
       <c r="B35">
-        <v>533</v>
+        <v>551</v>
       </c>
     </row>
     <row r="36" spans="1:2">
       <c r="A36" s="2">
-        <v>46218.35416666666</v>
+        <v>46220.35416666666</v>
       </c>
       <c r="B36">
-        <v>509</v>
+        <v>550</v>
       </c>
     </row>
     <row r="37" spans="1:2">
       <c r="A37" s="2">
-        <v>46218.36458333334</v>
+        <v>46220.36458333334</v>
       </c>
       <c r="B37">
-        <v>506</v>
+        <v>530</v>
       </c>
     </row>
     <row r="38" spans="1:2">
       <c r="A38" s="2">
-        <v>46218.375</v>
+        <v>46220.375</v>
       </c>
       <c r="B38">
-        <v>452</v>
+        <v>612</v>
       </c>
     </row>
     <row r="39" spans="1:2">
       <c r="A39" s="2">
-        <v>46218.38541666666</v>
+        <v>46220.38541666666</v>
       </c>
       <c r="B39">
-        <v>450</v>
+        <v>620</v>
       </c>
     </row>
     <row r="40" spans="1:2">
       <c r="A40" s="2">
-        <v>46218.39583333334</v>
+        <v>46220.39583333334</v>
       </c>
       <c r="B40">
-        <v>452</v>
+        <v>621</v>
       </c>
     </row>
     <row r="41" spans="1:2">
       <c r="A41" s="2">
-        <v>46218.40625</v>
+        <v>46220.40625</v>
       </c>
       <c r="B41">
-        <v>441</v>
+        <v>620</v>
       </c>
     </row>
     <row r="42" spans="1:2">
       <c r="A42" s="2">
-        <v>46218.41666666666</v>
+        <v>46220.41666666666</v>
       </c>
       <c r="B42">
-        <v>398</v>
+        <v>598</v>
       </c>
     </row>
     <row r="43" spans="1:2">
       <c r="A43" s="2">
-        <v>46218.42708333334</v>
+        <v>46220.42708333334</v>
       </c>
       <c r="B43">
-        <v>395</v>
+        <v>585</v>
       </c>
     </row>
     <row r="44" spans="1:2">
       <c r="A44" s="2">
-        <v>46218.4375</v>
+        <v>46220.4375</v>
       </c>
       <c r="B44">
-        <v>441</v>
+        <v>567</v>
       </c>
     </row>
     <row r="45" spans="1:2">
       <c r="A45" s="2">
-        <v>46218.44791666666</v>
+        <v>46220.44791666666</v>
       </c>
       <c r="B45">
-        <v>442</v>
+        <v>588</v>
       </c>
     </row>
     <row r="46" spans="1:2">
       <c r="A46" s="2">
-        <v>46218.45833333334</v>
+        <v>46220.45833333334</v>
       </c>
       <c r="B46">
-        <v>467</v>
+        <v>533</v>
       </c>
     </row>
     <row r="47" spans="1:2">
       <c r="A47" s="2">
-        <v>46218.46875</v>
+        <v>46220.46875</v>
       </c>
       <c r="B47">
-        <v>433</v>
+        <v>517</v>
       </c>
     </row>
     <row r="48" spans="1:2">
       <c r="A48" s="2">
-        <v>46218.47916666666</v>
+        <v>46220.47916666666</v>
       </c>
       <c r="B48">
-        <v>412</v>
+        <v>522</v>
       </c>
     </row>
     <row r="49" spans="1:2">
       <c r="A49" s="2">
-        <v>46218.48958333334</v>
+        <v>46220.48958333334</v>
       </c>
       <c r="B49">
-        <v>429</v>
+        <v>527</v>
       </c>
     </row>
     <row r="50" spans="1:2">
       <c r="A50" s="2">
-        <v>46218.5</v>
+        <v>46220.5</v>
       </c>
       <c r="B50">
-        <v>506</v>
+        <v>535</v>
       </c>
     </row>
     <row r="51" spans="1:2">
       <c r="A51" s="2">
-        <v>46218.51041666666</v>
+        <v>46220.51041666666</v>
       </c>
       <c r="B51">
-        <v>518</v>
+        <v>534</v>
       </c>
     </row>
     <row r="52" spans="1:2">
       <c r="A52" s="2">
-        <v>46218.52083333334</v>
+        <v>46220.52083333334</v>
       </c>
       <c r="B52">
-        <v>511</v>
+        <v>535</v>
       </c>
     </row>
     <row r="53" spans="1:2">
       <c r="A53" s="2">
-        <v>46218.53125</v>
+        <v>46220.53125</v>
       </c>
       <c r="B53">
-        <v>506</v>
+        <v>533</v>
       </c>
     </row>
     <row r="54" spans="1:2">
       <c r="A54" s="2">
-        <v>46218.54166666666</v>
+        <v>46220.54166666666</v>
       </c>
       <c r="B54">
-        <v>451</v>
+        <v>555</v>
       </c>
     </row>
     <row r="55" spans="1:2">
       <c r="A55" s="2">
-        <v>46218.55208333334</v>
+        <v>46220.55208333334</v>
       </c>
       <c r="B55">
-        <v>437</v>
+        <v>554</v>
       </c>
     </row>
     <row r="56" spans="1:2">
       <c r="A56" s="2">
-        <v>46218.5625</v>
+        <v>46220.5625</v>
       </c>
       <c r="B56">
-        <v>437</v>
+        <v>555</v>
       </c>
     </row>
     <row r="57" spans="1:2">
       <c r="A57" s="2">
-        <v>46218.57291666666</v>
+        <v>46220.57291666666</v>
       </c>
       <c r="B57">
-        <v>439</v>
+        <v>554</v>
       </c>
     </row>
     <row r="58" spans="1:2">
       <c r="A58" s="2">
-        <v>46218.58333333334</v>
+        <v>46220.58333333334</v>
       </c>
       <c r="B58">
-        <v>497</v>
+        <v>508</v>
       </c>
     </row>
     <row r="59" spans="1:2">
       <c r="A59" s="2">
-        <v>46218.59375</v>
+        <v>46220.59375</v>
       </c>
       <c r="B59">
-        <v>474</v>
+        <v>506</v>
       </c>
     </row>
     <row r="60" spans="1:2">
       <c r="A60" s="2">
-        <v>46218.60416666666</v>
+        <v>46220.60416666666</v>
       </c>
       <c r="B60">
-        <v>509</v>
+        <v>496</v>
       </c>
     </row>
     <row r="61" spans="1:2">
       <c r="A61" s="2">
-        <v>46218.61458333334</v>
+        <v>46220.61458333334</v>
       </c>
       <c r="B61">
-        <v>513</v>
+        <v>490</v>
       </c>
     </row>
     <row r="62" spans="1:2">
       <c r="A62" s="2">
-        <v>46218.625</v>
+        <v>46220.625</v>
       </c>
       <c r="B62">
-        <v>575</v>
+        <v>568</v>
       </c>
     </row>
     <row r="63" spans="1:2">
       <c r="A63" s="2">
-        <v>46218.63541666666</v>
+        <v>46220.63541666666</v>
       </c>
       <c r="B63">
         <v>579</v>
@@ -890,610 +890,2058 @@
     </row>
     <row r="64" spans="1:2">
       <c r="A64" s="2">
-        <v>46218.64583333334</v>
+        <v>46220.64583333334</v>
       </c>
       <c r="B64">
-        <v>662</v>
+        <v>557</v>
       </c>
     </row>
     <row r="65" spans="1:2">
       <c r="A65" s="2">
-        <v>46218.65625</v>
+        <v>46220.65625</v>
       </c>
       <c r="B65">
-        <v>760</v>
+        <v>557</v>
       </c>
     </row>
     <row r="66" spans="1:2">
       <c r="A66" s="2">
-        <v>46218.66666666666</v>
+        <v>46220.66666666666</v>
       </c>
       <c r="B66">
-        <v>793</v>
+        <v>600</v>
       </c>
     </row>
     <row r="67" spans="1:2">
       <c r="A67" s="2">
-        <v>46218.67708333334</v>
+        <v>46220.67708333334</v>
       </c>
       <c r="B67">
-        <v>811</v>
+        <v>632</v>
       </c>
     </row>
     <row r="68" spans="1:2">
       <c r="A68" s="2">
-        <v>46218.6875</v>
+        <v>46220.6875</v>
       </c>
       <c r="B68">
-        <v>700</v>
+        <v>640</v>
       </c>
     </row>
     <row r="69" spans="1:2">
       <c r="A69" s="2">
-        <v>46218.69791666666</v>
+        <v>46220.69791666666</v>
       </c>
       <c r="B69">
-        <v>694</v>
+        <v>649</v>
       </c>
     </row>
     <row r="70" spans="1:2">
       <c r="A70" s="2">
-        <v>46218.70833333334</v>
+        <v>46220.70833333334</v>
       </c>
       <c r="B70">
-        <v>740</v>
+        <v>656</v>
       </c>
     </row>
     <row r="71" spans="1:2">
       <c r="A71" s="2">
-        <v>46218.71875</v>
+        <v>46220.71875</v>
       </c>
       <c r="B71">
-        <v>669</v>
+        <v>662</v>
       </c>
     </row>
     <row r="72" spans="1:2">
       <c r="A72" s="2">
-        <v>46218.72916666666</v>
+        <v>46220.72916666666</v>
       </c>
       <c r="B72">
-        <v>637</v>
+        <v>669</v>
       </c>
     </row>
     <row r="73" spans="1:2">
       <c r="A73" s="2">
-        <v>46218.73958333334</v>
+        <v>46220.73958333334</v>
       </c>
       <c r="B73">
-        <v>635</v>
+        <v>671</v>
       </c>
     </row>
     <row r="74" spans="1:2">
       <c r="A74" s="2">
-        <v>46218.75</v>
+        <v>46220.75</v>
       </c>
       <c r="B74">
-        <v>635</v>
+        <v>698</v>
       </c>
     </row>
     <row r="75" spans="1:2">
       <c r="A75" s="2">
-        <v>46218.76041666666</v>
+        <v>46220.76041666666</v>
       </c>
       <c r="B75">
-        <v>606</v>
+        <v>702</v>
       </c>
     </row>
     <row r="76" spans="1:2">
       <c r="A76" s="2">
-        <v>46218.77083333334</v>
+        <v>46220.77083333334</v>
       </c>
       <c r="B76">
-        <v>601</v>
+        <v>701</v>
       </c>
     </row>
     <row r="77" spans="1:2">
       <c r="A77" s="2">
-        <v>46218.78125</v>
+        <v>46220.78125</v>
       </c>
       <c r="B77">
-        <v>603</v>
+        <v>704</v>
       </c>
     </row>
     <row r="78" spans="1:2">
       <c r="A78" s="2">
-        <v>46218.79166666666</v>
+        <v>46220.79166666666</v>
       </c>
       <c r="B78">
-        <v>662</v>
+        <v>698</v>
       </c>
     </row>
     <row r="79" spans="1:2">
       <c r="A79" s="2">
-        <v>46218.80208333334</v>
+        <v>46220.80208333334</v>
       </c>
       <c r="B79">
-        <v>667</v>
+        <v>701</v>
       </c>
     </row>
     <row r="80" spans="1:2">
       <c r="A80" s="2">
-        <v>46218.8125</v>
+        <v>46220.8125</v>
       </c>
       <c r="B80">
-        <v>684</v>
+        <v>704</v>
       </c>
     </row>
     <row r="81" spans="1:2">
       <c r="A81" s="2">
-        <v>46218.82291666666</v>
+        <v>46220.82291666666</v>
       </c>
       <c r="B81">
-        <v>687</v>
+        <v>705</v>
       </c>
     </row>
     <row r="82" spans="1:2">
       <c r="A82" s="2">
-        <v>46218.83333333334</v>
+        <v>46220.83333333334</v>
       </c>
       <c r="B82">
-        <v>781</v>
+        <v>719</v>
       </c>
     </row>
     <row r="83" spans="1:2">
       <c r="A83" s="2">
-        <v>46218.84375</v>
+        <v>46220.84375</v>
       </c>
       <c r="B83">
-        <v>788</v>
+        <v>719</v>
       </c>
     </row>
     <row r="84" spans="1:2">
       <c r="A84" s="2">
-        <v>46218.85416666666</v>
+        <v>46220.85416666666</v>
       </c>
       <c r="B84">
-        <v>788</v>
+        <v>720</v>
       </c>
     </row>
     <row r="85" spans="1:2">
       <c r="A85" s="2">
-        <v>46218.86458333334</v>
+        <v>46220.86458333334</v>
       </c>
       <c r="B85">
-        <v>788</v>
+        <v>735</v>
       </c>
     </row>
     <row r="86" spans="1:2">
       <c r="A86" s="2">
-        <v>46218.875</v>
+        <v>46220.875</v>
       </c>
       <c r="B86">
-        <v>642</v>
+        <v>852</v>
       </c>
     </row>
     <row r="87" spans="1:2">
       <c r="A87" s="2">
-        <v>46218.88541666666</v>
+        <v>46220.88541666666</v>
       </c>
       <c r="B87">
-        <v>640</v>
+        <v>853</v>
       </c>
     </row>
     <row r="88" spans="1:2">
       <c r="A88" s="2">
-        <v>46218.89583333334</v>
+        <v>46220.89583333334</v>
       </c>
       <c r="B88">
-        <v>650</v>
+        <v>768</v>
       </c>
     </row>
     <row r="89" spans="1:2">
       <c r="A89" s="2">
-        <v>46218.90625</v>
+        <v>46220.90625</v>
       </c>
       <c r="B89">
-        <v>650</v>
+        <v>756</v>
       </c>
     </row>
     <row r="90" spans="1:2">
       <c r="A90" s="2">
-        <v>46218.91666666666</v>
+        <v>46220.91666666666</v>
       </c>
       <c r="B90">
-        <v>603</v>
+        <v>661</v>
       </c>
     </row>
     <row r="91" spans="1:2">
       <c r="A91" s="2">
-        <v>46218.92708333334</v>
+        <v>46220.92708333334</v>
       </c>
       <c r="B91">
-        <v>591</v>
+        <v>639</v>
       </c>
     </row>
     <row r="92" spans="1:2">
       <c r="A92" s="2">
-        <v>46218.9375</v>
+        <v>46220.9375</v>
       </c>
       <c r="B92">
-        <v>592</v>
+        <v>636</v>
       </c>
     </row>
     <row r="93" spans="1:2">
       <c r="A93" s="2">
-        <v>46218.94791666666</v>
+        <v>46220.94791666666</v>
       </c>
       <c r="B93">
-        <v>591</v>
+        <v>638</v>
       </c>
     </row>
     <row r="94" spans="1:2">
       <c r="A94" s="2">
-        <v>46218.95833333334</v>
+        <v>46220.95833333334</v>
       </c>
       <c r="B94">
-        <v>561</v>
+        <v>697</v>
       </c>
     </row>
     <row r="95" spans="1:2">
       <c r="A95" s="2">
-        <v>46218.96875</v>
+        <v>46220.96875</v>
       </c>
       <c r="B95">
-        <v>558</v>
+        <v>702</v>
       </c>
     </row>
     <row r="96" spans="1:2">
       <c r="A96" s="2">
-        <v>46218.97916666666</v>
+        <v>46220.97916666666</v>
       </c>
       <c r="B96">
-        <v>555</v>
+        <v>702</v>
       </c>
     </row>
     <row r="97" spans="1:2">
       <c r="A97" s="2">
-        <v>46218.98958333334</v>
+        <v>46220.98958333334</v>
       </c>
       <c r="B97">
-        <v>556</v>
+        <v>694</v>
       </c>
     </row>
     <row r="98" spans="1:2">
       <c r="A98" s="2">
-        <v>46219</v>
+        <v>46221</v>
       </c>
       <c r="B98">
-        <v>491</v>
+        <v>686</v>
       </c>
     </row>
     <row r="99" spans="1:2">
       <c r="A99" s="2">
-        <v>46219.01041666666</v>
+        <v>46221.01041666666</v>
       </c>
       <c r="B99">
-        <v>484</v>
+        <v>678</v>
       </c>
     </row>
     <row r="100" spans="1:2">
       <c r="A100" s="2">
-        <v>46219.02083333334</v>
+        <v>46221.02083333334</v>
       </c>
       <c r="B100">
-        <v>479</v>
+        <v>679</v>
       </c>
     </row>
     <row r="101" spans="1:2">
       <c r="A101" s="2">
-        <v>46219.03125</v>
+        <v>46221.03125</v>
       </c>
       <c r="B101">
-        <v>483</v>
+        <v>677</v>
       </c>
     </row>
     <row r="102" spans="1:2">
       <c r="A102" s="2">
-        <v>46219.04166666666</v>
+        <v>46221.04166666666</v>
       </c>
       <c r="B102">
-        <v>485</v>
+        <v>680</v>
       </c>
     </row>
     <row r="103" spans="1:2">
       <c r="A103" s="2">
-        <v>46219.05208333334</v>
+        <v>46221.05208333334</v>
       </c>
       <c r="B103">
-        <v>484</v>
+        <v>678</v>
       </c>
     </row>
     <row r="104" spans="1:2">
       <c r="A104" s="2">
-        <v>46219.0625</v>
+        <v>46221.0625</v>
       </c>
       <c r="B104">
-        <v>484</v>
+        <v>678</v>
       </c>
     </row>
     <row r="105" spans="1:2">
       <c r="A105" s="2">
-        <v>46219.07291666666</v>
+        <v>46221.07291666666</v>
       </c>
       <c r="B105">
-        <v>484</v>
+        <v>678</v>
       </c>
     </row>
     <row r="106" spans="1:2">
       <c r="A106" s="2">
-        <v>46219.08333333334</v>
+        <v>46221.08333333334</v>
       </c>
       <c r="B106">
-        <v>485</v>
+        <v>677</v>
       </c>
     </row>
     <row r="107" spans="1:2">
       <c r="A107" s="2">
-        <v>46219.09375</v>
+        <v>46221.09375</v>
       </c>
       <c r="B107">
-        <v>484</v>
+        <v>677</v>
       </c>
     </row>
     <row r="108" spans="1:2">
       <c r="A108" s="2">
-        <v>46219.10416666666</v>
+        <v>46221.10416666666</v>
       </c>
       <c r="B108">
-        <v>484</v>
+        <v>678</v>
       </c>
     </row>
     <row r="109" spans="1:2">
       <c r="A109" s="2">
-        <v>46219.11458333334</v>
+        <v>46221.11458333334</v>
       </c>
       <c r="B109">
-        <v>484</v>
+        <v>675</v>
       </c>
     </row>
     <row r="110" spans="1:2">
       <c r="A110" s="2">
-        <v>46219.125</v>
+        <v>46221.125</v>
       </c>
       <c r="B110">
-        <v>484</v>
+        <v>681</v>
       </c>
     </row>
     <row r="111" spans="1:2">
       <c r="A111" s="2">
-        <v>46219.13541666666</v>
+        <v>46221.13541666666</v>
       </c>
       <c r="B111">
-        <v>484</v>
+        <v>681</v>
       </c>
     </row>
     <row r="112" spans="1:2">
       <c r="A112" s="2">
-        <v>46219.14583333334</v>
+        <v>46221.14583333334</v>
       </c>
       <c r="B112">
-        <v>484</v>
+        <v>684</v>
       </c>
     </row>
     <row r="113" spans="1:2">
       <c r="A113" s="2">
-        <v>46219.15625</v>
+        <v>46221.15625</v>
       </c>
       <c r="B113">
-        <v>484</v>
+        <v>684</v>
       </c>
     </row>
     <row r="114" spans="1:2">
       <c r="A114" s="2">
-        <v>46219.16666666666</v>
+        <v>46221.16666666666</v>
       </c>
       <c r="B114">
-        <v>483</v>
+        <v>686</v>
       </c>
     </row>
     <row r="115" spans="1:2">
       <c r="A115" s="2">
-        <v>46219.17708333334</v>
+        <v>46221.17708333334</v>
       </c>
       <c r="B115">
-        <v>484</v>
+        <v>683</v>
       </c>
     </row>
     <row r="116" spans="1:2">
       <c r="A116" s="2">
-        <v>46219.1875</v>
+        <v>46221.1875</v>
       </c>
       <c r="B116">
-        <v>484</v>
+        <v>684</v>
       </c>
     </row>
     <row r="117" spans="1:2">
       <c r="A117" s="2">
-        <v>46219.19791666666</v>
+        <v>46221.19791666666</v>
       </c>
       <c r="B117">
-        <v>485</v>
+        <v>684</v>
       </c>
     </row>
     <row r="118" spans="1:2">
       <c r="A118" s="2">
-        <v>46219.20833333334</v>
+        <v>46221.20833333334</v>
       </c>
       <c r="B118">
-        <v>510</v>
+        <v>685</v>
       </c>
     </row>
     <row r="119" spans="1:2">
       <c r="A119" s="2">
-        <v>46219.21875</v>
+        <v>46221.21875</v>
       </c>
       <c r="B119">
-        <v>512</v>
+        <v>690</v>
       </c>
     </row>
     <row r="120" spans="1:2">
       <c r="A120" s="2">
-        <v>46219.22916666666</v>
+        <v>46221.22916666666</v>
       </c>
       <c r="B120">
-        <v>512</v>
+        <v>689</v>
       </c>
     </row>
     <row r="121" spans="1:2">
       <c r="A121" s="2">
-        <v>46219.23958333334</v>
+        <v>46221.23958333334</v>
       </c>
       <c r="B121">
-        <v>515</v>
+        <v>688</v>
       </c>
     </row>
     <row r="122" spans="1:2">
       <c r="A122" s="2">
-        <v>46219.25</v>
+        <v>46221.25</v>
       </c>
       <c r="B122">
-        <v>561</v>
+        <v>745</v>
       </c>
     </row>
     <row r="123" spans="1:2">
       <c r="A123" s="2">
-        <v>46219.26041666666</v>
+        <v>46221.26041666666</v>
       </c>
       <c r="B123">
-        <v>566</v>
+        <v>741</v>
       </c>
     </row>
     <row r="124" spans="1:2">
       <c r="A124" s="2">
-        <v>46219.27083333334</v>
+        <v>46221.27083333334</v>
       </c>
       <c r="B124">
-        <v>593</v>
+        <v>737</v>
       </c>
     </row>
     <row r="125" spans="1:2">
       <c r="A125" s="2">
-        <v>46219.28125</v>
+        <v>46221.28125</v>
       </c>
       <c r="B125">
-        <v>595</v>
+        <v>734</v>
       </c>
     </row>
     <row r="126" spans="1:2">
       <c r="A126" s="2">
-        <v>46219.29166666666</v>
+        <v>46221.29166666666</v>
       </c>
       <c r="B126">
-        <v>592</v>
+        <v>752</v>
       </c>
     </row>
     <row r="127" spans="1:2">
       <c r="A127" s="2">
-        <v>46219.30208333334</v>
+        <v>46221.30208333334</v>
       </c>
       <c r="B127">
-        <v>593</v>
+        <v>750</v>
       </c>
     </row>
     <row r="128" spans="1:2">
       <c r="A128" s="2">
-        <v>46219.3125</v>
+        <v>46221.3125</v>
       </c>
       <c r="B128">
-        <v>587</v>
+        <v>750</v>
       </c>
     </row>
     <row r="129" spans="1:2">
       <c r="A129" s="2">
-        <v>46219.32291666666</v>
+        <v>46221.32291666666</v>
       </c>
       <c r="B129">
-        <v>558</v>
+        <v>750</v>
       </c>
     </row>
     <row r="130" spans="1:2">
       <c r="A130" s="2">
-        <v>46219.33333333334</v>
+        <v>46221.33333333334</v>
       </c>
       <c r="B130">
-        <v>554</v>
+        <v>756</v>
       </c>
     </row>
     <row r="131" spans="1:2">
       <c r="A131" s="2">
-        <v>46219.34375</v>
+        <v>46221.34375</v>
       </c>
       <c r="B131">
-        <v>556</v>
+        <v>753</v>
       </c>
     </row>
     <row r="132" spans="1:2">
       <c r="A132" s="2">
-        <v>46219.35416666666</v>
+        <v>46221.35416666666</v>
       </c>
       <c r="B132">
-        <v>582</v>
+        <v>752</v>
       </c>
     </row>
     <row r="133" spans="1:2">
       <c r="A133" s="2">
-        <v>46219.36458333334</v>
+        <v>46221.36458333334</v>
       </c>
       <c r="B133">
-        <v>584</v>
+        <v>750</v>
       </c>
     </row>
     <row r="134" spans="1:2">
       <c r="A134" s="2">
-        <v>46219.375</v>
+        <v>46221.375</v>
       </c>
       <c r="B134">
-        <v>552</v>
+        <v>540</v>
       </c>
     </row>
     <row r="135" spans="1:2">
       <c r="A135" s="2">
-        <v>46219.38541666666</v>
+        <v>46221.38541666666</v>
       </c>
       <c r="B135">
-        <v>540</v>
+        <v>506</v>
       </c>
     </row>
     <row r="136" spans="1:2">
       <c r="A136" s="2">
-        <v>46219.39583333334</v>
+        <v>46221.39583333334</v>
       </c>
       <c r="B136">
-        <v>548</v>
+        <v>505</v>
       </c>
     </row>
     <row r="137" spans="1:2">
       <c r="A137" s="2">
-        <v>46219.40625</v>
+        <v>46221.40625</v>
       </c>
       <c r="B137">
-        <v>553</v>
+        <v>502</v>
       </c>
     </row>
     <row r="138" spans="1:2">
       <c r="A138" s="2">
-        <v>46219.41666666666</v>
+        <v>46221.41666666666</v>
       </c>
       <c r="B138">
-        <v>420</v>
+        <v>472</v>
       </c>
     </row>
     <row r="139" spans="1:2">
       <c r="A139" s="2">
-        <v>46219.42708333334</v>
+        <v>46221.42708333334</v>
       </c>
       <c r="B139">
-        <v>461</v>
+        <v>470</v>
+      </c>
+    </row>
+    <row r="140" spans="1:2">
+      <c r="A140" s="2">
+        <v>46221.4375</v>
+      </c>
+      <c r="B140">
+        <v>471</v>
+      </c>
+    </row>
+    <row r="141" spans="1:2">
+      <c r="A141" s="2">
+        <v>46221.44791666666</v>
+      </c>
+      <c r="B141">
+        <v>471</v>
+      </c>
+    </row>
+    <row r="142" spans="1:2">
+      <c r="A142" s="2">
+        <v>46221.45833333334</v>
+      </c>
+      <c r="B142">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="143" spans="1:2">
+      <c r="A143" s="2">
+        <v>46221.46875</v>
+      </c>
+      <c r="B143">
+        <v>419</v>
+      </c>
+    </row>
+    <row r="144" spans="1:2">
+      <c r="A144" s="2">
+        <v>46221.47916666666</v>
+      </c>
+      <c r="B144">
+        <v>419</v>
+      </c>
+    </row>
+    <row r="145" spans="1:2">
+      <c r="A145" s="2">
+        <v>46221.48958333334</v>
+      </c>
+      <c r="B145">
+        <v>420</v>
+      </c>
+    </row>
+    <row r="146" spans="1:2">
+      <c r="A146" s="2">
+        <v>46221.5</v>
+      </c>
+      <c r="B146">
+        <v>405</v>
+      </c>
+    </row>
+    <row r="147" spans="1:2">
+      <c r="A147" s="2">
+        <v>46221.51041666666</v>
+      </c>
+      <c r="B147">
+        <v>406</v>
+      </c>
+    </row>
+    <row r="148" spans="1:2">
+      <c r="A148" s="2">
+        <v>46221.52083333334</v>
+      </c>
+      <c r="B148">
+        <v>406</v>
+      </c>
+    </row>
+    <row r="149" spans="1:2">
+      <c r="A149" s="2">
+        <v>46221.53125</v>
+      </c>
+      <c r="B149">
+        <v>406</v>
+      </c>
+    </row>
+    <row r="150" spans="1:2">
+      <c r="A150" s="2">
+        <v>46221.54166666666</v>
+      </c>
+      <c r="B150">
+        <v>404</v>
+      </c>
+    </row>
+    <row r="151" spans="1:2">
+      <c r="A151" s="2">
+        <v>46221.55208333334</v>
+      </c>
+      <c r="B151">
+        <v>402</v>
+      </c>
+    </row>
+    <row r="152" spans="1:2">
+      <c r="A152" s="2">
+        <v>46221.5625</v>
+      </c>
+      <c r="B152">
+        <v>403</v>
+      </c>
+    </row>
+    <row r="153" spans="1:2">
+      <c r="A153" s="2">
+        <v>46221.57291666666</v>
+      </c>
+      <c r="B153">
+        <v>405</v>
+      </c>
+    </row>
+    <row r="154" spans="1:2">
+      <c r="A154" s="2">
+        <v>46221.58333333334</v>
+      </c>
+      <c r="B154">
+        <v>424</v>
+      </c>
+    </row>
+    <row r="155" spans="1:2">
+      <c r="A155" s="2">
+        <v>46221.59375</v>
+      </c>
+      <c r="B155">
+        <v>419</v>
+      </c>
+    </row>
+    <row r="156" spans="1:2">
+      <c r="A156" s="2">
+        <v>46221.60416666666</v>
+      </c>
+      <c r="B156">
+        <v>425</v>
+      </c>
+    </row>
+    <row r="157" spans="1:2">
+      <c r="A157" s="2">
+        <v>46221.61458333334</v>
+      </c>
+      <c r="B157">
+        <v>437</v>
+      </c>
+    </row>
+    <row r="158" spans="1:2">
+      <c r="A158" s="2">
+        <v>46221.625</v>
+      </c>
+      <c r="B158">
+        <v>541</v>
+      </c>
+    </row>
+    <row r="159" spans="1:2">
+      <c r="A159" s="2">
+        <v>46221.63541666666</v>
+      </c>
+      <c r="B159">
+        <v>586</v>
+      </c>
+    </row>
+    <row r="160" spans="1:2">
+      <c r="A160" s="2">
+        <v>46221.64583333334</v>
+      </c>
+      <c r="B160">
+        <v>589</v>
+      </c>
+    </row>
+    <row r="161" spans="1:2">
+      <c r="A161" s="2">
+        <v>46221.65625</v>
+      </c>
+      <c r="B161">
+        <v>490</v>
+      </c>
+    </row>
+    <row r="162" spans="1:2">
+      <c r="A162" s="2">
+        <v>46221.66666666666</v>
+      </c>
+      <c r="B162">
+        <v>512</v>
+      </c>
+    </row>
+    <row r="163" spans="1:2">
+      <c r="A163" s="2">
+        <v>46221.67708333334</v>
+      </c>
+      <c r="B163">
+        <v>511</v>
+      </c>
+    </row>
+    <row r="164" spans="1:2">
+      <c r="A164" s="2">
+        <v>46221.6875</v>
+      </c>
+      <c r="B164">
+        <v>493</v>
+      </c>
+    </row>
+    <row r="165" spans="1:2">
+      <c r="A165" s="2">
+        <v>46221.69791666666</v>
+      </c>
+      <c r="B165">
+        <v>501</v>
+      </c>
+    </row>
+    <row r="166" spans="1:2">
+      <c r="A166" s="2">
+        <v>46221.70833333334</v>
+      </c>
+      <c r="B166">
+        <v>703</v>
+      </c>
+    </row>
+    <row r="167" spans="1:2">
+      <c r="A167" s="2">
+        <v>46221.71875</v>
+      </c>
+      <c r="B167">
+        <v>716</v>
+      </c>
+    </row>
+    <row r="168" spans="1:2">
+      <c r="A168" s="2">
+        <v>46221.72916666666</v>
+      </c>
+      <c r="B168">
+        <v>714</v>
+      </c>
+    </row>
+    <row r="169" spans="1:2">
+      <c r="A169" s="2">
+        <v>46221.73958333334</v>
+      </c>
+      <c r="B169">
+        <v>716</v>
+      </c>
+    </row>
+    <row r="170" spans="1:2">
+      <c r="A170" s="2">
+        <v>46221.75</v>
+      </c>
+      <c r="B170">
+        <v>778</v>
+      </c>
+    </row>
+    <row r="171" spans="1:2">
+      <c r="A171" s="2">
+        <v>46221.76041666666</v>
+      </c>
+      <c r="B171">
+        <v>785</v>
+      </c>
+    </row>
+    <row r="172" spans="1:2">
+      <c r="A172" s="2">
+        <v>46221.77083333334</v>
+      </c>
+      <c r="B172">
+        <v>763</v>
+      </c>
+    </row>
+    <row r="173" spans="1:2">
+      <c r="A173" s="2">
+        <v>46221.78125</v>
+      </c>
+      <c r="B173">
+        <v>763</v>
+      </c>
+    </row>
+    <row r="174" spans="1:2">
+      <c r="A174" s="2">
+        <v>46221.79166666666</v>
+      </c>
+      <c r="B174">
+        <v>770</v>
+      </c>
+    </row>
+    <row r="175" spans="1:2">
+      <c r="A175" s="2">
+        <v>46221.80208333334</v>
+      </c>
+      <c r="B175">
+        <v>774</v>
+      </c>
+    </row>
+    <row r="176" spans="1:2">
+      <c r="A176" s="2">
+        <v>46221.8125</v>
+      </c>
+      <c r="B176">
+        <v>773</v>
+      </c>
+    </row>
+    <row r="177" spans="1:2">
+      <c r="A177" s="2">
+        <v>46221.82291666666</v>
+      </c>
+      <c r="B177">
+        <v>772</v>
+      </c>
+    </row>
+    <row r="178" spans="1:2">
+      <c r="A178" s="2">
+        <v>46221.83333333334</v>
+      </c>
+      <c r="B178">
+        <v>785</v>
+      </c>
+    </row>
+    <row r="179" spans="1:2">
+      <c r="A179" s="2">
+        <v>46221.84375</v>
+      </c>
+      <c r="B179">
+        <v>786</v>
+      </c>
+    </row>
+    <row r="180" spans="1:2">
+      <c r="A180" s="2">
+        <v>46221.85416666666</v>
+      </c>
+      <c r="B180">
+        <v>784</v>
+      </c>
+    </row>
+    <row r="181" spans="1:2">
+      <c r="A181" s="2">
+        <v>46221.86458333334</v>
+      </c>
+      <c r="B181">
+        <v>788</v>
+      </c>
+    </row>
+    <row r="182" spans="1:2">
+      <c r="A182" s="2">
+        <v>46221.875</v>
+      </c>
+      <c r="B182">
+        <v>767</v>
+      </c>
+    </row>
+    <row r="183" spans="1:2">
+      <c r="A183" s="2">
+        <v>46221.88541666666</v>
+      </c>
+      <c r="B183">
+        <v>759</v>
+      </c>
+    </row>
+    <row r="184" spans="1:2">
+      <c r="A184" s="2">
+        <v>46221.89583333334</v>
+      </c>
+      <c r="B184">
+        <v>759</v>
+      </c>
+    </row>
+    <row r="185" spans="1:2">
+      <c r="A185" s="2">
+        <v>46221.90625</v>
+      </c>
+      <c r="B185">
+        <v>760</v>
+      </c>
+    </row>
+    <row r="186" spans="1:2">
+      <c r="A186" s="2">
+        <v>46221.91666666666</v>
+      </c>
+      <c r="B186">
+        <v>760</v>
+      </c>
+    </row>
+    <row r="187" spans="1:2">
+      <c r="A187" s="2">
+        <v>46221.92708333334</v>
+      </c>
+      <c r="B187">
+        <v>758</v>
+      </c>
+    </row>
+    <row r="188" spans="1:2">
+      <c r="A188" s="2">
+        <v>46221.9375</v>
+      </c>
+      <c r="B188">
+        <v>760</v>
+      </c>
+    </row>
+    <row r="189" spans="1:2">
+      <c r="A189" s="2">
+        <v>46221.94791666666</v>
+      </c>
+      <c r="B189">
+        <v>758</v>
+      </c>
+    </row>
+    <row r="190" spans="1:2">
+      <c r="A190" s="2">
+        <v>46221.95833333334</v>
+      </c>
+      <c r="B190">
+        <v>717</v>
+      </c>
+    </row>
+    <row r="191" spans="1:2">
+      <c r="A191" s="2">
+        <v>46221.96875</v>
+      </c>
+      <c r="B191">
+        <v>709</v>
+      </c>
+    </row>
+    <row r="192" spans="1:2">
+      <c r="A192" s="2">
+        <v>46221.97916666666</v>
+      </c>
+      <c r="B192">
+        <v>710</v>
+      </c>
+    </row>
+    <row r="193" spans="1:2">
+      <c r="A193" s="2">
+        <v>46221.98958333334</v>
+      </c>
+      <c r="B193">
+        <v>709</v>
+      </c>
+    </row>
+    <row r="194" spans="1:2">
+      <c r="A194" s="2">
+        <v>46222</v>
+      </c>
+      <c r="B194">
+        <v>674</v>
+      </c>
+    </row>
+    <row r="195" spans="1:2">
+      <c r="A195" s="2">
+        <v>46222.01041666666</v>
+      </c>
+      <c r="B195">
+        <v>665</v>
+      </c>
+    </row>
+    <row r="196" spans="1:2">
+      <c r="A196" s="2">
+        <v>46222.02083333334</v>
+      </c>
+      <c r="B196">
+        <v>672</v>
+      </c>
+    </row>
+    <row r="197" spans="1:2">
+      <c r="A197" s="2">
+        <v>46222.03125</v>
+      </c>
+      <c r="B197">
+        <v>671</v>
+      </c>
+    </row>
+    <row r="198" spans="1:2">
+      <c r="A198" s="2">
+        <v>46222.04166666666</v>
+      </c>
+      <c r="B198">
+        <v>625</v>
+      </c>
+    </row>
+    <row r="199" spans="1:2">
+      <c r="A199" s="2">
+        <v>46222.05208333334</v>
+      </c>
+      <c r="B199">
+        <v>623</v>
+      </c>
+    </row>
+    <row r="200" spans="1:2">
+      <c r="A200" s="2">
+        <v>46222.0625</v>
+      </c>
+      <c r="B200">
+        <v>622</v>
+      </c>
+    </row>
+    <row r="201" spans="1:2">
+      <c r="A201" s="2">
+        <v>46222.07291666666</v>
+      </c>
+      <c r="B201">
+        <v>622</v>
+      </c>
+    </row>
+    <row r="202" spans="1:2">
+      <c r="A202" s="2">
+        <v>46222.08333333334</v>
+      </c>
+      <c r="B202">
+        <v>650</v>
+      </c>
+    </row>
+    <row r="203" spans="1:2">
+      <c r="A203" s="2">
+        <v>46222.09375</v>
+      </c>
+      <c r="B203">
+        <v>651</v>
+      </c>
+    </row>
+    <row r="204" spans="1:2">
+      <c r="A204" s="2">
+        <v>46222.10416666666</v>
+      </c>
+      <c r="B204">
+        <v>652</v>
+      </c>
+    </row>
+    <row r="205" spans="1:2">
+      <c r="A205" s="2">
+        <v>46222.11458333334</v>
+      </c>
+      <c r="B205">
+        <v>651</v>
+      </c>
+    </row>
+    <row r="206" spans="1:2">
+      <c r="A206" s="2">
+        <v>46222.125</v>
+      </c>
+      <c r="B206">
+        <v>622</v>
+      </c>
+    </row>
+    <row r="207" spans="1:2">
+      <c r="A207" s="2">
+        <v>46222.13541666666</v>
+      </c>
+      <c r="B207">
+        <v>621</v>
+      </c>
+    </row>
+    <row r="208" spans="1:2">
+      <c r="A208" s="2">
+        <v>46222.14583333334</v>
+      </c>
+      <c r="B208">
+        <v>622</v>
+      </c>
+    </row>
+    <row r="209" spans="1:2">
+      <c r="A209" s="2">
+        <v>46222.15625</v>
+      </c>
+      <c r="B209">
+        <v>622</v>
+      </c>
+    </row>
+    <row r="210" spans="1:2">
+      <c r="A210" s="2">
+        <v>46222.16666666666</v>
+      </c>
+      <c r="B210">
+        <v>623</v>
+      </c>
+    </row>
+    <row r="211" spans="1:2">
+      <c r="A211" s="2">
+        <v>46222.17708333334</v>
+      </c>
+      <c r="B211">
+        <v>625</v>
+      </c>
+    </row>
+    <row r="212" spans="1:2">
+      <c r="A212" s="2">
+        <v>46222.1875</v>
+      </c>
+      <c r="B212">
+        <v>644</v>
+      </c>
+    </row>
+    <row r="213" spans="1:2">
+      <c r="A213" s="2">
+        <v>46222.19791666666</v>
+      </c>
+      <c r="B213">
+        <v>646</v>
+      </c>
+    </row>
+    <row r="214" spans="1:2">
+      <c r="A214" s="2">
+        <v>46222.20833333334</v>
+      </c>
+      <c r="B214">
+        <v>688</v>
+      </c>
+    </row>
+    <row r="215" spans="1:2">
+      <c r="A215" s="2">
+        <v>46222.21875</v>
+      </c>
+      <c r="B215">
+        <v>689</v>
+      </c>
+    </row>
+    <row r="216" spans="1:2">
+      <c r="A216" s="2">
+        <v>46222.22916666666</v>
+      </c>
+      <c r="B216">
+        <v>686</v>
+      </c>
+    </row>
+    <row r="217" spans="1:2">
+      <c r="A217" s="2">
+        <v>46222.23958333334</v>
+      </c>
+      <c r="B217">
+        <v>687</v>
+      </c>
+    </row>
+    <row r="218" spans="1:2">
+      <c r="A218" s="2">
+        <v>46222.25</v>
+      </c>
+      <c r="B218">
+        <v>816</v>
+      </c>
+    </row>
+    <row r="219" spans="1:2">
+      <c r="A219" s="2">
+        <v>46222.26041666666</v>
+      </c>
+      <c r="B219">
+        <v>828</v>
+      </c>
+    </row>
+    <row r="220" spans="1:2">
+      <c r="A220" s="2">
+        <v>46222.27083333334</v>
+      </c>
+      <c r="B220">
+        <v>827</v>
+      </c>
+    </row>
+    <row r="221" spans="1:2">
+      <c r="A221" s="2">
+        <v>46222.28125</v>
+      </c>
+      <c r="B221">
+        <v>820</v>
+      </c>
+    </row>
+    <row r="222" spans="1:2">
+      <c r="A222" s="2">
+        <v>46222.29166666666</v>
+      </c>
+      <c r="B222">
+        <v>520</v>
+      </c>
+    </row>
+    <row r="223" spans="1:2">
+      <c r="A223" s="2">
+        <v>46222.30208333334</v>
+      </c>
+      <c r="B223">
+        <v>507</v>
+      </c>
+    </row>
+    <row r="224" spans="1:2">
+      <c r="A224" s="2">
+        <v>46222.3125</v>
+      </c>
+      <c r="B224">
+        <v>517</v>
+      </c>
+    </row>
+    <row r="225" spans="1:2">
+      <c r="A225" s="2">
+        <v>46222.32291666666</v>
+      </c>
+      <c r="B225">
+        <v>517</v>
+      </c>
+    </row>
+    <row r="226" spans="1:2">
+      <c r="A226" s="2">
+        <v>46222.33333333334</v>
+      </c>
+      <c r="B226">
+        <v>488</v>
+      </c>
+    </row>
+    <row r="227" spans="1:2">
+      <c r="A227" s="2">
+        <v>46222.34375</v>
+      </c>
+      <c r="B227">
+        <v>483</v>
+      </c>
+    </row>
+    <row r="228" spans="1:2">
+      <c r="A228" s="2">
+        <v>46222.35416666666</v>
+      </c>
+      <c r="B228">
+        <v>533</v>
+      </c>
+    </row>
+    <row r="229" spans="1:2">
+      <c r="A229" s="2">
+        <v>46222.36458333334</v>
+      </c>
+      <c r="B229">
+        <v>540</v>
+      </c>
+    </row>
+    <row r="230" spans="1:2">
+      <c r="A230" s="2">
+        <v>46222.375</v>
+      </c>
+      <c r="B230">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="231" spans="1:2">
+      <c r="A231" s="2">
+        <v>46222.38541666666</v>
+      </c>
+      <c r="B231">
+        <v>387</v>
+      </c>
+    </row>
+    <row r="232" spans="1:2">
+      <c r="A232" s="2">
+        <v>46222.39583333334</v>
+      </c>
+      <c r="B232">
+        <v>398</v>
+      </c>
+    </row>
+    <row r="233" spans="1:2">
+      <c r="A233" s="2">
+        <v>46222.40625</v>
+      </c>
+      <c r="B233">
+        <v>398</v>
+      </c>
+    </row>
+    <row r="234" spans="1:2">
+      <c r="A234" s="2">
+        <v>46222.41666666666</v>
+      </c>
+      <c r="B234">
+        <v>393</v>
+      </c>
+    </row>
+    <row r="235" spans="1:2">
+      <c r="A235" s="2">
+        <v>46222.42708333334</v>
+      </c>
+      <c r="B235">
+        <v>379</v>
+      </c>
+    </row>
+    <row r="236" spans="1:2">
+      <c r="A236" s="2">
+        <v>46222.4375</v>
+      </c>
+      <c r="B236">
+        <v>386</v>
+      </c>
+    </row>
+    <row r="237" spans="1:2">
+      <c r="A237" s="2">
+        <v>46222.44791666666</v>
+      </c>
+      <c r="B237">
+        <v>386</v>
+      </c>
+    </row>
+    <row r="238" spans="1:2">
+      <c r="A238" s="2">
+        <v>46222.45833333334</v>
+      </c>
+      <c r="B238">
+        <v>399</v>
+      </c>
+    </row>
+    <row r="239" spans="1:2">
+      <c r="A239" s="2">
+        <v>46222.46875</v>
+      </c>
+      <c r="B239">
+        <v>398</v>
+      </c>
+    </row>
+    <row r="240" spans="1:2">
+      <c r="A240" s="2">
+        <v>46222.47916666666</v>
+      </c>
+      <c r="B240">
+        <v>397</v>
+      </c>
+    </row>
+    <row r="241" spans="1:2">
+      <c r="A241" s="2">
+        <v>46222.48958333334</v>
+      </c>
+      <c r="B241">
+        <v>397</v>
+      </c>
+    </row>
+    <row r="242" spans="1:2">
+      <c r="A242" s="2">
+        <v>46222.5</v>
+      </c>
+      <c r="B242">
+        <v>405</v>
+      </c>
+    </row>
+    <row r="243" spans="1:2">
+      <c r="A243" s="2">
+        <v>46222.51041666666</v>
+      </c>
+      <c r="B243">
+        <v>407</v>
+      </c>
+    </row>
+    <row r="244" spans="1:2">
+      <c r="A244" s="2">
+        <v>46222.52083333334</v>
+      </c>
+      <c r="B244">
+        <v>406</v>
+      </c>
+    </row>
+    <row r="245" spans="1:2">
+      <c r="A245" s="2">
+        <v>46222.53125</v>
+      </c>
+      <c r="B245">
+        <v>407</v>
+      </c>
+    </row>
+    <row r="246" spans="1:2">
+      <c r="A246" s="2">
+        <v>46222.54166666666</v>
+      </c>
+      <c r="B246">
+        <v>425</v>
+      </c>
+    </row>
+    <row r="247" spans="1:2">
+      <c r="A247" s="2">
+        <v>46222.55208333334</v>
+      </c>
+      <c r="B247">
+        <v>427</v>
+      </c>
+    </row>
+    <row r="248" spans="1:2">
+      <c r="A248" s="2">
+        <v>46222.5625</v>
+      </c>
+      <c r="B248">
+        <v>427</v>
+      </c>
+    </row>
+    <row r="249" spans="1:2">
+      <c r="A249" s="2">
+        <v>46222.57291666666</v>
+      </c>
+      <c r="B249">
+        <v>427</v>
+      </c>
+    </row>
+    <row r="250" spans="1:2">
+      <c r="A250" s="2">
+        <v>46222.58333333334</v>
+      </c>
+      <c r="B250">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="251" spans="1:2">
+      <c r="A251" s="2">
+        <v>46222.59375</v>
+      </c>
+      <c r="B251">
+        <v>437</v>
+      </c>
+    </row>
+    <row r="252" spans="1:2">
+      <c r="A252" s="2">
+        <v>46222.60416666666</v>
+      </c>
+      <c r="B252">
+        <v>431</v>
+      </c>
+    </row>
+    <row r="253" spans="1:2">
+      <c r="A253" s="2">
+        <v>46222.61458333334</v>
+      </c>
+      <c r="B253">
+        <v>430</v>
+      </c>
+    </row>
+    <row r="254" spans="1:2">
+      <c r="A254" s="2">
+        <v>46222.625</v>
+      </c>
+      <c r="B254">
+        <v>428</v>
+      </c>
+    </row>
+    <row r="255" spans="1:2">
+      <c r="A255" s="2">
+        <v>46222.63541666666</v>
+      </c>
+      <c r="B255">
+        <v>450</v>
+      </c>
+    </row>
+    <row r="256" spans="1:2">
+      <c r="A256" s="2">
+        <v>46222.64583333334</v>
+      </c>
+      <c r="B256">
+        <v>451</v>
+      </c>
+    </row>
+    <row r="257" spans="1:2">
+      <c r="A257" s="2">
+        <v>46222.65625</v>
+      </c>
+      <c r="B257">
+        <v>454</v>
+      </c>
+    </row>
+    <row r="258" spans="1:2">
+      <c r="A258" s="2">
+        <v>46222.66666666666</v>
+      </c>
+      <c r="B258">
+        <v>524</v>
+      </c>
+    </row>
+    <row r="259" spans="1:2">
+      <c r="A259" s="2">
+        <v>46222.67708333334</v>
+      </c>
+      <c r="B259">
+        <v>546</v>
+      </c>
+    </row>
+    <row r="260" spans="1:2">
+      <c r="A260" s="2">
+        <v>46222.6875</v>
+      </c>
+      <c r="B260">
+        <v>546</v>
+      </c>
+    </row>
+    <row r="261" spans="1:2">
+      <c r="A261" s="2">
+        <v>46222.69791666666</v>
+      </c>
+      <c r="B261">
+        <v>552</v>
+      </c>
+    </row>
+    <row r="262" spans="1:2">
+      <c r="A262" s="2">
+        <v>46222.70833333334</v>
+      </c>
+      <c r="B262">
+        <v>635</v>
+      </c>
+    </row>
+    <row r="263" spans="1:2">
+      <c r="A263" s="2">
+        <v>46222.71875</v>
+      </c>
+      <c r="B263">
+        <v>637</v>
+      </c>
+    </row>
+    <row r="264" spans="1:2">
+      <c r="A264" s="2">
+        <v>46222.72916666666</v>
+      </c>
+      <c r="B264">
+        <v>639</v>
+      </c>
+    </row>
+    <row r="265" spans="1:2">
+      <c r="A265" s="2">
+        <v>46222.73958333334</v>
+      </c>
+      <c r="B265">
+        <v>643</v>
+      </c>
+    </row>
+    <row r="266" spans="1:2">
+      <c r="A266" s="2">
+        <v>46222.75</v>
+      </c>
+      <c r="B266">
+        <v>883</v>
+      </c>
+    </row>
+    <row r="267" spans="1:2">
+      <c r="A267" s="2">
+        <v>46222.76041666666</v>
+      </c>
+      <c r="B267">
+        <v>945</v>
+      </c>
+    </row>
+    <row r="268" spans="1:2">
+      <c r="A268" s="2">
+        <v>46222.77083333334</v>
+      </c>
+      <c r="B268">
+        <v>944</v>
+      </c>
+    </row>
+    <row r="269" spans="1:2">
+      <c r="A269" s="2">
+        <v>46222.78125</v>
+      </c>
+      <c r="B269">
+        <v>936</v>
+      </c>
+    </row>
+    <row r="270" spans="1:2">
+      <c r="A270" s="2">
+        <v>46222.79166666666</v>
+      </c>
+      <c r="B270">
+        <v>937</v>
+      </c>
+    </row>
+    <row r="271" spans="1:2">
+      <c r="A271" s="2">
+        <v>46222.80208333334</v>
+      </c>
+      <c r="B271">
+        <v>940</v>
+      </c>
+    </row>
+    <row r="272" spans="1:2">
+      <c r="A272" s="2">
+        <v>46222.8125</v>
+      </c>
+      <c r="B272">
+        <v>940</v>
+      </c>
+    </row>
+    <row r="273" spans="1:2">
+      <c r="A273" s="2">
+        <v>46222.82291666666</v>
+      </c>
+      <c r="B273">
+        <v>941</v>
+      </c>
+    </row>
+    <row r="274" spans="1:2">
+      <c r="A274" s="2">
+        <v>46222.83333333334</v>
+      </c>
+      <c r="B274">
+        <v>962</v>
+      </c>
+    </row>
+    <row r="275" spans="1:2">
+      <c r="A275" s="2">
+        <v>46222.84375</v>
+      </c>
+      <c r="B275">
+        <v>977</v>
+      </c>
+    </row>
+    <row r="276" spans="1:2">
+      <c r="A276" s="2">
+        <v>46222.85416666666</v>
+      </c>
+      <c r="B276">
+        <v>953</v>
+      </c>
+    </row>
+    <row r="277" spans="1:2">
+      <c r="A277" s="2">
+        <v>46222.86458333334</v>
+      </c>
+      <c r="B277">
+        <v>973</v>
+      </c>
+    </row>
+    <row r="278" spans="1:2">
+      <c r="A278" s="2">
+        <v>46222.875</v>
+      </c>
+      <c r="B278">
+        <v>961</v>
+      </c>
+    </row>
+    <row r="279" spans="1:2">
+      <c r="A279" s="2">
+        <v>46222.88541666666</v>
+      </c>
+      <c r="B279">
+        <v>964</v>
+      </c>
+    </row>
+    <row r="280" spans="1:2">
+      <c r="A280" s="2">
+        <v>46222.89583333334</v>
+      </c>
+      <c r="B280">
+        <v>963</v>
+      </c>
+    </row>
+    <row r="281" spans="1:2">
+      <c r="A281" s="2">
+        <v>46222.90625</v>
+      </c>
+      <c r="B281">
+        <v>960</v>
+      </c>
+    </row>
+    <row r="282" spans="1:2">
+      <c r="A282" s="2">
+        <v>46222.91666666666</v>
+      </c>
+      <c r="B282">
+        <v>960</v>
+      </c>
+    </row>
+    <row r="283" spans="1:2">
+      <c r="A283" s="2">
+        <v>46222.92708333334</v>
+      </c>
+      <c r="B283">
+        <v>969</v>
+      </c>
+    </row>
+    <row r="284" spans="1:2">
+      <c r="A284" s="2">
+        <v>46222.9375</v>
+      </c>
+      <c r="B284">
+        <v>971</v>
+      </c>
+    </row>
+    <row r="285" spans="1:2">
+      <c r="A285" s="2">
+        <v>46222.94791666666</v>
+      </c>
+      <c r="B285">
+        <v>968</v>
+      </c>
+    </row>
+    <row r="286" spans="1:2">
+      <c r="A286" s="2">
+        <v>46222.95833333334</v>
+      </c>
+      <c r="B286">
+        <v>949</v>
+      </c>
+    </row>
+    <row r="287" spans="1:2">
+      <c r="A287" s="2">
+        <v>46222.96875</v>
+      </c>
+      <c r="B287">
+        <v>947</v>
+      </c>
+    </row>
+    <row r="288" spans="1:2">
+      <c r="A288" s="2">
+        <v>46222.97916666666</v>
+      </c>
+      <c r="B288">
+        <v>942</v>
+      </c>
+    </row>
+    <row r="289" spans="1:2">
+      <c r="A289" s="2">
+        <v>46222.98958333334</v>
+      </c>
+      <c r="B289">
+        <v>939</v>
+      </c>
+    </row>
+    <row r="290" spans="1:2">
+      <c r="A290" s="2">
+        <v>46223</v>
+      </c>
+      <c r="B290">
+        <v>775</v>
+      </c>
+    </row>
+    <row r="291" spans="1:2">
+      <c r="A291" s="2">
+        <v>46223.01041666666</v>
+      </c>
+      <c r="B291">
+        <v>739</v>
+      </c>
+    </row>
+    <row r="292" spans="1:2">
+      <c r="A292" s="2">
+        <v>46223.02083333334</v>
+      </c>
+      <c r="B292">
+        <v>736</v>
+      </c>
+    </row>
+    <row r="293" spans="1:2">
+      <c r="A293" s="2">
+        <v>46223.03125</v>
+      </c>
+      <c r="B293">
+        <v>735</v>
+      </c>
+    </row>
+    <row r="294" spans="1:2">
+      <c r="A294" s="2">
+        <v>46223.04166666666</v>
+      </c>
+      <c r="B294">
+        <v>736</v>
+      </c>
+    </row>
+    <row r="295" spans="1:2">
+      <c r="A295" s="2">
+        <v>46223.05208333334</v>
+      </c>
+      <c r="B295">
+        <v>736</v>
+      </c>
+    </row>
+    <row r="296" spans="1:2">
+      <c r="A296" s="2">
+        <v>46223.0625</v>
+      </c>
+      <c r="B296">
+        <v>735</v>
+      </c>
+    </row>
+    <row r="297" spans="1:2">
+      <c r="A297" s="2">
+        <v>46223.07291666666</v>
+      </c>
+      <c r="B297">
+        <v>734</v>
+      </c>
+    </row>
+    <row r="298" spans="1:2">
+      <c r="A298" s="2">
+        <v>46223.08333333334</v>
+      </c>
+      <c r="B298">
+        <v>746</v>
+      </c>
+    </row>
+    <row r="299" spans="1:2">
+      <c r="A299" s="2">
+        <v>46223.09375</v>
+      </c>
+      <c r="B299">
+        <v>744</v>
+      </c>
+    </row>
+    <row r="300" spans="1:2">
+      <c r="A300" s="2">
+        <v>46223.10416666666</v>
+      </c>
+      <c r="B300">
+        <v>744</v>
+      </c>
+    </row>
+    <row r="301" spans="1:2">
+      <c r="A301" s="2">
+        <v>46223.11458333334</v>
+      </c>
+      <c r="B301">
+        <v>744</v>
+      </c>
+    </row>
+    <row r="302" spans="1:2">
+      <c r="A302" s="2">
+        <v>46223.125</v>
+      </c>
+      <c r="B302">
+        <v>735</v>
+      </c>
+    </row>
+    <row r="303" spans="1:2">
+      <c r="A303" s="2">
+        <v>46223.13541666666</v>
+      </c>
+      <c r="B303">
+        <v>733</v>
+      </c>
+    </row>
+    <row r="304" spans="1:2">
+      <c r="A304" s="2">
+        <v>46223.14583333334</v>
+      </c>
+      <c r="B304">
+        <v>734</v>
+      </c>
+    </row>
+    <row r="305" spans="1:2">
+      <c r="A305" s="2">
+        <v>46223.15625</v>
+      </c>
+      <c r="B305">
+        <v>733</v>
+      </c>
+    </row>
+    <row r="306" spans="1:2">
+      <c r="A306" s="2">
+        <v>46223.16666666666</v>
+      </c>
+      <c r="B306">
+        <v>726</v>
+      </c>
+    </row>
+    <row r="307" spans="1:2">
+      <c r="A307" s="2">
+        <v>46223.17708333334</v>
+      </c>
+      <c r="B307">
+        <v>732</v>
+      </c>
+    </row>
+    <row r="308" spans="1:2">
+      <c r="A308" s="2">
+        <v>46223.1875</v>
+      </c>
+      <c r="B308">
+        <v>695</v>
+      </c>
+    </row>
+    <row r="309" spans="1:2">
+      <c r="A309" s="2">
+        <v>46223.19791666666</v>
+      </c>
+      <c r="B309">
+        <v>693</v>
+      </c>
+    </row>
+    <row r="310" spans="1:2">
+      <c r="A310" s="2">
+        <v>46223.20833333334</v>
+      </c>
+      <c r="B310">
+        <v>693</v>
+      </c>
+    </row>
+    <row r="311" spans="1:2">
+      <c r="A311" s="2">
+        <v>46223.21875</v>
+      </c>
+      <c r="B311">
+        <v>694</v>
+      </c>
+    </row>
+    <row r="312" spans="1:2">
+      <c r="A312" s="2">
+        <v>46223.22916666666</v>
+      </c>
+      <c r="B312">
+        <v>682</v>
+      </c>
+    </row>
+    <row r="313" spans="1:2">
+      <c r="A313" s="2">
+        <v>46223.23958333334</v>
+      </c>
+      <c r="B313">
+        <v>684</v>
+      </c>
+    </row>
+    <row r="314" spans="1:2">
+      <c r="A314" s="2">
+        <v>46223.25</v>
+      </c>
+      <c r="B314">
+        <v>731</v>
+      </c>
+    </row>
+    <row r="315" spans="1:2">
+      <c r="A315" s="2">
+        <v>46223.26041666666</v>
+      </c>
+      <c r="B315">
+        <v>746</v>
+      </c>
+    </row>
+    <row r="316" spans="1:2">
+      <c r="A316" s="2">
+        <v>46223.27083333334</v>
+      </c>
+      <c r="B316">
+        <v>746</v>
+      </c>
+    </row>
+    <row r="317" spans="1:2">
+      <c r="A317" s="2">
+        <v>46223.28125</v>
+      </c>
+      <c r="B317">
+        <v>730</v>
+      </c>
+    </row>
+    <row r="318" spans="1:2">
+      <c r="A318" s="2">
+        <v>46223.29166666666</v>
+      </c>
+      <c r="B318">
+        <v>669</v>
+      </c>
+    </row>
+    <row r="319" spans="1:2">
+      <c r="A319" s="2">
+        <v>46223.30208333334</v>
+      </c>
+      <c r="B319">
+        <v>668</v>
+      </c>
+    </row>
+    <row r="320" spans="1:2">
+      <c r="A320" s="2">
+        <v>46223.3125</v>
+      </c>
+      <c r="B320">
+        <v>670</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Updating the model for Rosiori
</commit_message>
<xml_diff>
--- a/data_fetching/Entsoe/Actual_Production_Hydro_River.xlsx
+++ b/data_fetching/Entsoe/Actual_Production_Hydro_River.xlsx
@@ -381,7 +381,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B148"/>
+  <dimension ref="A1:B419"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:2">
@@ -394,207 +394,207 @@
     </row>
     <row r="2" spans="1:2">
       <c r="A2" s="2">
-        <v>46245</v>
+        <v>46247</v>
       </c>
       <c r="B2">
-        <v>409</v>
+        <v>419</v>
       </c>
     </row>
     <row r="3" spans="1:2">
       <c r="A3" s="2">
-        <v>46245.01041666666</v>
+        <v>46247.01041666666</v>
       </c>
       <c r="B3">
-        <v>408</v>
+        <v>411</v>
       </c>
     </row>
     <row r="4" spans="1:2">
       <c r="A4" s="2">
-        <v>46245.02083333334</v>
+        <v>46247.02083333334</v>
       </c>
       <c r="B4">
-        <v>409</v>
+        <v>412</v>
       </c>
     </row>
     <row r="5" spans="1:2">
       <c r="A5" s="2">
-        <v>46245.03125</v>
+        <v>46247.03125</v>
       </c>
       <c r="B5">
-        <v>408</v>
+        <v>411</v>
       </c>
     </row>
     <row r="6" spans="1:2">
       <c r="A6" s="2">
-        <v>46245.04166666666</v>
+        <v>46247.04166666666</v>
       </c>
       <c r="B6">
-        <v>408</v>
+        <v>411</v>
       </c>
     </row>
     <row r="7" spans="1:2">
       <c r="A7" s="2">
-        <v>46245.05208333334</v>
+        <v>46247.05208333334</v>
       </c>
       <c r="B7">
-        <v>406</v>
+        <v>411</v>
       </c>
     </row>
     <row r="8" spans="1:2">
       <c r="A8" s="2">
-        <v>46245.0625</v>
+        <v>46247.0625</v>
       </c>
       <c r="B8">
-        <v>409</v>
+        <v>411</v>
       </c>
     </row>
     <row r="9" spans="1:2">
       <c r="A9" s="2">
-        <v>46245.07291666666</v>
+        <v>46247.07291666666</v>
       </c>
       <c r="B9">
-        <v>408</v>
+        <v>411</v>
       </c>
     </row>
     <row r="10" spans="1:2">
       <c r="A10" s="2">
-        <v>46245.08333333334</v>
+        <v>46247.08333333334</v>
       </c>
       <c r="B10">
-        <v>410</v>
+        <v>411</v>
       </c>
     </row>
     <row r="11" spans="1:2">
       <c r="A11" s="2">
-        <v>46245.09375</v>
+        <v>46247.09375</v>
       </c>
       <c r="B11">
-        <v>408</v>
+        <v>411</v>
       </c>
     </row>
     <row r="12" spans="1:2">
       <c r="A12" s="2">
-        <v>46245.10416666666</v>
+        <v>46247.10416666666</v>
       </c>
       <c r="B12">
-        <v>408</v>
+        <v>411</v>
       </c>
     </row>
     <row r="13" spans="1:2">
       <c r="A13" s="2">
-        <v>46245.11458333334</v>
+        <v>46247.11458333334</v>
       </c>
       <c r="B13">
-        <v>408</v>
+        <v>411</v>
       </c>
     </row>
     <row r="14" spans="1:2">
       <c r="A14" s="2">
-        <v>46245.125</v>
+        <v>46247.125</v>
       </c>
       <c r="B14">
-        <v>409</v>
+        <v>410</v>
       </c>
     </row>
     <row r="15" spans="1:2">
       <c r="A15" s="2">
-        <v>46245.13541666666</v>
+        <v>46247.13541666666</v>
       </c>
       <c r="B15">
-        <v>408</v>
+        <v>411</v>
       </c>
     </row>
     <row r="16" spans="1:2">
       <c r="A16" s="2">
-        <v>46245.14583333334</v>
+        <v>46247.14583333334</v>
       </c>
       <c r="B16">
-        <v>409</v>
+        <v>411</v>
       </c>
     </row>
     <row r="17" spans="1:2">
       <c r="A17" s="2">
-        <v>46245.15625</v>
+        <v>46247.15625</v>
       </c>
       <c r="B17">
-        <v>410</v>
+        <v>411</v>
       </c>
     </row>
     <row r="18" spans="1:2">
       <c r="A18" s="2">
-        <v>46245.16666666666</v>
+        <v>46247.16666666666</v>
       </c>
       <c r="B18">
-        <v>398</v>
+        <v>411</v>
       </c>
     </row>
     <row r="19" spans="1:2">
       <c r="A19" s="2">
-        <v>46245.17708333334</v>
+        <v>46247.17708333334</v>
       </c>
       <c r="B19">
-        <v>391</v>
+        <v>411</v>
       </c>
     </row>
     <row r="20" spans="1:2">
       <c r="A20" s="2">
-        <v>46245.1875</v>
+        <v>46247.1875</v>
       </c>
       <c r="B20">
-        <v>391</v>
+        <v>411</v>
       </c>
     </row>
     <row r="21" spans="1:2">
       <c r="A21" s="2">
-        <v>46245.19791666666</v>
+        <v>46247.19791666666</v>
       </c>
       <c r="B21">
-        <v>391</v>
+        <v>411</v>
       </c>
     </row>
     <row r="22" spans="1:2">
       <c r="A22" s="2">
-        <v>46245.20833333334</v>
+        <v>46247.20833333334</v>
       </c>
       <c r="B22">
-        <v>398</v>
+        <v>484</v>
       </c>
     </row>
     <row r="23" spans="1:2">
       <c r="A23" s="2">
-        <v>46245.21875</v>
+        <v>46247.21875</v>
       </c>
       <c r="B23">
-        <v>418</v>
+        <v>506</v>
       </c>
     </row>
     <row r="24" spans="1:2">
       <c r="A24" s="2">
-        <v>46245.22916666666</v>
+        <v>46247.22916666666</v>
       </c>
       <c r="B24">
-        <v>418</v>
+        <v>539</v>
       </c>
     </row>
     <row r="25" spans="1:2">
       <c r="A25" s="2">
-        <v>46245.23958333334</v>
+        <v>46247.23958333334</v>
       </c>
       <c r="B25">
-        <v>416</v>
+        <v>540</v>
       </c>
     </row>
     <row r="26" spans="1:2">
       <c r="A26" s="2">
-        <v>46245.25</v>
+        <v>46247.25</v>
       </c>
       <c r="B26">
-        <v>489</v>
+        <v>467</v>
       </c>
     </row>
     <row r="27" spans="1:2">
       <c r="A27" s="2">
-        <v>46245.26041666666</v>
+        <v>46247.26041666666</v>
       </c>
       <c r="B27">
         <v>492</v>
@@ -602,279 +602,279 @@
     </row>
     <row r="28" spans="1:2">
       <c r="A28" s="2">
-        <v>46245.27083333334</v>
+        <v>46247.27083333334</v>
       </c>
       <c r="B28">
-        <v>490</v>
+        <v>524</v>
       </c>
     </row>
     <row r="29" spans="1:2">
       <c r="A29" s="2">
-        <v>46245.28125</v>
+        <v>46247.28125</v>
       </c>
       <c r="B29">
-        <v>490</v>
+        <v>615</v>
       </c>
     </row>
     <row r="30" spans="1:2">
       <c r="A30" s="2">
-        <v>46245.29166666666</v>
+        <v>46247.29166666666</v>
       </c>
       <c r="B30">
-        <v>491</v>
+        <v>666</v>
       </c>
     </row>
     <row r="31" spans="1:2">
       <c r="A31" s="2">
-        <v>46245.30208333334</v>
+        <v>46247.30208333334</v>
       </c>
       <c r="B31">
-        <v>490</v>
+        <v>669</v>
       </c>
     </row>
     <row r="32" spans="1:2">
       <c r="A32" s="2">
-        <v>46245.3125</v>
+        <v>46247.3125</v>
       </c>
       <c r="B32">
-        <v>490</v>
+        <v>672</v>
       </c>
     </row>
     <row r="33" spans="1:2">
       <c r="A33" s="2">
-        <v>46245.32291666666</v>
+        <v>46247.32291666666</v>
       </c>
       <c r="B33">
-        <v>488</v>
+        <v>660</v>
       </c>
     </row>
     <row r="34" spans="1:2">
       <c r="A34" s="2">
-        <v>46245.33333333334</v>
+        <v>46247.33333333334</v>
       </c>
       <c r="B34">
-        <v>459</v>
+        <v>496</v>
       </c>
     </row>
     <row r="35" spans="1:2">
       <c r="A35" s="2">
-        <v>46245.34375</v>
+        <v>46247.34375</v>
       </c>
       <c r="B35">
-        <v>455</v>
+        <v>486</v>
       </c>
     </row>
     <row r="36" spans="1:2">
       <c r="A36" s="2">
-        <v>46245.35416666666</v>
+        <v>46247.35416666666</v>
       </c>
       <c r="B36">
-        <v>472</v>
+        <v>431</v>
       </c>
     </row>
     <row r="37" spans="1:2">
       <c r="A37" s="2">
-        <v>46245.36458333334</v>
+        <v>46247.36458333334</v>
       </c>
       <c r="B37">
-        <v>471</v>
+        <v>438</v>
       </c>
     </row>
     <row r="38" spans="1:2">
       <c r="A38" s="2">
-        <v>46245.375</v>
+        <v>46247.375</v>
       </c>
       <c r="B38">
-        <v>410</v>
+        <v>450</v>
       </c>
     </row>
     <row r="39" spans="1:2">
       <c r="A39" s="2">
-        <v>46245.38541666666</v>
+        <v>46247.38541666666</v>
       </c>
       <c r="B39">
-        <v>405</v>
+        <v>451</v>
       </c>
     </row>
     <row r="40" spans="1:2">
       <c r="A40" s="2">
-        <v>46245.39583333334</v>
+        <v>46247.39583333334</v>
       </c>
       <c r="B40">
-        <v>407</v>
+        <v>451</v>
       </c>
     </row>
     <row r="41" spans="1:2">
       <c r="A41" s="2">
-        <v>46245.40625</v>
+        <v>46247.40625</v>
       </c>
       <c r="B41">
-        <v>403</v>
+        <v>450</v>
       </c>
     </row>
     <row r="42" spans="1:2">
       <c r="A42" s="2">
-        <v>46245.41666666666</v>
+        <v>46247.41666666666</v>
       </c>
       <c r="B42">
-        <v>274</v>
+        <v>266</v>
       </c>
     </row>
     <row r="43" spans="1:2">
       <c r="A43" s="2">
-        <v>46245.42708333334</v>
+        <v>46247.42708333334</v>
       </c>
       <c r="B43">
-        <v>262</v>
+        <v>257</v>
       </c>
     </row>
     <row r="44" spans="1:2">
       <c r="A44" s="2">
-        <v>46245.4375</v>
+        <v>46247.4375</v>
       </c>
       <c r="B44">
-        <v>266</v>
+        <v>257</v>
       </c>
     </row>
     <row r="45" spans="1:2">
       <c r="A45" s="2">
-        <v>46245.44791666666</v>
+        <v>46247.44791666666</v>
       </c>
       <c r="B45">
-        <v>265</v>
+        <v>256</v>
       </c>
     </row>
     <row r="46" spans="1:2">
       <c r="A46" s="2">
-        <v>46245.45833333334</v>
+        <v>46247.45833333334</v>
       </c>
       <c r="B46">
-        <v>261</v>
+        <v>273</v>
       </c>
     </row>
     <row r="47" spans="1:2">
       <c r="A47" s="2">
-        <v>46245.46875</v>
+        <v>46247.46875</v>
       </c>
       <c r="B47">
-        <v>261</v>
+        <v>274</v>
       </c>
     </row>
     <row r="48" spans="1:2">
       <c r="A48" s="2">
-        <v>46245.47916666666</v>
+        <v>46247.47916666666</v>
       </c>
       <c r="B48">
-        <v>261</v>
+        <v>267</v>
       </c>
     </row>
     <row r="49" spans="1:2">
       <c r="A49" s="2">
-        <v>46245.48958333334</v>
+        <v>46247.48958333334</v>
       </c>
       <c r="B49">
-        <v>261</v>
+        <v>267</v>
       </c>
     </row>
     <row r="50" spans="1:2">
       <c r="A50" s="2">
-        <v>46245.5</v>
+        <v>46247.5</v>
       </c>
       <c r="B50">
-        <v>282</v>
+        <v>230</v>
       </c>
     </row>
     <row r="51" spans="1:2">
       <c r="A51" s="2">
-        <v>46245.51041666666</v>
+        <v>46247.51041666666</v>
       </c>
       <c r="B51">
-        <v>278</v>
+        <v>228</v>
       </c>
     </row>
     <row r="52" spans="1:2">
       <c r="A52" s="2">
-        <v>46245.52083333334</v>
+        <v>46247.52083333334</v>
       </c>
       <c r="B52">
-        <v>280</v>
+        <v>228</v>
       </c>
     </row>
     <row r="53" spans="1:2">
       <c r="A53" s="2">
-        <v>46245.53125</v>
+        <v>46247.53125</v>
       </c>
       <c r="B53">
-        <v>280</v>
+        <v>228</v>
       </c>
     </row>
     <row r="54" spans="1:2">
       <c r="A54" s="2">
-        <v>46245.54166666666</v>
+        <v>46247.54166666666</v>
       </c>
       <c r="B54">
-        <v>282</v>
+        <v>216</v>
       </c>
     </row>
     <row r="55" spans="1:2">
       <c r="A55" s="2">
-        <v>46245.55208333334</v>
+        <v>46247.55208333334</v>
       </c>
       <c r="B55">
-        <v>280</v>
+        <v>213</v>
       </c>
     </row>
     <row r="56" spans="1:2">
       <c r="A56" s="2">
-        <v>46245.5625</v>
+        <v>46247.5625</v>
       </c>
       <c r="B56">
-        <v>279</v>
+        <v>215</v>
       </c>
     </row>
     <row r="57" spans="1:2">
       <c r="A57" s="2">
-        <v>46245.57291666666</v>
+        <v>46247.57291666666</v>
       </c>
       <c r="B57">
-        <v>279</v>
+        <v>212</v>
       </c>
     </row>
     <row r="58" spans="1:2">
       <c r="A58" s="2">
-        <v>46245.58333333334</v>
+        <v>46247.58333333334</v>
       </c>
       <c r="B58">
-        <v>271</v>
+        <v>208</v>
       </c>
     </row>
     <row r="59" spans="1:2">
       <c r="A59" s="2">
-        <v>46245.59375</v>
+        <v>46247.59375</v>
       </c>
       <c r="B59">
-        <v>246</v>
+        <v>207</v>
       </c>
     </row>
     <row r="60" spans="1:2">
       <c r="A60" s="2">
-        <v>46245.60416666666</v>
+        <v>46247.60416666666</v>
       </c>
       <c r="B60">
-        <v>274</v>
+        <v>208</v>
       </c>
     </row>
     <row r="61" spans="1:2">
       <c r="A61" s="2">
-        <v>46245.61458333334</v>
+        <v>46247.61458333334</v>
       </c>
       <c r="B61">
-        <v>277</v>
+        <v>211</v>
       </c>
     </row>
     <row r="62" spans="1:2">
       <c r="A62" s="2">
-        <v>46245.625</v>
+        <v>46247.625</v>
       </c>
       <c r="B62">
         <v>273</v>
@@ -882,690 +882,2858 @@
     </row>
     <row r="63" spans="1:2">
       <c r="A63" s="2">
-        <v>46245.63541666666</v>
+        <v>46247.63541666666</v>
       </c>
       <c r="B63">
-        <v>275</v>
+        <v>276</v>
       </c>
     </row>
     <row r="64" spans="1:2">
       <c r="A64" s="2">
-        <v>46245.64583333334</v>
+        <v>46247.64583333334</v>
       </c>
       <c r="B64">
-        <v>274</v>
+        <v>276</v>
       </c>
     </row>
     <row r="65" spans="1:2">
       <c r="A65" s="2">
-        <v>46245.65625</v>
+        <v>46247.65625</v>
       </c>
       <c r="B65">
-        <v>274</v>
+        <v>276</v>
       </c>
     </row>
     <row r="66" spans="1:2">
       <c r="A66" s="2">
-        <v>46245.66666666666</v>
+        <v>46247.66666666666</v>
       </c>
       <c r="B66">
-        <v>278</v>
+        <v>299</v>
       </c>
     </row>
     <row r="67" spans="1:2">
       <c r="A67" s="2">
-        <v>46245.67708333334</v>
+        <v>46247.67708333334</v>
       </c>
       <c r="B67">
-        <v>280</v>
+        <v>302</v>
       </c>
     </row>
     <row r="68" spans="1:2">
       <c r="A68" s="2">
-        <v>46245.6875</v>
+        <v>46247.6875</v>
       </c>
       <c r="B68">
-        <v>279</v>
+        <v>321</v>
       </c>
     </row>
     <row r="69" spans="1:2">
       <c r="A69" s="2">
-        <v>46245.69791666666</v>
+        <v>46247.69791666666</v>
       </c>
       <c r="B69">
-        <v>297</v>
+        <v>333</v>
       </c>
     </row>
     <row r="70" spans="1:2">
       <c r="A70" s="2">
-        <v>46245.70833333334</v>
+        <v>46247.70833333334</v>
       </c>
       <c r="B70">
-        <v>527</v>
+        <v>560</v>
       </c>
     </row>
     <row r="71" spans="1:2">
       <c r="A71" s="2">
-        <v>46245.71875</v>
+        <v>46247.71875</v>
       </c>
       <c r="B71">
-        <v>549</v>
+        <v>594</v>
       </c>
     </row>
     <row r="72" spans="1:2">
       <c r="A72" s="2">
-        <v>46245.72916666666</v>
+        <v>46247.72916666666</v>
       </c>
       <c r="B72">
-        <v>546</v>
+        <v>589</v>
       </c>
     </row>
     <row r="73" spans="1:2">
       <c r="A73" s="2">
-        <v>46245.73958333334</v>
+        <v>46247.73958333334</v>
       </c>
       <c r="B73">
-        <v>546</v>
+        <v>594</v>
       </c>
     </row>
     <row r="74" spans="1:2">
       <c r="A74" s="2">
-        <v>46245.75</v>
+        <v>46247.75</v>
       </c>
       <c r="B74">
-        <v>682</v>
+        <v>668</v>
       </c>
     </row>
     <row r="75" spans="1:2">
       <c r="A75" s="2">
-        <v>46245.76041666666</v>
+        <v>46247.76041666666</v>
       </c>
       <c r="B75">
-        <v>714</v>
+        <v>687</v>
       </c>
     </row>
     <row r="76" spans="1:2">
       <c r="A76" s="2">
-        <v>46245.77083333334</v>
+        <v>46247.77083333334</v>
       </c>
       <c r="B76">
-        <v>715</v>
+        <v>687</v>
       </c>
     </row>
     <row r="77" spans="1:2">
       <c r="A77" s="2">
-        <v>46245.78125</v>
+        <v>46247.78125</v>
       </c>
       <c r="B77">
-        <v>718</v>
+        <v>680</v>
       </c>
     </row>
     <row r="78" spans="1:2">
       <c r="A78" s="2">
-        <v>46245.79166666666</v>
+        <v>46247.79166666666</v>
       </c>
       <c r="B78">
-        <v>712</v>
+        <v>683</v>
       </c>
     </row>
     <row r="79" spans="1:2">
       <c r="A79" s="2">
-        <v>46245.80208333334</v>
+        <v>46247.80208333334</v>
       </c>
       <c r="B79">
-        <v>719</v>
+        <v>692</v>
       </c>
     </row>
     <row r="80" spans="1:2">
       <c r="A80" s="2">
-        <v>46245.8125</v>
+        <v>46247.8125</v>
       </c>
       <c r="B80">
-        <v>719</v>
+        <v>690</v>
       </c>
     </row>
     <row r="81" spans="1:2">
       <c r="A81" s="2">
-        <v>46245.82291666666</v>
+        <v>46247.82291666666</v>
       </c>
       <c r="B81">
-        <v>720</v>
+        <v>690</v>
       </c>
     </row>
     <row r="82" spans="1:2">
       <c r="A82" s="2">
-        <v>46245.83333333334</v>
+        <v>46247.83333333334</v>
       </c>
       <c r="B82">
-        <v>679</v>
+        <v>682</v>
       </c>
     </row>
     <row r="83" spans="1:2">
       <c r="A83" s="2">
-        <v>46245.84375</v>
+        <v>46247.84375</v>
       </c>
       <c r="B83">
-        <v>676</v>
+        <v>680</v>
       </c>
     </row>
     <row r="84" spans="1:2">
       <c r="A84" s="2">
-        <v>46245.85416666666</v>
+        <v>46247.85416666666</v>
       </c>
       <c r="B84">
-        <v>674</v>
+        <v>679</v>
       </c>
     </row>
     <row r="85" spans="1:2">
       <c r="A85" s="2">
-        <v>46245.86458333334</v>
+        <v>46247.86458333334</v>
       </c>
       <c r="B85">
-        <v>671</v>
+        <v>678</v>
       </c>
     </row>
     <row r="86" spans="1:2">
       <c r="A86" s="2">
-        <v>46245.875</v>
+        <v>46247.875</v>
       </c>
       <c r="B86">
-        <v>640</v>
+        <v>674</v>
       </c>
     </row>
     <row r="87" spans="1:2">
       <c r="A87" s="2">
-        <v>46245.88541666666</v>
+        <v>46247.88541666666</v>
       </c>
       <c r="B87">
-        <v>634</v>
+        <v>672</v>
       </c>
     </row>
     <row r="88" spans="1:2">
       <c r="A88" s="2">
-        <v>46245.89583333334</v>
+        <v>46247.89583333334</v>
       </c>
       <c r="B88">
-        <v>648</v>
+        <v>674</v>
       </c>
     </row>
     <row r="89" spans="1:2">
       <c r="A89" s="2">
-        <v>46245.90625</v>
+        <v>46247.90625</v>
       </c>
       <c r="B89">
-        <v>650</v>
+        <v>684</v>
       </c>
     </row>
     <row r="90" spans="1:2">
       <c r="A90" s="2">
-        <v>46245.91666666666</v>
+        <v>46247.91666666666</v>
       </c>
       <c r="B90">
-        <v>670</v>
+        <v>684</v>
       </c>
     </row>
     <row r="91" spans="1:2">
       <c r="A91" s="2">
-        <v>46245.92708333334</v>
+        <v>46247.92708333334</v>
       </c>
       <c r="B91">
-        <v>679</v>
+        <v>677</v>
       </c>
     </row>
     <row r="92" spans="1:2">
       <c r="A92" s="2">
-        <v>46245.9375</v>
+        <v>46247.9375</v>
       </c>
       <c r="B92">
-        <v>683</v>
+        <v>682</v>
       </c>
     </row>
     <row r="93" spans="1:2">
       <c r="A93" s="2">
-        <v>46245.94791666666</v>
+        <v>46247.94791666666</v>
       </c>
       <c r="B93">
-        <v>679</v>
+        <v>675</v>
       </c>
     </row>
     <row r="94" spans="1:2">
       <c r="A94" s="2">
-        <v>46245.95833333334</v>
+        <v>46247.95833333334</v>
       </c>
       <c r="B94">
-        <v>634</v>
+        <v>492</v>
       </c>
     </row>
     <row r="95" spans="1:2">
       <c r="A95" s="2">
-        <v>46245.96875</v>
+        <v>46247.96875</v>
       </c>
       <c r="B95">
-        <v>632</v>
+        <v>473</v>
       </c>
     </row>
     <row r="96" spans="1:2">
       <c r="A96" s="2">
-        <v>46245.97916666666</v>
+        <v>46247.97916666666</v>
       </c>
       <c r="B96">
-        <v>635</v>
+        <v>477</v>
       </c>
     </row>
     <row r="97" spans="1:2">
       <c r="A97" s="2">
-        <v>46245.98958333334</v>
+        <v>46247.98958333334</v>
       </c>
       <c r="B97">
-        <v>628</v>
+        <v>477</v>
       </c>
     </row>
     <row r="98" spans="1:2">
       <c r="A98" s="2">
-        <v>46246</v>
+        <v>46248</v>
       </c>
       <c r="B98">
-        <v>529</v>
+        <v>438</v>
       </c>
     </row>
     <row r="99" spans="1:2">
       <c r="A99" s="2">
-        <v>46246.01041666666</v>
+        <v>46248.01041666666</v>
       </c>
       <c r="B99">
-        <v>522</v>
+        <v>431</v>
       </c>
     </row>
     <row r="100" spans="1:2">
       <c r="A100" s="2">
-        <v>46246.02083333334</v>
+        <v>46248.02083333334</v>
       </c>
       <c r="B100">
-        <v>522</v>
+        <v>431</v>
       </c>
     </row>
     <row r="101" spans="1:2">
       <c r="A101" s="2">
-        <v>46246.03125</v>
+        <v>46248.03125</v>
       </c>
       <c r="B101">
-        <v>521</v>
+        <v>431</v>
       </c>
     </row>
     <row r="102" spans="1:2">
       <c r="A102" s="2">
-        <v>46246.04166666666</v>
+        <v>46248.04166666666</v>
       </c>
       <c r="B102">
-        <v>522</v>
+        <v>430</v>
       </c>
     </row>
     <row r="103" spans="1:2">
       <c r="A103" s="2">
-        <v>46246.05208333334</v>
+        <v>46248.05208333334</v>
       </c>
       <c r="B103">
-        <v>523</v>
+        <v>429</v>
       </c>
     </row>
     <row r="104" spans="1:2">
       <c r="A104" s="2">
-        <v>46246.0625</v>
+        <v>46248.0625</v>
       </c>
       <c r="B104">
-        <v>522</v>
+        <v>429</v>
       </c>
     </row>
     <row r="105" spans="1:2">
       <c r="A105" s="2">
-        <v>46246.07291666666</v>
+        <v>46248.07291666666</v>
       </c>
       <c r="B105">
-        <v>522</v>
+        <v>429</v>
       </c>
     </row>
     <row r="106" spans="1:2">
       <c r="A106" s="2">
-        <v>46246.08333333334</v>
+        <v>46248.08333333334</v>
       </c>
       <c r="B106">
-        <v>452</v>
+        <v>417</v>
       </c>
     </row>
     <row r="107" spans="1:2">
       <c r="A107" s="2">
-        <v>46246.09375</v>
+        <v>46248.09375</v>
       </c>
       <c r="B107">
-        <v>445</v>
+        <v>417</v>
       </c>
     </row>
     <row r="108" spans="1:2">
       <c r="A108" s="2">
-        <v>46246.10416666666</v>
+        <v>46248.10416666666</v>
       </c>
       <c r="B108">
-        <v>445</v>
+        <v>418</v>
       </c>
     </row>
     <row r="109" spans="1:2">
       <c r="A109" s="2">
-        <v>46246.11458333334</v>
+        <v>46248.11458333334</v>
       </c>
       <c r="B109">
-        <v>445</v>
+        <v>418</v>
       </c>
     </row>
     <row r="110" spans="1:2">
       <c r="A110" s="2">
-        <v>46246.125</v>
+        <v>46248.125</v>
       </c>
       <c r="B110">
-        <v>431</v>
+        <v>420</v>
       </c>
     </row>
     <row r="111" spans="1:2">
       <c r="A111" s="2">
-        <v>46246.13541666666</v>
+        <v>46248.13541666666</v>
       </c>
       <c r="B111">
-        <v>429</v>
+        <v>420</v>
       </c>
     </row>
     <row r="112" spans="1:2">
       <c r="A112" s="2">
-        <v>46246.14583333334</v>
+        <v>46248.14583333334</v>
       </c>
       <c r="B112">
-        <v>430</v>
+        <v>420</v>
       </c>
     </row>
     <row r="113" spans="1:2">
       <c r="A113" s="2">
-        <v>46246.15625</v>
+        <v>46248.15625</v>
       </c>
       <c r="B113">
-        <v>429</v>
+        <v>420</v>
       </c>
     </row>
     <row r="114" spans="1:2">
       <c r="A114" s="2">
-        <v>46246.16666666666</v>
+        <v>46248.16666666666</v>
       </c>
       <c r="B114">
-        <v>419</v>
+        <v>433</v>
       </c>
     </row>
     <row r="115" spans="1:2">
       <c r="A115" s="2">
-        <v>46246.17708333334</v>
+        <v>46248.17708333334</v>
       </c>
       <c r="B115">
-        <v>419</v>
+        <v>437</v>
       </c>
     </row>
     <row r="116" spans="1:2">
       <c r="A116" s="2">
-        <v>46246.1875</v>
+        <v>46248.1875</v>
       </c>
       <c r="B116">
-        <v>419</v>
+        <v>437</v>
       </c>
     </row>
     <row r="117" spans="1:2">
       <c r="A117" s="2">
-        <v>46246.19791666666</v>
+        <v>46248.19791666666</v>
       </c>
       <c r="B117">
-        <v>420</v>
+        <v>442</v>
       </c>
     </row>
     <row r="118" spans="1:2">
       <c r="A118" s="2">
-        <v>46246.20833333334</v>
+        <v>46248.20833333334</v>
       </c>
       <c r="B118">
-        <v>395</v>
+        <v>454</v>
       </c>
     </row>
     <row r="119" spans="1:2">
       <c r="A119" s="2">
-        <v>46246.21875</v>
+        <v>46248.21875</v>
       </c>
       <c r="B119">
-        <v>415</v>
+        <v>454</v>
       </c>
     </row>
     <row r="120" spans="1:2">
       <c r="A120" s="2">
-        <v>46246.22916666666</v>
+        <v>46248.22916666666</v>
       </c>
       <c r="B120">
-        <v>415</v>
+        <v>454</v>
       </c>
     </row>
     <row r="121" spans="1:2">
       <c r="A121" s="2">
-        <v>46246.23958333334</v>
+        <v>46248.23958333334</v>
       </c>
       <c r="B121">
-        <v>417</v>
+        <v>450</v>
       </c>
     </row>
     <row r="122" spans="1:2">
       <c r="A122" s="2">
-        <v>46246.25</v>
+        <v>46248.25</v>
       </c>
       <c r="B122">
-        <v>486</v>
+        <v>499</v>
       </c>
     </row>
     <row r="123" spans="1:2">
       <c r="A123" s="2">
-        <v>46246.26041666666</v>
+        <v>46248.26041666666</v>
       </c>
       <c r="B123">
-        <v>494</v>
+        <v>513</v>
       </c>
     </row>
     <row r="124" spans="1:2">
       <c r="A124" s="2">
-        <v>46246.27083333334</v>
+        <v>46248.27083333334</v>
       </c>
       <c r="B124">
-        <v>493</v>
+        <v>512</v>
       </c>
     </row>
     <row r="125" spans="1:2">
       <c r="A125" s="2">
-        <v>46246.28125</v>
+        <v>46248.28125</v>
       </c>
       <c r="B125">
-        <v>492</v>
+        <v>505</v>
       </c>
     </row>
     <row r="126" spans="1:2">
       <c r="A126" s="2">
-        <v>46246.29166666666</v>
+        <v>46248.29166666666</v>
       </c>
       <c r="B126">
-        <v>485</v>
+        <v>500</v>
       </c>
     </row>
     <row r="127" spans="1:2">
       <c r="A127" s="2">
-        <v>46246.30208333334</v>
+        <v>46248.30208333334</v>
       </c>
       <c r="B127">
-        <v>483</v>
+        <v>499</v>
       </c>
     </row>
     <row r="128" spans="1:2">
       <c r="A128" s="2">
-        <v>46246.3125</v>
+        <v>46248.3125</v>
       </c>
       <c r="B128">
-        <v>484</v>
+        <v>500</v>
       </c>
     </row>
     <row r="129" spans="1:2">
       <c r="A129" s="2">
-        <v>46246.32291666666</v>
+        <v>46248.32291666666</v>
       </c>
       <c r="B129">
-        <v>484</v>
+        <v>498</v>
       </c>
     </row>
     <row r="130" spans="1:2">
       <c r="A130" s="2">
-        <v>46246.33333333334</v>
+        <v>46248.33333333334</v>
       </c>
       <c r="B130">
-        <v>440</v>
+        <v>485</v>
       </c>
     </row>
     <row r="131" spans="1:2">
       <c r="A131" s="2">
-        <v>46246.34375</v>
+        <v>46248.34375</v>
       </c>
       <c r="B131">
-        <v>430</v>
+        <v>484</v>
       </c>
     </row>
     <row r="132" spans="1:2">
       <c r="A132" s="2">
-        <v>46246.35416666666</v>
+        <v>46248.35416666666</v>
       </c>
       <c r="B132">
-        <v>432</v>
+        <v>485</v>
       </c>
     </row>
     <row r="133" spans="1:2">
       <c r="A133" s="2">
-        <v>46246.36458333334</v>
+        <v>46248.36458333334</v>
       </c>
       <c r="B133">
-        <v>429</v>
+        <v>493</v>
       </c>
     </row>
     <row r="134" spans="1:2">
       <c r="A134" s="2">
-        <v>46246.375</v>
+        <v>46248.375</v>
       </c>
       <c r="B134">
-        <v>262</v>
+        <v>358</v>
       </c>
     </row>
     <row r="135" spans="1:2">
       <c r="A135" s="2">
-        <v>46246.38541666666</v>
+        <v>46248.38541666666</v>
       </c>
       <c r="B135">
-        <v>254</v>
+        <v>351</v>
       </c>
     </row>
     <row r="136" spans="1:2">
       <c r="A136" s="2">
-        <v>46246.39583333334</v>
+        <v>46248.39583333334</v>
       </c>
       <c r="B136">
-        <v>255</v>
+        <v>351</v>
       </c>
     </row>
     <row r="137" spans="1:2">
       <c r="A137" s="2">
-        <v>46246.40625</v>
+        <v>46248.40625</v>
       </c>
       <c r="B137">
-        <v>266</v>
+        <v>350</v>
       </c>
     </row>
     <row r="138" spans="1:2">
       <c r="A138" s="2">
-        <v>46246.41666666666</v>
+        <v>46248.41666666666</v>
       </c>
       <c r="B138">
-        <v>239</v>
+        <v>350</v>
       </c>
     </row>
     <row r="139" spans="1:2">
       <c r="A139" s="2">
-        <v>46246.42708333334</v>
+        <v>46248.42708333334</v>
       </c>
       <c r="B139">
-        <v>236</v>
+        <v>346</v>
       </c>
     </row>
     <row r="140" spans="1:2">
       <c r="A140" s="2">
-        <v>46246.4375</v>
+        <v>46248.4375</v>
       </c>
       <c r="B140">
-        <v>235</v>
+        <v>349</v>
       </c>
     </row>
     <row r="141" spans="1:2">
       <c r="A141" s="2">
-        <v>46246.44791666666</v>
+        <v>46248.44791666666</v>
       </c>
       <c r="B141">
-        <v>235</v>
+        <v>348</v>
       </c>
     </row>
     <row r="142" spans="1:2">
       <c r="A142" s="2">
-        <v>46246.45833333334</v>
+        <v>46248.45833333334</v>
       </c>
       <c r="B142">
-        <v>245</v>
+        <v>340</v>
       </c>
     </row>
     <row r="143" spans="1:2">
       <c r="A143" s="2">
-        <v>46246.46875</v>
+        <v>46248.46875</v>
       </c>
       <c r="B143">
-        <v>245</v>
+        <v>325</v>
       </c>
     </row>
     <row r="144" spans="1:2">
       <c r="A144" s="2">
-        <v>46246.47916666666</v>
+        <v>46248.47916666666</v>
       </c>
       <c r="B144">
-        <v>245</v>
+        <v>325</v>
       </c>
     </row>
     <row r="145" spans="1:2">
       <c r="A145" s="2">
-        <v>46246.48958333334</v>
+        <v>46248.48958333334</v>
       </c>
       <c r="B145">
-        <v>245</v>
+        <v>325</v>
       </c>
     </row>
     <row r="146" spans="1:2">
       <c r="A146" s="2">
-        <v>46246.5</v>
+        <v>46248.5</v>
       </c>
       <c r="B146">
-        <v>245</v>
+        <v>321</v>
       </c>
     </row>
     <row r="147" spans="1:2">
       <c r="A147" s="2">
-        <v>46246.51041666666</v>
+        <v>46248.51041666666</v>
       </c>
       <c r="B147">
-        <v>245</v>
+        <v>317</v>
       </c>
     </row>
     <row r="148" spans="1:2">
       <c r="A148" s="2">
-        <v>46246.52083333334</v>
+        <v>46248.52083333334</v>
       </c>
       <c r="B148">
+        <v>318</v>
+      </c>
+    </row>
+    <row r="149" spans="1:2">
+      <c r="A149" s="2">
+        <v>46248.53125</v>
+      </c>
+      <c r="B149">
+        <v>318</v>
+      </c>
+    </row>
+    <row r="150" spans="1:2">
+      <c r="A150" s="2">
+        <v>46248.54166666666</v>
+      </c>
+      <c r="B150">
+        <v>297</v>
+      </c>
+    </row>
+    <row r="151" spans="1:2">
+      <c r="A151" s="2">
+        <v>46248.55208333334</v>
+      </c>
+      <c r="B151">
+        <v>321</v>
+      </c>
+    </row>
+    <row r="152" spans="1:2">
+      <c r="A152" s="2">
+        <v>46248.5625</v>
+      </c>
+      <c r="B152">
+        <v>311</v>
+      </c>
+    </row>
+    <row r="153" spans="1:2">
+      <c r="A153" s="2">
+        <v>46248.57291666666</v>
+      </c>
+      <c r="B153">
+        <v>310</v>
+      </c>
+    </row>
+    <row r="154" spans="1:2">
+      <c r="A154" s="2">
+        <v>46248.58333333334</v>
+      </c>
+      <c r="B154">
+        <v>311</v>
+      </c>
+    </row>
+    <row r="155" spans="1:2">
+      <c r="A155" s="2">
+        <v>46248.59375</v>
+      </c>
+      <c r="B155">
+        <v>312</v>
+      </c>
+    </row>
+    <row r="156" spans="1:2">
+      <c r="A156" s="2">
+        <v>46248.60416666666</v>
+      </c>
+      <c r="B156">
+        <v>312</v>
+      </c>
+    </row>
+    <row r="157" spans="1:2">
+      <c r="A157" s="2">
+        <v>46248.61458333334</v>
+      </c>
+      <c r="B157">
+        <v>312</v>
+      </c>
+    </row>
+    <row r="158" spans="1:2">
+      <c r="A158" s="2">
+        <v>46248.625</v>
+      </c>
+      <c r="B158">
+        <v>318</v>
+      </c>
+    </row>
+    <row r="159" spans="1:2">
+      <c r="A159" s="2">
+        <v>46248.63541666666</v>
+      </c>
+      <c r="B159">
+        <v>319</v>
+      </c>
+    </row>
+    <row r="160" spans="1:2">
+      <c r="A160" s="2">
+        <v>46248.64583333334</v>
+      </c>
+      <c r="B160">
+        <v>318</v>
+      </c>
+    </row>
+    <row r="161" spans="1:2">
+      <c r="A161" s="2">
+        <v>46248.65625</v>
+      </c>
+      <c r="B161">
+        <v>317</v>
+      </c>
+    </row>
+    <row r="162" spans="1:2">
+      <c r="A162" s="2">
+        <v>46248.66666666666</v>
+      </c>
+      <c r="B162">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="163" spans="1:2">
+      <c r="A163" s="2">
+        <v>46248.67708333334</v>
+      </c>
+      <c r="B163">
+        <v>437</v>
+      </c>
+    </row>
+    <row r="164" spans="1:2">
+      <c r="A164" s="2">
+        <v>46248.6875</v>
+      </c>
+      <c r="B164">
+        <v>437</v>
+      </c>
+    </row>
+    <row r="165" spans="1:2">
+      <c r="A165" s="2">
+        <v>46248.69791666666</v>
+      </c>
+      <c r="B165">
+        <v>444</v>
+      </c>
+    </row>
+    <row r="166" spans="1:2">
+      <c r="A166" s="2">
+        <v>46248.70833333334</v>
+      </c>
+      <c r="B166">
+        <v>691</v>
+      </c>
+    </row>
+    <row r="167" spans="1:2">
+      <c r="A167" s="2">
+        <v>46248.71875</v>
+      </c>
+      <c r="B167">
+        <v>709</v>
+      </c>
+    </row>
+    <row r="168" spans="1:2">
+      <c r="A168" s="2">
+        <v>46248.72916666666</v>
+      </c>
+      <c r="B168">
+        <v>710</v>
+      </c>
+    </row>
+    <row r="169" spans="1:2">
+      <c r="A169" s="2">
+        <v>46248.73958333334</v>
+      </c>
+      <c r="B169">
+        <v>687</v>
+      </c>
+    </row>
+    <row r="170" spans="1:2">
+      <c r="A170" s="2">
+        <v>46248.75</v>
+      </c>
+      <c r="B170">
+        <v>698</v>
+      </c>
+    </row>
+    <row r="171" spans="1:2">
+      <c r="A171" s="2">
+        <v>46248.76041666666</v>
+      </c>
+      <c r="B171">
+        <v>702</v>
+      </c>
+    </row>
+    <row r="172" spans="1:2">
+      <c r="A172" s="2">
+        <v>46248.77083333334</v>
+      </c>
+      <c r="B172">
+        <v>701</v>
+      </c>
+    </row>
+    <row r="173" spans="1:2">
+      <c r="A173" s="2">
+        <v>46248.78125</v>
+      </c>
+      <c r="B173">
+        <v>705</v>
+      </c>
+    </row>
+    <row r="174" spans="1:2">
+      <c r="A174" s="2">
+        <v>46248.79166666666</v>
+      </c>
+      <c r="B174">
+        <v>752</v>
+      </c>
+    </row>
+    <row r="175" spans="1:2">
+      <c r="A175" s="2">
+        <v>46248.80208333334</v>
+      </c>
+      <c r="B175">
+        <v>759</v>
+      </c>
+    </row>
+    <row r="176" spans="1:2">
+      <c r="A176" s="2">
+        <v>46248.8125</v>
+      </c>
+      <c r="B176">
+        <v>723</v>
+      </c>
+    </row>
+    <row r="177" spans="1:2">
+      <c r="A177" s="2">
+        <v>46248.82291666666</v>
+      </c>
+      <c r="B177">
+        <v>723</v>
+      </c>
+    </row>
+    <row r="178" spans="1:2">
+      <c r="A178" s="2">
+        <v>46248.83333333334</v>
+      </c>
+      <c r="B178">
+        <v>705</v>
+      </c>
+    </row>
+    <row r="179" spans="1:2">
+      <c r="A179" s="2">
+        <v>46248.84375</v>
+      </c>
+      <c r="B179">
+        <v>705</v>
+      </c>
+    </row>
+    <row r="180" spans="1:2">
+      <c r="A180" s="2">
+        <v>46248.85416666666</v>
+      </c>
+      <c r="B180">
+        <v>707</v>
+      </c>
+    </row>
+    <row r="181" spans="1:2">
+      <c r="A181" s="2">
+        <v>46248.86458333334</v>
+      </c>
+      <c r="B181">
+        <v>703</v>
+      </c>
+    </row>
+    <row r="182" spans="1:2">
+      <c r="A182" s="2">
+        <v>46248.875</v>
+      </c>
+      <c r="B182">
+        <v>702</v>
+      </c>
+    </row>
+    <row r="183" spans="1:2">
+      <c r="A183" s="2">
+        <v>46248.88541666666</v>
+      </c>
+      <c r="B183">
+        <v>701</v>
+      </c>
+    </row>
+    <row r="184" spans="1:2">
+      <c r="A184" s="2">
+        <v>46248.89583333334</v>
+      </c>
+      <c r="B184">
+        <v>720</v>
+      </c>
+    </row>
+    <row r="185" spans="1:2">
+      <c r="A185" s="2">
+        <v>46248.90625</v>
+      </c>
+      <c r="B185">
+        <v>719</v>
+      </c>
+    </row>
+    <row r="186" spans="1:2">
+      <c r="A186" s="2">
+        <v>46248.91666666666</v>
+      </c>
+      <c r="B186">
+        <v>700</v>
+      </c>
+    </row>
+    <row r="187" spans="1:2">
+      <c r="A187" s="2">
+        <v>46248.92708333334</v>
+      </c>
+      <c r="B187">
+        <v>696</v>
+      </c>
+    </row>
+    <row r="188" spans="1:2">
+      <c r="A188" s="2">
+        <v>46248.9375</v>
+      </c>
+      <c r="B188">
+        <v>697</v>
+      </c>
+    </row>
+    <row r="189" spans="1:2">
+      <c r="A189" s="2">
+        <v>46248.94791666666</v>
+      </c>
+      <c r="B189">
+        <v>695</v>
+      </c>
+    </row>
+    <row r="190" spans="1:2">
+      <c r="A190" s="2">
+        <v>46248.95833333334</v>
+      </c>
+      <c r="B190">
+        <v>626</v>
+      </c>
+    </row>
+    <row r="191" spans="1:2">
+      <c r="A191" s="2">
+        <v>46248.96875</v>
+      </c>
+      <c r="B191">
+        <v>619</v>
+      </c>
+    </row>
+    <row r="192" spans="1:2">
+      <c r="A192" s="2">
+        <v>46248.97916666666</v>
+      </c>
+      <c r="B192">
+        <v>620</v>
+      </c>
+    </row>
+    <row r="193" spans="1:2">
+      <c r="A193" s="2">
+        <v>46248.98958333334</v>
+      </c>
+      <c r="B193">
+        <v>616</v>
+      </c>
+    </row>
+    <row r="194" spans="1:2">
+      <c r="A194" s="2">
+        <v>46249</v>
+      </c>
+      <c r="B194">
+        <v>524</v>
+      </c>
+    </row>
+    <row r="195" spans="1:2">
+      <c r="A195" s="2">
+        <v>46249.01041666666</v>
+      </c>
+      <c r="B195">
+        <v>522</v>
+      </c>
+    </row>
+    <row r="196" spans="1:2">
+      <c r="A196" s="2">
+        <v>46249.02083333334</v>
+      </c>
+      <c r="B196">
+        <v>521</v>
+      </c>
+    </row>
+    <row r="197" spans="1:2">
+      <c r="A197" s="2">
+        <v>46249.03125</v>
+      </c>
+      <c r="B197">
+        <v>520</v>
+      </c>
+    </row>
+    <row r="198" spans="1:2">
+      <c r="A198" s="2">
+        <v>46249.04166666666</v>
+      </c>
+      <c r="B198">
+        <v>481</v>
+      </c>
+    </row>
+    <row r="199" spans="1:2">
+      <c r="A199" s="2">
+        <v>46249.05208333334</v>
+      </c>
+      <c r="B199">
+        <v>479</v>
+      </c>
+    </row>
+    <row r="200" spans="1:2">
+      <c r="A200" s="2">
+        <v>46249.0625</v>
+      </c>
+      <c r="B200">
+        <v>480</v>
+      </c>
+    </row>
+    <row r="201" spans="1:2">
+      <c r="A201" s="2">
+        <v>46249.07291666666</v>
+      </c>
+      <c r="B201">
+        <v>478</v>
+      </c>
+    </row>
+    <row r="202" spans="1:2">
+      <c r="A202" s="2">
+        <v>46249.08333333334</v>
+      </c>
+      <c r="B202">
+        <v>479</v>
+      </c>
+    </row>
+    <row r="203" spans="1:2">
+      <c r="A203" s="2">
+        <v>46249.09375</v>
+      </c>
+      <c r="B203">
+        <v>479</v>
+      </c>
+    </row>
+    <row r="204" spans="1:2">
+      <c r="A204" s="2">
+        <v>46249.10416666666</v>
+      </c>
+      <c r="B204">
+        <v>479</v>
+      </c>
+    </row>
+    <row r="205" spans="1:2">
+      <c r="A205" s="2">
+        <v>46249.11458333334</v>
+      </c>
+      <c r="B205">
+        <v>475</v>
+      </c>
+    </row>
+    <row r="206" spans="1:2">
+      <c r="A206" s="2">
+        <v>46249.125</v>
+      </c>
+      <c r="B206">
+        <v>487</v>
+      </c>
+    </row>
+    <row r="207" spans="1:2">
+      <c r="A207" s="2">
+        <v>46249.13541666666</v>
+      </c>
+      <c r="B207">
+        <v>485</v>
+      </c>
+    </row>
+    <row r="208" spans="1:2">
+      <c r="A208" s="2">
+        <v>46249.14583333334</v>
+      </c>
+      <c r="B208">
+        <v>485</v>
+      </c>
+    </row>
+    <row r="209" spans="1:2">
+      <c r="A209" s="2">
+        <v>46249.15625</v>
+      </c>
+      <c r="B209">
+        <v>484</v>
+      </c>
+    </row>
+    <row r="210" spans="1:2">
+      <c r="A210" s="2">
+        <v>46249.16666666666</v>
+      </c>
+      <c r="B210">
+        <v>485</v>
+      </c>
+    </row>
+    <row r="211" spans="1:2">
+      <c r="A211" s="2">
+        <v>46249.17708333334</v>
+      </c>
+      <c r="B211">
+        <v>485</v>
+      </c>
+    </row>
+    <row r="212" spans="1:2">
+      <c r="A212" s="2">
+        <v>46249.1875</v>
+      </c>
+      <c r="B212">
+        <v>485</v>
+      </c>
+    </row>
+    <row r="213" spans="1:2">
+      <c r="A213" s="2">
+        <v>46249.19791666666</v>
+      </c>
+      <c r="B213">
+        <v>484</v>
+      </c>
+    </row>
+    <row r="214" spans="1:2">
+      <c r="A214" s="2">
+        <v>46249.20833333334</v>
+      </c>
+      <c r="B214">
+        <v>412</v>
+      </c>
+    </row>
+    <row r="215" spans="1:2">
+      <c r="A215" s="2">
+        <v>46249.21875</v>
+      </c>
+      <c r="B215">
+        <v>412</v>
+      </c>
+    </row>
+    <row r="216" spans="1:2">
+      <c r="A216" s="2">
+        <v>46249.22916666666</v>
+      </c>
+      <c r="B216">
+        <v>413</v>
+      </c>
+    </row>
+    <row r="217" spans="1:2">
+      <c r="A217" s="2">
+        <v>46249.23958333334</v>
+      </c>
+      <c r="B217">
+        <v>412</v>
+      </c>
+    </row>
+    <row r="218" spans="1:2">
+      <c r="A218" s="2">
+        <v>46249.25</v>
+      </c>
+      <c r="B218">
+        <v>461</v>
+      </c>
+    </row>
+    <row r="219" spans="1:2">
+      <c r="A219" s="2">
+        <v>46249.26041666666</v>
+      </c>
+      <c r="B219">
+        <v>476</v>
+      </c>
+    </row>
+    <row r="220" spans="1:2">
+      <c r="A220" s="2">
+        <v>46249.27083333334</v>
+      </c>
+      <c r="B220">
+        <v>476</v>
+      </c>
+    </row>
+    <row r="221" spans="1:2">
+      <c r="A221" s="2">
+        <v>46249.28125</v>
+      </c>
+      <c r="B221">
+        <v>477</v>
+      </c>
+    </row>
+    <row r="222" spans="1:2">
+      <c r="A222" s="2">
+        <v>46249.29166666666</v>
+      </c>
+      <c r="B222">
+        <v>454</v>
+      </c>
+    </row>
+    <row r="223" spans="1:2">
+      <c r="A223" s="2">
+        <v>46249.30208333334</v>
+      </c>
+      <c r="B223">
+        <v>452</v>
+      </c>
+    </row>
+    <row r="224" spans="1:2">
+      <c r="A224" s="2">
+        <v>46249.3125</v>
+      </c>
+      <c r="B224">
+        <v>451</v>
+      </c>
+    </row>
+    <row r="225" spans="1:2">
+      <c r="A225" s="2">
+        <v>46249.32291666666</v>
+      </c>
+      <c r="B225">
+        <v>450</v>
+      </c>
+    </row>
+    <row r="226" spans="1:2">
+      <c r="A226" s="2">
+        <v>46249.33333333334</v>
+      </c>
+      <c r="B226">
+        <v>329</v>
+      </c>
+    </row>
+    <row r="227" spans="1:2">
+      <c r="A227" s="2">
+        <v>46249.34375</v>
+      </c>
+      <c r="B227">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="228" spans="1:2">
+      <c r="A228" s="2">
+        <v>46249.35416666666</v>
+      </c>
+      <c r="B228">
+        <v>359</v>
+      </c>
+    </row>
+    <row r="229" spans="1:2">
+      <c r="A229" s="2">
+        <v>46249.36458333334</v>
+      </c>
+      <c r="B229">
+        <v>368</v>
+      </c>
+    </row>
+    <row r="230" spans="1:2">
+      <c r="A230" s="2">
+        <v>46249.375</v>
+      </c>
+      <c r="B230">
+        <v>325</v>
+      </c>
+    </row>
+    <row r="231" spans="1:2">
+      <c r="A231" s="2">
+        <v>46249.38541666666</v>
+      </c>
+      <c r="B231">
+        <v>284</v>
+      </c>
+    </row>
+    <row r="232" spans="1:2">
+      <c r="A232" s="2">
+        <v>46249.39583333334</v>
+      </c>
+      <c r="B232">
+        <v>282</v>
+      </c>
+    </row>
+    <row r="233" spans="1:2">
+      <c r="A233" s="2">
+        <v>46249.40625</v>
+      </c>
+      <c r="B233">
+        <v>282</v>
+      </c>
+    </row>
+    <row r="234" spans="1:2">
+      <c r="A234" s="2">
+        <v>46249.41666666666</v>
+      </c>
+      <c r="B234">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="235" spans="1:2">
+      <c r="A235" s="2">
+        <v>46249.42708333334</v>
+      </c>
+      <c r="B235">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="236" spans="1:2">
+      <c r="A236" s="2">
+        <v>46249.4375</v>
+      </c>
+      <c r="B236">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="237" spans="1:2">
+      <c r="A237" s="2">
+        <v>46249.44791666666</v>
+      </c>
+      <c r="B237">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="238" spans="1:2">
+      <c r="A238" s="2">
+        <v>46249.45833333334</v>
+      </c>
+      <c r="B238">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="239" spans="1:2">
+      <c r="A239" s="2">
+        <v>46249.46875</v>
+      </c>
+      <c r="B239">
+        <v>285</v>
+      </c>
+    </row>
+    <row r="240" spans="1:2">
+      <c r="A240" s="2">
+        <v>46249.47916666666</v>
+      </c>
+      <c r="B240">
+        <v>284</v>
+      </c>
+    </row>
+    <row r="241" spans="1:2">
+      <c r="A241" s="2">
+        <v>46249.48958333334</v>
+      </c>
+      <c r="B241">
+        <v>284</v>
+      </c>
+    </row>
+    <row r="242" spans="1:2">
+      <c r="A242" s="2">
+        <v>46249.5</v>
+      </c>
+      <c r="B242">
+        <v>282</v>
+      </c>
+    </row>
+    <row r="243" spans="1:2">
+      <c r="A243" s="2">
+        <v>46249.51041666666</v>
+      </c>
+      <c r="B243">
+        <v>279</v>
+      </c>
+    </row>
+    <row r="244" spans="1:2">
+      <c r="A244" s="2">
+        <v>46249.52083333334</v>
+      </c>
+      <c r="B244">
+        <v>284</v>
+      </c>
+    </row>
+    <row r="245" spans="1:2">
+      <c r="A245" s="2">
+        <v>46249.53125</v>
+      </c>
+      <c r="B245">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="246" spans="1:2">
+      <c r="A246" s="2">
+        <v>46249.54166666666</v>
+      </c>
+      <c r="B246">
+        <v>285</v>
+      </c>
+    </row>
+    <row r="247" spans="1:2">
+      <c r="A247" s="2">
+        <v>46249.55208333334</v>
+      </c>
+      <c r="B247">
+        <v>284</v>
+      </c>
+    </row>
+    <row r="248" spans="1:2">
+      <c r="A248" s="2">
+        <v>46249.5625</v>
+      </c>
+      <c r="B248">
+        <v>285</v>
+      </c>
+    </row>
+    <row r="249" spans="1:2">
+      <c r="A249" s="2">
+        <v>46249.57291666666</v>
+      </c>
+      <c r="B249">
+        <v>265</v>
+      </c>
+    </row>
+    <row r="250" spans="1:2">
+      <c r="A250" s="2">
+        <v>46249.58333333334</v>
+      </c>
+      <c r="B250">
+        <v>280</v>
+      </c>
+    </row>
+    <row r="251" spans="1:2">
+      <c r="A251" s="2">
+        <v>46249.59375</v>
+      </c>
+      <c r="B251">
+        <v>282</v>
+      </c>
+    </row>
+    <row r="252" spans="1:2">
+      <c r="A252" s="2">
+        <v>46249.60416666666</v>
+      </c>
+      <c r="B252">
+        <v>282</v>
+      </c>
+    </row>
+    <row r="253" spans="1:2">
+      <c r="A253" s="2">
+        <v>46249.61458333334</v>
+      </c>
+      <c r="B253">
+        <v>282</v>
+      </c>
+    </row>
+    <row r="254" spans="1:2">
+      <c r="A254" s="2">
+        <v>46249.625</v>
+      </c>
+      <c r="B254">
+        <v>265</v>
+      </c>
+    </row>
+    <row r="255" spans="1:2">
+      <c r="A255" s="2">
+        <v>46249.63541666666</v>
+      </c>
+      <c r="B255">
+        <v>264</v>
+      </c>
+    </row>
+    <row r="256" spans="1:2">
+      <c r="A256" s="2">
+        <v>46249.64583333334</v>
+      </c>
+      <c r="B256">
+        <v>264</v>
+      </c>
+    </row>
+    <row r="257" spans="1:2">
+      <c r="A257" s="2">
+        <v>46249.65625</v>
+      </c>
+      <c r="B257">
+        <v>265</v>
+      </c>
+    </row>
+    <row r="258" spans="1:2">
+      <c r="A258" s="2">
+        <v>46249.66666666666</v>
+      </c>
+      <c r="B258">
+        <v>284</v>
+      </c>
+    </row>
+    <row r="259" spans="1:2">
+      <c r="A259" s="2">
+        <v>46249.67708333334</v>
+      </c>
+      <c r="B259">
+        <v>286</v>
+      </c>
+    </row>
+    <row r="260" spans="1:2">
+      <c r="A260" s="2">
+        <v>46249.6875</v>
+      </c>
+      <c r="B260">
+        <v>286</v>
+      </c>
+    </row>
+    <row r="261" spans="1:2">
+      <c r="A261" s="2">
+        <v>46249.69791666666</v>
+      </c>
+      <c r="B261">
+        <v>286</v>
+      </c>
+    </row>
+    <row r="262" spans="1:2">
+      <c r="A262" s="2">
+        <v>46249.70833333334</v>
+      </c>
+      <c r="B262">
+        <v>466</v>
+      </c>
+    </row>
+    <row r="263" spans="1:2">
+      <c r="A263" s="2">
+        <v>46249.71875</v>
+      </c>
+      <c r="B263">
+        <v>651</v>
+      </c>
+    </row>
+    <row r="264" spans="1:2">
+      <c r="A264" s="2">
+        <v>46249.72916666666</v>
+      </c>
+      <c r="B264">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="265" spans="1:2">
+      <c r="A265" s="2">
+        <v>46249.73958333334</v>
+      </c>
+      <c r="B265">
+        <v>657</v>
+      </c>
+    </row>
+    <row r="266" spans="1:2">
+      <c r="A266" s="2">
+        <v>46249.75</v>
+      </c>
+      <c r="B266">
+        <v>718</v>
+      </c>
+    </row>
+    <row r="267" spans="1:2">
+      <c r="A267" s="2">
+        <v>46249.76041666666</v>
+      </c>
+      <c r="B267">
+        <v>724</v>
+      </c>
+    </row>
+    <row r="268" spans="1:2">
+      <c r="A268" s="2">
+        <v>46249.77083333334</v>
+      </c>
+      <c r="B268">
+        <v>721</v>
+      </c>
+    </row>
+    <row r="269" spans="1:2">
+      <c r="A269" s="2">
+        <v>46249.78125</v>
+      </c>
+      <c r="B269">
+        <v>724</v>
+      </c>
+    </row>
+    <row r="270" spans="1:2">
+      <c r="A270" s="2">
+        <v>46249.79166666666</v>
+      </c>
+      <c r="B270">
+        <v>698</v>
+      </c>
+    </row>
+    <row r="271" spans="1:2">
+      <c r="A271" s="2">
+        <v>46249.80208333334</v>
+      </c>
+      <c r="B271">
+        <v>700</v>
+      </c>
+    </row>
+    <row r="272" spans="1:2">
+      <c r="A272" s="2">
+        <v>46249.8125</v>
+      </c>
+      <c r="B272">
+        <v>702</v>
+      </c>
+    </row>
+    <row r="273" spans="1:2">
+      <c r="A273" s="2">
+        <v>46249.82291666666</v>
+      </c>
+      <c r="B273">
+        <v>702</v>
+      </c>
+    </row>
+    <row r="274" spans="1:2">
+      <c r="A274" s="2">
+        <v>46249.83333333334</v>
+      </c>
+      <c r="B274">
+        <v>716</v>
+      </c>
+    </row>
+    <row r="275" spans="1:2">
+      <c r="A275" s="2">
+        <v>46249.84375</v>
+      </c>
+      <c r="B275">
+        <v>719</v>
+      </c>
+    </row>
+    <row r="276" spans="1:2">
+      <c r="A276" s="2">
+        <v>46249.85416666666</v>
+      </c>
+      <c r="B276">
+        <v>720</v>
+      </c>
+    </row>
+    <row r="277" spans="1:2">
+      <c r="A277" s="2">
+        <v>46249.86458333334</v>
+      </c>
+      <c r="B277">
+        <v>719</v>
+      </c>
+    </row>
+    <row r="278" spans="1:2">
+      <c r="A278" s="2">
+        <v>46249.875</v>
+      </c>
+      <c r="B278">
+        <v>707</v>
+      </c>
+    </row>
+    <row r="279" spans="1:2">
+      <c r="A279" s="2">
+        <v>46249.88541666666</v>
+      </c>
+      <c r="B279">
+        <v>703</v>
+      </c>
+    </row>
+    <row r="280" spans="1:2">
+      <c r="A280" s="2">
+        <v>46249.89583333334</v>
+      </c>
+      <c r="B280">
+        <v>703</v>
+      </c>
+    </row>
+    <row r="281" spans="1:2">
+      <c r="A281" s="2">
+        <v>46249.90625</v>
+      </c>
+      <c r="B281">
+        <v>714</v>
+      </c>
+    </row>
+    <row r="282" spans="1:2">
+      <c r="A282" s="2">
+        <v>46249.91666666666</v>
+      </c>
+      <c r="B282">
+        <v>709</v>
+      </c>
+    </row>
+    <row r="283" spans="1:2">
+      <c r="A283" s="2">
+        <v>46249.92708333334</v>
+      </c>
+      <c r="B283">
+        <v>695</v>
+      </c>
+    </row>
+    <row r="284" spans="1:2">
+      <c r="A284" s="2">
+        <v>46249.9375</v>
+      </c>
+      <c r="B284">
+        <v>697</v>
+      </c>
+    </row>
+    <row r="285" spans="1:2">
+      <c r="A285" s="2">
+        <v>46249.94791666666</v>
+      </c>
+      <c r="B285">
+        <v>695</v>
+      </c>
+    </row>
+    <row r="286" spans="1:2">
+      <c r="A286" s="2">
+        <v>46249.95833333334</v>
+      </c>
+      <c r="B286">
+        <v>626</v>
+      </c>
+    </row>
+    <row r="287" spans="1:2">
+      <c r="A287" s="2">
+        <v>46249.96875</v>
+      </c>
+      <c r="B287">
+        <v>623</v>
+      </c>
+    </row>
+    <row r="288" spans="1:2">
+      <c r="A288" s="2">
+        <v>46249.97916666666</v>
+      </c>
+      <c r="B288">
+        <v>625</v>
+      </c>
+    </row>
+    <row r="289" spans="1:2">
+      <c r="A289" s="2">
+        <v>46249.98958333334</v>
+      </c>
+      <c r="B289">
+        <v>622</v>
+      </c>
+    </row>
+    <row r="290" spans="1:2">
+      <c r="A290" s="2">
+        <v>46250</v>
+      </c>
+      <c r="B290">
+        <v>511</v>
+      </c>
+    </row>
+    <row r="291" spans="1:2">
+      <c r="A291" s="2">
+        <v>46250.01041666666</v>
+      </c>
+      <c r="B291">
+        <v>503</v>
+      </c>
+    </row>
+    <row r="292" spans="1:2">
+      <c r="A292" s="2">
+        <v>46250.02083333334</v>
+      </c>
+      <c r="B292">
+        <v>503</v>
+      </c>
+    </row>
+    <row r="293" spans="1:2">
+      <c r="A293" s="2">
+        <v>46250.03125</v>
+      </c>
+      <c r="B293">
+        <v>504</v>
+      </c>
+    </row>
+    <row r="294" spans="1:2">
+      <c r="A294" s="2">
+        <v>46250.04166666666</v>
+      </c>
+      <c r="B294">
+        <v>506</v>
+      </c>
+    </row>
+    <row r="295" spans="1:2">
+      <c r="A295" s="2">
+        <v>46250.05208333334</v>
+      </c>
+      <c r="B295">
+        <v>504</v>
+      </c>
+    </row>
+    <row r="296" spans="1:2">
+      <c r="A296" s="2">
+        <v>46250.0625</v>
+      </c>
+      <c r="B296">
+        <v>505</v>
+      </c>
+    </row>
+    <row r="297" spans="1:2">
+      <c r="A297" s="2">
+        <v>46250.07291666666</v>
+      </c>
+      <c r="B297">
+        <v>504</v>
+      </c>
+    </row>
+    <row r="298" spans="1:2">
+      <c r="A298" s="2">
+        <v>46250.08333333334</v>
+      </c>
+      <c r="B298">
+        <v>504</v>
+      </c>
+    </row>
+    <row r="299" spans="1:2">
+      <c r="A299" s="2">
+        <v>46250.09375</v>
+      </c>
+      <c r="B299">
+        <v>504</v>
+      </c>
+    </row>
+    <row r="300" spans="1:2">
+      <c r="A300" s="2">
+        <v>46250.10416666666</v>
+      </c>
+      <c r="B300">
+        <v>504</v>
+      </c>
+    </row>
+    <row r="301" spans="1:2">
+      <c r="A301" s="2">
+        <v>46250.11458333334</v>
+      </c>
+      <c r="B301">
+        <v>503</v>
+      </c>
+    </row>
+    <row r="302" spans="1:2">
+      <c r="A302" s="2">
+        <v>46250.125</v>
+      </c>
+      <c r="B302">
+        <v>506</v>
+      </c>
+    </row>
+    <row r="303" spans="1:2">
+      <c r="A303" s="2">
+        <v>46250.13541666666</v>
+      </c>
+      <c r="B303">
+        <v>505</v>
+      </c>
+    </row>
+    <row r="304" spans="1:2">
+      <c r="A304" s="2">
+        <v>46250.14583333334</v>
+      </c>
+      <c r="B304">
+        <v>504</v>
+      </c>
+    </row>
+    <row r="305" spans="1:2">
+      <c r="A305" s="2">
+        <v>46250.15625</v>
+      </c>
+      <c r="B305">
+        <v>504</v>
+      </c>
+    </row>
+    <row r="306" spans="1:2">
+      <c r="A306" s="2">
+        <v>46250.16666666666</v>
+      </c>
+      <c r="B306">
+        <v>506</v>
+      </c>
+    </row>
+    <row r="307" spans="1:2">
+      <c r="A307" s="2">
+        <v>46250.17708333334</v>
+      </c>
+      <c r="B307">
+        <v>503</v>
+      </c>
+    </row>
+    <row r="308" spans="1:2">
+      <c r="A308" s="2">
+        <v>46250.1875</v>
+      </c>
+      <c r="B308">
+        <v>503</v>
+      </c>
+    </row>
+    <row r="309" spans="1:2">
+      <c r="A309" s="2">
+        <v>46250.19791666666</v>
+      </c>
+      <c r="B309">
+        <v>501</v>
+      </c>
+    </row>
+    <row r="310" spans="1:2">
+      <c r="A310" s="2">
+        <v>46250.20833333334</v>
+      </c>
+      <c r="B310">
+        <v>450</v>
+      </c>
+    </row>
+    <row r="311" spans="1:2">
+      <c r="A311" s="2">
+        <v>46250.21875</v>
+      </c>
+      <c r="B311">
+        <v>453</v>
+      </c>
+    </row>
+    <row r="312" spans="1:2">
+      <c r="A312" s="2">
+        <v>46250.22916666666</v>
+      </c>
+      <c r="B312">
+        <v>453</v>
+      </c>
+    </row>
+    <row r="313" spans="1:2">
+      <c r="A313" s="2">
+        <v>46250.23958333334</v>
+      </c>
+      <c r="B313">
+        <v>456</v>
+      </c>
+    </row>
+    <row r="314" spans="1:2">
+      <c r="A314" s="2">
+        <v>46250.25</v>
+      </c>
+      <c r="B314">
+        <v>509</v>
+      </c>
+    </row>
+    <row r="315" spans="1:2">
+      <c r="A315" s="2">
+        <v>46250.26041666666</v>
+      </c>
+      <c r="B315">
+        <v>510</v>
+      </c>
+    </row>
+    <row r="316" spans="1:2">
+      <c r="A316" s="2">
+        <v>46250.27083333334</v>
+      </c>
+      <c r="B316">
+        <v>506</v>
+      </c>
+    </row>
+    <row r="317" spans="1:2">
+      <c r="A317" s="2">
+        <v>46250.28125</v>
+      </c>
+      <c r="B317">
+        <v>506</v>
+      </c>
+    </row>
+    <row r="318" spans="1:2">
+      <c r="A318" s="2">
+        <v>46250.29166666666</v>
+      </c>
+      <c r="B318">
+        <v>506</v>
+      </c>
+    </row>
+    <row r="319" spans="1:2">
+      <c r="A319" s="2">
+        <v>46250.30208333334</v>
+      </c>
+      <c r="B319">
+        <v>502</v>
+      </c>
+    </row>
+    <row r="320" spans="1:2">
+      <c r="A320" s="2">
+        <v>46250.3125</v>
+      </c>
+      <c r="B320">
+        <v>504</v>
+      </c>
+    </row>
+    <row r="321" spans="1:2">
+      <c r="A321" s="2">
+        <v>46250.32291666666</v>
+      </c>
+      <c r="B321">
+        <v>503</v>
+      </c>
+    </row>
+    <row r="322" spans="1:2">
+      <c r="A322" s="2">
+        <v>46250.33333333334</v>
+      </c>
+      <c r="B322">
+        <v>445</v>
+      </c>
+    </row>
+    <row r="323" spans="1:2">
+      <c r="A323" s="2">
+        <v>46250.34375</v>
+      </c>
+      <c r="B323">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="324" spans="1:2">
+      <c r="A324" s="2">
+        <v>46250.35416666666</v>
+      </c>
+      <c r="B324">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="325" spans="1:2">
+      <c r="A325" s="2">
+        <v>46250.36458333334</v>
+      </c>
+      <c r="B325">
+        <v>437</v>
+      </c>
+    </row>
+    <row r="326" spans="1:2">
+      <c r="A326" s="2">
+        <v>46250.375</v>
+      </c>
+      <c r="B326">
+        <v>281</v>
+      </c>
+    </row>
+    <row r="327" spans="1:2">
+      <c r="A327" s="2">
+        <v>46250.38541666666</v>
+      </c>
+      <c r="B327">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="328" spans="1:2">
+      <c r="A328" s="2">
+        <v>46250.39583333334</v>
+      </c>
+      <c r="B328">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="329" spans="1:2">
+      <c r="A329" s="2">
+        <v>46250.40625</v>
+      </c>
+      <c r="B329">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="330" spans="1:2">
+      <c r="A330" s="2">
+        <v>46250.41666666666</v>
+      </c>
+      <c r="B330">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="331" spans="1:2">
+      <c r="A331" s="2">
+        <v>46250.42708333334</v>
+      </c>
+      <c r="B331">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="332" spans="1:2">
+      <c r="A332" s="2">
+        <v>46250.4375</v>
+      </c>
+      <c r="B332">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="333" spans="1:2">
+      <c r="A333" s="2">
+        <v>46250.44791666666</v>
+      </c>
+      <c r="B333">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="334" spans="1:2">
+      <c r="A334" s="2">
+        <v>46250.45833333334</v>
+      </c>
+      <c r="B334">
+        <v>255</v>
+      </c>
+    </row>
+    <row r="335" spans="1:2">
+      <c r="A335" s="2">
+        <v>46250.46875</v>
+      </c>
+      <c r="B335">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="336" spans="1:2">
+      <c r="A336" s="2">
+        <v>46250.47916666666</v>
+      </c>
+      <c r="B336">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="337" spans="1:2">
+      <c r="A337" s="2">
+        <v>46250.48958333334</v>
+      </c>
+      <c r="B337">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="338" spans="1:2">
+      <c r="A338" s="2">
+        <v>46250.5</v>
+      </c>
+      <c r="B338">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="339" spans="1:2">
+      <c r="A339" s="2">
+        <v>46250.51041666666</v>
+      </c>
+      <c r="B339">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="340" spans="1:2">
+      <c r="A340" s="2">
+        <v>46250.52083333334</v>
+      </c>
+      <c r="B340">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="341" spans="1:2">
+      <c r="A341" s="2">
+        <v>46250.53125</v>
+      </c>
+      <c r="B341">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="342" spans="1:2">
+      <c r="A342" s="2">
+        <v>46250.54166666666</v>
+      </c>
+      <c r="B342">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="343" spans="1:2">
+      <c r="A343" s="2">
+        <v>46250.55208333334</v>
+      </c>
+      <c r="B343">
         <v>246</v>
+      </c>
+    </row>
+    <row r="344" spans="1:2">
+      <c r="A344" s="2">
+        <v>46250.5625</v>
+      </c>
+      <c r="B344">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="345" spans="1:2">
+      <c r="A345" s="2">
+        <v>46250.57291666666</v>
+      </c>
+      <c r="B345">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="346" spans="1:2">
+      <c r="A346" s="2">
+        <v>46250.58333333334</v>
+      </c>
+      <c r="B346">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="347" spans="1:2">
+      <c r="A347" s="2">
+        <v>46250.59375</v>
+      </c>
+      <c r="B347">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="348" spans="1:2">
+      <c r="A348" s="2">
+        <v>46250.60416666666</v>
+      </c>
+      <c r="B348">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="349" spans="1:2">
+      <c r="A349" s="2">
+        <v>46250.61458333334</v>
+      </c>
+      <c r="B349">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="350" spans="1:2">
+      <c r="A350" s="2">
+        <v>46250.625</v>
+      </c>
+      <c r="B350">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="351" spans="1:2">
+      <c r="A351" s="2">
+        <v>46250.63541666666</v>
+      </c>
+      <c r="B351">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="352" spans="1:2">
+      <c r="A352" s="2">
+        <v>46250.64583333334</v>
+      </c>
+      <c r="B352">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="353" spans="1:2">
+      <c r="A353" s="2">
+        <v>46250.65625</v>
+      </c>
+      <c r="B353">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="354" spans="1:2">
+      <c r="A354" s="2">
+        <v>46250.66666666666</v>
+      </c>
+      <c r="B354">
+        <v>285</v>
+      </c>
+    </row>
+    <row r="355" spans="1:2">
+      <c r="A355" s="2">
+        <v>46250.67708333334</v>
+      </c>
+      <c r="B355">
+        <v>286</v>
+      </c>
+    </row>
+    <row r="356" spans="1:2">
+      <c r="A356" s="2">
+        <v>46250.6875</v>
+      </c>
+      <c r="B356">
+        <v>274</v>
+      </c>
+    </row>
+    <row r="357" spans="1:2">
+      <c r="A357" s="2">
+        <v>46250.69791666666</v>
+      </c>
+      <c r="B357">
+        <v>284</v>
+      </c>
+    </row>
+    <row r="358" spans="1:2">
+      <c r="A358" s="2">
+        <v>46250.70833333334</v>
+      </c>
+      <c r="B358">
+        <v>582</v>
+      </c>
+    </row>
+    <row r="359" spans="1:2">
+      <c r="A359" s="2">
+        <v>46250.71875</v>
+      </c>
+      <c r="B359">
+        <v>606</v>
+      </c>
+    </row>
+    <row r="360" spans="1:2">
+      <c r="A360" s="2">
+        <v>46250.72916666666</v>
+      </c>
+      <c r="B360">
+        <v>607</v>
+      </c>
+    </row>
+    <row r="361" spans="1:2">
+      <c r="A361" s="2">
+        <v>46250.73958333334</v>
+      </c>
+      <c r="B361">
+        <v>646</v>
+      </c>
+    </row>
+    <row r="362" spans="1:2">
+      <c r="A362" s="2">
+        <v>46250.75</v>
+      </c>
+      <c r="B362">
+        <v>672</v>
+      </c>
+    </row>
+    <row r="363" spans="1:2">
+      <c r="A363" s="2">
+        <v>46250.76041666666</v>
+      </c>
+      <c r="B363">
+        <v>680</v>
+      </c>
+    </row>
+    <row r="364" spans="1:2">
+      <c r="A364" s="2">
+        <v>46250.77083333334</v>
+      </c>
+      <c r="B364">
+        <v>677</v>
+      </c>
+    </row>
+    <row r="365" spans="1:2">
+      <c r="A365" s="2">
+        <v>46250.78125</v>
+      </c>
+      <c r="B365">
+        <v>677</v>
+      </c>
+    </row>
+    <row r="366" spans="1:2">
+      <c r="A366" s="2">
+        <v>46250.79166666666</v>
+      </c>
+      <c r="B366">
+        <v>656</v>
+      </c>
+    </row>
+    <row r="367" spans="1:2">
+      <c r="A367" s="2">
+        <v>46250.80208333334</v>
+      </c>
+      <c r="B367">
+        <v>659</v>
+      </c>
+    </row>
+    <row r="368" spans="1:2">
+      <c r="A368" s="2">
+        <v>46250.8125</v>
+      </c>
+      <c r="B368">
+        <v>657</v>
+      </c>
+    </row>
+    <row r="369" spans="1:2">
+      <c r="A369" s="2">
+        <v>46250.82291666666</v>
+      </c>
+      <c r="B369">
+        <v>661</v>
+      </c>
+    </row>
+    <row r="370" spans="1:2">
+      <c r="A370" s="2">
+        <v>46250.83333333334</v>
+      </c>
+      <c r="B370">
+        <v>682</v>
+      </c>
+    </row>
+    <row r="371" spans="1:2">
+      <c r="A371" s="2">
+        <v>46250.84375</v>
+      </c>
+      <c r="B371">
+        <v>684</v>
+      </c>
+    </row>
+    <row r="372" spans="1:2">
+      <c r="A372" s="2">
+        <v>46250.85416666666</v>
+      </c>
+      <c r="B372">
+        <v>683</v>
+      </c>
+    </row>
+    <row r="373" spans="1:2">
+      <c r="A373" s="2">
+        <v>46250.86458333334</v>
+      </c>
+      <c r="B373">
+        <v>690</v>
+      </c>
+    </row>
+    <row r="374" spans="1:2">
+      <c r="A374" s="2">
+        <v>46250.875</v>
+      </c>
+      <c r="B374">
+        <v>667</v>
+      </c>
+    </row>
+    <row r="375" spans="1:2">
+      <c r="A375" s="2">
+        <v>46250.88541666666</v>
+      </c>
+      <c r="B375">
+        <v>666</v>
+      </c>
+    </row>
+    <row r="376" spans="1:2">
+      <c r="A376" s="2">
+        <v>46250.89583333334</v>
+      </c>
+      <c r="B376">
+        <v>665</v>
+      </c>
+    </row>
+    <row r="377" spans="1:2">
+      <c r="A377" s="2">
+        <v>46250.90625</v>
+      </c>
+      <c r="B377">
+        <v>673</v>
+      </c>
+    </row>
+    <row r="378" spans="1:2">
+      <c r="A378" s="2">
+        <v>46250.91666666666</v>
+      </c>
+      <c r="B378">
+        <v>664</v>
+      </c>
+    </row>
+    <row r="379" spans="1:2">
+      <c r="A379" s="2">
+        <v>46250.92708333334</v>
+      </c>
+      <c r="B379">
+        <v>662</v>
+      </c>
+    </row>
+    <row r="380" spans="1:2">
+      <c r="A380" s="2">
+        <v>46250.9375</v>
+      </c>
+      <c r="B380">
+        <v>662</v>
+      </c>
+    </row>
+    <row r="381" spans="1:2">
+      <c r="A381" s="2">
+        <v>46250.94791666666</v>
+      </c>
+      <c r="B381">
+        <v>660</v>
+      </c>
+    </row>
+    <row r="382" spans="1:2">
+      <c r="A382" s="2">
+        <v>46250.95833333334</v>
+      </c>
+      <c r="B382">
+        <v>600</v>
+      </c>
+    </row>
+    <row r="383" spans="1:2">
+      <c r="A383" s="2">
+        <v>46250.96875</v>
+      </c>
+      <c r="B383">
+        <v>595</v>
+      </c>
+    </row>
+    <row r="384" spans="1:2">
+      <c r="A384" s="2">
+        <v>46250.97916666666</v>
+      </c>
+      <c r="B384">
+        <v>595</v>
+      </c>
+    </row>
+    <row r="385" spans="1:2">
+      <c r="A385" s="2">
+        <v>46250.98958333334</v>
+      </c>
+      <c r="B385">
+        <v>593</v>
+      </c>
+    </row>
+    <row r="386" spans="1:2">
+      <c r="A386" s="2">
+        <v>46251</v>
+      </c>
+      <c r="B386">
+        <v>510</v>
+      </c>
+    </row>
+    <row r="387" spans="1:2">
+      <c r="A387" s="2">
+        <v>46251.01041666666</v>
+      </c>
+      <c r="B387">
+        <v>507</v>
+      </c>
+    </row>
+    <row r="388" spans="1:2">
+      <c r="A388" s="2">
+        <v>46251.02083333334</v>
+      </c>
+      <c r="B388">
+        <v>509</v>
+      </c>
+    </row>
+    <row r="389" spans="1:2">
+      <c r="A389" s="2">
+        <v>46251.03125</v>
+      </c>
+      <c r="B389">
+        <v>507</v>
+      </c>
+    </row>
+    <row r="390" spans="1:2">
+      <c r="A390" s="2">
+        <v>46251.04166666666</v>
+      </c>
+      <c r="B390">
+        <v>409</v>
+      </c>
+    </row>
+    <row r="391" spans="1:2">
+      <c r="A391" s="2">
+        <v>46251.05208333334</v>
+      </c>
+      <c r="B391">
+        <v>406</v>
+      </c>
+    </row>
+    <row r="392" spans="1:2">
+      <c r="A392" s="2">
+        <v>46251.0625</v>
+      </c>
+      <c r="B392">
+        <v>405</v>
+      </c>
+    </row>
+    <row r="393" spans="1:2">
+      <c r="A393" s="2">
+        <v>46251.07291666666</v>
+      </c>
+      <c r="B393">
+        <v>405</v>
+      </c>
+    </row>
+    <row r="394" spans="1:2">
+      <c r="A394" s="2">
+        <v>46251.08333333334</v>
+      </c>
+      <c r="B394">
+        <v>407</v>
+      </c>
+    </row>
+    <row r="395" spans="1:2">
+      <c r="A395" s="2">
+        <v>46251.09375</v>
+      </c>
+      <c r="B395">
+        <v>406</v>
+      </c>
+    </row>
+    <row r="396" spans="1:2">
+      <c r="A396" s="2">
+        <v>46251.10416666666</v>
+      </c>
+      <c r="B396">
+        <v>406</v>
+      </c>
+    </row>
+    <row r="397" spans="1:2">
+      <c r="A397" s="2">
+        <v>46251.11458333334</v>
+      </c>
+      <c r="B397">
+        <v>406</v>
+      </c>
+    </row>
+    <row r="398" spans="1:2">
+      <c r="A398" s="2">
+        <v>46251.125</v>
+      </c>
+      <c r="B398">
+        <v>406</v>
+      </c>
+    </row>
+    <row r="399" spans="1:2">
+      <c r="A399" s="2">
+        <v>46251.13541666666</v>
+      </c>
+      <c r="B399">
+        <v>405</v>
+      </c>
+    </row>
+    <row r="400" spans="1:2">
+      <c r="A400" s="2">
+        <v>46251.14583333334</v>
+      </c>
+      <c r="B400">
+        <v>405</v>
+      </c>
+    </row>
+    <row r="401" spans="1:2">
+      <c r="A401" s="2">
+        <v>46251.15625</v>
+      </c>
+      <c r="B401">
+        <v>409</v>
+      </c>
+    </row>
+    <row r="402" spans="1:2">
+      <c r="A402" s="2">
+        <v>46251.16666666666</v>
+      </c>
+      <c r="B402">
+        <v>481</v>
+      </c>
+    </row>
+    <row r="403" spans="1:2">
+      <c r="A403" s="2">
+        <v>46251.17708333334</v>
+      </c>
+      <c r="B403">
+        <v>477</v>
+      </c>
+    </row>
+    <row r="404" spans="1:2">
+      <c r="A404" s="2">
+        <v>46251.1875</v>
+      </c>
+      <c r="B404">
+        <v>482</v>
+      </c>
+    </row>
+    <row r="405" spans="1:2">
+      <c r="A405" s="2">
+        <v>46251.19791666666</v>
+      </c>
+      <c r="B405">
+        <v>484</v>
+      </c>
+    </row>
+    <row r="406" spans="1:2">
+      <c r="A406" s="2">
+        <v>46251.20833333334</v>
+      </c>
+      <c r="B406">
+        <v>487</v>
+      </c>
+    </row>
+    <row r="407" spans="1:2">
+      <c r="A407" s="2">
+        <v>46251.21875</v>
+      </c>
+      <c r="B407">
+        <v>481</v>
+      </c>
+    </row>
+    <row r="408" spans="1:2">
+      <c r="A408" s="2">
+        <v>46251.22916666666</v>
+      </c>
+      <c r="B408">
+        <v>481</v>
+      </c>
+    </row>
+    <row r="409" spans="1:2">
+      <c r="A409" s="2">
+        <v>46251.23958333334</v>
+      </c>
+      <c r="B409">
+        <v>480</v>
+      </c>
+    </row>
+    <row r="410" spans="1:2">
+      <c r="A410" s="2">
+        <v>46251.25</v>
+      </c>
+      <c r="B410">
+        <v>510</v>
+      </c>
+    </row>
+    <row r="411" spans="1:2">
+      <c r="A411" s="2">
+        <v>46251.26041666666</v>
+      </c>
+      <c r="B411">
+        <v>511</v>
+      </c>
+    </row>
+    <row r="412" spans="1:2">
+      <c r="A412" s="2">
+        <v>46251.27083333334</v>
+      </c>
+      <c r="B412">
+        <v>511</v>
+      </c>
+    </row>
+    <row r="413" spans="1:2">
+      <c r="A413" s="2">
+        <v>46251.28125</v>
+      </c>
+      <c r="B413">
+        <v>512</v>
+      </c>
+    </row>
+    <row r="414" spans="1:2">
+      <c r="A414" s="2">
+        <v>46251.29166666666</v>
+      </c>
+      <c r="B414">
+        <v>494</v>
+      </c>
+    </row>
+    <row r="415" spans="1:2">
+      <c r="A415" s="2">
+        <v>46251.30208333334</v>
+      </c>
+      <c r="B415">
+        <v>493</v>
+      </c>
+    </row>
+    <row r="416" spans="1:2">
+      <c r="A416" s="2">
+        <v>46251.3125</v>
+      </c>
+      <c r="B416">
+        <v>492</v>
+      </c>
+    </row>
+    <row r="417" spans="1:2">
+      <c r="A417" s="2">
+        <v>46251.32291666666</v>
+      </c>
+      <c r="B417">
+        <v>491</v>
+      </c>
+    </row>
+    <row r="418" spans="1:2">
+      <c r="A418" s="2">
+        <v>46251.33333333334</v>
+      </c>
+      <c r="B418">
+        <v>466</v>
+      </c>
+    </row>
+    <row r="419" spans="1:2">
+      <c r="A419" s="2">
+        <v>46251.34375</v>
+      </c>
+      <c r="B419">
+        <v>460</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Updating hte model for Necaluxan
</commit_message>
<xml_diff>
--- a/data_fetching/Entsoe/Actual_Production_Hydro_River.xlsx
+++ b/data_fetching/Entsoe/Actual_Production_Hydro_River.xlsx
@@ -381,7 +381,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B131"/>
+  <dimension ref="A1:B127"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:2">
@@ -394,151 +394,151 @@
     </row>
     <row r="2" spans="1:2">
       <c r="A2" s="2">
-        <v>46253</v>
+        <v>46258</v>
       </c>
       <c r="B2">
-        <v>455</v>
+        <v>408</v>
       </c>
     </row>
     <row r="3" spans="1:2">
       <c r="A3" s="2">
-        <v>46253.01041666666</v>
+        <v>46258.01041666666</v>
       </c>
       <c r="B3">
-        <v>439</v>
+        <v>400</v>
       </c>
     </row>
     <row r="4" spans="1:2">
       <c r="A4" s="2">
-        <v>46253.02083333334</v>
+        <v>46258.02083333334</v>
       </c>
       <c r="B4">
-        <v>439</v>
+        <v>398</v>
       </c>
     </row>
     <row r="5" spans="1:2">
       <c r="A5" s="2">
-        <v>46253.03125</v>
+        <v>46258.03125</v>
       </c>
       <c r="B5">
-        <v>438</v>
+        <v>399</v>
       </c>
     </row>
     <row r="6" spans="1:2">
       <c r="A6" s="2">
-        <v>46253.04166666666</v>
+        <v>46258.04166666666</v>
       </c>
       <c r="B6">
-        <v>383</v>
+        <v>400</v>
       </c>
     </row>
     <row r="7" spans="1:2">
       <c r="A7" s="2">
-        <v>46253.05208333334</v>
+        <v>46258.05208333334</v>
       </c>
       <c r="B7">
-        <v>369</v>
+        <v>399</v>
       </c>
     </row>
     <row r="8" spans="1:2">
       <c r="A8" s="2">
-        <v>46253.0625</v>
+        <v>46258.0625</v>
       </c>
       <c r="B8">
-        <v>369</v>
+        <v>399</v>
       </c>
     </row>
     <row r="9" spans="1:2">
       <c r="A9" s="2">
-        <v>46253.07291666666</v>
+        <v>46258.07291666666</v>
       </c>
       <c r="B9">
-        <v>368</v>
+        <v>381</v>
       </c>
     </row>
     <row r="10" spans="1:2">
       <c r="A10" s="2">
-        <v>46253.08333333334</v>
+        <v>46258.08333333334</v>
       </c>
       <c r="B10">
-        <v>330</v>
+        <v>381</v>
       </c>
     </row>
     <row r="11" spans="1:2">
       <c r="A11" s="2">
-        <v>46253.09375</v>
+        <v>46258.09375</v>
       </c>
       <c r="B11">
-        <v>328</v>
+        <v>380</v>
       </c>
     </row>
     <row r="12" spans="1:2">
       <c r="A12" s="2">
-        <v>46253.10416666666</v>
+        <v>46258.10416666666</v>
       </c>
       <c r="B12">
-        <v>329</v>
+        <v>380</v>
       </c>
     </row>
     <row r="13" spans="1:2">
       <c r="A13" s="2">
-        <v>46253.11458333334</v>
+        <v>46258.11458333334</v>
       </c>
       <c r="B13">
-        <v>328</v>
+        <v>379</v>
       </c>
     </row>
     <row r="14" spans="1:2">
       <c r="A14" s="2">
-        <v>46253.125</v>
+        <v>46258.125</v>
       </c>
       <c r="B14">
-        <v>317</v>
+        <v>380</v>
       </c>
     </row>
     <row r="15" spans="1:2">
       <c r="A15" s="2">
-        <v>46253.13541666666</v>
+        <v>46258.13541666666</v>
       </c>
       <c r="B15">
-        <v>317</v>
+        <v>380</v>
       </c>
     </row>
     <row r="16" spans="1:2">
       <c r="A16" s="2">
-        <v>46253.14583333334</v>
+        <v>46258.14583333334</v>
       </c>
       <c r="B16">
-        <v>317</v>
+        <v>380</v>
       </c>
     </row>
     <row r="17" spans="1:2">
       <c r="A17" s="2">
-        <v>46253.15625</v>
+        <v>46258.15625</v>
       </c>
       <c r="B17">
-        <v>319</v>
+        <v>380</v>
       </c>
     </row>
     <row r="18" spans="1:2">
       <c r="A18" s="2">
-        <v>46253.16666666666</v>
+        <v>46258.16666666666</v>
       </c>
       <c r="B18">
-        <v>388</v>
+        <v>402</v>
       </c>
     </row>
     <row r="19" spans="1:2">
       <c r="A19" s="2">
-        <v>46253.17708333334</v>
+        <v>46258.17708333334</v>
       </c>
       <c r="B19">
-        <v>393</v>
+        <v>403</v>
       </c>
     </row>
     <row r="20" spans="1:2">
       <c r="A20" s="2">
-        <v>46253.1875</v>
+        <v>46258.1875</v>
       </c>
       <c r="B20">
         <v>403</v>
@@ -546,890 +546,858 @@
     </row>
     <row r="21" spans="1:2">
       <c r="A21" s="2">
-        <v>46253.19791666666</v>
+        <v>46258.19791666666</v>
       </c>
       <c r="B21">
-        <v>403</v>
+        <v>407</v>
       </c>
     </row>
     <row r="22" spans="1:2">
       <c r="A22" s="2">
-        <v>46253.20833333334</v>
+        <v>46258.20833333334</v>
       </c>
       <c r="B22">
-        <v>500</v>
+        <v>539</v>
       </c>
     </row>
     <row r="23" spans="1:2">
       <c r="A23" s="2">
-        <v>46253.21875</v>
+        <v>46258.21875</v>
       </c>
       <c r="B23">
-        <v>498</v>
+        <v>542</v>
       </c>
     </row>
     <row r="24" spans="1:2">
       <c r="A24" s="2">
-        <v>46253.22916666666</v>
+        <v>46258.22916666666</v>
       </c>
       <c r="B24">
-        <v>518</v>
+        <v>538</v>
       </c>
     </row>
     <row r="25" spans="1:2">
       <c r="A25" s="2">
-        <v>46253.23958333334</v>
+        <v>46258.23958333334</v>
       </c>
       <c r="B25">
-        <v>516</v>
+        <v>559</v>
       </c>
     </row>
     <row r="26" spans="1:2">
       <c r="A26" s="2">
-        <v>46253.25</v>
+        <v>46258.25</v>
       </c>
       <c r="B26">
-        <v>551</v>
+        <v>547</v>
       </c>
     </row>
     <row r="27" spans="1:2">
       <c r="A27" s="2">
-        <v>46253.26041666666</v>
+        <v>46258.26041666666</v>
       </c>
       <c r="B27">
-        <v>555</v>
+        <v>540</v>
       </c>
     </row>
     <row r="28" spans="1:2">
       <c r="A28" s="2">
-        <v>46253.27083333334</v>
+        <v>46258.27083333334</v>
       </c>
       <c r="B28">
-        <v>559</v>
+        <v>547</v>
       </c>
     </row>
     <row r="29" spans="1:2">
       <c r="A29" s="2">
-        <v>46253.28125</v>
+        <v>46258.28125</v>
       </c>
       <c r="B29">
-        <v>579</v>
+        <v>547</v>
       </c>
     </row>
     <row r="30" spans="1:2">
       <c r="A30" s="2">
-        <v>46253.29166666666</v>
+        <v>46258.29166666666</v>
       </c>
       <c r="B30">
-        <v>572</v>
+        <v>538</v>
       </c>
     </row>
     <row r="31" spans="1:2">
       <c r="A31" s="2">
-        <v>46253.30208333334</v>
+        <v>46258.30208333334</v>
       </c>
       <c r="B31">
-        <v>571</v>
+        <v>527</v>
       </c>
     </row>
     <row r="32" spans="1:2">
       <c r="A32" s="2">
-        <v>46253.3125</v>
+        <v>46258.3125</v>
       </c>
       <c r="B32">
-        <v>570</v>
+        <v>524</v>
       </c>
     </row>
     <row r="33" spans="1:2">
       <c r="A33" s="2">
-        <v>46253.32291666666</v>
+        <v>46258.32291666666</v>
       </c>
       <c r="B33">
-        <v>569</v>
+        <v>524</v>
       </c>
     </row>
     <row r="34" spans="1:2">
       <c r="A34" s="2">
-        <v>46253.33333333334</v>
+        <v>46258.33333333334</v>
       </c>
       <c r="B34">
-        <v>503</v>
+        <v>534</v>
       </c>
     </row>
     <row r="35" spans="1:2">
       <c r="A35" s="2">
-        <v>46253.34375</v>
+        <v>46258.34375</v>
       </c>
       <c r="B35">
-        <v>489</v>
+        <v>536</v>
       </c>
     </row>
     <row r="36" spans="1:2">
       <c r="A36" s="2">
-        <v>46253.35416666666</v>
+        <v>46258.35416666666</v>
       </c>
       <c r="B36">
-        <v>494</v>
+        <v>529</v>
       </c>
     </row>
     <row r="37" spans="1:2">
       <c r="A37" s="2">
-        <v>46253.36458333334</v>
+        <v>46258.36458333334</v>
       </c>
       <c r="B37">
-        <v>499</v>
+        <v>529</v>
       </c>
     </row>
     <row r="38" spans="1:2">
       <c r="A38" s="2">
-        <v>46253.375</v>
+        <v>46258.375</v>
       </c>
       <c r="B38">
-        <v>422</v>
+        <v>424</v>
       </c>
     </row>
     <row r="39" spans="1:2">
       <c r="A39" s="2">
-        <v>46253.38541666666</v>
+        <v>46258.38541666666</v>
       </c>
       <c r="B39">
-        <v>412</v>
+        <v>415</v>
       </c>
     </row>
     <row r="40" spans="1:2">
       <c r="A40" s="2">
-        <v>46253.39583333334</v>
+        <v>46258.39583333334</v>
       </c>
       <c r="B40">
-        <v>417</v>
+        <v>414</v>
       </c>
     </row>
     <row r="41" spans="1:2">
       <c r="A41" s="2">
-        <v>46253.40625</v>
+        <v>46258.40625</v>
       </c>
       <c r="B41">
-        <v>410</v>
+        <v>412</v>
       </c>
     </row>
     <row r="42" spans="1:2">
       <c r="A42" s="2">
-        <v>46253.41666666666</v>
+        <v>46258.41666666666</v>
       </c>
       <c r="B42">
-        <v>307</v>
+        <v>236</v>
       </c>
     </row>
     <row r="43" spans="1:2">
       <c r="A43" s="2">
-        <v>46253.42708333334</v>
+        <v>46258.42708333334</v>
       </c>
       <c r="B43">
-        <v>337</v>
+        <v>230</v>
       </c>
     </row>
     <row r="44" spans="1:2">
       <c r="A44" s="2">
-        <v>46253.4375</v>
+        <v>46258.4375</v>
       </c>
       <c r="B44">
-        <v>339</v>
+        <v>265</v>
       </c>
     </row>
     <row r="45" spans="1:2">
       <c r="A45" s="2">
-        <v>46253.44791666666</v>
+        <v>46258.44791666666</v>
       </c>
       <c r="B45">
-        <v>337</v>
+        <v>268</v>
       </c>
     </row>
     <row r="46" spans="1:2">
       <c r="A46" s="2">
-        <v>46253.45833333334</v>
+        <v>46258.45833333334</v>
       </c>
       <c r="B46">
-        <v>341</v>
+        <v>283</v>
       </c>
     </row>
     <row r="47" spans="1:2">
       <c r="A47" s="2">
-        <v>46253.46875</v>
+        <v>46258.46875</v>
       </c>
       <c r="B47">
-        <v>342</v>
+        <v>298</v>
       </c>
     </row>
     <row r="48" spans="1:2">
       <c r="A48" s="2">
-        <v>46253.47916666666</v>
+        <v>46258.47916666666</v>
       </c>
       <c r="B48">
-        <v>339</v>
+        <v>291</v>
       </c>
     </row>
     <row r="49" spans="1:2">
       <c r="A49" s="2">
-        <v>46253.48958333334</v>
+        <v>46258.48958333334</v>
       </c>
       <c r="B49">
-        <v>336</v>
+        <v>293</v>
       </c>
     </row>
     <row r="50" spans="1:2">
       <c r="A50" s="2">
-        <v>46253.5</v>
+        <v>46258.5</v>
       </c>
       <c r="B50">
-        <v>290</v>
+        <v>298</v>
       </c>
     </row>
     <row r="51" spans="1:2">
       <c r="A51" s="2">
-        <v>46253.51041666666</v>
+        <v>46258.51041666666</v>
       </c>
       <c r="B51">
-        <v>279</v>
+        <v>297</v>
       </c>
     </row>
     <row r="52" spans="1:2">
       <c r="A52" s="2">
-        <v>46253.52083333334</v>
+        <v>46258.52083333334</v>
       </c>
       <c r="B52">
-        <v>280</v>
+        <v>293</v>
       </c>
     </row>
     <row r="53" spans="1:2">
       <c r="A53" s="2">
-        <v>46253.53125</v>
+        <v>46258.53125</v>
       </c>
       <c r="B53">
-        <v>278</v>
+        <v>287</v>
       </c>
     </row>
     <row r="54" spans="1:2">
       <c r="A54" s="2">
-        <v>46253.54166666666</v>
+        <v>46258.54166666666</v>
       </c>
       <c r="B54">
-        <v>219</v>
+        <v>269</v>
       </c>
     </row>
     <row r="55" spans="1:2">
       <c r="A55" s="2">
-        <v>46253.55208333334</v>
+        <v>46258.55208333334</v>
       </c>
       <c r="B55">
-        <v>214</v>
+        <v>269</v>
       </c>
     </row>
     <row r="56" spans="1:2">
       <c r="A56" s="2">
-        <v>46253.5625</v>
+        <v>46258.5625</v>
       </c>
       <c r="B56">
-        <v>215</v>
+        <v>264</v>
       </c>
     </row>
     <row r="57" spans="1:2">
       <c r="A57" s="2">
-        <v>46253.57291666666</v>
+        <v>46258.57291666666</v>
       </c>
       <c r="B57">
-        <v>234</v>
+        <v>263</v>
       </c>
     </row>
     <row r="58" spans="1:2">
       <c r="A58" s="2">
-        <v>46253.58333333334</v>
+        <v>46258.58333333334</v>
       </c>
       <c r="B58">
-        <v>239</v>
+        <v>261</v>
       </c>
     </row>
     <row r="59" spans="1:2">
       <c r="A59" s="2">
-        <v>46253.59375</v>
+        <v>46258.59375</v>
       </c>
       <c r="B59">
-        <v>261</v>
+        <v>266</v>
       </c>
     </row>
     <row r="60" spans="1:2">
       <c r="A60" s="2">
-        <v>46253.60416666666</v>
+        <v>46258.60416666666</v>
       </c>
       <c r="B60">
-        <v>258</v>
+        <v>250</v>
       </c>
     </row>
     <row r="61" spans="1:2">
       <c r="A61" s="2">
-        <v>46253.61458333334</v>
+        <v>46258.61458333334</v>
       </c>
       <c r="B61">
-        <v>265</v>
+        <v>250</v>
       </c>
     </row>
     <row r="62" spans="1:2">
       <c r="A62" s="2">
-        <v>46253.625</v>
+        <v>46258.625</v>
       </c>
       <c r="B62">
-        <v>293</v>
+        <v>256</v>
       </c>
     </row>
     <row r="63" spans="1:2">
       <c r="A63" s="2">
-        <v>46253.63541666666</v>
+        <v>46258.63541666666</v>
       </c>
       <c r="B63">
-        <v>295</v>
+        <v>256</v>
       </c>
     </row>
     <row r="64" spans="1:2">
       <c r="A64" s="2">
-        <v>46253.64583333334</v>
+        <v>46258.64583333334</v>
       </c>
       <c r="B64">
-        <v>295</v>
+        <v>253</v>
       </c>
     </row>
     <row r="65" spans="1:2">
       <c r="A65" s="2">
-        <v>46253.65625</v>
+        <v>46258.65625</v>
       </c>
       <c r="B65">
-        <v>299</v>
+        <v>233</v>
       </c>
     </row>
     <row r="66" spans="1:2">
       <c r="A66" s="2">
-        <v>46253.66666666666</v>
+        <v>46258.66666666666</v>
       </c>
       <c r="B66">
-        <v>479</v>
+        <v>519</v>
       </c>
     </row>
     <row r="67" spans="1:2">
       <c r="A67" s="2">
-        <v>46253.67708333334</v>
+        <v>46258.67708333334</v>
       </c>
       <c r="B67">
-        <v>495</v>
+        <v>484</v>
       </c>
     </row>
     <row r="68" spans="1:2">
       <c r="A68" s="2">
-        <v>46253.6875</v>
+        <v>46258.6875</v>
       </c>
       <c r="B68">
-        <v>492</v>
+        <v>475</v>
       </c>
     </row>
     <row r="69" spans="1:2">
       <c r="A69" s="2">
-        <v>46253.69791666666</v>
+        <v>46258.69791666666</v>
       </c>
       <c r="B69">
-        <v>506</v>
+        <v>482</v>
       </c>
     </row>
     <row r="70" spans="1:2">
       <c r="A70" s="2">
-        <v>46253.70833333334</v>
+        <v>46258.70833333334</v>
       </c>
       <c r="B70">
-        <v>614</v>
+        <v>634</v>
       </c>
     </row>
     <row r="71" spans="1:2">
       <c r="A71" s="2">
-        <v>46253.71875</v>
+        <v>46258.71875</v>
       </c>
       <c r="B71">
-        <v>624</v>
+        <v>657</v>
       </c>
     </row>
     <row r="72" spans="1:2">
       <c r="A72" s="2">
-        <v>46253.72916666666</v>
+        <v>46258.72916666666</v>
       </c>
       <c r="B72">
-        <v>626</v>
+        <v>664</v>
       </c>
     </row>
     <row r="73" spans="1:2">
       <c r="A73" s="2">
-        <v>46253.73958333334</v>
+        <v>46258.73958333334</v>
       </c>
       <c r="B73">
-        <v>623</v>
+        <v>670</v>
       </c>
     </row>
     <row r="74" spans="1:2">
       <c r="A74" s="2">
-        <v>46253.75</v>
+        <v>46258.75</v>
       </c>
       <c r="B74">
-        <v>623</v>
+        <v>702</v>
       </c>
     </row>
     <row r="75" spans="1:2">
       <c r="A75" s="2">
-        <v>46253.76041666666</v>
+        <v>46258.76041666666</v>
       </c>
       <c r="B75">
-        <v>0</v>
+        <v>706</v>
       </c>
     </row>
     <row r="76" spans="1:2">
       <c r="A76" s="2">
-        <v>46253.77083333334</v>
+        <v>46258.77083333334</v>
       </c>
       <c r="B76">
-        <v>670</v>
+        <v>706</v>
       </c>
     </row>
     <row r="77" spans="1:2">
       <c r="A77" s="2">
-        <v>46253.78125</v>
+        <v>46258.78125</v>
       </c>
       <c r="B77">
-        <v>662</v>
+        <v>707</v>
       </c>
     </row>
     <row r="78" spans="1:2">
       <c r="A78" s="2">
-        <v>46253.79166666666</v>
+        <v>46258.79166666666</v>
       </c>
       <c r="B78">
-        <v>662</v>
+        <v>702</v>
       </c>
     </row>
     <row r="79" spans="1:2">
       <c r="A79" s="2">
-        <v>46253.80208333334</v>
+        <v>46258.80208333334</v>
       </c>
       <c r="B79">
-        <v>671</v>
+        <v>705</v>
       </c>
     </row>
     <row r="80" spans="1:2">
       <c r="A80" s="2">
-        <v>46253.8125</v>
+        <v>46258.8125</v>
       </c>
       <c r="B80">
-        <v>670</v>
+        <v>704</v>
       </c>
     </row>
     <row r="81" spans="1:2">
       <c r="A81" s="2">
-        <v>46253.82291666666</v>
+        <v>46258.82291666666</v>
       </c>
       <c r="B81">
-        <v>691</v>
+        <v>703</v>
       </c>
     </row>
     <row r="82" spans="1:2">
       <c r="A82" s="2">
-        <v>46253.83333333334</v>
+        <v>46258.83333333334</v>
       </c>
       <c r="B82">
-        <v>679</v>
+        <v>698</v>
       </c>
     </row>
     <row r="83" spans="1:2">
       <c r="A83" s="2">
-        <v>46253.84375</v>
+        <v>46258.84375</v>
       </c>
       <c r="B83">
-        <v>700</v>
+        <v>699</v>
       </c>
     </row>
     <row r="84" spans="1:2">
       <c r="A84" s="2">
-        <v>46253.85416666666</v>
+        <v>46258.85416666666</v>
       </c>
       <c r="B84">
-        <v>710</v>
+        <v>701</v>
       </c>
     </row>
     <row r="85" spans="1:2">
       <c r="A85" s="2">
-        <v>46253.86458333334</v>
+        <v>46258.86458333334</v>
       </c>
       <c r="B85">
-        <v>710</v>
+        <v>701</v>
       </c>
     </row>
     <row r="86" spans="1:2">
       <c r="A86" s="2">
-        <v>46253.875</v>
+        <v>46258.875</v>
       </c>
       <c r="B86">
-        <v>691</v>
+        <v>675</v>
       </c>
     </row>
     <row r="87" spans="1:2">
       <c r="A87" s="2">
-        <v>46253.88541666666</v>
+        <v>46258.88541666666</v>
       </c>
       <c r="B87">
-        <v>689</v>
+        <v>673</v>
       </c>
     </row>
     <row r="88" spans="1:2">
       <c r="A88" s="2">
-        <v>46253.89583333334</v>
+        <v>46258.89583333334</v>
       </c>
       <c r="B88">
-        <v>688</v>
+        <v>673</v>
       </c>
     </row>
     <row r="89" spans="1:2">
       <c r="A89" s="2">
-        <v>46253.90625</v>
+        <v>46258.90625</v>
       </c>
       <c r="B89">
-        <v>696</v>
+        <v>684</v>
       </c>
     </row>
     <row r="90" spans="1:2">
       <c r="A90" s="2">
-        <v>46253.91666666666</v>
+        <v>46258.91666666666</v>
       </c>
       <c r="B90">
-        <v>653</v>
+        <v>660</v>
       </c>
     </row>
     <row r="91" spans="1:2">
       <c r="A91" s="2">
-        <v>46253.92708333334</v>
+        <v>46258.92708333334</v>
       </c>
       <c r="B91">
-        <v>649</v>
+        <v>661</v>
       </c>
     </row>
     <row r="92" spans="1:2">
       <c r="A92" s="2">
-        <v>46253.9375</v>
+        <v>46258.9375</v>
       </c>
       <c r="B92">
-        <v>649</v>
+        <v>661</v>
       </c>
     </row>
     <row r="93" spans="1:2">
       <c r="A93" s="2">
-        <v>46253.94791666666</v>
+        <v>46258.94791666666</v>
       </c>
       <c r="B93">
-        <v>647</v>
+        <v>661</v>
       </c>
     </row>
     <row r="94" spans="1:2">
       <c r="A94" s="2">
-        <v>46253.95833333334</v>
+        <v>46258.95833333334</v>
       </c>
       <c r="B94">
-        <v>603</v>
+        <v>654</v>
       </c>
     </row>
     <row r="95" spans="1:2">
       <c r="A95" s="2">
-        <v>46253.96875</v>
+        <v>46258.96875</v>
       </c>
       <c r="B95">
-        <v>601</v>
+        <v>648</v>
       </c>
     </row>
     <row r="96" spans="1:2">
       <c r="A96" s="2">
-        <v>46253.97916666666</v>
+        <v>46258.97916666666</v>
       </c>
       <c r="B96">
-        <v>604</v>
+        <v>647</v>
       </c>
     </row>
     <row r="97" spans="1:2">
       <c r="A97" s="2">
-        <v>46253.98958333334</v>
+        <v>46258.98958333334</v>
       </c>
       <c r="B97">
-        <v>588</v>
+        <v>660</v>
       </c>
     </row>
     <row r="98" spans="1:2">
       <c r="A98" s="2">
-        <v>46254</v>
+        <v>46259</v>
       </c>
       <c r="B98">
-        <v>469</v>
+        <v>531</v>
       </c>
     </row>
     <row r="99" spans="1:2">
       <c r="A99" s="2">
-        <v>46254.01041666666</v>
+        <v>46259.01041666666</v>
       </c>
       <c r="B99">
-        <v>463</v>
+        <v>528</v>
       </c>
     </row>
     <row r="100" spans="1:2">
       <c r="A100" s="2">
-        <v>46254.02083333334</v>
+        <v>46259.02083333334</v>
       </c>
       <c r="B100">
-        <v>462</v>
+        <v>529</v>
       </c>
     </row>
     <row r="101" spans="1:2">
       <c r="A101" s="2">
-        <v>46254.03125</v>
+        <v>46259.03125</v>
       </c>
       <c r="B101">
-        <v>462</v>
+        <v>529</v>
       </c>
     </row>
     <row r="102" spans="1:2">
       <c r="A102" s="2">
-        <v>46254.04166666666</v>
+        <v>46259.04166666666</v>
       </c>
       <c r="B102">
-        <v>464</v>
+        <v>498</v>
       </c>
     </row>
     <row r="103" spans="1:2">
       <c r="A103" s="2">
-        <v>46254.05208333334</v>
+        <v>46259.05208333334</v>
       </c>
       <c r="B103">
-        <v>464</v>
+        <v>495</v>
       </c>
     </row>
     <row r="104" spans="1:2">
       <c r="A104" s="2">
-        <v>46254.0625</v>
+        <v>46259.0625</v>
       </c>
       <c r="B104">
-        <v>464</v>
+        <v>495</v>
       </c>
     </row>
     <row r="105" spans="1:2">
       <c r="A105" s="2">
-        <v>46254.07291666666</v>
+        <v>46259.07291666666</v>
       </c>
       <c r="B105">
-        <v>463</v>
+        <v>495</v>
       </c>
     </row>
     <row r="106" spans="1:2">
       <c r="A106" s="2">
-        <v>46254.08333333334</v>
+        <v>46259.08333333334</v>
       </c>
       <c r="B106">
-        <v>462</v>
+        <v>482</v>
       </c>
     </row>
     <row r="107" spans="1:2">
       <c r="A107" s="2">
-        <v>46254.09375</v>
+        <v>46259.09375</v>
       </c>
       <c r="B107">
-        <v>461</v>
+        <v>476</v>
       </c>
     </row>
     <row r="108" spans="1:2">
       <c r="A108" s="2">
-        <v>46254.10416666666</v>
+        <v>46259.10416666666</v>
       </c>
       <c r="B108">
-        <v>462</v>
+        <v>474</v>
       </c>
     </row>
     <row r="109" spans="1:2">
       <c r="A109" s="2">
-        <v>46254.11458333334</v>
+        <v>46259.11458333334</v>
       </c>
       <c r="B109">
-        <v>462</v>
+        <v>475</v>
       </c>
     </row>
     <row r="110" spans="1:2">
       <c r="A110" s="2">
-        <v>46254.125</v>
+        <v>46259.125</v>
       </c>
       <c r="B110">
-        <v>395</v>
+        <v>403</v>
       </c>
     </row>
     <row r="111" spans="1:2">
       <c r="A111" s="2">
-        <v>46254.13541666666</v>
+        <v>46259.13541666666</v>
       </c>
       <c r="B111">
-        <v>385</v>
+        <v>424</v>
       </c>
     </row>
     <row r="112" spans="1:2">
       <c r="A112" s="2">
-        <v>46254.14583333334</v>
+        <v>46259.14583333334</v>
       </c>
       <c r="B112">
-        <v>385</v>
+        <v>424</v>
       </c>
     </row>
     <row r="113" spans="1:2">
       <c r="A113" s="2">
-        <v>46254.15625</v>
+        <v>46259.15625</v>
       </c>
       <c r="B113">
-        <v>387</v>
+        <v>424</v>
       </c>
     </row>
     <row r="114" spans="1:2">
       <c r="A114" s="2">
-        <v>46254.16666666666</v>
+        <v>46259.16666666666</v>
       </c>
       <c r="B114">
-        <v>468</v>
+        <v>445</v>
       </c>
     </row>
     <row r="115" spans="1:2">
       <c r="A115" s="2">
-        <v>46254.17708333334</v>
+        <v>46259.17708333334</v>
       </c>
       <c r="B115">
-        <v>469</v>
+        <v>447</v>
       </c>
     </row>
     <row r="116" spans="1:2">
       <c r="A116" s="2">
-        <v>46254.1875</v>
+        <v>46259.1875</v>
       </c>
       <c r="B116">
-        <v>470</v>
+        <v>447</v>
       </c>
     </row>
     <row r="117" spans="1:2">
       <c r="A117" s="2">
-        <v>46254.19791666666</v>
+        <v>46259.19791666666</v>
       </c>
       <c r="B117">
-        <v>470</v>
+        <v>448</v>
       </c>
     </row>
     <row r="118" spans="1:2">
       <c r="A118" s="2">
-        <v>46254.20833333334</v>
+        <v>46259.20833333334</v>
       </c>
       <c r="B118">
-        <v>500</v>
+        <v>554</v>
       </c>
     </row>
     <row r="119" spans="1:2">
       <c r="A119" s="2">
-        <v>46254.21875</v>
+        <v>46259.21875</v>
       </c>
       <c r="B119">
-        <v>502</v>
+        <v>567</v>
       </c>
     </row>
     <row r="120" spans="1:2">
       <c r="A120" s="2">
-        <v>46254.22916666666</v>
+        <v>46259.22916666666</v>
       </c>
       <c r="B120">
-        <v>503</v>
+        <v>574</v>
       </c>
     </row>
     <row r="121" spans="1:2">
       <c r="A121" s="2">
-        <v>46254.23958333334</v>
+        <v>46259.23958333334</v>
       </c>
       <c r="B121">
-        <v>500</v>
+        <v>575</v>
       </c>
     </row>
     <row r="122" spans="1:2">
       <c r="A122" s="2">
-        <v>46254.25</v>
+        <v>46259.25</v>
       </c>
       <c r="B122">
-        <v>511</v>
+        <v>565</v>
       </c>
     </row>
     <row r="123" spans="1:2">
       <c r="A123" s="2">
-        <v>46254.26041666666</v>
+        <v>46259.26041666666</v>
       </c>
       <c r="B123">
-        <v>516</v>
+        <v>559</v>
       </c>
     </row>
     <row r="124" spans="1:2">
       <c r="A124" s="2">
-        <v>46254.27083333334</v>
+        <v>46259.27083333334</v>
       </c>
       <c r="B124">
-        <v>515</v>
+        <v>559</v>
       </c>
     </row>
     <row r="125" spans="1:2">
       <c r="A125" s="2">
-        <v>46254.28125</v>
+        <v>46259.28125</v>
       </c>
       <c r="B125">
-        <v>514</v>
+        <v>561</v>
       </c>
     </row>
     <row r="126" spans="1:2">
       <c r="A126" s="2">
-        <v>46254.29166666666</v>
+        <v>46259.29166666666</v>
       </c>
       <c r="B126">
-        <v>509</v>
+        <v>539</v>
       </c>
     </row>
     <row r="127" spans="1:2">
       <c r="A127" s="2">
-        <v>46254.30208333334</v>
+        <v>46259.30208333334</v>
       </c>
       <c r="B127">
-        <v>508</v>
-      </c>
-    </row>
-    <row r="128" spans="1:2">
-      <c r="A128" s="2">
-        <v>46254.3125</v>
-      </c>
-      <c r="B128">
-        <v>506</v>
-      </c>
-    </row>
-    <row r="129" spans="1:2">
-      <c r="A129" s="2">
-        <v>46254.32291666666</v>
-      </c>
-      <c r="B129">
-        <v>504</v>
-      </c>
-    </row>
-    <row r="130" spans="1:2">
-      <c r="A130" s="2">
-        <v>46254.33333333334</v>
-      </c>
-      <c r="B130">
-        <v>476</v>
-      </c>
-    </row>
-    <row r="131" spans="1:2">
-      <c r="A131" s="2">
-        <v>46254.34375</v>
-      </c>
-      <c r="B131">
-        <v>517</v>
+        <v>528</v>
       </c>
     </row>
   </sheetData>

</xml_diff>